<commit_message>
Aggiornamento automatico del 13/09/2026 alle 19:03
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3826,8 +3826,12 @@
           <t>Monza</t>
         </is>
       </c>
-      <c r="G30" s="71" t="n"/>
-      <c r="H30" s="71" t="n"/>
+      <c r="G30" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I30" s="72">
         <f>IF(OR($G30="",$H30=""),"",IF($G30&gt;$H30,"1",IF($G30=$H30,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 13/09/2026 alle 21:23
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3874,8 +3874,12 @@
           <t>Bologna</t>
         </is>
       </c>
-      <c r="G31" s="71" t="n"/>
-      <c r="H31" s="71" t="n"/>
+      <c r="G31" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I31" s="72">
         <f>IF(OR($G31="",$H31=""),"",IF($G31&gt;$H31,"1",IF($G31=$H31,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 13/09/2026 alle 23:31
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3646,8 +3646,12 @@
           <t>Juventus</t>
         </is>
       </c>
-      <c r="G26" s="71" t="n"/>
-      <c r="H26" s="71" t="n"/>
+      <c r="G26" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I26" s="72">
         <f>IF(OR($G26="",$H26=""),"",IF($G26&gt;$H26,"1",IF($G26=$H26,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 14/09/2026 alle 21:55
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3742,8 +3742,12 @@
           <t>Roma</t>
         </is>
       </c>
-      <c r="G28" s="71" t="n"/>
-      <c r="H28" s="71" t="n"/>
+      <c r="G28" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I28" s="72">
         <f>IF(OR($G28="",$H28=""),"",IF($G28&gt;$H28,"1",IF($G28=$H28,"X","2")))</f>
         <v/>
@@ -3786,8 +3790,12 @@
           <t>Parma</t>
         </is>
       </c>
-      <c r="G29" s="71" t="n"/>
-      <c r="H29" s="71" t="n"/>
+      <c r="G29" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I29" s="72">
         <f>IF(OR($G29="",$H29=""),"",IF($G29&gt;$H29,"1",IF($G29=$H29,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 15/09/2026 alle 00:57
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3934,8 +3934,12 @@
           <t>Udinese</t>
         </is>
       </c>
-      <c r="G32" s="71" t="n"/>
-      <c r="H32" s="71" t="n"/>
+      <c r="G32" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H32" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I32" s="72">
         <f>IF(OR($G32="",$H32=""),"",IF($G32&gt;$H32,"1",IF($G32=$H32,"X","2")))</f>
         <v/>
@@ -4400,12 +4404,12 @@
       </c>
       <c r="C43" s="25" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="D43" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="E43" s="70" t="inlineStr">
@@ -4449,7 +4453,7 @@
       </c>
       <c r="D44" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="E44" s="70" t="inlineStr">
@@ -4493,7 +4497,7 @@
       </c>
       <c r="D45" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E45" s="70" t="inlineStr">
@@ -4532,12 +4536,12 @@
       </c>
       <c r="C46" s="25" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="D46" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E46" s="70" t="inlineStr">
@@ -4576,12 +4580,12 @@
       </c>
       <c r="C47" s="25" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="D47" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E47" s="70" t="inlineStr">
@@ -4625,7 +4629,7 @@
       </c>
       <c r="D48" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E48" s="70" t="inlineStr">
@@ -4669,7 +4673,7 @@
       </c>
       <c r="D49" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E49" s="70" t="inlineStr">
@@ -4708,12 +4712,12 @@
       </c>
       <c r="C50" s="25" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="E50" s="70" t="inlineStr">
@@ -4757,7 +4761,7 @@
       </c>
       <c r="D51" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E51" s="70" t="inlineStr">
@@ -4796,12 +4800,12 @@
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="D52" s="25" t="inlineStr">
         <is>
-          <t>da definire</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="E52" s="70" t="inlineStr">

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/09/2026 alle 21:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -7224,21 +7224,61 @@
         <f>IF(Partite!$F33="","",Partite!$F33)</f>
         <v/>
       </c>
-      <c r="E33" s="71" t="n"/>
-      <c r="F33" s="71" t="n"/>
-      <c r="G33" s="71" t="n"/>
-      <c r="H33" s="71" t="n"/>
-      <c r="I33" s="71" t="n"/>
-      <c r="J33" s="71" t="n"/>
-      <c r="K33" s="71" t="n"/>
-      <c r="L33" s="71" t="n"/>
-      <c r="M33" s="71" t="n"/>
-      <c r="N33" s="71" t="n"/>
-      <c r="O33" s="71" t="n"/>
-      <c r="P33" s="71" t="n"/>
-      <c r="Q33" s="71" t="n"/>
-      <c r="R33" s="71" t="n"/>
-      <c r="S33" s="71" t="n"/>
+      <c r="E33" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F33" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I33" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L33" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O33" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q33" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R33" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S33" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="74">
@@ -7257,21 +7297,61 @@
         <f>IF(Partite!$F34="","",Partite!$F34)</f>
         <v/>
       </c>
-      <c r="E34" s="71" t="n"/>
-      <c r="F34" s="71" t="n"/>
-      <c r="G34" s="71" t="n"/>
-      <c r="H34" s="71" t="n"/>
-      <c r="I34" s="71" t="n"/>
-      <c r="J34" s="71" t="n"/>
-      <c r="K34" s="71" t="n"/>
-      <c r="L34" s="71" t="n"/>
-      <c r="M34" s="71" t="n"/>
-      <c r="N34" s="71" t="n"/>
-      <c r="O34" s="71" t="n"/>
-      <c r="P34" s="71" t="n"/>
-      <c r="Q34" s="71" t="n"/>
-      <c r="R34" s="71" t="n"/>
-      <c r="S34" s="71" t="n"/>
+      <c r="E34" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F34" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O34" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S34" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="74">
@@ -7290,21 +7370,61 @@
         <f>IF(Partite!$F35="","",Partite!$F35)</f>
         <v/>
       </c>
-      <c r="E35" s="71" t="n"/>
-      <c r="F35" s="71" t="n"/>
-      <c r="G35" s="71" t="n"/>
-      <c r="H35" s="71" t="n"/>
-      <c r="I35" s="71" t="n"/>
-      <c r="J35" s="71" t="n"/>
-      <c r="K35" s="71" t="n"/>
-      <c r="L35" s="71" t="n"/>
-      <c r="M35" s="71" t="n"/>
-      <c r="N35" s="71" t="n"/>
-      <c r="O35" s="71" t="n"/>
-      <c r="P35" s="71" t="n"/>
-      <c r="Q35" s="71" t="n"/>
-      <c r="R35" s="71" t="n"/>
-      <c r="S35" s="71" t="n"/>
+      <c r="E35" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F35" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I35" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L35" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O35" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P35" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="74">
@@ -7323,21 +7443,61 @@
         <f>IF(Partite!$F36="","",Partite!$F36)</f>
         <v/>
       </c>
-      <c r="E36" s="71" t="n"/>
-      <c r="F36" s="71" t="n"/>
-      <c r="G36" s="71" t="n"/>
-      <c r="H36" s="71" t="n"/>
-      <c r="I36" s="71" t="n"/>
-      <c r="J36" s="71" t="n"/>
-      <c r="K36" s="71" t="n"/>
-      <c r="L36" s="71" t="n"/>
-      <c r="M36" s="71" t="n"/>
-      <c r="N36" s="71" t="n"/>
-      <c r="O36" s="71" t="n"/>
-      <c r="P36" s="71" t="n"/>
-      <c r="Q36" s="71" t="n"/>
-      <c r="R36" s="71" t="n"/>
-      <c r="S36" s="71" t="n"/>
+      <c r="E36" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F36" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I36" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J36" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L36" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N36" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O36" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P36" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q36" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R36" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="74">
@@ -7356,21 +7516,61 @@
         <f>IF(Partite!$F37="","",Partite!$F37)</f>
         <v/>
       </c>
-      <c r="E37" s="71" t="n"/>
-      <c r="F37" s="71" t="n"/>
-      <c r="G37" s="71" t="n"/>
-      <c r="H37" s="71" t="n"/>
-      <c r="I37" s="71" t="n"/>
-      <c r="J37" s="71" t="n"/>
-      <c r="K37" s="71" t="n"/>
-      <c r="L37" s="71" t="n"/>
-      <c r="M37" s="71" t="n"/>
-      <c r="N37" s="71" t="n"/>
-      <c r="O37" s="71" t="n"/>
-      <c r="P37" s="71" t="n"/>
-      <c r="Q37" s="71" t="n"/>
-      <c r="R37" s="71" t="n"/>
-      <c r="S37" s="71" t="n"/>
+      <c r="E37" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F37" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I37" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L37" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O37" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q37" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R37" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="74">
@@ -7389,21 +7589,61 @@
         <f>IF(Partite!$F38="","",Partite!$F38)</f>
         <v/>
       </c>
-      <c r="E38" s="71" t="n"/>
-      <c r="F38" s="71" t="n"/>
-      <c r="G38" s="71" t="n"/>
-      <c r="H38" s="71" t="n"/>
-      <c r="I38" s="71" t="n"/>
-      <c r="J38" s="71" t="n"/>
-      <c r="K38" s="71" t="n"/>
-      <c r="L38" s="71" t="n"/>
-      <c r="M38" s="71" t="n"/>
-      <c r="N38" s="71" t="n"/>
-      <c r="O38" s="71" t="n"/>
-      <c r="P38" s="71" t="n"/>
-      <c r="Q38" s="71" t="n"/>
-      <c r="R38" s="71" t="n"/>
-      <c r="S38" s="71" t="n"/>
+      <c r="E38" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F38" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L38" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N38" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S38" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="74">
@@ -7422,21 +7662,61 @@
         <f>IF(Partite!$F39="","",Partite!$F39)</f>
         <v/>
       </c>
-      <c r="E39" s="71" t="n"/>
-      <c r="F39" s="71" t="n"/>
-      <c r="G39" s="71" t="n"/>
-      <c r="H39" s="71" t="n"/>
-      <c r="I39" s="71" t="n"/>
-      <c r="J39" s="71" t="n"/>
-      <c r="K39" s="71" t="n"/>
-      <c r="L39" s="71" t="n"/>
-      <c r="M39" s="71" t="n"/>
-      <c r="N39" s="71" t="n"/>
-      <c r="O39" s="71" t="n"/>
-      <c r="P39" s="71" t="n"/>
-      <c r="Q39" s="71" t="n"/>
-      <c r="R39" s="71" t="n"/>
-      <c r="S39" s="71" t="n"/>
+      <c r="E39" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F39" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H39" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I39" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K39" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L39" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N39" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O39" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q39" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R39" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" s="71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="74">
@@ -7455,21 +7735,61 @@
         <f>IF(Partite!$F40="","",Partite!$F40)</f>
         <v/>
       </c>
-      <c r="E40" s="71" t="n"/>
-      <c r="F40" s="71" t="n"/>
-      <c r="G40" s="71" t="n"/>
-      <c r="H40" s="71" t="n"/>
-      <c r="I40" s="71" t="n"/>
-      <c r="J40" s="71" t="n"/>
-      <c r="K40" s="71" t="n"/>
-      <c r="L40" s="71" t="n"/>
-      <c r="M40" s="71" t="n"/>
-      <c r="N40" s="71" t="n"/>
-      <c r="O40" s="71" t="n"/>
-      <c r="P40" s="71" t="n"/>
-      <c r="Q40" s="71" t="n"/>
-      <c r="R40" s="71" t="n"/>
-      <c r="S40" s="71" t="n"/>
+      <c r="E40" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I40" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R40" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="74">
@@ -7488,21 +7808,61 @@
         <f>IF(Partite!$F41="","",Partite!$F41)</f>
         <v/>
       </c>
-      <c r="E41" s="71" t="n"/>
-      <c r="F41" s="71" t="n"/>
-      <c r="G41" s="71" t="n"/>
-      <c r="H41" s="71" t="n"/>
-      <c r="I41" s="71" t="n"/>
-      <c r="J41" s="71" t="n"/>
-      <c r="K41" s="71" t="n"/>
-      <c r="L41" s="71" t="n"/>
-      <c r="M41" s="71" t="n"/>
-      <c r="N41" s="71" t="n"/>
-      <c r="O41" s="71" t="n"/>
-      <c r="P41" s="71" t="n"/>
-      <c r="Q41" s="71" t="n"/>
-      <c r="R41" s="71" t="n"/>
-      <c r="S41" s="71" t="n"/>
+      <c r="E41" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F41" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J41" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N41" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q41" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S41" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="74">
@@ -7521,21 +7881,61 @@
         <f>IF(Partite!$F42="","",Partite!$F42)</f>
         <v/>
       </c>
-      <c r="E42" s="71" t="n"/>
-      <c r="F42" s="71" t="n"/>
-      <c r="G42" s="71" t="n"/>
-      <c r="H42" s="71" t="n"/>
-      <c r="I42" s="71" t="n"/>
-      <c r="J42" s="71" t="n"/>
-      <c r="K42" s="71" t="n"/>
-      <c r="L42" s="71" t="n"/>
-      <c r="M42" s="71" t="n"/>
-      <c r="N42" s="71" t="n"/>
-      <c r="O42" s="71" t="n"/>
-      <c r="P42" s="71" t="n"/>
-      <c r="Q42" s="71" t="n"/>
-      <c r="R42" s="71" t="n"/>
-      <c r="S42" s="71" t="n"/>
+      <c r="E42" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I42" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L42" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M42" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O42" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P42" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="69">

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/09/2026 alle 23:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3982,8 +3982,12 @@
           <t>Sassuolo</t>
         </is>
       </c>
-      <c r="G33" s="71" t="n"/>
-      <c r="H33" s="71" t="n"/>
+      <c r="G33" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I33" s="76">
         <f>IF(OR($G33="",$H33=""),"",IF($G33&gt;$H33,"1",IF($G33=$H33,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 19/09/2026 alle 18:07
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4030,8 +4030,12 @@
           <t>Torino</t>
         </is>
       </c>
-      <c r="G34" s="71" t="n"/>
-      <c r="H34" s="71" t="n"/>
+      <c r="G34" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I34" s="76">
         <f>IF(OR($G34="",$H34=""),"",IF($G34&gt;$H34,"1",IF($G34=$H34,"X","2")))</f>
         <v/>
@@ -4074,8 +4078,12 @@
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="G35" s="71" t="n"/>
-      <c r="H35" s="71" t="n"/>
+      <c r="G35" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I35" s="76">
         <f>IF(OR($G35="",$H35=""),"",IF($G35&gt;$H35,"1",IF($G35=$H35,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 19/09/2026 alle 20:35
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4126,8 +4126,12 @@
           <t>Inter</t>
         </is>
       </c>
-      <c r="G36" s="71" t="n"/>
-      <c r="H36" s="71" t="n"/>
+      <c r="G36" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I36" s="76">
         <f>IF(OR($G36="",$H36=""),"",IF($G36&gt;$H36,"1",IF($G36=$H36,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 19/09/2026 alle 22:58
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4174,8 +4174,12 @@
           <t>Lazio</t>
         </is>
       </c>
-      <c r="G37" s="71" t="n"/>
-      <c r="H37" s="71" t="n"/>
+      <c r="G37" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I37" s="76">
         <f>IF(OR($G37="",$H37=""),"",IF($G37&gt;$H37,"1",IF($G37=$H37,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 14:57
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -1595,11 +1595,11 @@
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$7)+COUNTIF(Punti!$D$3:$D$52,Config!$D$6)+COUNTIF(Punti!$D$3:$D$52,Config!$D$10)+COUNTIF(Punti!$D$3:$D$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$7)+COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$6)+COUNTIF(Punti!$D$3:$D$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
@@ -1629,11 +1629,11 @@
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$7)+COUNTIF(Punti!$E$3:$E$52,Config!$D$6)+COUNTIF(Punti!$E$3:$E$52,Config!$D$10)+COUNTIF(Punti!$E$3:$E$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$7)+COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$6)+COUNTIF(Punti!$E$3:$E$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
@@ -1663,11 +1663,11 @@
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$7)+COUNTIF(Punti!$F$3:$F$52,Config!$D$6)+COUNTIF(Punti!$F$3:$F$52,Config!$D$10)+COUNTIF(Punti!$F$3:$F$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$7)+COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$6)+COUNTIF(Punti!$F$3:$F$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
@@ -1697,11 +1697,11 @@
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$7)+COUNTIF(Punti!$G$3:$G$52,Config!$D$6)+COUNTIF(Punti!$G$3:$G$52,Config!$D$10)+COUNTIF(Punti!$G$3:$G$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$7)+COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$6)+COUNTIF(Punti!$G$3:$G$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
@@ -1731,11 +1731,11 @@
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$7)+COUNTIF(Punti!$H$3:$H$52,Config!$D$6)+COUNTIF(Punti!$H$3:$H$52,Config!$D$10)+COUNTIF(Punti!$H$3:$H$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$7)+COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$6)+COUNTIF(Punti!$H$3:$H$52,Config!$D$9)</f>
+        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
@@ -4222,8 +4222,12 @@
           <t>Napoli</t>
         </is>
       </c>
-      <c r="G38" s="71" t="n"/>
-      <c r="H38" s="71" t="n"/>
+      <c r="G38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I38" s="76">
         <f>IF(OR($G38="",$H38=""),"",IF($G38&gt;$H38,"1",IF($G38=$H38,"X","2")))</f>
         <v/>
@@ -8313,7 +8317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T52"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8329,11 +8333,6 @@
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="9" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -8351,7 +8350,7 @@
       <c r="H1" s="2" t="n"/>
       <c r="J1" s="35" t="inlineStr">
         <is>
-          <t>servizio: a sinistra il segno effettivo (dichiarato, o dedotto dal punteggio), a destra il punteggio scritto. Servono a vedere chi era da solo.</t>
+          <t>servizio: il segno effettivo di ognuno, dichiarato o dedotto dal punteggio.</t>
         </is>
       </c>
     </row>
@@ -8408,26 +8407,6 @@
         <v/>
       </c>
       <c r="N2" s="60">
-        <f>Config!$A$10</f>
-        <v/>
-      </c>
-      <c r="P2" s="60">
-        <f>Config!$A$6</f>
-        <v/>
-      </c>
-      <c r="Q2" s="60">
-        <f>Config!$A$7</f>
-        <v/>
-      </c>
-      <c r="R2" s="60">
-        <f>Config!$A$8</f>
-        <v/>
-      </c>
-      <c r="S2" s="60">
-        <f>Config!$A$9</f>
-        <v/>
-      </c>
-      <c r="T2" s="60">
         <f>Config!$A$10</f>
         <v/>
       </c>
@@ -8446,23 +8425,23 @@
         <v/>
       </c>
       <c r="D3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$F3&lt;&gt;"",Pronostici!$G3&lt;&gt;"",Pronostici!$F3=Partite!$G3,Pronostici!$G3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$P3)=1),Config!$D$9,Config!$D$6),IF(AND($J3&lt;&gt;"",$J3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$J3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$F3&lt;&gt;"",Pronostici!$G3&lt;&gt;"",Pronostici!$F3=Partite!$G3,Pronostici!$G3=Partite!$H3),Config!$D$6,IF(AND($J3&lt;&gt;"",$J3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$I3&lt;&gt;"",Pronostici!$J3&lt;&gt;"",Pronostici!$I3=Partite!$G3,Pronostici!$J3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$Q3)=1),Config!$D$9,Config!$D$6),IF(AND($K3&lt;&gt;"",$K3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$K3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$I3&lt;&gt;"",Pronostici!$J3&lt;&gt;"",Pronostici!$I3=Partite!$G3,Pronostici!$J3=Partite!$H3),Config!$D$6,IF(AND($K3&lt;&gt;"",$K3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$L3&lt;&gt;"",Pronostici!$M3&lt;&gt;"",Pronostici!$L3=Partite!$G3,Pronostici!$M3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$R3)=1),Config!$D$9,Config!$D$6),IF(AND($L3&lt;&gt;"",$L3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$L3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$L3&lt;&gt;"",Pronostici!$M3&lt;&gt;"",Pronostici!$L3=Partite!$G3,Pronostici!$M3=Partite!$H3),Config!$D$6,IF(AND($L3&lt;&gt;"",$L3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$O3&lt;&gt;"",Pronostici!$P3&lt;&gt;"",Pronostici!$O3=Partite!$G3,Pronostici!$P3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$S3)=1),Config!$D$9,Config!$D$6),IF(AND($M3&lt;&gt;"",$M3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$M3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$O3&lt;&gt;"",Pronostici!$P3&lt;&gt;"",Pronostici!$O3=Partite!$G3,Pronostici!$P3=Partite!$H3),Config!$D$6,IF(AND($M3&lt;&gt;"",$M3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$R3&lt;&gt;"",Pronostici!$S3&lt;&gt;"",Pronostici!$R3=Partite!$G3,Pronostici!$S3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$T3)=1),Config!$D$9,Config!$D$6),IF(AND($N3&lt;&gt;"",$N3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$N3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$R3&lt;&gt;"",Pronostici!$S3&lt;&gt;"",Pronostici!$R3=Partite!$G3,Pronostici!$S3=Partite!$H3),Config!$D$6,IF(AND($N3&lt;&gt;"",$N3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J3" s="63">
@@ -8483,26 +8462,6 @@
       </c>
       <c r="N3" s="63">
         <f>IF(Pronostici!$Q3&lt;&gt;"",UPPER(Pronostici!$Q3),IF(OR(Pronostici!$R3="",Pronostici!$S3=""),"",IF(Pronostici!$R3&gt;Pronostici!$S3,"1",IF(Pronostici!$R3=Pronostici!$S3,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P3" s="63">
-        <f>IF(OR(Pronostici!$F3="",Pronostici!$G3=""),"",Pronostici!$F3&amp;" a "&amp;Pronostici!$G3)</f>
-        <v/>
-      </c>
-      <c r="Q3" s="63">
-        <f>IF(OR(Pronostici!$I3="",Pronostici!$J3=""),"",Pronostici!$I3&amp;" a "&amp;Pronostici!$J3)</f>
-        <v/>
-      </c>
-      <c r="R3" s="63">
-        <f>IF(OR(Pronostici!$L3="",Pronostici!$M3=""),"",Pronostici!$L3&amp;" a "&amp;Pronostici!$M3)</f>
-        <v/>
-      </c>
-      <c r="S3" s="63">
-        <f>IF(OR(Pronostici!$O3="",Pronostici!$P3=""),"",Pronostici!$O3&amp;" a "&amp;Pronostici!$P3)</f>
-        <v/>
-      </c>
-      <c r="T3" s="63">
-        <f>IF(OR(Pronostici!$R3="",Pronostici!$S3=""),"",Pronostici!$R3&amp;" a "&amp;Pronostici!$S3)</f>
         <v/>
       </c>
     </row>
@@ -8520,23 +8479,23 @@
         <v/>
       </c>
       <c r="D4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$F4&lt;&gt;"",Pronostici!$G4&lt;&gt;"",Pronostici!$F4=Partite!$G4,Pronostici!$G4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$P4)=1),Config!$D$9,Config!$D$6),IF(AND($J4&lt;&gt;"",$J4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$J4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$F4&lt;&gt;"",Pronostici!$G4&lt;&gt;"",Pronostici!$F4=Partite!$G4,Pronostici!$G4=Partite!$H4),Config!$D$6,IF(AND($J4&lt;&gt;"",$J4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$I4&lt;&gt;"",Pronostici!$J4&lt;&gt;"",Pronostici!$I4=Partite!$G4,Pronostici!$J4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$Q4)=1),Config!$D$9,Config!$D$6),IF(AND($K4&lt;&gt;"",$K4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$K4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$I4&lt;&gt;"",Pronostici!$J4&lt;&gt;"",Pronostici!$I4=Partite!$G4,Pronostici!$J4=Partite!$H4),Config!$D$6,IF(AND($K4&lt;&gt;"",$K4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$L4&lt;&gt;"",Pronostici!$M4&lt;&gt;"",Pronostici!$L4=Partite!$G4,Pronostici!$M4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$R4)=1),Config!$D$9,Config!$D$6),IF(AND($L4&lt;&gt;"",$L4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$L4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$L4&lt;&gt;"",Pronostici!$M4&lt;&gt;"",Pronostici!$L4=Partite!$G4,Pronostici!$M4=Partite!$H4),Config!$D$6,IF(AND($L4&lt;&gt;"",$L4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$O4&lt;&gt;"",Pronostici!$P4&lt;&gt;"",Pronostici!$O4=Partite!$G4,Pronostici!$P4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$S4)=1),Config!$D$9,Config!$D$6),IF(AND($M4&lt;&gt;"",$M4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$M4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$O4&lt;&gt;"",Pronostici!$P4&lt;&gt;"",Pronostici!$O4=Partite!$G4,Pronostici!$P4=Partite!$H4),Config!$D$6,IF(AND($M4&lt;&gt;"",$M4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$R4&lt;&gt;"",Pronostici!$S4&lt;&gt;"",Pronostici!$R4=Partite!$G4,Pronostici!$S4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$T4)=1),Config!$D$9,Config!$D$6),IF(AND($N4&lt;&gt;"",$N4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$N4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$R4&lt;&gt;"",Pronostici!$S4&lt;&gt;"",Pronostici!$R4=Partite!$G4,Pronostici!$S4=Partite!$H4),Config!$D$6,IF(AND($N4&lt;&gt;"",$N4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J4" s="63">
@@ -8557,26 +8516,6 @@
       </c>
       <c r="N4" s="63">
         <f>IF(Pronostici!$Q4&lt;&gt;"",UPPER(Pronostici!$Q4),IF(OR(Pronostici!$R4="",Pronostici!$S4=""),"",IF(Pronostici!$R4&gt;Pronostici!$S4,"1",IF(Pronostici!$R4=Pronostici!$S4,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P4" s="63">
-        <f>IF(OR(Pronostici!$F4="",Pronostici!$G4=""),"",Pronostici!$F4&amp;" a "&amp;Pronostici!$G4)</f>
-        <v/>
-      </c>
-      <c r="Q4" s="63">
-        <f>IF(OR(Pronostici!$I4="",Pronostici!$J4=""),"",Pronostici!$I4&amp;" a "&amp;Pronostici!$J4)</f>
-        <v/>
-      </c>
-      <c r="R4" s="63">
-        <f>IF(OR(Pronostici!$L4="",Pronostici!$M4=""),"",Pronostici!$L4&amp;" a "&amp;Pronostici!$M4)</f>
-        <v/>
-      </c>
-      <c r="S4" s="63">
-        <f>IF(OR(Pronostici!$O4="",Pronostici!$P4=""),"",Pronostici!$O4&amp;" a "&amp;Pronostici!$P4)</f>
-        <v/>
-      </c>
-      <c r="T4" s="63">
-        <f>IF(OR(Pronostici!$R4="",Pronostici!$S4=""),"",Pronostici!$R4&amp;" a "&amp;Pronostici!$S4)</f>
         <v/>
       </c>
     </row>
@@ -8594,23 +8533,23 @@
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$F5&lt;&gt;"",Pronostici!$G5&lt;&gt;"",Pronostici!$F5=Partite!$G5,Pronostici!$G5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$P5)=1),Config!$D$9,Config!$D$6),IF(AND($J5&lt;&gt;"",$J5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$J5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$F5&lt;&gt;"",Pronostici!$G5&lt;&gt;"",Pronostici!$F5=Partite!$G5,Pronostici!$G5=Partite!$H5),Config!$D$6,IF(AND($J5&lt;&gt;"",$J5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$I5&lt;&gt;"",Pronostici!$J5&lt;&gt;"",Pronostici!$I5=Partite!$G5,Pronostici!$J5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$Q5)=1),Config!$D$9,Config!$D$6),IF(AND($K5&lt;&gt;"",$K5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$K5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$I5&lt;&gt;"",Pronostici!$J5&lt;&gt;"",Pronostici!$I5=Partite!$G5,Pronostici!$J5=Partite!$H5),Config!$D$6,IF(AND($K5&lt;&gt;"",$K5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$L5&lt;&gt;"",Pronostici!$M5&lt;&gt;"",Pronostici!$L5=Partite!$G5,Pronostici!$M5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$R5)=1),Config!$D$9,Config!$D$6),IF(AND($L5&lt;&gt;"",$L5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$L5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$L5&lt;&gt;"",Pronostici!$M5&lt;&gt;"",Pronostici!$L5=Partite!$G5,Pronostici!$M5=Partite!$H5),Config!$D$6,IF(AND($L5&lt;&gt;"",$L5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$O5&lt;&gt;"",Pronostici!$P5&lt;&gt;"",Pronostici!$O5=Partite!$G5,Pronostici!$P5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$S5)=1),Config!$D$9,Config!$D$6),IF(AND($M5&lt;&gt;"",$M5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$M5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$O5&lt;&gt;"",Pronostici!$P5&lt;&gt;"",Pronostici!$O5=Partite!$G5,Pronostici!$P5=Partite!$H5),Config!$D$6,IF(AND($M5&lt;&gt;"",$M5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$R5&lt;&gt;"",Pronostici!$S5&lt;&gt;"",Pronostici!$R5=Partite!$G5,Pronostici!$S5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$T5)=1),Config!$D$9,Config!$D$6),IF(AND($N5&lt;&gt;"",$N5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$N5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$R5&lt;&gt;"",Pronostici!$S5&lt;&gt;"",Pronostici!$R5=Partite!$G5,Pronostici!$S5=Partite!$H5),Config!$D$6,IF(AND($N5&lt;&gt;"",$N5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J5" s="63">
@@ -8631,26 +8570,6 @@
       </c>
       <c r="N5" s="63">
         <f>IF(Pronostici!$Q5&lt;&gt;"",UPPER(Pronostici!$Q5),IF(OR(Pronostici!$R5="",Pronostici!$S5=""),"",IF(Pronostici!$R5&gt;Pronostici!$S5,"1",IF(Pronostici!$R5=Pronostici!$S5,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P5" s="63">
-        <f>IF(OR(Pronostici!$F5="",Pronostici!$G5=""),"",Pronostici!$F5&amp;" a "&amp;Pronostici!$G5)</f>
-        <v/>
-      </c>
-      <c r="Q5" s="63">
-        <f>IF(OR(Pronostici!$I5="",Pronostici!$J5=""),"",Pronostici!$I5&amp;" a "&amp;Pronostici!$J5)</f>
-        <v/>
-      </c>
-      <c r="R5" s="63">
-        <f>IF(OR(Pronostici!$L5="",Pronostici!$M5=""),"",Pronostici!$L5&amp;" a "&amp;Pronostici!$M5)</f>
-        <v/>
-      </c>
-      <c r="S5" s="63">
-        <f>IF(OR(Pronostici!$O5="",Pronostici!$P5=""),"",Pronostici!$O5&amp;" a "&amp;Pronostici!$P5)</f>
-        <v/>
-      </c>
-      <c r="T5" s="63">
-        <f>IF(OR(Pronostici!$R5="",Pronostici!$S5=""),"",Pronostici!$R5&amp;" a "&amp;Pronostici!$S5)</f>
         <v/>
       </c>
     </row>
@@ -8668,23 +8587,23 @@
         <v/>
       </c>
       <c r="D6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$F6&lt;&gt;"",Pronostici!$G6&lt;&gt;"",Pronostici!$F6=Partite!$G6,Pronostici!$G6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$P6)=1),Config!$D$9,Config!$D$6),IF(AND($J6&lt;&gt;"",$J6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$J6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$F6&lt;&gt;"",Pronostici!$G6&lt;&gt;"",Pronostici!$F6=Partite!$G6,Pronostici!$G6=Partite!$H6),Config!$D$6,IF(AND($J6&lt;&gt;"",$J6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$I6&lt;&gt;"",Pronostici!$J6&lt;&gt;"",Pronostici!$I6=Partite!$G6,Pronostici!$J6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$Q6)=1),Config!$D$9,Config!$D$6),IF(AND($K6&lt;&gt;"",$K6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$K6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$I6&lt;&gt;"",Pronostici!$J6&lt;&gt;"",Pronostici!$I6=Partite!$G6,Pronostici!$J6=Partite!$H6),Config!$D$6,IF(AND($K6&lt;&gt;"",$K6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$L6&lt;&gt;"",Pronostici!$M6&lt;&gt;"",Pronostici!$L6=Partite!$G6,Pronostici!$M6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$R6)=1),Config!$D$9,Config!$D$6),IF(AND($L6&lt;&gt;"",$L6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$L6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$L6&lt;&gt;"",Pronostici!$M6&lt;&gt;"",Pronostici!$L6=Partite!$G6,Pronostici!$M6=Partite!$H6),Config!$D$6,IF(AND($L6&lt;&gt;"",$L6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$O6&lt;&gt;"",Pronostici!$P6&lt;&gt;"",Pronostici!$O6=Partite!$G6,Pronostici!$P6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$S6)=1),Config!$D$9,Config!$D$6),IF(AND($M6&lt;&gt;"",$M6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$M6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$O6&lt;&gt;"",Pronostici!$P6&lt;&gt;"",Pronostici!$O6=Partite!$G6,Pronostici!$P6=Partite!$H6),Config!$D$6,IF(AND($M6&lt;&gt;"",$M6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$R6&lt;&gt;"",Pronostici!$S6&lt;&gt;"",Pronostici!$R6=Partite!$G6,Pronostici!$S6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$T6)=1),Config!$D$9,Config!$D$6),IF(AND($N6&lt;&gt;"",$N6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$N6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$R6&lt;&gt;"",Pronostici!$S6&lt;&gt;"",Pronostici!$R6=Partite!$G6,Pronostici!$S6=Partite!$H6),Config!$D$6,IF(AND($N6&lt;&gt;"",$N6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J6" s="63">
@@ -8705,26 +8624,6 @@
       </c>
       <c r="N6" s="63">
         <f>IF(Pronostici!$Q6&lt;&gt;"",UPPER(Pronostici!$Q6),IF(OR(Pronostici!$R6="",Pronostici!$S6=""),"",IF(Pronostici!$R6&gt;Pronostici!$S6,"1",IF(Pronostici!$R6=Pronostici!$S6,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P6" s="63">
-        <f>IF(OR(Pronostici!$F6="",Pronostici!$G6=""),"",Pronostici!$F6&amp;" a "&amp;Pronostici!$G6)</f>
-        <v/>
-      </c>
-      <c r="Q6" s="63">
-        <f>IF(OR(Pronostici!$I6="",Pronostici!$J6=""),"",Pronostici!$I6&amp;" a "&amp;Pronostici!$J6)</f>
-        <v/>
-      </c>
-      <c r="R6" s="63">
-        <f>IF(OR(Pronostici!$L6="",Pronostici!$M6=""),"",Pronostici!$L6&amp;" a "&amp;Pronostici!$M6)</f>
-        <v/>
-      </c>
-      <c r="S6" s="63">
-        <f>IF(OR(Pronostici!$O6="",Pronostici!$P6=""),"",Pronostici!$O6&amp;" a "&amp;Pronostici!$P6)</f>
-        <v/>
-      </c>
-      <c r="T6" s="63">
-        <f>IF(OR(Pronostici!$R6="",Pronostici!$S6=""),"",Pronostici!$R6&amp;" a "&amp;Pronostici!$S6)</f>
         <v/>
       </c>
     </row>
@@ -8742,23 +8641,23 @@
         <v/>
       </c>
       <c r="D7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$F7&lt;&gt;"",Pronostici!$G7&lt;&gt;"",Pronostici!$F7=Partite!$G7,Pronostici!$G7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$P7)=1),Config!$D$9,Config!$D$6),IF(AND($J7&lt;&gt;"",$J7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$J7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$F7&lt;&gt;"",Pronostici!$G7&lt;&gt;"",Pronostici!$F7=Partite!$G7,Pronostici!$G7=Partite!$H7),Config!$D$6,IF(AND($J7&lt;&gt;"",$J7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$I7&lt;&gt;"",Pronostici!$J7&lt;&gt;"",Pronostici!$I7=Partite!$G7,Pronostici!$J7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$Q7)=1),Config!$D$9,Config!$D$6),IF(AND($K7&lt;&gt;"",$K7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$K7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$I7&lt;&gt;"",Pronostici!$J7&lt;&gt;"",Pronostici!$I7=Partite!$G7,Pronostici!$J7=Partite!$H7),Config!$D$6,IF(AND($K7&lt;&gt;"",$K7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$L7&lt;&gt;"",Pronostici!$M7&lt;&gt;"",Pronostici!$L7=Partite!$G7,Pronostici!$M7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$R7)=1),Config!$D$9,Config!$D$6),IF(AND($L7&lt;&gt;"",$L7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$L7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$L7&lt;&gt;"",Pronostici!$M7&lt;&gt;"",Pronostici!$L7=Partite!$G7,Pronostici!$M7=Partite!$H7),Config!$D$6,IF(AND($L7&lt;&gt;"",$L7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$O7&lt;&gt;"",Pronostici!$P7&lt;&gt;"",Pronostici!$O7=Partite!$G7,Pronostici!$P7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$S7)=1),Config!$D$9,Config!$D$6),IF(AND($M7&lt;&gt;"",$M7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$M7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$O7&lt;&gt;"",Pronostici!$P7&lt;&gt;"",Pronostici!$O7=Partite!$G7,Pronostici!$P7=Partite!$H7),Config!$D$6,IF(AND($M7&lt;&gt;"",$M7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$R7&lt;&gt;"",Pronostici!$S7&lt;&gt;"",Pronostici!$R7=Partite!$G7,Pronostici!$S7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$T7)=1),Config!$D$9,Config!$D$6),IF(AND($N7&lt;&gt;"",$N7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$N7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$R7&lt;&gt;"",Pronostici!$S7&lt;&gt;"",Pronostici!$R7=Partite!$G7,Pronostici!$S7=Partite!$H7),Config!$D$6,IF(AND($N7&lt;&gt;"",$N7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J7" s="63">
@@ -8779,26 +8678,6 @@
       </c>
       <c r="N7" s="63">
         <f>IF(Pronostici!$Q7&lt;&gt;"",UPPER(Pronostici!$Q7),IF(OR(Pronostici!$R7="",Pronostici!$S7=""),"",IF(Pronostici!$R7&gt;Pronostici!$S7,"1",IF(Pronostici!$R7=Pronostici!$S7,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P7" s="63">
-        <f>IF(OR(Pronostici!$F7="",Pronostici!$G7=""),"",Pronostici!$F7&amp;" a "&amp;Pronostici!$G7)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="63">
-        <f>IF(OR(Pronostici!$I7="",Pronostici!$J7=""),"",Pronostici!$I7&amp;" a "&amp;Pronostici!$J7)</f>
-        <v/>
-      </c>
-      <c r="R7" s="63">
-        <f>IF(OR(Pronostici!$L7="",Pronostici!$M7=""),"",Pronostici!$L7&amp;" a "&amp;Pronostici!$M7)</f>
-        <v/>
-      </c>
-      <c r="S7" s="63">
-        <f>IF(OR(Pronostici!$O7="",Pronostici!$P7=""),"",Pronostici!$O7&amp;" a "&amp;Pronostici!$P7)</f>
-        <v/>
-      </c>
-      <c r="T7" s="63">
-        <f>IF(OR(Pronostici!$R7="",Pronostici!$S7=""),"",Pronostici!$R7&amp;" a "&amp;Pronostici!$S7)</f>
         <v/>
       </c>
     </row>
@@ -8816,23 +8695,23 @@
         <v/>
       </c>
       <c r="D8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$F8&lt;&gt;"",Pronostici!$G8&lt;&gt;"",Pronostici!$F8=Partite!$G8,Pronostici!$G8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$P8)=1),Config!$D$9,Config!$D$6),IF(AND($J8&lt;&gt;"",$J8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$J8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$F8&lt;&gt;"",Pronostici!$G8&lt;&gt;"",Pronostici!$F8=Partite!$G8,Pronostici!$G8=Partite!$H8),Config!$D$6,IF(AND($J8&lt;&gt;"",$J8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$I8&lt;&gt;"",Pronostici!$J8&lt;&gt;"",Pronostici!$I8=Partite!$G8,Pronostici!$J8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$Q8)=1),Config!$D$9,Config!$D$6),IF(AND($K8&lt;&gt;"",$K8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$K8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$I8&lt;&gt;"",Pronostici!$J8&lt;&gt;"",Pronostici!$I8=Partite!$G8,Pronostici!$J8=Partite!$H8),Config!$D$6,IF(AND($K8&lt;&gt;"",$K8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$L8&lt;&gt;"",Pronostici!$M8&lt;&gt;"",Pronostici!$L8=Partite!$G8,Pronostici!$M8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$R8)=1),Config!$D$9,Config!$D$6),IF(AND($L8&lt;&gt;"",$L8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$L8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$L8&lt;&gt;"",Pronostici!$M8&lt;&gt;"",Pronostici!$L8=Partite!$G8,Pronostici!$M8=Partite!$H8),Config!$D$6,IF(AND($L8&lt;&gt;"",$L8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$O8&lt;&gt;"",Pronostici!$P8&lt;&gt;"",Pronostici!$O8=Partite!$G8,Pronostici!$P8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$S8)=1),Config!$D$9,Config!$D$6),IF(AND($M8&lt;&gt;"",$M8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$M8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$O8&lt;&gt;"",Pronostici!$P8&lt;&gt;"",Pronostici!$O8=Partite!$G8,Pronostici!$P8=Partite!$H8),Config!$D$6,IF(AND($M8&lt;&gt;"",$M8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$R8&lt;&gt;"",Pronostici!$S8&lt;&gt;"",Pronostici!$R8=Partite!$G8,Pronostici!$S8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$T8)=1),Config!$D$9,Config!$D$6),IF(AND($N8&lt;&gt;"",$N8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$N8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$R8&lt;&gt;"",Pronostici!$S8&lt;&gt;"",Pronostici!$R8=Partite!$G8,Pronostici!$S8=Partite!$H8),Config!$D$6,IF(AND($N8&lt;&gt;"",$N8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J8" s="63">
@@ -8853,26 +8732,6 @@
       </c>
       <c r="N8" s="63">
         <f>IF(Pronostici!$Q8&lt;&gt;"",UPPER(Pronostici!$Q8),IF(OR(Pronostici!$R8="",Pronostici!$S8=""),"",IF(Pronostici!$R8&gt;Pronostici!$S8,"1",IF(Pronostici!$R8=Pronostici!$S8,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P8" s="63">
-        <f>IF(OR(Pronostici!$F8="",Pronostici!$G8=""),"",Pronostici!$F8&amp;" a "&amp;Pronostici!$G8)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="63">
-        <f>IF(OR(Pronostici!$I8="",Pronostici!$J8=""),"",Pronostici!$I8&amp;" a "&amp;Pronostici!$J8)</f>
-        <v/>
-      </c>
-      <c r="R8" s="63">
-        <f>IF(OR(Pronostici!$L8="",Pronostici!$M8=""),"",Pronostici!$L8&amp;" a "&amp;Pronostici!$M8)</f>
-        <v/>
-      </c>
-      <c r="S8" s="63">
-        <f>IF(OR(Pronostici!$O8="",Pronostici!$P8=""),"",Pronostici!$O8&amp;" a "&amp;Pronostici!$P8)</f>
-        <v/>
-      </c>
-      <c r="T8" s="63">
-        <f>IF(OR(Pronostici!$R8="",Pronostici!$S8=""),"",Pronostici!$R8&amp;" a "&amp;Pronostici!$S8)</f>
         <v/>
       </c>
     </row>
@@ -8890,23 +8749,23 @@
         <v/>
       </c>
       <c r="D9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$F9&lt;&gt;"",Pronostici!$G9&lt;&gt;"",Pronostici!$F9=Partite!$G9,Pronostici!$G9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$P9)=1),Config!$D$9,Config!$D$6),IF(AND($J9&lt;&gt;"",$J9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$J9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$F9&lt;&gt;"",Pronostici!$G9&lt;&gt;"",Pronostici!$F9=Partite!$G9,Pronostici!$G9=Partite!$H9),Config!$D$6,IF(AND($J9&lt;&gt;"",$J9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$I9&lt;&gt;"",Pronostici!$J9&lt;&gt;"",Pronostici!$I9=Partite!$G9,Pronostici!$J9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$Q9)=1),Config!$D$9,Config!$D$6),IF(AND($K9&lt;&gt;"",$K9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$K9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$I9&lt;&gt;"",Pronostici!$J9&lt;&gt;"",Pronostici!$I9=Partite!$G9,Pronostici!$J9=Partite!$H9),Config!$D$6,IF(AND($K9&lt;&gt;"",$K9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$L9&lt;&gt;"",Pronostici!$M9&lt;&gt;"",Pronostici!$L9=Partite!$G9,Pronostici!$M9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$R9)=1),Config!$D$9,Config!$D$6),IF(AND($L9&lt;&gt;"",$L9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$L9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$L9&lt;&gt;"",Pronostici!$M9&lt;&gt;"",Pronostici!$L9=Partite!$G9,Pronostici!$M9=Partite!$H9),Config!$D$6,IF(AND($L9&lt;&gt;"",$L9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$O9&lt;&gt;"",Pronostici!$P9&lt;&gt;"",Pronostici!$O9=Partite!$G9,Pronostici!$P9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$S9)=1),Config!$D$9,Config!$D$6),IF(AND($M9&lt;&gt;"",$M9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$M9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$O9&lt;&gt;"",Pronostici!$P9&lt;&gt;"",Pronostici!$O9=Partite!$G9,Pronostici!$P9=Partite!$H9),Config!$D$6,IF(AND($M9&lt;&gt;"",$M9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$R9&lt;&gt;"",Pronostici!$S9&lt;&gt;"",Pronostici!$R9=Partite!$G9,Pronostici!$S9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$T9)=1),Config!$D$9,Config!$D$6),IF(AND($N9&lt;&gt;"",$N9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$N9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$R9&lt;&gt;"",Pronostici!$S9&lt;&gt;"",Pronostici!$R9=Partite!$G9,Pronostici!$S9=Partite!$H9),Config!$D$6,IF(AND($N9&lt;&gt;"",$N9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J9" s="63">
@@ -8927,26 +8786,6 @@
       </c>
       <c r="N9" s="63">
         <f>IF(Pronostici!$Q9&lt;&gt;"",UPPER(Pronostici!$Q9),IF(OR(Pronostici!$R9="",Pronostici!$S9=""),"",IF(Pronostici!$R9&gt;Pronostici!$S9,"1",IF(Pronostici!$R9=Pronostici!$S9,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P9" s="63">
-        <f>IF(OR(Pronostici!$F9="",Pronostici!$G9=""),"",Pronostici!$F9&amp;" a "&amp;Pronostici!$G9)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="63">
-        <f>IF(OR(Pronostici!$I9="",Pronostici!$J9=""),"",Pronostici!$I9&amp;" a "&amp;Pronostici!$J9)</f>
-        <v/>
-      </c>
-      <c r="R9" s="63">
-        <f>IF(OR(Pronostici!$L9="",Pronostici!$M9=""),"",Pronostici!$L9&amp;" a "&amp;Pronostici!$M9)</f>
-        <v/>
-      </c>
-      <c r="S9" s="63">
-        <f>IF(OR(Pronostici!$O9="",Pronostici!$P9=""),"",Pronostici!$O9&amp;" a "&amp;Pronostici!$P9)</f>
-        <v/>
-      </c>
-      <c r="T9" s="63">
-        <f>IF(OR(Pronostici!$R9="",Pronostici!$S9=""),"",Pronostici!$R9&amp;" a "&amp;Pronostici!$S9)</f>
         <v/>
       </c>
     </row>
@@ -8964,23 +8803,23 @@
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$F10&lt;&gt;"",Pronostici!$G10&lt;&gt;"",Pronostici!$F10=Partite!$G10,Pronostici!$G10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$P10)=1),Config!$D$9,Config!$D$6),IF(AND($J10&lt;&gt;"",$J10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$J10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$F10&lt;&gt;"",Pronostici!$G10&lt;&gt;"",Pronostici!$F10=Partite!$G10,Pronostici!$G10=Partite!$H10),Config!$D$6,IF(AND($J10&lt;&gt;"",$J10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$I10&lt;&gt;"",Pronostici!$J10&lt;&gt;"",Pronostici!$I10=Partite!$G10,Pronostici!$J10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$Q10)=1),Config!$D$9,Config!$D$6),IF(AND($K10&lt;&gt;"",$K10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$K10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$I10&lt;&gt;"",Pronostici!$J10&lt;&gt;"",Pronostici!$I10=Partite!$G10,Pronostici!$J10=Partite!$H10),Config!$D$6,IF(AND($K10&lt;&gt;"",$K10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$L10&lt;&gt;"",Pronostici!$M10&lt;&gt;"",Pronostici!$L10=Partite!$G10,Pronostici!$M10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$R10)=1),Config!$D$9,Config!$D$6),IF(AND($L10&lt;&gt;"",$L10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$L10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$L10&lt;&gt;"",Pronostici!$M10&lt;&gt;"",Pronostici!$L10=Partite!$G10,Pronostici!$M10=Partite!$H10),Config!$D$6,IF(AND($L10&lt;&gt;"",$L10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$O10&lt;&gt;"",Pronostici!$P10&lt;&gt;"",Pronostici!$O10=Partite!$G10,Pronostici!$P10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$S10)=1),Config!$D$9,Config!$D$6),IF(AND($M10&lt;&gt;"",$M10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$M10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$O10&lt;&gt;"",Pronostici!$P10&lt;&gt;"",Pronostici!$O10=Partite!$G10,Pronostici!$P10=Partite!$H10),Config!$D$6,IF(AND($M10&lt;&gt;"",$M10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$R10&lt;&gt;"",Pronostici!$S10&lt;&gt;"",Pronostici!$R10=Partite!$G10,Pronostici!$S10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$T10)=1),Config!$D$9,Config!$D$6),IF(AND($N10&lt;&gt;"",$N10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$N10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$R10&lt;&gt;"",Pronostici!$S10&lt;&gt;"",Pronostici!$R10=Partite!$G10,Pronostici!$S10=Partite!$H10),Config!$D$6,IF(AND($N10&lt;&gt;"",$N10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J10" s="63">
@@ -9001,26 +8840,6 @@
       </c>
       <c r="N10" s="63">
         <f>IF(Pronostici!$Q10&lt;&gt;"",UPPER(Pronostici!$Q10),IF(OR(Pronostici!$R10="",Pronostici!$S10=""),"",IF(Pronostici!$R10&gt;Pronostici!$S10,"1",IF(Pronostici!$R10=Pronostici!$S10,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P10" s="63">
-        <f>IF(OR(Pronostici!$F10="",Pronostici!$G10=""),"",Pronostici!$F10&amp;" a "&amp;Pronostici!$G10)</f>
-        <v/>
-      </c>
-      <c r="Q10" s="63">
-        <f>IF(OR(Pronostici!$I10="",Pronostici!$J10=""),"",Pronostici!$I10&amp;" a "&amp;Pronostici!$J10)</f>
-        <v/>
-      </c>
-      <c r="R10" s="63">
-        <f>IF(OR(Pronostici!$L10="",Pronostici!$M10=""),"",Pronostici!$L10&amp;" a "&amp;Pronostici!$M10)</f>
-        <v/>
-      </c>
-      <c r="S10" s="63">
-        <f>IF(OR(Pronostici!$O10="",Pronostici!$P10=""),"",Pronostici!$O10&amp;" a "&amp;Pronostici!$P10)</f>
-        <v/>
-      </c>
-      <c r="T10" s="63">
-        <f>IF(OR(Pronostici!$R10="",Pronostici!$S10=""),"",Pronostici!$R10&amp;" a "&amp;Pronostici!$S10)</f>
         <v/>
       </c>
     </row>
@@ -9038,23 +8857,23 @@
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$F11&lt;&gt;"",Pronostici!$G11&lt;&gt;"",Pronostici!$F11=Partite!$G11,Pronostici!$G11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$P11)=1),Config!$D$9,Config!$D$6),IF(AND($J11&lt;&gt;"",$J11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$J11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$F11&lt;&gt;"",Pronostici!$G11&lt;&gt;"",Pronostici!$F11=Partite!$G11,Pronostici!$G11=Partite!$H11),Config!$D$6,IF(AND($J11&lt;&gt;"",$J11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$I11&lt;&gt;"",Pronostici!$J11&lt;&gt;"",Pronostici!$I11=Partite!$G11,Pronostici!$J11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$Q11)=1),Config!$D$9,Config!$D$6),IF(AND($K11&lt;&gt;"",$K11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$K11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$I11&lt;&gt;"",Pronostici!$J11&lt;&gt;"",Pronostici!$I11=Partite!$G11,Pronostici!$J11=Partite!$H11),Config!$D$6,IF(AND($K11&lt;&gt;"",$K11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$L11&lt;&gt;"",Pronostici!$M11&lt;&gt;"",Pronostici!$L11=Partite!$G11,Pronostici!$M11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$R11)=1),Config!$D$9,Config!$D$6),IF(AND($L11&lt;&gt;"",$L11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$L11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$L11&lt;&gt;"",Pronostici!$M11&lt;&gt;"",Pronostici!$L11=Partite!$G11,Pronostici!$M11=Partite!$H11),Config!$D$6,IF(AND($L11&lt;&gt;"",$L11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$O11&lt;&gt;"",Pronostici!$P11&lt;&gt;"",Pronostici!$O11=Partite!$G11,Pronostici!$P11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$S11)=1),Config!$D$9,Config!$D$6),IF(AND($M11&lt;&gt;"",$M11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$M11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$O11&lt;&gt;"",Pronostici!$P11&lt;&gt;"",Pronostici!$O11=Partite!$G11,Pronostici!$P11=Partite!$H11),Config!$D$6,IF(AND($M11&lt;&gt;"",$M11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$R11&lt;&gt;"",Pronostici!$S11&lt;&gt;"",Pronostici!$R11=Partite!$G11,Pronostici!$S11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$T11)=1),Config!$D$9,Config!$D$6),IF(AND($N11&lt;&gt;"",$N11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$N11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$R11&lt;&gt;"",Pronostici!$S11&lt;&gt;"",Pronostici!$R11=Partite!$G11,Pronostici!$S11=Partite!$H11),Config!$D$6,IF(AND($N11&lt;&gt;"",$N11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J11" s="63">
@@ -9075,26 +8894,6 @@
       </c>
       <c r="N11" s="63">
         <f>IF(Pronostici!$Q11&lt;&gt;"",UPPER(Pronostici!$Q11),IF(OR(Pronostici!$R11="",Pronostici!$S11=""),"",IF(Pronostici!$R11&gt;Pronostici!$S11,"1",IF(Pronostici!$R11=Pronostici!$S11,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P11" s="63">
-        <f>IF(OR(Pronostici!$F11="",Pronostici!$G11=""),"",Pronostici!$F11&amp;" a "&amp;Pronostici!$G11)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="63">
-        <f>IF(OR(Pronostici!$I11="",Pronostici!$J11=""),"",Pronostici!$I11&amp;" a "&amp;Pronostici!$J11)</f>
-        <v/>
-      </c>
-      <c r="R11" s="63">
-        <f>IF(OR(Pronostici!$L11="",Pronostici!$M11=""),"",Pronostici!$L11&amp;" a "&amp;Pronostici!$M11)</f>
-        <v/>
-      </c>
-      <c r="S11" s="63">
-        <f>IF(OR(Pronostici!$O11="",Pronostici!$P11=""),"",Pronostici!$O11&amp;" a "&amp;Pronostici!$P11)</f>
-        <v/>
-      </c>
-      <c r="T11" s="63">
-        <f>IF(OR(Pronostici!$R11="",Pronostici!$S11=""),"",Pronostici!$R11&amp;" a "&amp;Pronostici!$S11)</f>
         <v/>
       </c>
     </row>
@@ -9112,23 +8911,23 @@
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$F12&lt;&gt;"",Pronostici!$G12&lt;&gt;"",Pronostici!$F12=Partite!$G12,Pronostici!$G12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$P12)=1),Config!$D$9,Config!$D$6),IF(AND($J12&lt;&gt;"",$J12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$J12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$F12&lt;&gt;"",Pronostici!$G12&lt;&gt;"",Pronostici!$F12=Partite!$G12,Pronostici!$G12=Partite!$H12),Config!$D$6,IF(AND($J12&lt;&gt;"",$J12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$I12&lt;&gt;"",Pronostici!$J12&lt;&gt;"",Pronostici!$I12=Partite!$G12,Pronostici!$J12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$Q12)=1),Config!$D$9,Config!$D$6),IF(AND($K12&lt;&gt;"",$K12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$K12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$I12&lt;&gt;"",Pronostici!$J12&lt;&gt;"",Pronostici!$I12=Partite!$G12,Pronostici!$J12=Partite!$H12),Config!$D$6,IF(AND($K12&lt;&gt;"",$K12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$L12&lt;&gt;"",Pronostici!$M12&lt;&gt;"",Pronostici!$L12=Partite!$G12,Pronostici!$M12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$R12)=1),Config!$D$9,Config!$D$6),IF(AND($L12&lt;&gt;"",$L12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$L12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$L12&lt;&gt;"",Pronostici!$M12&lt;&gt;"",Pronostici!$L12=Partite!$G12,Pronostici!$M12=Partite!$H12),Config!$D$6,IF(AND($L12&lt;&gt;"",$L12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$O12&lt;&gt;"",Pronostici!$P12&lt;&gt;"",Pronostici!$O12=Partite!$G12,Pronostici!$P12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$S12)=1),Config!$D$9,Config!$D$6),IF(AND($M12&lt;&gt;"",$M12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$M12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$O12&lt;&gt;"",Pronostici!$P12&lt;&gt;"",Pronostici!$O12=Partite!$G12,Pronostici!$P12=Partite!$H12),Config!$D$6,IF(AND($M12&lt;&gt;"",$M12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$R12&lt;&gt;"",Pronostici!$S12&lt;&gt;"",Pronostici!$R12=Partite!$G12,Pronostici!$S12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$T12)=1),Config!$D$9,Config!$D$6),IF(AND($N12&lt;&gt;"",$N12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$N12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$R12&lt;&gt;"",Pronostici!$S12&lt;&gt;"",Pronostici!$R12=Partite!$G12,Pronostici!$S12=Partite!$H12),Config!$D$6,IF(AND($N12&lt;&gt;"",$N12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J12" s="63">
@@ -9149,26 +8948,6 @@
       </c>
       <c r="N12" s="63">
         <f>IF(Pronostici!$Q12&lt;&gt;"",UPPER(Pronostici!$Q12),IF(OR(Pronostici!$R12="",Pronostici!$S12=""),"",IF(Pronostici!$R12&gt;Pronostici!$S12,"1",IF(Pronostici!$R12=Pronostici!$S12,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P12" s="63">
-        <f>IF(OR(Pronostici!$F12="",Pronostici!$G12=""),"",Pronostici!$F12&amp;" a "&amp;Pronostici!$G12)</f>
-        <v/>
-      </c>
-      <c r="Q12" s="63">
-        <f>IF(OR(Pronostici!$I12="",Pronostici!$J12=""),"",Pronostici!$I12&amp;" a "&amp;Pronostici!$J12)</f>
-        <v/>
-      </c>
-      <c r="R12" s="63">
-        <f>IF(OR(Pronostici!$L12="",Pronostici!$M12=""),"",Pronostici!$L12&amp;" a "&amp;Pronostici!$M12)</f>
-        <v/>
-      </c>
-      <c r="S12" s="63">
-        <f>IF(OR(Pronostici!$O12="",Pronostici!$P12=""),"",Pronostici!$O12&amp;" a "&amp;Pronostici!$P12)</f>
-        <v/>
-      </c>
-      <c r="T12" s="63">
-        <f>IF(OR(Pronostici!$R12="",Pronostici!$S12=""),"",Pronostici!$R12&amp;" a "&amp;Pronostici!$S12)</f>
         <v/>
       </c>
     </row>
@@ -9186,23 +8965,23 @@
         <v/>
       </c>
       <c r="D13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$F13&lt;&gt;"",Pronostici!$G13&lt;&gt;"",Pronostici!$F13=Partite!$G13,Pronostici!$G13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$P13)=1),Config!$D$9,Config!$D$6),IF(AND($J13&lt;&gt;"",$J13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$J13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$F13&lt;&gt;"",Pronostici!$G13&lt;&gt;"",Pronostici!$F13=Partite!$G13,Pronostici!$G13=Partite!$H13),Config!$D$6,IF(AND($J13&lt;&gt;"",$J13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$I13&lt;&gt;"",Pronostici!$J13&lt;&gt;"",Pronostici!$I13=Partite!$G13,Pronostici!$J13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$Q13)=1),Config!$D$9,Config!$D$6),IF(AND($K13&lt;&gt;"",$K13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$K13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$I13&lt;&gt;"",Pronostici!$J13&lt;&gt;"",Pronostici!$I13=Partite!$G13,Pronostici!$J13=Partite!$H13),Config!$D$6,IF(AND($K13&lt;&gt;"",$K13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$L13&lt;&gt;"",Pronostici!$M13&lt;&gt;"",Pronostici!$L13=Partite!$G13,Pronostici!$M13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$R13)=1),Config!$D$9,Config!$D$6),IF(AND($L13&lt;&gt;"",$L13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$L13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$L13&lt;&gt;"",Pronostici!$M13&lt;&gt;"",Pronostici!$L13=Partite!$G13,Pronostici!$M13=Partite!$H13),Config!$D$6,IF(AND($L13&lt;&gt;"",$L13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$O13&lt;&gt;"",Pronostici!$P13&lt;&gt;"",Pronostici!$O13=Partite!$G13,Pronostici!$P13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$S13)=1),Config!$D$9,Config!$D$6),IF(AND($M13&lt;&gt;"",$M13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$M13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$O13&lt;&gt;"",Pronostici!$P13&lt;&gt;"",Pronostici!$O13=Partite!$G13,Pronostici!$P13=Partite!$H13),Config!$D$6,IF(AND($M13&lt;&gt;"",$M13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$R13&lt;&gt;"",Pronostici!$S13&lt;&gt;"",Pronostici!$R13=Partite!$G13,Pronostici!$S13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$T13)=1),Config!$D$9,Config!$D$6),IF(AND($N13&lt;&gt;"",$N13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$N13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$R13&lt;&gt;"",Pronostici!$S13&lt;&gt;"",Pronostici!$R13=Partite!$G13,Pronostici!$S13=Partite!$H13),Config!$D$6,IF(AND($N13&lt;&gt;"",$N13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J13" s="63">
@@ -9223,26 +9002,6 @@
       </c>
       <c r="N13" s="63">
         <f>IF(Pronostici!$Q13&lt;&gt;"",UPPER(Pronostici!$Q13),IF(OR(Pronostici!$R13="",Pronostici!$S13=""),"",IF(Pronostici!$R13&gt;Pronostici!$S13,"1",IF(Pronostici!$R13=Pronostici!$S13,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P13" s="63">
-        <f>IF(OR(Pronostici!$F13="",Pronostici!$G13=""),"",Pronostici!$F13&amp;" a "&amp;Pronostici!$G13)</f>
-        <v/>
-      </c>
-      <c r="Q13" s="63">
-        <f>IF(OR(Pronostici!$I13="",Pronostici!$J13=""),"",Pronostici!$I13&amp;" a "&amp;Pronostici!$J13)</f>
-        <v/>
-      </c>
-      <c r="R13" s="63">
-        <f>IF(OR(Pronostici!$L13="",Pronostici!$M13=""),"",Pronostici!$L13&amp;" a "&amp;Pronostici!$M13)</f>
-        <v/>
-      </c>
-      <c r="S13" s="63">
-        <f>IF(OR(Pronostici!$O13="",Pronostici!$P13=""),"",Pronostici!$O13&amp;" a "&amp;Pronostici!$P13)</f>
-        <v/>
-      </c>
-      <c r="T13" s="63">
-        <f>IF(OR(Pronostici!$R13="",Pronostici!$S13=""),"",Pronostici!$R13&amp;" a "&amp;Pronostici!$S13)</f>
         <v/>
       </c>
     </row>
@@ -9260,23 +9019,23 @@
         <v/>
       </c>
       <c r="D14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$F14&lt;&gt;"",Pronostici!$G14&lt;&gt;"",Pronostici!$F14=Partite!$G14,Pronostici!$G14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$P14)=1),Config!$D$9,Config!$D$6),IF(AND($J14&lt;&gt;"",$J14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$J14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$F14&lt;&gt;"",Pronostici!$G14&lt;&gt;"",Pronostici!$F14=Partite!$G14,Pronostici!$G14=Partite!$H14),Config!$D$6,IF(AND($J14&lt;&gt;"",$J14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$I14&lt;&gt;"",Pronostici!$J14&lt;&gt;"",Pronostici!$I14=Partite!$G14,Pronostici!$J14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$Q14)=1),Config!$D$9,Config!$D$6),IF(AND($K14&lt;&gt;"",$K14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$K14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$I14&lt;&gt;"",Pronostici!$J14&lt;&gt;"",Pronostici!$I14=Partite!$G14,Pronostici!$J14=Partite!$H14),Config!$D$6,IF(AND($K14&lt;&gt;"",$K14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$L14&lt;&gt;"",Pronostici!$M14&lt;&gt;"",Pronostici!$L14=Partite!$G14,Pronostici!$M14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$R14)=1),Config!$D$9,Config!$D$6),IF(AND($L14&lt;&gt;"",$L14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$L14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$L14&lt;&gt;"",Pronostici!$M14&lt;&gt;"",Pronostici!$L14=Partite!$G14,Pronostici!$M14=Partite!$H14),Config!$D$6,IF(AND($L14&lt;&gt;"",$L14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$O14&lt;&gt;"",Pronostici!$P14&lt;&gt;"",Pronostici!$O14=Partite!$G14,Pronostici!$P14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$S14)=1),Config!$D$9,Config!$D$6),IF(AND($M14&lt;&gt;"",$M14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$M14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$O14&lt;&gt;"",Pronostici!$P14&lt;&gt;"",Pronostici!$O14=Partite!$G14,Pronostici!$P14=Partite!$H14),Config!$D$6,IF(AND($M14&lt;&gt;"",$M14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$R14&lt;&gt;"",Pronostici!$S14&lt;&gt;"",Pronostici!$R14=Partite!$G14,Pronostici!$S14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$T14)=1),Config!$D$9,Config!$D$6),IF(AND($N14&lt;&gt;"",$N14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$N14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$R14&lt;&gt;"",Pronostici!$S14&lt;&gt;"",Pronostici!$R14=Partite!$G14,Pronostici!$S14=Partite!$H14),Config!$D$6,IF(AND($N14&lt;&gt;"",$N14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J14" s="63">
@@ -9297,26 +9056,6 @@
       </c>
       <c r="N14" s="63">
         <f>IF(Pronostici!$Q14&lt;&gt;"",UPPER(Pronostici!$Q14),IF(OR(Pronostici!$R14="",Pronostici!$S14=""),"",IF(Pronostici!$R14&gt;Pronostici!$S14,"1",IF(Pronostici!$R14=Pronostici!$S14,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P14" s="63">
-        <f>IF(OR(Pronostici!$F14="",Pronostici!$G14=""),"",Pronostici!$F14&amp;" a "&amp;Pronostici!$G14)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="63">
-        <f>IF(OR(Pronostici!$I14="",Pronostici!$J14=""),"",Pronostici!$I14&amp;" a "&amp;Pronostici!$J14)</f>
-        <v/>
-      </c>
-      <c r="R14" s="63">
-        <f>IF(OR(Pronostici!$L14="",Pronostici!$M14=""),"",Pronostici!$L14&amp;" a "&amp;Pronostici!$M14)</f>
-        <v/>
-      </c>
-      <c r="S14" s="63">
-        <f>IF(OR(Pronostici!$O14="",Pronostici!$P14=""),"",Pronostici!$O14&amp;" a "&amp;Pronostici!$P14)</f>
-        <v/>
-      </c>
-      <c r="T14" s="63">
-        <f>IF(OR(Pronostici!$R14="",Pronostici!$S14=""),"",Pronostici!$R14&amp;" a "&amp;Pronostici!$S14)</f>
         <v/>
       </c>
     </row>
@@ -9334,23 +9073,23 @@
         <v/>
       </c>
       <c r="D15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$F15&lt;&gt;"",Pronostici!$G15&lt;&gt;"",Pronostici!$F15=Partite!$G15,Pronostici!$G15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$P15)=1),Config!$D$9,Config!$D$6),IF(AND($J15&lt;&gt;"",$J15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$J15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$F15&lt;&gt;"",Pronostici!$G15&lt;&gt;"",Pronostici!$F15=Partite!$G15,Pronostici!$G15=Partite!$H15),Config!$D$6,IF(AND($J15&lt;&gt;"",$J15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$I15&lt;&gt;"",Pronostici!$J15&lt;&gt;"",Pronostici!$I15=Partite!$G15,Pronostici!$J15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$Q15)=1),Config!$D$9,Config!$D$6),IF(AND($K15&lt;&gt;"",$K15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$K15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$I15&lt;&gt;"",Pronostici!$J15&lt;&gt;"",Pronostici!$I15=Partite!$G15,Pronostici!$J15=Partite!$H15),Config!$D$6,IF(AND($K15&lt;&gt;"",$K15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$L15&lt;&gt;"",Pronostici!$M15&lt;&gt;"",Pronostici!$L15=Partite!$G15,Pronostici!$M15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$R15)=1),Config!$D$9,Config!$D$6),IF(AND($L15&lt;&gt;"",$L15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$L15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$L15&lt;&gt;"",Pronostici!$M15&lt;&gt;"",Pronostici!$L15=Partite!$G15,Pronostici!$M15=Partite!$H15),Config!$D$6,IF(AND($L15&lt;&gt;"",$L15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$O15&lt;&gt;"",Pronostici!$P15&lt;&gt;"",Pronostici!$O15=Partite!$G15,Pronostici!$P15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$S15)=1),Config!$D$9,Config!$D$6),IF(AND($M15&lt;&gt;"",$M15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$M15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$O15&lt;&gt;"",Pronostici!$P15&lt;&gt;"",Pronostici!$O15=Partite!$G15,Pronostici!$P15=Partite!$H15),Config!$D$6,IF(AND($M15&lt;&gt;"",$M15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$R15&lt;&gt;"",Pronostici!$S15&lt;&gt;"",Pronostici!$R15=Partite!$G15,Pronostici!$S15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$T15)=1),Config!$D$9,Config!$D$6),IF(AND($N15&lt;&gt;"",$N15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$N15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$R15&lt;&gt;"",Pronostici!$S15&lt;&gt;"",Pronostici!$R15=Partite!$G15,Pronostici!$S15=Partite!$H15),Config!$D$6,IF(AND($N15&lt;&gt;"",$N15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J15" s="63">
@@ -9371,26 +9110,6 @@
       </c>
       <c r="N15" s="63">
         <f>IF(Pronostici!$Q15&lt;&gt;"",UPPER(Pronostici!$Q15),IF(OR(Pronostici!$R15="",Pronostici!$S15=""),"",IF(Pronostici!$R15&gt;Pronostici!$S15,"1",IF(Pronostici!$R15=Pronostici!$S15,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P15" s="63">
-        <f>IF(OR(Pronostici!$F15="",Pronostici!$G15=""),"",Pronostici!$F15&amp;" a "&amp;Pronostici!$G15)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="63">
-        <f>IF(OR(Pronostici!$I15="",Pronostici!$J15=""),"",Pronostici!$I15&amp;" a "&amp;Pronostici!$J15)</f>
-        <v/>
-      </c>
-      <c r="R15" s="63">
-        <f>IF(OR(Pronostici!$L15="",Pronostici!$M15=""),"",Pronostici!$L15&amp;" a "&amp;Pronostici!$M15)</f>
-        <v/>
-      </c>
-      <c r="S15" s="63">
-        <f>IF(OR(Pronostici!$O15="",Pronostici!$P15=""),"",Pronostici!$O15&amp;" a "&amp;Pronostici!$P15)</f>
-        <v/>
-      </c>
-      <c r="T15" s="63">
-        <f>IF(OR(Pronostici!$R15="",Pronostici!$S15=""),"",Pronostici!$R15&amp;" a "&amp;Pronostici!$S15)</f>
         <v/>
       </c>
     </row>
@@ -9408,23 +9127,23 @@
         <v/>
       </c>
       <c r="D16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$F16&lt;&gt;"",Pronostici!$G16&lt;&gt;"",Pronostici!$F16=Partite!$G16,Pronostici!$G16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$P16)=1),Config!$D$9,Config!$D$6),IF(AND($J16&lt;&gt;"",$J16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$J16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$F16&lt;&gt;"",Pronostici!$G16&lt;&gt;"",Pronostici!$F16=Partite!$G16,Pronostici!$G16=Partite!$H16),Config!$D$6,IF(AND($J16&lt;&gt;"",$J16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$I16&lt;&gt;"",Pronostici!$J16&lt;&gt;"",Pronostici!$I16=Partite!$G16,Pronostici!$J16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$Q16)=1),Config!$D$9,Config!$D$6),IF(AND($K16&lt;&gt;"",$K16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$K16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$I16&lt;&gt;"",Pronostici!$J16&lt;&gt;"",Pronostici!$I16=Partite!$G16,Pronostici!$J16=Partite!$H16),Config!$D$6,IF(AND($K16&lt;&gt;"",$K16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$L16&lt;&gt;"",Pronostici!$M16&lt;&gt;"",Pronostici!$L16=Partite!$G16,Pronostici!$M16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$R16)=1),Config!$D$9,Config!$D$6),IF(AND($L16&lt;&gt;"",$L16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$L16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$L16&lt;&gt;"",Pronostici!$M16&lt;&gt;"",Pronostici!$L16=Partite!$G16,Pronostici!$M16=Partite!$H16),Config!$D$6,IF(AND($L16&lt;&gt;"",$L16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$O16&lt;&gt;"",Pronostici!$P16&lt;&gt;"",Pronostici!$O16=Partite!$G16,Pronostici!$P16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$S16)=1),Config!$D$9,Config!$D$6),IF(AND($M16&lt;&gt;"",$M16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$M16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$O16&lt;&gt;"",Pronostici!$P16&lt;&gt;"",Pronostici!$O16=Partite!$G16,Pronostici!$P16=Partite!$H16),Config!$D$6,IF(AND($M16&lt;&gt;"",$M16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$R16&lt;&gt;"",Pronostici!$S16&lt;&gt;"",Pronostici!$R16=Partite!$G16,Pronostici!$S16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$T16)=1),Config!$D$9,Config!$D$6),IF(AND($N16&lt;&gt;"",$N16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$N16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$R16&lt;&gt;"",Pronostici!$S16&lt;&gt;"",Pronostici!$R16=Partite!$G16,Pronostici!$S16=Partite!$H16),Config!$D$6,IF(AND($N16&lt;&gt;"",$N16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J16" s="63">
@@ -9445,26 +9164,6 @@
       </c>
       <c r="N16" s="63">
         <f>IF(Pronostici!$Q16&lt;&gt;"",UPPER(Pronostici!$Q16),IF(OR(Pronostici!$R16="",Pronostici!$S16=""),"",IF(Pronostici!$R16&gt;Pronostici!$S16,"1",IF(Pronostici!$R16=Pronostici!$S16,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P16" s="63">
-        <f>IF(OR(Pronostici!$F16="",Pronostici!$G16=""),"",Pronostici!$F16&amp;" a "&amp;Pronostici!$G16)</f>
-        <v/>
-      </c>
-      <c r="Q16" s="63">
-        <f>IF(OR(Pronostici!$I16="",Pronostici!$J16=""),"",Pronostici!$I16&amp;" a "&amp;Pronostici!$J16)</f>
-        <v/>
-      </c>
-      <c r="R16" s="63">
-        <f>IF(OR(Pronostici!$L16="",Pronostici!$M16=""),"",Pronostici!$L16&amp;" a "&amp;Pronostici!$M16)</f>
-        <v/>
-      </c>
-      <c r="S16" s="63">
-        <f>IF(OR(Pronostici!$O16="",Pronostici!$P16=""),"",Pronostici!$O16&amp;" a "&amp;Pronostici!$P16)</f>
-        <v/>
-      </c>
-      <c r="T16" s="63">
-        <f>IF(OR(Pronostici!$R16="",Pronostici!$S16=""),"",Pronostici!$R16&amp;" a "&amp;Pronostici!$S16)</f>
         <v/>
       </c>
     </row>
@@ -9482,23 +9181,23 @@
         <v/>
       </c>
       <c r="D17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$F17&lt;&gt;"",Pronostici!$G17&lt;&gt;"",Pronostici!$F17=Partite!$G17,Pronostici!$G17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$P17)=1),Config!$D$9,Config!$D$6),IF(AND($J17&lt;&gt;"",$J17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$J17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$F17&lt;&gt;"",Pronostici!$G17&lt;&gt;"",Pronostici!$F17=Partite!$G17,Pronostici!$G17=Partite!$H17),Config!$D$6,IF(AND($J17&lt;&gt;"",$J17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$I17&lt;&gt;"",Pronostici!$J17&lt;&gt;"",Pronostici!$I17=Partite!$G17,Pronostici!$J17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$Q17)=1),Config!$D$9,Config!$D$6),IF(AND($K17&lt;&gt;"",$K17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$K17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$I17&lt;&gt;"",Pronostici!$J17&lt;&gt;"",Pronostici!$I17=Partite!$G17,Pronostici!$J17=Partite!$H17),Config!$D$6,IF(AND($K17&lt;&gt;"",$K17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$L17&lt;&gt;"",Pronostici!$M17&lt;&gt;"",Pronostici!$L17=Partite!$G17,Pronostici!$M17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$R17)=1),Config!$D$9,Config!$D$6),IF(AND($L17&lt;&gt;"",$L17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$L17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$L17&lt;&gt;"",Pronostici!$M17&lt;&gt;"",Pronostici!$L17=Partite!$G17,Pronostici!$M17=Partite!$H17),Config!$D$6,IF(AND($L17&lt;&gt;"",$L17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$O17&lt;&gt;"",Pronostici!$P17&lt;&gt;"",Pronostici!$O17=Partite!$G17,Pronostici!$P17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$S17)=1),Config!$D$9,Config!$D$6),IF(AND($M17&lt;&gt;"",$M17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$M17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$O17&lt;&gt;"",Pronostici!$P17&lt;&gt;"",Pronostici!$O17=Partite!$G17,Pronostici!$P17=Partite!$H17),Config!$D$6,IF(AND($M17&lt;&gt;"",$M17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$R17&lt;&gt;"",Pronostici!$S17&lt;&gt;"",Pronostici!$R17=Partite!$G17,Pronostici!$S17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$T17)=1),Config!$D$9,Config!$D$6),IF(AND($N17&lt;&gt;"",$N17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$N17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$R17&lt;&gt;"",Pronostici!$S17&lt;&gt;"",Pronostici!$R17=Partite!$G17,Pronostici!$S17=Partite!$H17),Config!$D$6,IF(AND($N17&lt;&gt;"",$N17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J17" s="63">
@@ -9519,26 +9218,6 @@
       </c>
       <c r="N17" s="63">
         <f>IF(Pronostici!$Q17&lt;&gt;"",UPPER(Pronostici!$Q17),IF(OR(Pronostici!$R17="",Pronostici!$S17=""),"",IF(Pronostici!$R17&gt;Pronostici!$S17,"1",IF(Pronostici!$R17=Pronostici!$S17,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P17" s="63">
-        <f>IF(OR(Pronostici!$F17="",Pronostici!$G17=""),"",Pronostici!$F17&amp;" a "&amp;Pronostici!$G17)</f>
-        <v/>
-      </c>
-      <c r="Q17" s="63">
-        <f>IF(OR(Pronostici!$I17="",Pronostici!$J17=""),"",Pronostici!$I17&amp;" a "&amp;Pronostici!$J17)</f>
-        <v/>
-      </c>
-      <c r="R17" s="63">
-        <f>IF(OR(Pronostici!$L17="",Pronostici!$M17=""),"",Pronostici!$L17&amp;" a "&amp;Pronostici!$M17)</f>
-        <v/>
-      </c>
-      <c r="S17" s="63">
-        <f>IF(OR(Pronostici!$O17="",Pronostici!$P17=""),"",Pronostici!$O17&amp;" a "&amp;Pronostici!$P17)</f>
-        <v/>
-      </c>
-      <c r="T17" s="63">
-        <f>IF(OR(Pronostici!$R17="",Pronostici!$S17=""),"",Pronostici!$R17&amp;" a "&amp;Pronostici!$S17)</f>
         <v/>
       </c>
     </row>
@@ -9556,23 +9235,23 @@
         <v/>
       </c>
       <c r="D18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$F18&lt;&gt;"",Pronostici!$G18&lt;&gt;"",Pronostici!$F18=Partite!$G18,Pronostici!$G18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$P18)=1),Config!$D$9,Config!$D$6),IF(AND($J18&lt;&gt;"",$J18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$J18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$F18&lt;&gt;"",Pronostici!$G18&lt;&gt;"",Pronostici!$F18=Partite!$G18,Pronostici!$G18=Partite!$H18),Config!$D$6,IF(AND($J18&lt;&gt;"",$J18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$I18&lt;&gt;"",Pronostici!$J18&lt;&gt;"",Pronostici!$I18=Partite!$G18,Pronostici!$J18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$Q18)=1),Config!$D$9,Config!$D$6),IF(AND($K18&lt;&gt;"",$K18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$K18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$I18&lt;&gt;"",Pronostici!$J18&lt;&gt;"",Pronostici!$I18=Partite!$G18,Pronostici!$J18=Partite!$H18),Config!$D$6,IF(AND($K18&lt;&gt;"",$K18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$L18&lt;&gt;"",Pronostici!$M18&lt;&gt;"",Pronostici!$L18=Partite!$G18,Pronostici!$M18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$R18)=1),Config!$D$9,Config!$D$6),IF(AND($L18&lt;&gt;"",$L18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$L18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$L18&lt;&gt;"",Pronostici!$M18&lt;&gt;"",Pronostici!$L18=Partite!$G18,Pronostici!$M18=Partite!$H18),Config!$D$6,IF(AND($L18&lt;&gt;"",$L18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$O18&lt;&gt;"",Pronostici!$P18&lt;&gt;"",Pronostici!$O18=Partite!$G18,Pronostici!$P18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$S18)=1),Config!$D$9,Config!$D$6),IF(AND($M18&lt;&gt;"",$M18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$M18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$O18&lt;&gt;"",Pronostici!$P18&lt;&gt;"",Pronostici!$O18=Partite!$G18,Pronostici!$P18=Partite!$H18),Config!$D$6,IF(AND($M18&lt;&gt;"",$M18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$R18&lt;&gt;"",Pronostici!$S18&lt;&gt;"",Pronostici!$R18=Partite!$G18,Pronostici!$S18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$T18)=1),Config!$D$9,Config!$D$6),IF(AND($N18&lt;&gt;"",$N18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$N18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$R18&lt;&gt;"",Pronostici!$S18&lt;&gt;"",Pronostici!$R18=Partite!$G18,Pronostici!$S18=Partite!$H18),Config!$D$6,IF(AND($N18&lt;&gt;"",$N18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J18" s="63">
@@ -9593,26 +9272,6 @@
       </c>
       <c r="N18" s="63">
         <f>IF(Pronostici!$Q18&lt;&gt;"",UPPER(Pronostici!$Q18),IF(OR(Pronostici!$R18="",Pronostici!$S18=""),"",IF(Pronostici!$R18&gt;Pronostici!$S18,"1",IF(Pronostici!$R18=Pronostici!$S18,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P18" s="63">
-        <f>IF(OR(Pronostici!$F18="",Pronostici!$G18=""),"",Pronostici!$F18&amp;" a "&amp;Pronostici!$G18)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="63">
-        <f>IF(OR(Pronostici!$I18="",Pronostici!$J18=""),"",Pronostici!$I18&amp;" a "&amp;Pronostici!$J18)</f>
-        <v/>
-      </c>
-      <c r="R18" s="63">
-        <f>IF(OR(Pronostici!$L18="",Pronostici!$M18=""),"",Pronostici!$L18&amp;" a "&amp;Pronostici!$M18)</f>
-        <v/>
-      </c>
-      <c r="S18" s="63">
-        <f>IF(OR(Pronostici!$O18="",Pronostici!$P18=""),"",Pronostici!$O18&amp;" a "&amp;Pronostici!$P18)</f>
-        <v/>
-      </c>
-      <c r="T18" s="63">
-        <f>IF(OR(Pronostici!$R18="",Pronostici!$S18=""),"",Pronostici!$R18&amp;" a "&amp;Pronostici!$S18)</f>
         <v/>
       </c>
     </row>
@@ -9630,23 +9289,23 @@
         <v/>
       </c>
       <c r="D19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$F19&lt;&gt;"",Pronostici!$G19&lt;&gt;"",Pronostici!$F19=Partite!$G19,Pronostici!$G19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$P19)=1),Config!$D$9,Config!$D$6),IF(AND($J19&lt;&gt;"",$J19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$J19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$F19&lt;&gt;"",Pronostici!$G19&lt;&gt;"",Pronostici!$F19=Partite!$G19,Pronostici!$G19=Partite!$H19),Config!$D$6,IF(AND($J19&lt;&gt;"",$J19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$I19&lt;&gt;"",Pronostici!$J19&lt;&gt;"",Pronostici!$I19=Partite!$G19,Pronostici!$J19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$Q19)=1),Config!$D$9,Config!$D$6),IF(AND($K19&lt;&gt;"",$K19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$K19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$I19&lt;&gt;"",Pronostici!$J19&lt;&gt;"",Pronostici!$I19=Partite!$G19,Pronostici!$J19=Partite!$H19),Config!$D$6,IF(AND($K19&lt;&gt;"",$K19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$L19&lt;&gt;"",Pronostici!$M19&lt;&gt;"",Pronostici!$L19=Partite!$G19,Pronostici!$M19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$R19)=1),Config!$D$9,Config!$D$6),IF(AND($L19&lt;&gt;"",$L19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$L19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$L19&lt;&gt;"",Pronostici!$M19&lt;&gt;"",Pronostici!$L19=Partite!$G19,Pronostici!$M19=Partite!$H19),Config!$D$6,IF(AND($L19&lt;&gt;"",$L19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$O19&lt;&gt;"",Pronostici!$P19&lt;&gt;"",Pronostici!$O19=Partite!$G19,Pronostici!$P19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$S19)=1),Config!$D$9,Config!$D$6),IF(AND($M19&lt;&gt;"",$M19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$M19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$O19&lt;&gt;"",Pronostici!$P19&lt;&gt;"",Pronostici!$O19=Partite!$G19,Pronostici!$P19=Partite!$H19),Config!$D$6,IF(AND($M19&lt;&gt;"",$M19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$R19&lt;&gt;"",Pronostici!$S19&lt;&gt;"",Pronostici!$R19=Partite!$G19,Pronostici!$S19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$T19)=1),Config!$D$9,Config!$D$6),IF(AND($N19&lt;&gt;"",$N19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$N19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$R19&lt;&gt;"",Pronostici!$S19&lt;&gt;"",Pronostici!$R19=Partite!$G19,Pronostici!$S19=Partite!$H19),Config!$D$6,IF(AND($N19&lt;&gt;"",$N19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J19" s="63">
@@ -9667,26 +9326,6 @@
       </c>
       <c r="N19" s="63">
         <f>IF(Pronostici!$Q19&lt;&gt;"",UPPER(Pronostici!$Q19),IF(OR(Pronostici!$R19="",Pronostici!$S19=""),"",IF(Pronostici!$R19&gt;Pronostici!$S19,"1",IF(Pronostici!$R19=Pronostici!$S19,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P19" s="63">
-        <f>IF(OR(Pronostici!$F19="",Pronostici!$G19=""),"",Pronostici!$F19&amp;" a "&amp;Pronostici!$G19)</f>
-        <v/>
-      </c>
-      <c r="Q19" s="63">
-        <f>IF(OR(Pronostici!$I19="",Pronostici!$J19=""),"",Pronostici!$I19&amp;" a "&amp;Pronostici!$J19)</f>
-        <v/>
-      </c>
-      <c r="R19" s="63">
-        <f>IF(OR(Pronostici!$L19="",Pronostici!$M19=""),"",Pronostici!$L19&amp;" a "&amp;Pronostici!$M19)</f>
-        <v/>
-      </c>
-      <c r="S19" s="63">
-        <f>IF(OR(Pronostici!$O19="",Pronostici!$P19=""),"",Pronostici!$O19&amp;" a "&amp;Pronostici!$P19)</f>
-        <v/>
-      </c>
-      <c r="T19" s="63">
-        <f>IF(OR(Pronostici!$R19="",Pronostici!$S19=""),"",Pronostici!$R19&amp;" a "&amp;Pronostici!$S19)</f>
         <v/>
       </c>
     </row>
@@ -9704,23 +9343,23 @@
         <v/>
       </c>
       <c r="D20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$F20&lt;&gt;"",Pronostici!$G20&lt;&gt;"",Pronostici!$F20=Partite!$G20,Pronostici!$G20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$P20)=1),Config!$D$9,Config!$D$6),IF(AND($J20&lt;&gt;"",$J20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$J20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$F20&lt;&gt;"",Pronostici!$G20&lt;&gt;"",Pronostici!$F20=Partite!$G20,Pronostici!$G20=Partite!$H20),Config!$D$6,IF(AND($J20&lt;&gt;"",$J20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$I20&lt;&gt;"",Pronostici!$J20&lt;&gt;"",Pronostici!$I20=Partite!$G20,Pronostici!$J20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$Q20)=1),Config!$D$9,Config!$D$6),IF(AND($K20&lt;&gt;"",$K20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$K20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$I20&lt;&gt;"",Pronostici!$J20&lt;&gt;"",Pronostici!$I20=Partite!$G20,Pronostici!$J20=Partite!$H20),Config!$D$6,IF(AND($K20&lt;&gt;"",$K20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$L20&lt;&gt;"",Pronostici!$M20&lt;&gt;"",Pronostici!$L20=Partite!$G20,Pronostici!$M20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$R20)=1),Config!$D$9,Config!$D$6),IF(AND($L20&lt;&gt;"",$L20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$L20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$L20&lt;&gt;"",Pronostici!$M20&lt;&gt;"",Pronostici!$L20=Partite!$G20,Pronostici!$M20=Partite!$H20),Config!$D$6,IF(AND($L20&lt;&gt;"",$L20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$O20&lt;&gt;"",Pronostici!$P20&lt;&gt;"",Pronostici!$O20=Partite!$G20,Pronostici!$P20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$S20)=1),Config!$D$9,Config!$D$6),IF(AND($M20&lt;&gt;"",$M20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$M20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$O20&lt;&gt;"",Pronostici!$P20&lt;&gt;"",Pronostici!$O20=Partite!$G20,Pronostici!$P20=Partite!$H20),Config!$D$6,IF(AND($M20&lt;&gt;"",$M20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$R20&lt;&gt;"",Pronostici!$S20&lt;&gt;"",Pronostici!$R20=Partite!$G20,Pronostici!$S20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$T20)=1),Config!$D$9,Config!$D$6),IF(AND($N20&lt;&gt;"",$N20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$N20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$R20&lt;&gt;"",Pronostici!$S20&lt;&gt;"",Pronostici!$R20=Partite!$G20,Pronostici!$S20=Partite!$H20),Config!$D$6,IF(AND($N20&lt;&gt;"",$N20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J20" s="63">
@@ -9741,26 +9380,6 @@
       </c>
       <c r="N20" s="63">
         <f>IF(Pronostici!$Q20&lt;&gt;"",UPPER(Pronostici!$Q20),IF(OR(Pronostici!$R20="",Pronostici!$S20=""),"",IF(Pronostici!$R20&gt;Pronostici!$S20,"1",IF(Pronostici!$R20=Pronostici!$S20,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P20" s="63">
-        <f>IF(OR(Pronostici!$F20="",Pronostici!$G20=""),"",Pronostici!$F20&amp;" a "&amp;Pronostici!$G20)</f>
-        <v/>
-      </c>
-      <c r="Q20" s="63">
-        <f>IF(OR(Pronostici!$I20="",Pronostici!$J20=""),"",Pronostici!$I20&amp;" a "&amp;Pronostici!$J20)</f>
-        <v/>
-      </c>
-      <c r="R20" s="63">
-        <f>IF(OR(Pronostici!$L20="",Pronostici!$M20=""),"",Pronostici!$L20&amp;" a "&amp;Pronostici!$M20)</f>
-        <v/>
-      </c>
-      <c r="S20" s="63">
-        <f>IF(OR(Pronostici!$O20="",Pronostici!$P20=""),"",Pronostici!$O20&amp;" a "&amp;Pronostici!$P20)</f>
-        <v/>
-      </c>
-      <c r="T20" s="63">
-        <f>IF(OR(Pronostici!$R20="",Pronostici!$S20=""),"",Pronostici!$R20&amp;" a "&amp;Pronostici!$S20)</f>
         <v/>
       </c>
     </row>
@@ -9778,23 +9397,23 @@
         <v/>
       </c>
       <c r="D21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$F21&lt;&gt;"",Pronostici!$G21&lt;&gt;"",Pronostici!$F21=Partite!$G21,Pronostici!$G21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$P21)=1),Config!$D$9,Config!$D$6),IF(AND($J21&lt;&gt;"",$J21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$J21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$F21&lt;&gt;"",Pronostici!$G21&lt;&gt;"",Pronostici!$F21=Partite!$G21,Pronostici!$G21=Partite!$H21),Config!$D$6,IF(AND($J21&lt;&gt;"",$J21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$I21&lt;&gt;"",Pronostici!$J21&lt;&gt;"",Pronostici!$I21=Partite!$G21,Pronostici!$J21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$Q21)=1),Config!$D$9,Config!$D$6),IF(AND($K21&lt;&gt;"",$K21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$K21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$I21&lt;&gt;"",Pronostici!$J21&lt;&gt;"",Pronostici!$I21=Partite!$G21,Pronostici!$J21=Partite!$H21),Config!$D$6,IF(AND($K21&lt;&gt;"",$K21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$L21&lt;&gt;"",Pronostici!$M21&lt;&gt;"",Pronostici!$L21=Partite!$G21,Pronostici!$M21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$R21)=1),Config!$D$9,Config!$D$6),IF(AND($L21&lt;&gt;"",$L21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$L21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$L21&lt;&gt;"",Pronostici!$M21&lt;&gt;"",Pronostici!$L21=Partite!$G21,Pronostici!$M21=Partite!$H21),Config!$D$6,IF(AND($L21&lt;&gt;"",$L21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$O21&lt;&gt;"",Pronostici!$P21&lt;&gt;"",Pronostici!$O21=Partite!$G21,Pronostici!$P21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$S21)=1),Config!$D$9,Config!$D$6),IF(AND($M21&lt;&gt;"",$M21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$M21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$O21&lt;&gt;"",Pronostici!$P21&lt;&gt;"",Pronostici!$O21=Partite!$G21,Pronostici!$P21=Partite!$H21),Config!$D$6,IF(AND($M21&lt;&gt;"",$M21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$R21&lt;&gt;"",Pronostici!$S21&lt;&gt;"",Pronostici!$R21=Partite!$G21,Pronostici!$S21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$T21)=1),Config!$D$9,Config!$D$6),IF(AND($N21&lt;&gt;"",$N21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$N21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$R21&lt;&gt;"",Pronostici!$S21&lt;&gt;"",Pronostici!$R21=Partite!$G21,Pronostici!$S21=Partite!$H21),Config!$D$6,IF(AND($N21&lt;&gt;"",$N21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J21" s="63">
@@ -9815,26 +9434,6 @@
       </c>
       <c r="N21" s="63">
         <f>IF(Pronostici!$Q21&lt;&gt;"",UPPER(Pronostici!$Q21),IF(OR(Pronostici!$R21="",Pronostici!$S21=""),"",IF(Pronostici!$R21&gt;Pronostici!$S21,"1",IF(Pronostici!$R21=Pronostici!$S21,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P21" s="63">
-        <f>IF(OR(Pronostici!$F21="",Pronostici!$G21=""),"",Pronostici!$F21&amp;" a "&amp;Pronostici!$G21)</f>
-        <v/>
-      </c>
-      <c r="Q21" s="63">
-        <f>IF(OR(Pronostici!$I21="",Pronostici!$J21=""),"",Pronostici!$I21&amp;" a "&amp;Pronostici!$J21)</f>
-        <v/>
-      </c>
-      <c r="R21" s="63">
-        <f>IF(OR(Pronostici!$L21="",Pronostici!$M21=""),"",Pronostici!$L21&amp;" a "&amp;Pronostici!$M21)</f>
-        <v/>
-      </c>
-      <c r="S21" s="63">
-        <f>IF(OR(Pronostici!$O21="",Pronostici!$P21=""),"",Pronostici!$O21&amp;" a "&amp;Pronostici!$P21)</f>
-        <v/>
-      </c>
-      <c r="T21" s="63">
-        <f>IF(OR(Pronostici!$R21="",Pronostici!$S21=""),"",Pronostici!$R21&amp;" a "&amp;Pronostici!$S21)</f>
         <v/>
       </c>
     </row>
@@ -9852,23 +9451,23 @@
         <v/>
       </c>
       <c r="D22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$F22&lt;&gt;"",Pronostici!$G22&lt;&gt;"",Pronostici!$F22=Partite!$G22,Pronostici!$G22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$P22)=1),Config!$D$9,Config!$D$6),IF(AND($J22&lt;&gt;"",$J22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$J22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$F22&lt;&gt;"",Pronostici!$G22&lt;&gt;"",Pronostici!$F22=Partite!$G22,Pronostici!$G22=Partite!$H22),Config!$D$6,IF(AND($J22&lt;&gt;"",$J22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$I22&lt;&gt;"",Pronostici!$J22&lt;&gt;"",Pronostici!$I22=Partite!$G22,Pronostici!$J22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$Q22)=1),Config!$D$9,Config!$D$6),IF(AND($K22&lt;&gt;"",$K22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$K22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$I22&lt;&gt;"",Pronostici!$J22&lt;&gt;"",Pronostici!$I22=Partite!$G22,Pronostici!$J22=Partite!$H22),Config!$D$6,IF(AND($K22&lt;&gt;"",$K22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$L22&lt;&gt;"",Pronostici!$M22&lt;&gt;"",Pronostici!$L22=Partite!$G22,Pronostici!$M22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$R22)=1),Config!$D$9,Config!$D$6),IF(AND($L22&lt;&gt;"",$L22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$L22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$L22&lt;&gt;"",Pronostici!$M22&lt;&gt;"",Pronostici!$L22=Partite!$G22,Pronostici!$M22=Partite!$H22),Config!$D$6,IF(AND($L22&lt;&gt;"",$L22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$O22&lt;&gt;"",Pronostici!$P22&lt;&gt;"",Pronostici!$O22=Partite!$G22,Pronostici!$P22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$S22)=1),Config!$D$9,Config!$D$6),IF(AND($M22&lt;&gt;"",$M22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$M22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$O22&lt;&gt;"",Pronostici!$P22&lt;&gt;"",Pronostici!$O22=Partite!$G22,Pronostici!$P22=Partite!$H22),Config!$D$6,IF(AND($M22&lt;&gt;"",$M22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$R22&lt;&gt;"",Pronostici!$S22&lt;&gt;"",Pronostici!$R22=Partite!$G22,Pronostici!$S22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$T22)=1),Config!$D$9,Config!$D$6),IF(AND($N22&lt;&gt;"",$N22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$N22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$R22&lt;&gt;"",Pronostici!$S22&lt;&gt;"",Pronostici!$R22=Partite!$G22,Pronostici!$S22=Partite!$H22),Config!$D$6,IF(AND($N22&lt;&gt;"",$N22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J22" s="63">
@@ -9889,26 +9488,6 @@
       </c>
       <c r="N22" s="63">
         <f>IF(Pronostici!$Q22&lt;&gt;"",UPPER(Pronostici!$Q22),IF(OR(Pronostici!$R22="",Pronostici!$S22=""),"",IF(Pronostici!$R22&gt;Pronostici!$S22,"1",IF(Pronostici!$R22=Pronostici!$S22,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P22" s="63">
-        <f>IF(OR(Pronostici!$F22="",Pronostici!$G22=""),"",Pronostici!$F22&amp;" a "&amp;Pronostici!$G22)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="63">
-        <f>IF(OR(Pronostici!$I22="",Pronostici!$J22=""),"",Pronostici!$I22&amp;" a "&amp;Pronostici!$J22)</f>
-        <v/>
-      </c>
-      <c r="R22" s="63">
-        <f>IF(OR(Pronostici!$L22="",Pronostici!$M22=""),"",Pronostici!$L22&amp;" a "&amp;Pronostici!$M22)</f>
-        <v/>
-      </c>
-      <c r="S22" s="63">
-        <f>IF(OR(Pronostici!$O22="",Pronostici!$P22=""),"",Pronostici!$O22&amp;" a "&amp;Pronostici!$P22)</f>
-        <v/>
-      </c>
-      <c r="T22" s="63">
-        <f>IF(OR(Pronostici!$R22="",Pronostici!$S22=""),"",Pronostici!$R22&amp;" a "&amp;Pronostici!$S22)</f>
         <v/>
       </c>
     </row>
@@ -9926,23 +9505,23 @@
         <v/>
       </c>
       <c r="D23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$F23&lt;&gt;"",Pronostici!$G23&lt;&gt;"",Pronostici!$F23=Partite!$G23,Pronostici!$G23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$P23)=1),Config!$D$9,Config!$D$6),IF(AND($J23&lt;&gt;"",$J23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$J23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$F23&lt;&gt;"",Pronostici!$G23&lt;&gt;"",Pronostici!$F23=Partite!$G23,Pronostici!$G23=Partite!$H23),Config!$D$6,IF(AND($J23&lt;&gt;"",$J23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$I23&lt;&gt;"",Pronostici!$J23&lt;&gt;"",Pronostici!$I23=Partite!$G23,Pronostici!$J23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$Q23)=1),Config!$D$9,Config!$D$6),IF(AND($K23&lt;&gt;"",$K23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$K23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$I23&lt;&gt;"",Pronostici!$J23&lt;&gt;"",Pronostici!$I23=Partite!$G23,Pronostici!$J23=Partite!$H23),Config!$D$6,IF(AND($K23&lt;&gt;"",$K23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$L23&lt;&gt;"",Pronostici!$M23&lt;&gt;"",Pronostici!$L23=Partite!$G23,Pronostici!$M23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$R23)=1),Config!$D$9,Config!$D$6),IF(AND($L23&lt;&gt;"",$L23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$L23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$L23&lt;&gt;"",Pronostici!$M23&lt;&gt;"",Pronostici!$L23=Partite!$G23,Pronostici!$M23=Partite!$H23),Config!$D$6,IF(AND($L23&lt;&gt;"",$L23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$O23&lt;&gt;"",Pronostici!$P23&lt;&gt;"",Pronostici!$O23=Partite!$G23,Pronostici!$P23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$S23)=1),Config!$D$9,Config!$D$6),IF(AND($M23&lt;&gt;"",$M23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$M23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$O23&lt;&gt;"",Pronostici!$P23&lt;&gt;"",Pronostici!$O23=Partite!$G23,Pronostici!$P23=Partite!$H23),Config!$D$6,IF(AND($M23&lt;&gt;"",$M23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$R23&lt;&gt;"",Pronostici!$S23&lt;&gt;"",Pronostici!$R23=Partite!$G23,Pronostici!$S23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$T23)=1),Config!$D$9,Config!$D$6),IF(AND($N23&lt;&gt;"",$N23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$N23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$R23&lt;&gt;"",Pronostici!$S23&lt;&gt;"",Pronostici!$R23=Partite!$G23,Pronostici!$S23=Partite!$H23),Config!$D$6,IF(AND($N23&lt;&gt;"",$N23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J23" s="63">
@@ -9963,26 +9542,6 @@
       </c>
       <c r="N23" s="63">
         <f>IF(Pronostici!$Q23&lt;&gt;"",UPPER(Pronostici!$Q23),IF(OR(Pronostici!$R23="",Pronostici!$S23=""),"",IF(Pronostici!$R23&gt;Pronostici!$S23,"1",IF(Pronostici!$R23=Pronostici!$S23,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P23" s="63">
-        <f>IF(OR(Pronostici!$F23="",Pronostici!$G23=""),"",Pronostici!$F23&amp;" a "&amp;Pronostici!$G23)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="63">
-        <f>IF(OR(Pronostici!$I23="",Pronostici!$J23=""),"",Pronostici!$I23&amp;" a "&amp;Pronostici!$J23)</f>
-        <v/>
-      </c>
-      <c r="R23" s="63">
-        <f>IF(OR(Pronostici!$L23="",Pronostici!$M23=""),"",Pronostici!$L23&amp;" a "&amp;Pronostici!$M23)</f>
-        <v/>
-      </c>
-      <c r="S23" s="63">
-        <f>IF(OR(Pronostici!$O23="",Pronostici!$P23=""),"",Pronostici!$O23&amp;" a "&amp;Pronostici!$P23)</f>
-        <v/>
-      </c>
-      <c r="T23" s="63">
-        <f>IF(OR(Pronostici!$R23="",Pronostici!$S23=""),"",Pronostici!$R23&amp;" a "&amp;Pronostici!$S23)</f>
         <v/>
       </c>
     </row>
@@ -10000,23 +9559,23 @@
         <v/>
       </c>
       <c r="D24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$F24&lt;&gt;"",Pronostici!$G24&lt;&gt;"",Pronostici!$F24=Partite!$G24,Pronostici!$G24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$P24)=1),Config!$D$9,Config!$D$6),IF(AND($J24&lt;&gt;"",$J24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$J24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$F24&lt;&gt;"",Pronostici!$G24&lt;&gt;"",Pronostici!$F24=Partite!$G24,Pronostici!$G24=Partite!$H24),Config!$D$6,IF(AND($J24&lt;&gt;"",$J24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$I24&lt;&gt;"",Pronostici!$J24&lt;&gt;"",Pronostici!$I24=Partite!$G24,Pronostici!$J24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$Q24)=1),Config!$D$9,Config!$D$6),IF(AND($K24&lt;&gt;"",$K24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$K24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$I24&lt;&gt;"",Pronostici!$J24&lt;&gt;"",Pronostici!$I24=Partite!$G24,Pronostici!$J24=Partite!$H24),Config!$D$6,IF(AND($K24&lt;&gt;"",$K24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$L24&lt;&gt;"",Pronostici!$M24&lt;&gt;"",Pronostici!$L24=Partite!$G24,Pronostici!$M24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$R24)=1),Config!$D$9,Config!$D$6),IF(AND($L24&lt;&gt;"",$L24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$L24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$L24&lt;&gt;"",Pronostici!$M24&lt;&gt;"",Pronostici!$L24=Partite!$G24,Pronostici!$M24=Partite!$H24),Config!$D$6,IF(AND($L24&lt;&gt;"",$L24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$O24&lt;&gt;"",Pronostici!$P24&lt;&gt;"",Pronostici!$O24=Partite!$G24,Pronostici!$P24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$S24)=1),Config!$D$9,Config!$D$6),IF(AND($M24&lt;&gt;"",$M24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$M24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$O24&lt;&gt;"",Pronostici!$P24&lt;&gt;"",Pronostici!$O24=Partite!$G24,Pronostici!$P24=Partite!$H24),Config!$D$6,IF(AND($M24&lt;&gt;"",$M24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$R24&lt;&gt;"",Pronostici!$S24&lt;&gt;"",Pronostici!$R24=Partite!$G24,Pronostici!$S24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$T24)=1),Config!$D$9,Config!$D$6),IF(AND($N24&lt;&gt;"",$N24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$N24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$R24&lt;&gt;"",Pronostici!$S24&lt;&gt;"",Pronostici!$R24=Partite!$G24,Pronostici!$S24=Partite!$H24),Config!$D$6,IF(AND($N24&lt;&gt;"",$N24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J24" s="63">
@@ -10037,26 +9596,6 @@
       </c>
       <c r="N24" s="63">
         <f>IF(Pronostici!$Q24&lt;&gt;"",UPPER(Pronostici!$Q24),IF(OR(Pronostici!$R24="",Pronostici!$S24=""),"",IF(Pronostici!$R24&gt;Pronostici!$S24,"1",IF(Pronostici!$R24=Pronostici!$S24,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P24" s="63">
-        <f>IF(OR(Pronostici!$F24="",Pronostici!$G24=""),"",Pronostici!$F24&amp;" a "&amp;Pronostici!$G24)</f>
-        <v/>
-      </c>
-      <c r="Q24" s="63">
-        <f>IF(OR(Pronostici!$I24="",Pronostici!$J24=""),"",Pronostici!$I24&amp;" a "&amp;Pronostici!$J24)</f>
-        <v/>
-      </c>
-      <c r="R24" s="63">
-        <f>IF(OR(Pronostici!$L24="",Pronostici!$M24=""),"",Pronostici!$L24&amp;" a "&amp;Pronostici!$M24)</f>
-        <v/>
-      </c>
-      <c r="S24" s="63">
-        <f>IF(OR(Pronostici!$O24="",Pronostici!$P24=""),"",Pronostici!$O24&amp;" a "&amp;Pronostici!$P24)</f>
-        <v/>
-      </c>
-      <c r="T24" s="63">
-        <f>IF(OR(Pronostici!$R24="",Pronostici!$S24=""),"",Pronostici!$R24&amp;" a "&amp;Pronostici!$S24)</f>
         <v/>
       </c>
     </row>
@@ -10074,23 +9613,23 @@
         <v/>
       </c>
       <c r="D25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$F25&lt;&gt;"",Pronostici!$G25&lt;&gt;"",Pronostici!$F25=Partite!$G25,Pronostici!$G25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$P25)=1),Config!$D$9,Config!$D$6),IF(AND($J25&lt;&gt;"",$J25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$J25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$F25&lt;&gt;"",Pronostici!$G25&lt;&gt;"",Pronostici!$F25=Partite!$G25,Pronostici!$G25=Partite!$H25),Config!$D$6,IF(AND($J25&lt;&gt;"",$J25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$I25&lt;&gt;"",Pronostici!$J25&lt;&gt;"",Pronostici!$I25=Partite!$G25,Pronostici!$J25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$Q25)=1),Config!$D$9,Config!$D$6),IF(AND($K25&lt;&gt;"",$K25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$K25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$I25&lt;&gt;"",Pronostici!$J25&lt;&gt;"",Pronostici!$I25=Partite!$G25,Pronostici!$J25=Partite!$H25),Config!$D$6,IF(AND($K25&lt;&gt;"",$K25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$L25&lt;&gt;"",Pronostici!$M25&lt;&gt;"",Pronostici!$L25=Partite!$G25,Pronostici!$M25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$R25)=1),Config!$D$9,Config!$D$6),IF(AND($L25&lt;&gt;"",$L25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$L25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$L25&lt;&gt;"",Pronostici!$M25&lt;&gt;"",Pronostici!$L25=Partite!$G25,Pronostici!$M25=Partite!$H25),Config!$D$6,IF(AND($L25&lt;&gt;"",$L25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$O25&lt;&gt;"",Pronostici!$P25&lt;&gt;"",Pronostici!$O25=Partite!$G25,Pronostici!$P25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$S25)=1),Config!$D$9,Config!$D$6),IF(AND($M25&lt;&gt;"",$M25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$M25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$O25&lt;&gt;"",Pronostici!$P25&lt;&gt;"",Pronostici!$O25=Partite!$G25,Pronostici!$P25=Partite!$H25),Config!$D$6,IF(AND($M25&lt;&gt;"",$M25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$R25&lt;&gt;"",Pronostici!$S25&lt;&gt;"",Pronostici!$R25=Partite!$G25,Pronostici!$S25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$T25)=1),Config!$D$9,Config!$D$6),IF(AND($N25&lt;&gt;"",$N25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$N25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$R25&lt;&gt;"",Pronostici!$S25&lt;&gt;"",Pronostici!$R25=Partite!$G25,Pronostici!$S25=Partite!$H25),Config!$D$6,IF(AND($N25&lt;&gt;"",$N25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J25" s="63">
@@ -10111,26 +9650,6 @@
       </c>
       <c r="N25" s="63">
         <f>IF(Pronostici!$Q25&lt;&gt;"",UPPER(Pronostici!$Q25),IF(OR(Pronostici!$R25="",Pronostici!$S25=""),"",IF(Pronostici!$R25&gt;Pronostici!$S25,"1",IF(Pronostici!$R25=Pronostici!$S25,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P25" s="63">
-        <f>IF(OR(Pronostici!$F25="",Pronostici!$G25=""),"",Pronostici!$F25&amp;" a "&amp;Pronostici!$G25)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="63">
-        <f>IF(OR(Pronostici!$I25="",Pronostici!$J25=""),"",Pronostici!$I25&amp;" a "&amp;Pronostici!$J25)</f>
-        <v/>
-      </c>
-      <c r="R25" s="63">
-        <f>IF(OR(Pronostici!$L25="",Pronostici!$M25=""),"",Pronostici!$L25&amp;" a "&amp;Pronostici!$M25)</f>
-        <v/>
-      </c>
-      <c r="S25" s="63">
-        <f>IF(OR(Pronostici!$O25="",Pronostici!$P25=""),"",Pronostici!$O25&amp;" a "&amp;Pronostici!$P25)</f>
-        <v/>
-      </c>
-      <c r="T25" s="63">
-        <f>IF(OR(Pronostici!$R25="",Pronostici!$S25=""),"",Pronostici!$R25&amp;" a "&amp;Pronostici!$S25)</f>
         <v/>
       </c>
     </row>
@@ -10148,23 +9667,23 @@
         <v/>
       </c>
       <c r="D26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$F26&lt;&gt;"",Pronostici!$G26&lt;&gt;"",Pronostici!$F26=Partite!$G26,Pronostici!$G26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$P26)=1),Config!$D$9,Config!$D$6),IF(AND($J26&lt;&gt;"",$J26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$J26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$F26&lt;&gt;"",Pronostici!$G26&lt;&gt;"",Pronostici!$F26=Partite!$G26,Pronostici!$G26=Partite!$H26),Config!$D$6,IF(AND($J26&lt;&gt;"",$J26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$I26&lt;&gt;"",Pronostici!$J26&lt;&gt;"",Pronostici!$I26=Partite!$G26,Pronostici!$J26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$Q26)=1),Config!$D$9,Config!$D$6),IF(AND($K26&lt;&gt;"",$K26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$K26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$I26&lt;&gt;"",Pronostici!$J26&lt;&gt;"",Pronostici!$I26=Partite!$G26,Pronostici!$J26=Partite!$H26),Config!$D$6,IF(AND($K26&lt;&gt;"",$K26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$L26&lt;&gt;"",Pronostici!$M26&lt;&gt;"",Pronostici!$L26=Partite!$G26,Pronostici!$M26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$R26)=1),Config!$D$9,Config!$D$6),IF(AND($L26&lt;&gt;"",$L26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$L26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$L26&lt;&gt;"",Pronostici!$M26&lt;&gt;"",Pronostici!$L26=Partite!$G26,Pronostici!$M26=Partite!$H26),Config!$D$6,IF(AND($L26&lt;&gt;"",$L26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$O26&lt;&gt;"",Pronostici!$P26&lt;&gt;"",Pronostici!$O26=Partite!$G26,Pronostici!$P26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$S26)=1),Config!$D$9,Config!$D$6),IF(AND($M26&lt;&gt;"",$M26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$M26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$O26&lt;&gt;"",Pronostici!$P26&lt;&gt;"",Pronostici!$O26=Partite!$G26,Pronostici!$P26=Partite!$H26),Config!$D$6,IF(AND($M26&lt;&gt;"",$M26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$R26&lt;&gt;"",Pronostici!$S26&lt;&gt;"",Pronostici!$R26=Partite!$G26,Pronostici!$S26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$T26)=1),Config!$D$9,Config!$D$6),IF(AND($N26&lt;&gt;"",$N26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$N26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$R26&lt;&gt;"",Pronostici!$S26&lt;&gt;"",Pronostici!$R26=Partite!$G26,Pronostici!$S26=Partite!$H26),Config!$D$6,IF(AND($N26&lt;&gt;"",$N26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J26" s="63">
@@ -10185,26 +9704,6 @@
       </c>
       <c r="N26" s="63">
         <f>IF(Pronostici!$Q26&lt;&gt;"",UPPER(Pronostici!$Q26),IF(OR(Pronostici!$R26="",Pronostici!$S26=""),"",IF(Pronostici!$R26&gt;Pronostici!$S26,"1",IF(Pronostici!$R26=Pronostici!$S26,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P26" s="63">
-        <f>IF(OR(Pronostici!$F26="",Pronostici!$G26=""),"",Pronostici!$F26&amp;" a "&amp;Pronostici!$G26)</f>
-        <v/>
-      </c>
-      <c r="Q26" s="63">
-        <f>IF(OR(Pronostici!$I26="",Pronostici!$J26=""),"",Pronostici!$I26&amp;" a "&amp;Pronostici!$J26)</f>
-        <v/>
-      </c>
-      <c r="R26" s="63">
-        <f>IF(OR(Pronostici!$L26="",Pronostici!$M26=""),"",Pronostici!$L26&amp;" a "&amp;Pronostici!$M26)</f>
-        <v/>
-      </c>
-      <c r="S26" s="63">
-        <f>IF(OR(Pronostici!$O26="",Pronostici!$P26=""),"",Pronostici!$O26&amp;" a "&amp;Pronostici!$P26)</f>
-        <v/>
-      </c>
-      <c r="T26" s="63">
-        <f>IF(OR(Pronostici!$R26="",Pronostici!$S26=""),"",Pronostici!$R26&amp;" a "&amp;Pronostici!$S26)</f>
         <v/>
       </c>
     </row>
@@ -10222,23 +9721,23 @@
         <v/>
       </c>
       <c r="D27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$F27&lt;&gt;"",Pronostici!$G27&lt;&gt;"",Pronostici!$F27=Partite!$G27,Pronostici!$G27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$P27)=1),Config!$D$9,Config!$D$6),IF(AND($J27&lt;&gt;"",$J27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$J27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$F27&lt;&gt;"",Pronostici!$G27&lt;&gt;"",Pronostici!$F27=Partite!$G27,Pronostici!$G27=Partite!$H27),Config!$D$6,IF(AND($J27&lt;&gt;"",$J27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$I27&lt;&gt;"",Pronostici!$J27&lt;&gt;"",Pronostici!$I27=Partite!$G27,Pronostici!$J27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$Q27)=1),Config!$D$9,Config!$D$6),IF(AND($K27&lt;&gt;"",$K27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$K27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$I27&lt;&gt;"",Pronostici!$J27&lt;&gt;"",Pronostici!$I27=Partite!$G27,Pronostici!$J27=Partite!$H27),Config!$D$6,IF(AND($K27&lt;&gt;"",$K27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$L27&lt;&gt;"",Pronostici!$M27&lt;&gt;"",Pronostici!$L27=Partite!$G27,Pronostici!$M27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$R27)=1),Config!$D$9,Config!$D$6),IF(AND($L27&lt;&gt;"",$L27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$L27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$L27&lt;&gt;"",Pronostici!$M27&lt;&gt;"",Pronostici!$L27=Partite!$G27,Pronostici!$M27=Partite!$H27),Config!$D$6,IF(AND($L27&lt;&gt;"",$L27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$O27&lt;&gt;"",Pronostici!$P27&lt;&gt;"",Pronostici!$O27=Partite!$G27,Pronostici!$P27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$S27)=1),Config!$D$9,Config!$D$6),IF(AND($M27&lt;&gt;"",$M27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$M27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$O27&lt;&gt;"",Pronostici!$P27&lt;&gt;"",Pronostici!$O27=Partite!$G27,Pronostici!$P27=Partite!$H27),Config!$D$6,IF(AND($M27&lt;&gt;"",$M27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$R27&lt;&gt;"",Pronostici!$S27&lt;&gt;"",Pronostici!$R27=Partite!$G27,Pronostici!$S27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$T27)=1),Config!$D$9,Config!$D$6),IF(AND($N27&lt;&gt;"",$N27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$N27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$R27&lt;&gt;"",Pronostici!$S27&lt;&gt;"",Pronostici!$R27=Partite!$G27,Pronostici!$S27=Partite!$H27),Config!$D$6,IF(AND($N27&lt;&gt;"",$N27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J27" s="63">
@@ -10259,26 +9758,6 @@
       </c>
       <c r="N27" s="63">
         <f>IF(Pronostici!$Q27&lt;&gt;"",UPPER(Pronostici!$Q27),IF(OR(Pronostici!$R27="",Pronostici!$S27=""),"",IF(Pronostici!$R27&gt;Pronostici!$S27,"1",IF(Pronostici!$R27=Pronostici!$S27,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P27" s="63">
-        <f>IF(OR(Pronostici!$F27="",Pronostici!$G27=""),"",Pronostici!$F27&amp;" a "&amp;Pronostici!$G27)</f>
-        <v/>
-      </c>
-      <c r="Q27" s="63">
-        <f>IF(OR(Pronostici!$I27="",Pronostici!$J27=""),"",Pronostici!$I27&amp;" a "&amp;Pronostici!$J27)</f>
-        <v/>
-      </c>
-      <c r="R27" s="63">
-        <f>IF(OR(Pronostici!$L27="",Pronostici!$M27=""),"",Pronostici!$L27&amp;" a "&amp;Pronostici!$M27)</f>
-        <v/>
-      </c>
-      <c r="S27" s="63">
-        <f>IF(OR(Pronostici!$O27="",Pronostici!$P27=""),"",Pronostici!$O27&amp;" a "&amp;Pronostici!$P27)</f>
-        <v/>
-      </c>
-      <c r="T27" s="63">
-        <f>IF(OR(Pronostici!$R27="",Pronostici!$S27=""),"",Pronostici!$R27&amp;" a "&amp;Pronostici!$S27)</f>
         <v/>
       </c>
     </row>
@@ -10296,23 +9775,23 @@
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$F28&lt;&gt;"",Pronostici!$G28&lt;&gt;"",Pronostici!$F28=Partite!$G28,Pronostici!$G28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$P28)=1),Config!$D$9,Config!$D$6),IF(AND($J28&lt;&gt;"",$J28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$J28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$F28&lt;&gt;"",Pronostici!$G28&lt;&gt;"",Pronostici!$F28=Partite!$G28,Pronostici!$G28=Partite!$H28),Config!$D$6,IF(AND($J28&lt;&gt;"",$J28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$I28&lt;&gt;"",Pronostici!$J28&lt;&gt;"",Pronostici!$I28=Partite!$G28,Pronostici!$J28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$Q28)=1),Config!$D$9,Config!$D$6),IF(AND($K28&lt;&gt;"",$K28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$K28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$I28&lt;&gt;"",Pronostici!$J28&lt;&gt;"",Pronostici!$I28=Partite!$G28,Pronostici!$J28=Partite!$H28),Config!$D$6,IF(AND($K28&lt;&gt;"",$K28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$L28&lt;&gt;"",Pronostici!$M28&lt;&gt;"",Pronostici!$L28=Partite!$G28,Pronostici!$M28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$R28)=1),Config!$D$9,Config!$D$6),IF(AND($L28&lt;&gt;"",$L28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$L28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$L28&lt;&gt;"",Pronostici!$M28&lt;&gt;"",Pronostici!$L28=Partite!$G28,Pronostici!$M28=Partite!$H28),Config!$D$6,IF(AND($L28&lt;&gt;"",$L28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$O28&lt;&gt;"",Pronostici!$P28&lt;&gt;"",Pronostici!$O28=Partite!$G28,Pronostici!$P28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$S28)=1),Config!$D$9,Config!$D$6),IF(AND($M28&lt;&gt;"",$M28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$M28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$O28&lt;&gt;"",Pronostici!$P28&lt;&gt;"",Pronostici!$O28=Partite!$G28,Pronostici!$P28=Partite!$H28),Config!$D$6,IF(AND($M28&lt;&gt;"",$M28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$R28&lt;&gt;"",Pronostici!$S28&lt;&gt;"",Pronostici!$R28=Partite!$G28,Pronostici!$S28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$T28)=1),Config!$D$9,Config!$D$6),IF(AND($N28&lt;&gt;"",$N28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$N28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$R28&lt;&gt;"",Pronostici!$S28&lt;&gt;"",Pronostici!$R28=Partite!$G28,Pronostici!$S28=Partite!$H28),Config!$D$6,IF(AND($N28&lt;&gt;"",$N28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J28" s="63">
@@ -10333,26 +9812,6 @@
       </c>
       <c r="N28" s="63">
         <f>IF(Pronostici!$Q28&lt;&gt;"",UPPER(Pronostici!$Q28),IF(OR(Pronostici!$R28="",Pronostici!$S28=""),"",IF(Pronostici!$R28&gt;Pronostici!$S28,"1",IF(Pronostici!$R28=Pronostici!$S28,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P28" s="63">
-        <f>IF(OR(Pronostici!$F28="",Pronostici!$G28=""),"",Pronostici!$F28&amp;" a "&amp;Pronostici!$G28)</f>
-        <v/>
-      </c>
-      <c r="Q28" s="63">
-        <f>IF(OR(Pronostici!$I28="",Pronostici!$J28=""),"",Pronostici!$I28&amp;" a "&amp;Pronostici!$J28)</f>
-        <v/>
-      </c>
-      <c r="R28" s="63">
-        <f>IF(OR(Pronostici!$L28="",Pronostici!$M28=""),"",Pronostici!$L28&amp;" a "&amp;Pronostici!$M28)</f>
-        <v/>
-      </c>
-      <c r="S28" s="63">
-        <f>IF(OR(Pronostici!$O28="",Pronostici!$P28=""),"",Pronostici!$O28&amp;" a "&amp;Pronostici!$P28)</f>
-        <v/>
-      </c>
-      <c r="T28" s="63">
-        <f>IF(OR(Pronostici!$R28="",Pronostici!$S28=""),"",Pronostici!$R28&amp;" a "&amp;Pronostici!$S28)</f>
         <v/>
       </c>
     </row>
@@ -10370,23 +9829,23 @@
         <v/>
       </c>
       <c r="D29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$F29&lt;&gt;"",Pronostici!$G29&lt;&gt;"",Pronostici!$F29=Partite!$G29,Pronostici!$G29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$P29)=1),Config!$D$9,Config!$D$6),IF(AND($J29&lt;&gt;"",$J29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$J29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$F29&lt;&gt;"",Pronostici!$G29&lt;&gt;"",Pronostici!$F29=Partite!$G29,Pronostici!$G29=Partite!$H29),Config!$D$6,IF(AND($J29&lt;&gt;"",$J29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$I29&lt;&gt;"",Pronostici!$J29&lt;&gt;"",Pronostici!$I29=Partite!$G29,Pronostici!$J29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$Q29)=1),Config!$D$9,Config!$D$6),IF(AND($K29&lt;&gt;"",$K29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$K29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$I29&lt;&gt;"",Pronostici!$J29&lt;&gt;"",Pronostici!$I29=Partite!$G29,Pronostici!$J29=Partite!$H29),Config!$D$6,IF(AND($K29&lt;&gt;"",$K29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$L29&lt;&gt;"",Pronostici!$M29&lt;&gt;"",Pronostici!$L29=Partite!$G29,Pronostici!$M29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$R29)=1),Config!$D$9,Config!$D$6),IF(AND($L29&lt;&gt;"",$L29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$L29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$L29&lt;&gt;"",Pronostici!$M29&lt;&gt;"",Pronostici!$L29=Partite!$G29,Pronostici!$M29=Partite!$H29),Config!$D$6,IF(AND($L29&lt;&gt;"",$L29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$O29&lt;&gt;"",Pronostici!$P29&lt;&gt;"",Pronostici!$O29=Partite!$G29,Pronostici!$P29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$S29)=1),Config!$D$9,Config!$D$6),IF(AND($M29&lt;&gt;"",$M29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$M29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$O29&lt;&gt;"",Pronostici!$P29&lt;&gt;"",Pronostici!$O29=Partite!$G29,Pronostici!$P29=Partite!$H29),Config!$D$6,IF(AND($M29&lt;&gt;"",$M29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$R29&lt;&gt;"",Pronostici!$S29&lt;&gt;"",Pronostici!$R29=Partite!$G29,Pronostici!$S29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$T29)=1),Config!$D$9,Config!$D$6),IF(AND($N29&lt;&gt;"",$N29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$N29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$R29&lt;&gt;"",Pronostici!$S29&lt;&gt;"",Pronostici!$R29=Partite!$G29,Pronostici!$S29=Partite!$H29),Config!$D$6,IF(AND($N29&lt;&gt;"",$N29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J29" s="63">
@@ -10407,26 +9866,6 @@
       </c>
       <c r="N29" s="63">
         <f>IF(Pronostici!$Q29&lt;&gt;"",UPPER(Pronostici!$Q29),IF(OR(Pronostici!$R29="",Pronostici!$S29=""),"",IF(Pronostici!$R29&gt;Pronostici!$S29,"1",IF(Pronostici!$R29=Pronostici!$S29,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P29" s="63">
-        <f>IF(OR(Pronostici!$F29="",Pronostici!$G29=""),"",Pronostici!$F29&amp;" a "&amp;Pronostici!$G29)</f>
-        <v/>
-      </c>
-      <c r="Q29" s="63">
-        <f>IF(OR(Pronostici!$I29="",Pronostici!$J29=""),"",Pronostici!$I29&amp;" a "&amp;Pronostici!$J29)</f>
-        <v/>
-      </c>
-      <c r="R29" s="63">
-        <f>IF(OR(Pronostici!$L29="",Pronostici!$M29=""),"",Pronostici!$L29&amp;" a "&amp;Pronostici!$M29)</f>
-        <v/>
-      </c>
-      <c r="S29" s="63">
-        <f>IF(OR(Pronostici!$O29="",Pronostici!$P29=""),"",Pronostici!$O29&amp;" a "&amp;Pronostici!$P29)</f>
-        <v/>
-      </c>
-      <c r="T29" s="63">
-        <f>IF(OR(Pronostici!$R29="",Pronostici!$S29=""),"",Pronostici!$R29&amp;" a "&amp;Pronostici!$S29)</f>
         <v/>
       </c>
     </row>
@@ -10444,23 +9883,23 @@
         <v/>
       </c>
       <c r="D30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$F30&lt;&gt;"",Pronostici!$G30&lt;&gt;"",Pronostici!$F30=Partite!$G30,Pronostici!$G30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$P30)=1),Config!$D$9,Config!$D$6),IF(AND($J30&lt;&gt;"",$J30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$J30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$F30&lt;&gt;"",Pronostici!$G30&lt;&gt;"",Pronostici!$F30=Partite!$G30,Pronostici!$G30=Partite!$H30),Config!$D$6,IF(AND($J30&lt;&gt;"",$J30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$I30&lt;&gt;"",Pronostici!$J30&lt;&gt;"",Pronostici!$I30=Partite!$G30,Pronostici!$J30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$Q30)=1),Config!$D$9,Config!$D$6),IF(AND($K30&lt;&gt;"",$K30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$K30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$I30&lt;&gt;"",Pronostici!$J30&lt;&gt;"",Pronostici!$I30=Partite!$G30,Pronostici!$J30=Partite!$H30),Config!$D$6,IF(AND($K30&lt;&gt;"",$K30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$L30&lt;&gt;"",Pronostici!$M30&lt;&gt;"",Pronostici!$L30=Partite!$G30,Pronostici!$M30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$R30)=1),Config!$D$9,Config!$D$6),IF(AND($L30&lt;&gt;"",$L30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$L30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$L30&lt;&gt;"",Pronostici!$M30&lt;&gt;"",Pronostici!$L30=Partite!$G30,Pronostici!$M30=Partite!$H30),Config!$D$6,IF(AND($L30&lt;&gt;"",$L30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$O30&lt;&gt;"",Pronostici!$P30&lt;&gt;"",Pronostici!$O30=Partite!$G30,Pronostici!$P30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$S30)=1),Config!$D$9,Config!$D$6),IF(AND($M30&lt;&gt;"",$M30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$M30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$O30&lt;&gt;"",Pronostici!$P30&lt;&gt;"",Pronostici!$O30=Partite!$G30,Pronostici!$P30=Partite!$H30),Config!$D$6,IF(AND($M30&lt;&gt;"",$M30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$R30&lt;&gt;"",Pronostici!$S30&lt;&gt;"",Pronostici!$R30=Partite!$G30,Pronostici!$S30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$T30)=1),Config!$D$9,Config!$D$6),IF(AND($N30&lt;&gt;"",$N30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$N30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$R30&lt;&gt;"",Pronostici!$S30&lt;&gt;"",Pronostici!$R30=Partite!$G30,Pronostici!$S30=Partite!$H30),Config!$D$6,IF(AND($N30&lt;&gt;"",$N30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J30" s="63">
@@ -10481,26 +9920,6 @@
       </c>
       <c r="N30" s="63">
         <f>IF(Pronostici!$Q30&lt;&gt;"",UPPER(Pronostici!$Q30),IF(OR(Pronostici!$R30="",Pronostici!$S30=""),"",IF(Pronostici!$R30&gt;Pronostici!$S30,"1",IF(Pronostici!$R30=Pronostici!$S30,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P30" s="63">
-        <f>IF(OR(Pronostici!$F30="",Pronostici!$G30=""),"",Pronostici!$F30&amp;" a "&amp;Pronostici!$G30)</f>
-        <v/>
-      </c>
-      <c r="Q30" s="63">
-        <f>IF(OR(Pronostici!$I30="",Pronostici!$J30=""),"",Pronostici!$I30&amp;" a "&amp;Pronostici!$J30)</f>
-        <v/>
-      </c>
-      <c r="R30" s="63">
-        <f>IF(OR(Pronostici!$L30="",Pronostici!$M30=""),"",Pronostici!$L30&amp;" a "&amp;Pronostici!$M30)</f>
-        <v/>
-      </c>
-      <c r="S30" s="63">
-        <f>IF(OR(Pronostici!$O30="",Pronostici!$P30=""),"",Pronostici!$O30&amp;" a "&amp;Pronostici!$P30)</f>
-        <v/>
-      </c>
-      <c r="T30" s="63">
-        <f>IF(OR(Pronostici!$R30="",Pronostici!$S30=""),"",Pronostici!$R30&amp;" a "&amp;Pronostici!$S30)</f>
         <v/>
       </c>
     </row>
@@ -10518,23 +9937,23 @@
         <v/>
       </c>
       <c r="D31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$F31&lt;&gt;"",Pronostici!$G31&lt;&gt;"",Pronostici!$F31=Partite!$G31,Pronostici!$G31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$P31)=1),Config!$D$9,Config!$D$6),IF(AND($J31&lt;&gt;"",$J31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$J31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$F31&lt;&gt;"",Pronostici!$G31&lt;&gt;"",Pronostici!$F31=Partite!$G31,Pronostici!$G31=Partite!$H31),Config!$D$6,IF(AND($J31&lt;&gt;"",$J31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$I31&lt;&gt;"",Pronostici!$J31&lt;&gt;"",Pronostici!$I31=Partite!$G31,Pronostici!$J31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$Q31)=1),Config!$D$9,Config!$D$6),IF(AND($K31&lt;&gt;"",$K31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$K31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$I31&lt;&gt;"",Pronostici!$J31&lt;&gt;"",Pronostici!$I31=Partite!$G31,Pronostici!$J31=Partite!$H31),Config!$D$6,IF(AND($K31&lt;&gt;"",$K31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$L31&lt;&gt;"",Pronostici!$M31&lt;&gt;"",Pronostici!$L31=Partite!$G31,Pronostici!$M31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$R31)=1),Config!$D$9,Config!$D$6),IF(AND($L31&lt;&gt;"",$L31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$L31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$L31&lt;&gt;"",Pronostici!$M31&lt;&gt;"",Pronostici!$L31=Partite!$G31,Pronostici!$M31=Partite!$H31),Config!$D$6,IF(AND($L31&lt;&gt;"",$L31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$O31&lt;&gt;"",Pronostici!$P31&lt;&gt;"",Pronostici!$O31=Partite!$G31,Pronostici!$P31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$S31)=1),Config!$D$9,Config!$D$6),IF(AND($M31&lt;&gt;"",$M31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$M31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$O31&lt;&gt;"",Pronostici!$P31&lt;&gt;"",Pronostici!$O31=Partite!$G31,Pronostici!$P31=Partite!$H31),Config!$D$6,IF(AND($M31&lt;&gt;"",$M31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$R31&lt;&gt;"",Pronostici!$S31&lt;&gt;"",Pronostici!$R31=Partite!$G31,Pronostici!$S31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$T31)=1),Config!$D$9,Config!$D$6),IF(AND($N31&lt;&gt;"",$N31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$N31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$R31&lt;&gt;"",Pronostici!$S31&lt;&gt;"",Pronostici!$R31=Partite!$G31,Pronostici!$S31=Partite!$H31),Config!$D$6,IF(AND($N31&lt;&gt;"",$N31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J31" s="63">
@@ -10555,26 +9974,6 @@
       </c>
       <c r="N31" s="63">
         <f>IF(Pronostici!$Q31&lt;&gt;"",UPPER(Pronostici!$Q31),IF(OR(Pronostici!$R31="",Pronostici!$S31=""),"",IF(Pronostici!$R31&gt;Pronostici!$S31,"1",IF(Pronostici!$R31=Pronostici!$S31,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P31" s="63">
-        <f>IF(OR(Pronostici!$F31="",Pronostici!$G31=""),"",Pronostici!$F31&amp;" a "&amp;Pronostici!$G31)</f>
-        <v/>
-      </c>
-      <c r="Q31" s="63">
-        <f>IF(OR(Pronostici!$I31="",Pronostici!$J31=""),"",Pronostici!$I31&amp;" a "&amp;Pronostici!$J31)</f>
-        <v/>
-      </c>
-      <c r="R31" s="63">
-        <f>IF(OR(Pronostici!$L31="",Pronostici!$M31=""),"",Pronostici!$L31&amp;" a "&amp;Pronostici!$M31)</f>
-        <v/>
-      </c>
-      <c r="S31" s="63">
-        <f>IF(OR(Pronostici!$O31="",Pronostici!$P31=""),"",Pronostici!$O31&amp;" a "&amp;Pronostici!$P31)</f>
-        <v/>
-      </c>
-      <c r="T31" s="63">
-        <f>IF(OR(Pronostici!$R31="",Pronostici!$S31=""),"",Pronostici!$R31&amp;" a "&amp;Pronostici!$S31)</f>
         <v/>
       </c>
     </row>
@@ -10592,23 +9991,23 @@
         <v/>
       </c>
       <c r="D32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$F32&lt;&gt;"",Pronostici!$G32&lt;&gt;"",Pronostici!$F32=Partite!$G32,Pronostici!$G32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$P32)=1),Config!$D$9,Config!$D$6),IF(AND($J32&lt;&gt;"",$J32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$J32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$F32&lt;&gt;"",Pronostici!$G32&lt;&gt;"",Pronostici!$F32=Partite!$G32,Pronostici!$G32=Partite!$H32),Config!$D$6,IF(AND($J32&lt;&gt;"",$J32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$I32&lt;&gt;"",Pronostici!$J32&lt;&gt;"",Pronostici!$I32=Partite!$G32,Pronostici!$J32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$Q32)=1),Config!$D$9,Config!$D$6),IF(AND($K32&lt;&gt;"",$K32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$K32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$I32&lt;&gt;"",Pronostici!$J32&lt;&gt;"",Pronostici!$I32=Partite!$G32,Pronostici!$J32=Partite!$H32),Config!$D$6,IF(AND($K32&lt;&gt;"",$K32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$L32&lt;&gt;"",Pronostici!$M32&lt;&gt;"",Pronostici!$L32=Partite!$G32,Pronostici!$M32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$R32)=1),Config!$D$9,Config!$D$6),IF(AND($L32&lt;&gt;"",$L32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$L32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$L32&lt;&gt;"",Pronostici!$M32&lt;&gt;"",Pronostici!$L32=Partite!$G32,Pronostici!$M32=Partite!$H32),Config!$D$6,IF(AND($L32&lt;&gt;"",$L32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$O32&lt;&gt;"",Pronostici!$P32&lt;&gt;"",Pronostici!$O32=Partite!$G32,Pronostici!$P32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$S32)=1),Config!$D$9,Config!$D$6),IF(AND($M32&lt;&gt;"",$M32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$M32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$O32&lt;&gt;"",Pronostici!$P32&lt;&gt;"",Pronostici!$O32=Partite!$G32,Pronostici!$P32=Partite!$H32),Config!$D$6,IF(AND($M32&lt;&gt;"",$M32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$R32&lt;&gt;"",Pronostici!$S32&lt;&gt;"",Pronostici!$R32=Partite!$G32,Pronostici!$S32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$T32)=1),Config!$D$9,Config!$D$6),IF(AND($N32&lt;&gt;"",$N32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$N32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$R32&lt;&gt;"",Pronostici!$S32&lt;&gt;"",Pronostici!$R32=Partite!$G32,Pronostici!$S32=Partite!$H32),Config!$D$6,IF(AND($N32&lt;&gt;"",$N32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J32" s="63">
@@ -10629,26 +10028,6 @@
       </c>
       <c r="N32" s="63">
         <f>IF(Pronostici!$Q32&lt;&gt;"",UPPER(Pronostici!$Q32),IF(OR(Pronostici!$R32="",Pronostici!$S32=""),"",IF(Pronostici!$R32&gt;Pronostici!$S32,"1",IF(Pronostici!$R32=Pronostici!$S32,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P32" s="63">
-        <f>IF(OR(Pronostici!$F32="",Pronostici!$G32=""),"",Pronostici!$F32&amp;" a "&amp;Pronostici!$G32)</f>
-        <v/>
-      </c>
-      <c r="Q32" s="63">
-        <f>IF(OR(Pronostici!$I32="",Pronostici!$J32=""),"",Pronostici!$I32&amp;" a "&amp;Pronostici!$J32)</f>
-        <v/>
-      </c>
-      <c r="R32" s="63">
-        <f>IF(OR(Pronostici!$L32="",Pronostici!$M32=""),"",Pronostici!$L32&amp;" a "&amp;Pronostici!$M32)</f>
-        <v/>
-      </c>
-      <c r="S32" s="63">
-        <f>IF(OR(Pronostici!$O32="",Pronostici!$P32=""),"",Pronostici!$O32&amp;" a "&amp;Pronostici!$P32)</f>
-        <v/>
-      </c>
-      <c r="T32" s="63">
-        <f>IF(OR(Pronostici!$R32="",Pronostici!$S32=""),"",Pronostici!$R32&amp;" a "&amp;Pronostici!$S32)</f>
         <v/>
       </c>
     </row>
@@ -10666,23 +10045,23 @@
         <v/>
       </c>
       <c r="D33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$F33&lt;&gt;"",Pronostici!$G33&lt;&gt;"",Pronostici!$F33=Partite!$G33,Pronostici!$G33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$P33)=1),Config!$D$9,Config!$D$6),IF(AND($J33&lt;&gt;"",$J33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$J33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$F33&lt;&gt;"",Pronostici!$G33&lt;&gt;"",Pronostici!$F33=Partite!$G33,Pronostici!$G33=Partite!$H33),Config!$D$6,IF(AND($J33&lt;&gt;"",$J33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$I33&lt;&gt;"",Pronostici!$J33&lt;&gt;"",Pronostici!$I33=Partite!$G33,Pronostici!$J33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$Q33)=1),Config!$D$9,Config!$D$6),IF(AND($K33&lt;&gt;"",$K33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$K33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$I33&lt;&gt;"",Pronostici!$J33&lt;&gt;"",Pronostici!$I33=Partite!$G33,Pronostici!$J33=Partite!$H33),Config!$D$6,IF(AND($K33&lt;&gt;"",$K33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$L33&lt;&gt;"",Pronostici!$M33&lt;&gt;"",Pronostici!$L33=Partite!$G33,Pronostici!$M33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$R33)=1),Config!$D$9,Config!$D$6),IF(AND($L33&lt;&gt;"",$L33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$L33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$L33&lt;&gt;"",Pronostici!$M33&lt;&gt;"",Pronostici!$L33=Partite!$G33,Pronostici!$M33=Partite!$H33),Config!$D$6,IF(AND($L33&lt;&gt;"",$L33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$O33&lt;&gt;"",Pronostici!$P33&lt;&gt;"",Pronostici!$O33=Partite!$G33,Pronostici!$P33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$S33)=1),Config!$D$9,Config!$D$6),IF(AND($M33&lt;&gt;"",$M33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$M33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$O33&lt;&gt;"",Pronostici!$P33&lt;&gt;"",Pronostici!$O33=Partite!$G33,Pronostici!$P33=Partite!$H33),Config!$D$6,IF(AND($M33&lt;&gt;"",$M33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$R33&lt;&gt;"",Pronostici!$S33&lt;&gt;"",Pronostici!$R33=Partite!$G33,Pronostici!$S33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$T33)=1),Config!$D$9,Config!$D$6),IF(AND($N33&lt;&gt;"",$N33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$N33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$R33&lt;&gt;"",Pronostici!$S33&lt;&gt;"",Pronostici!$R33=Partite!$G33,Pronostici!$S33=Partite!$H33),Config!$D$6,IF(AND($N33&lt;&gt;"",$N33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J33" s="63">
@@ -10703,26 +10082,6 @@
       </c>
       <c r="N33" s="63">
         <f>IF(Pronostici!$Q33&lt;&gt;"",UPPER(Pronostici!$Q33),IF(OR(Pronostici!$R33="",Pronostici!$S33=""),"",IF(Pronostici!$R33&gt;Pronostici!$S33,"1",IF(Pronostici!$R33=Pronostici!$S33,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P33" s="63">
-        <f>IF(OR(Pronostici!$F33="",Pronostici!$G33=""),"",Pronostici!$F33&amp;" a "&amp;Pronostici!$G33)</f>
-        <v/>
-      </c>
-      <c r="Q33" s="63">
-        <f>IF(OR(Pronostici!$I33="",Pronostici!$J33=""),"",Pronostici!$I33&amp;" a "&amp;Pronostici!$J33)</f>
-        <v/>
-      </c>
-      <c r="R33" s="63">
-        <f>IF(OR(Pronostici!$L33="",Pronostici!$M33=""),"",Pronostici!$L33&amp;" a "&amp;Pronostici!$M33)</f>
-        <v/>
-      </c>
-      <c r="S33" s="63">
-        <f>IF(OR(Pronostici!$O33="",Pronostici!$P33=""),"",Pronostici!$O33&amp;" a "&amp;Pronostici!$P33)</f>
-        <v/>
-      </c>
-      <c r="T33" s="63">
-        <f>IF(OR(Pronostici!$R33="",Pronostici!$S33=""),"",Pronostici!$R33&amp;" a "&amp;Pronostici!$S33)</f>
         <v/>
       </c>
     </row>
@@ -10740,23 +10099,23 @@
         <v/>
       </c>
       <c r="D34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$F34&lt;&gt;"",Pronostici!$G34&lt;&gt;"",Pronostici!$F34=Partite!$G34,Pronostici!$G34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$P34)=1),Config!$D$9,Config!$D$6),IF(AND($J34&lt;&gt;"",$J34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$J34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$F34&lt;&gt;"",Pronostici!$G34&lt;&gt;"",Pronostici!$F34=Partite!$G34,Pronostici!$G34=Partite!$H34),Config!$D$6,IF(AND($J34&lt;&gt;"",$J34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$I34&lt;&gt;"",Pronostici!$J34&lt;&gt;"",Pronostici!$I34=Partite!$G34,Pronostici!$J34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$Q34)=1),Config!$D$9,Config!$D$6),IF(AND($K34&lt;&gt;"",$K34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$K34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$I34&lt;&gt;"",Pronostici!$J34&lt;&gt;"",Pronostici!$I34=Partite!$G34,Pronostici!$J34=Partite!$H34),Config!$D$6,IF(AND($K34&lt;&gt;"",$K34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$L34&lt;&gt;"",Pronostici!$M34&lt;&gt;"",Pronostici!$L34=Partite!$G34,Pronostici!$M34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$R34)=1),Config!$D$9,Config!$D$6),IF(AND($L34&lt;&gt;"",$L34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$L34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$L34&lt;&gt;"",Pronostici!$M34&lt;&gt;"",Pronostici!$L34=Partite!$G34,Pronostici!$M34=Partite!$H34),Config!$D$6,IF(AND($L34&lt;&gt;"",$L34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$O34&lt;&gt;"",Pronostici!$P34&lt;&gt;"",Pronostici!$O34=Partite!$G34,Pronostici!$P34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$S34)=1),Config!$D$9,Config!$D$6),IF(AND($M34&lt;&gt;"",$M34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$M34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$O34&lt;&gt;"",Pronostici!$P34&lt;&gt;"",Pronostici!$O34=Partite!$G34,Pronostici!$P34=Partite!$H34),Config!$D$6,IF(AND($M34&lt;&gt;"",$M34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$R34&lt;&gt;"",Pronostici!$S34&lt;&gt;"",Pronostici!$R34=Partite!$G34,Pronostici!$S34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$T34)=1),Config!$D$9,Config!$D$6),IF(AND($N34&lt;&gt;"",$N34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$N34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$R34&lt;&gt;"",Pronostici!$S34&lt;&gt;"",Pronostici!$R34=Partite!$G34,Pronostici!$S34=Partite!$H34),Config!$D$6,IF(AND($N34&lt;&gt;"",$N34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J34" s="63">
@@ -10777,26 +10136,6 @@
       </c>
       <c r="N34" s="63">
         <f>IF(Pronostici!$Q34&lt;&gt;"",UPPER(Pronostici!$Q34),IF(OR(Pronostici!$R34="",Pronostici!$S34=""),"",IF(Pronostici!$R34&gt;Pronostici!$S34,"1",IF(Pronostici!$R34=Pronostici!$S34,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P34" s="63">
-        <f>IF(OR(Pronostici!$F34="",Pronostici!$G34=""),"",Pronostici!$F34&amp;" a "&amp;Pronostici!$G34)</f>
-        <v/>
-      </c>
-      <c r="Q34" s="63">
-        <f>IF(OR(Pronostici!$I34="",Pronostici!$J34=""),"",Pronostici!$I34&amp;" a "&amp;Pronostici!$J34)</f>
-        <v/>
-      </c>
-      <c r="R34" s="63">
-        <f>IF(OR(Pronostici!$L34="",Pronostici!$M34=""),"",Pronostici!$L34&amp;" a "&amp;Pronostici!$M34)</f>
-        <v/>
-      </c>
-      <c r="S34" s="63">
-        <f>IF(OR(Pronostici!$O34="",Pronostici!$P34=""),"",Pronostici!$O34&amp;" a "&amp;Pronostici!$P34)</f>
-        <v/>
-      </c>
-      <c r="T34" s="63">
-        <f>IF(OR(Pronostici!$R34="",Pronostici!$S34=""),"",Pronostici!$R34&amp;" a "&amp;Pronostici!$S34)</f>
         <v/>
       </c>
     </row>
@@ -10814,23 +10153,23 @@
         <v/>
       </c>
       <c r="D35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$F35&lt;&gt;"",Pronostici!$G35&lt;&gt;"",Pronostici!$F35=Partite!$G35,Pronostici!$G35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$P35)=1),Config!$D$9,Config!$D$6),IF(AND($J35&lt;&gt;"",$J35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$J35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$F35&lt;&gt;"",Pronostici!$G35&lt;&gt;"",Pronostici!$F35=Partite!$G35,Pronostici!$G35=Partite!$H35),Config!$D$6,IF(AND($J35&lt;&gt;"",$J35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$I35&lt;&gt;"",Pronostici!$J35&lt;&gt;"",Pronostici!$I35=Partite!$G35,Pronostici!$J35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$Q35)=1),Config!$D$9,Config!$D$6),IF(AND($K35&lt;&gt;"",$K35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$K35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$I35&lt;&gt;"",Pronostici!$J35&lt;&gt;"",Pronostici!$I35=Partite!$G35,Pronostici!$J35=Partite!$H35),Config!$D$6,IF(AND($K35&lt;&gt;"",$K35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$L35&lt;&gt;"",Pronostici!$M35&lt;&gt;"",Pronostici!$L35=Partite!$G35,Pronostici!$M35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$R35)=1),Config!$D$9,Config!$D$6),IF(AND($L35&lt;&gt;"",$L35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$L35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$L35&lt;&gt;"",Pronostici!$M35&lt;&gt;"",Pronostici!$L35=Partite!$G35,Pronostici!$M35=Partite!$H35),Config!$D$6,IF(AND($L35&lt;&gt;"",$L35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$O35&lt;&gt;"",Pronostici!$P35&lt;&gt;"",Pronostici!$O35=Partite!$G35,Pronostici!$P35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$S35)=1),Config!$D$9,Config!$D$6),IF(AND($M35&lt;&gt;"",$M35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$M35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$O35&lt;&gt;"",Pronostici!$P35&lt;&gt;"",Pronostici!$O35=Partite!$G35,Pronostici!$P35=Partite!$H35),Config!$D$6,IF(AND($M35&lt;&gt;"",$M35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$R35&lt;&gt;"",Pronostici!$S35&lt;&gt;"",Pronostici!$R35=Partite!$G35,Pronostici!$S35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$T35)=1),Config!$D$9,Config!$D$6),IF(AND($N35&lt;&gt;"",$N35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$N35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$R35&lt;&gt;"",Pronostici!$S35&lt;&gt;"",Pronostici!$R35=Partite!$G35,Pronostici!$S35=Partite!$H35),Config!$D$6,IF(AND($N35&lt;&gt;"",$N35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J35" s="63">
@@ -10851,26 +10190,6 @@
       </c>
       <c r="N35" s="63">
         <f>IF(Pronostici!$Q35&lt;&gt;"",UPPER(Pronostici!$Q35),IF(OR(Pronostici!$R35="",Pronostici!$S35=""),"",IF(Pronostici!$R35&gt;Pronostici!$S35,"1",IF(Pronostici!$R35=Pronostici!$S35,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P35" s="63">
-        <f>IF(OR(Pronostici!$F35="",Pronostici!$G35=""),"",Pronostici!$F35&amp;" a "&amp;Pronostici!$G35)</f>
-        <v/>
-      </c>
-      <c r="Q35" s="63">
-        <f>IF(OR(Pronostici!$I35="",Pronostici!$J35=""),"",Pronostici!$I35&amp;" a "&amp;Pronostici!$J35)</f>
-        <v/>
-      </c>
-      <c r="R35" s="63">
-        <f>IF(OR(Pronostici!$L35="",Pronostici!$M35=""),"",Pronostici!$L35&amp;" a "&amp;Pronostici!$M35)</f>
-        <v/>
-      </c>
-      <c r="S35" s="63">
-        <f>IF(OR(Pronostici!$O35="",Pronostici!$P35=""),"",Pronostici!$O35&amp;" a "&amp;Pronostici!$P35)</f>
-        <v/>
-      </c>
-      <c r="T35" s="63">
-        <f>IF(OR(Pronostici!$R35="",Pronostici!$S35=""),"",Pronostici!$R35&amp;" a "&amp;Pronostici!$S35)</f>
         <v/>
       </c>
     </row>
@@ -10888,23 +10207,23 @@
         <v/>
       </c>
       <c r="D36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$F36&lt;&gt;"",Pronostici!$G36&lt;&gt;"",Pronostici!$F36=Partite!$G36,Pronostici!$G36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$P36)=1),Config!$D$9,Config!$D$6),IF(AND($J36&lt;&gt;"",$J36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$J36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$F36&lt;&gt;"",Pronostici!$G36&lt;&gt;"",Pronostici!$F36=Partite!$G36,Pronostici!$G36=Partite!$H36),Config!$D$6,IF(AND($J36&lt;&gt;"",$J36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$I36&lt;&gt;"",Pronostici!$J36&lt;&gt;"",Pronostici!$I36=Partite!$G36,Pronostici!$J36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$Q36)=1),Config!$D$9,Config!$D$6),IF(AND($K36&lt;&gt;"",$K36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$K36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$I36&lt;&gt;"",Pronostici!$J36&lt;&gt;"",Pronostici!$I36=Partite!$G36,Pronostici!$J36=Partite!$H36),Config!$D$6,IF(AND($K36&lt;&gt;"",$K36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$L36&lt;&gt;"",Pronostici!$M36&lt;&gt;"",Pronostici!$L36=Partite!$G36,Pronostici!$M36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$R36)=1),Config!$D$9,Config!$D$6),IF(AND($L36&lt;&gt;"",$L36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$L36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$L36&lt;&gt;"",Pronostici!$M36&lt;&gt;"",Pronostici!$L36=Partite!$G36,Pronostici!$M36=Partite!$H36),Config!$D$6,IF(AND($L36&lt;&gt;"",$L36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$O36&lt;&gt;"",Pronostici!$P36&lt;&gt;"",Pronostici!$O36=Partite!$G36,Pronostici!$P36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$S36)=1),Config!$D$9,Config!$D$6),IF(AND($M36&lt;&gt;"",$M36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$M36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$O36&lt;&gt;"",Pronostici!$P36&lt;&gt;"",Pronostici!$O36=Partite!$G36,Pronostici!$P36=Partite!$H36),Config!$D$6,IF(AND($M36&lt;&gt;"",$M36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$R36&lt;&gt;"",Pronostici!$S36&lt;&gt;"",Pronostici!$R36=Partite!$G36,Pronostici!$S36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$T36)=1),Config!$D$9,Config!$D$6),IF(AND($N36&lt;&gt;"",$N36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$N36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$R36&lt;&gt;"",Pronostici!$S36&lt;&gt;"",Pronostici!$R36=Partite!$G36,Pronostici!$S36=Partite!$H36),Config!$D$6,IF(AND($N36&lt;&gt;"",$N36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J36" s="63">
@@ -10925,26 +10244,6 @@
       </c>
       <c r="N36" s="63">
         <f>IF(Pronostici!$Q36&lt;&gt;"",UPPER(Pronostici!$Q36),IF(OR(Pronostici!$R36="",Pronostici!$S36=""),"",IF(Pronostici!$R36&gt;Pronostici!$S36,"1",IF(Pronostici!$R36=Pronostici!$S36,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P36" s="63">
-        <f>IF(OR(Pronostici!$F36="",Pronostici!$G36=""),"",Pronostici!$F36&amp;" a "&amp;Pronostici!$G36)</f>
-        <v/>
-      </c>
-      <c r="Q36" s="63">
-        <f>IF(OR(Pronostici!$I36="",Pronostici!$J36=""),"",Pronostici!$I36&amp;" a "&amp;Pronostici!$J36)</f>
-        <v/>
-      </c>
-      <c r="R36" s="63">
-        <f>IF(OR(Pronostici!$L36="",Pronostici!$M36=""),"",Pronostici!$L36&amp;" a "&amp;Pronostici!$M36)</f>
-        <v/>
-      </c>
-      <c r="S36" s="63">
-        <f>IF(OR(Pronostici!$O36="",Pronostici!$P36=""),"",Pronostici!$O36&amp;" a "&amp;Pronostici!$P36)</f>
-        <v/>
-      </c>
-      <c r="T36" s="63">
-        <f>IF(OR(Pronostici!$R36="",Pronostici!$S36=""),"",Pronostici!$R36&amp;" a "&amp;Pronostici!$S36)</f>
         <v/>
       </c>
     </row>
@@ -10962,23 +10261,23 @@
         <v/>
       </c>
       <c r="D37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$F37&lt;&gt;"",Pronostici!$G37&lt;&gt;"",Pronostici!$F37=Partite!$G37,Pronostici!$G37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$P37)=1),Config!$D$9,Config!$D$6),IF(AND($J37&lt;&gt;"",$J37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$J37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$F37&lt;&gt;"",Pronostici!$G37&lt;&gt;"",Pronostici!$F37=Partite!$G37,Pronostici!$G37=Partite!$H37),Config!$D$6,IF(AND($J37&lt;&gt;"",$J37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$I37&lt;&gt;"",Pronostici!$J37&lt;&gt;"",Pronostici!$I37=Partite!$G37,Pronostici!$J37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$Q37)=1),Config!$D$9,Config!$D$6),IF(AND($K37&lt;&gt;"",$K37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$K37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$I37&lt;&gt;"",Pronostici!$J37&lt;&gt;"",Pronostici!$I37=Partite!$G37,Pronostici!$J37=Partite!$H37),Config!$D$6,IF(AND($K37&lt;&gt;"",$K37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$L37&lt;&gt;"",Pronostici!$M37&lt;&gt;"",Pronostici!$L37=Partite!$G37,Pronostici!$M37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$R37)=1),Config!$D$9,Config!$D$6),IF(AND($L37&lt;&gt;"",$L37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$L37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$L37&lt;&gt;"",Pronostici!$M37&lt;&gt;"",Pronostici!$L37=Partite!$G37,Pronostici!$M37=Partite!$H37),Config!$D$6,IF(AND($L37&lt;&gt;"",$L37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$O37&lt;&gt;"",Pronostici!$P37&lt;&gt;"",Pronostici!$O37=Partite!$G37,Pronostici!$P37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$S37)=1),Config!$D$9,Config!$D$6),IF(AND($M37&lt;&gt;"",$M37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$M37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$O37&lt;&gt;"",Pronostici!$P37&lt;&gt;"",Pronostici!$O37=Partite!$G37,Pronostici!$P37=Partite!$H37),Config!$D$6,IF(AND($M37&lt;&gt;"",$M37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$R37&lt;&gt;"",Pronostici!$S37&lt;&gt;"",Pronostici!$R37=Partite!$G37,Pronostici!$S37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$T37)=1),Config!$D$9,Config!$D$6),IF(AND($N37&lt;&gt;"",$N37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$N37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$R37&lt;&gt;"",Pronostici!$S37&lt;&gt;"",Pronostici!$R37=Partite!$G37,Pronostici!$S37=Partite!$H37),Config!$D$6,IF(AND($N37&lt;&gt;"",$N37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J37" s="63">
@@ -10999,26 +10298,6 @@
       </c>
       <c r="N37" s="63">
         <f>IF(Pronostici!$Q37&lt;&gt;"",UPPER(Pronostici!$Q37),IF(OR(Pronostici!$R37="",Pronostici!$S37=""),"",IF(Pronostici!$R37&gt;Pronostici!$S37,"1",IF(Pronostici!$R37=Pronostici!$S37,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P37" s="63">
-        <f>IF(OR(Pronostici!$F37="",Pronostici!$G37=""),"",Pronostici!$F37&amp;" a "&amp;Pronostici!$G37)</f>
-        <v/>
-      </c>
-      <c r="Q37" s="63">
-        <f>IF(OR(Pronostici!$I37="",Pronostici!$J37=""),"",Pronostici!$I37&amp;" a "&amp;Pronostici!$J37)</f>
-        <v/>
-      </c>
-      <c r="R37" s="63">
-        <f>IF(OR(Pronostici!$L37="",Pronostici!$M37=""),"",Pronostici!$L37&amp;" a "&amp;Pronostici!$M37)</f>
-        <v/>
-      </c>
-      <c r="S37" s="63">
-        <f>IF(OR(Pronostici!$O37="",Pronostici!$P37=""),"",Pronostici!$O37&amp;" a "&amp;Pronostici!$P37)</f>
-        <v/>
-      </c>
-      <c r="T37" s="63">
-        <f>IF(OR(Pronostici!$R37="",Pronostici!$S37=""),"",Pronostici!$R37&amp;" a "&amp;Pronostici!$S37)</f>
         <v/>
       </c>
     </row>
@@ -11036,23 +10315,23 @@
         <v/>
       </c>
       <c r="D38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$F38&lt;&gt;"",Pronostici!$G38&lt;&gt;"",Pronostici!$F38=Partite!$G38,Pronostici!$G38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$P38)=1),Config!$D$9,Config!$D$6),IF(AND($J38&lt;&gt;"",$J38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$J38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$F38&lt;&gt;"",Pronostici!$G38&lt;&gt;"",Pronostici!$F38=Partite!$G38,Pronostici!$G38=Partite!$H38),Config!$D$6,IF(AND($J38&lt;&gt;"",$J38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$I38&lt;&gt;"",Pronostici!$J38&lt;&gt;"",Pronostici!$I38=Partite!$G38,Pronostici!$J38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$Q38)=1),Config!$D$9,Config!$D$6),IF(AND($K38&lt;&gt;"",$K38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$K38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$I38&lt;&gt;"",Pronostici!$J38&lt;&gt;"",Pronostici!$I38=Partite!$G38,Pronostici!$J38=Partite!$H38),Config!$D$6,IF(AND($K38&lt;&gt;"",$K38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$L38&lt;&gt;"",Pronostici!$M38&lt;&gt;"",Pronostici!$L38=Partite!$G38,Pronostici!$M38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$R38)=1),Config!$D$9,Config!$D$6),IF(AND($L38&lt;&gt;"",$L38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$L38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$L38&lt;&gt;"",Pronostici!$M38&lt;&gt;"",Pronostici!$L38=Partite!$G38,Pronostici!$M38=Partite!$H38),Config!$D$6,IF(AND($L38&lt;&gt;"",$L38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$O38&lt;&gt;"",Pronostici!$P38&lt;&gt;"",Pronostici!$O38=Partite!$G38,Pronostici!$P38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$S38)=1),Config!$D$9,Config!$D$6),IF(AND($M38&lt;&gt;"",$M38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$M38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$O38&lt;&gt;"",Pronostici!$P38&lt;&gt;"",Pronostici!$O38=Partite!$G38,Pronostici!$P38=Partite!$H38),Config!$D$6,IF(AND($M38&lt;&gt;"",$M38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$R38&lt;&gt;"",Pronostici!$S38&lt;&gt;"",Pronostici!$R38=Partite!$G38,Pronostici!$S38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$T38)=1),Config!$D$9,Config!$D$6),IF(AND($N38&lt;&gt;"",$N38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$N38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$R38&lt;&gt;"",Pronostici!$S38&lt;&gt;"",Pronostici!$R38=Partite!$G38,Pronostici!$S38=Partite!$H38),Config!$D$6,IF(AND($N38&lt;&gt;"",$N38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J38" s="63">
@@ -11073,26 +10352,6 @@
       </c>
       <c r="N38" s="63">
         <f>IF(Pronostici!$Q38&lt;&gt;"",UPPER(Pronostici!$Q38),IF(OR(Pronostici!$R38="",Pronostici!$S38=""),"",IF(Pronostici!$R38&gt;Pronostici!$S38,"1",IF(Pronostici!$R38=Pronostici!$S38,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P38" s="63">
-        <f>IF(OR(Pronostici!$F38="",Pronostici!$G38=""),"",Pronostici!$F38&amp;" a "&amp;Pronostici!$G38)</f>
-        <v/>
-      </c>
-      <c r="Q38" s="63">
-        <f>IF(OR(Pronostici!$I38="",Pronostici!$J38=""),"",Pronostici!$I38&amp;" a "&amp;Pronostici!$J38)</f>
-        <v/>
-      </c>
-      <c r="R38" s="63">
-        <f>IF(OR(Pronostici!$L38="",Pronostici!$M38=""),"",Pronostici!$L38&amp;" a "&amp;Pronostici!$M38)</f>
-        <v/>
-      </c>
-      <c r="S38" s="63">
-        <f>IF(OR(Pronostici!$O38="",Pronostici!$P38=""),"",Pronostici!$O38&amp;" a "&amp;Pronostici!$P38)</f>
-        <v/>
-      </c>
-      <c r="T38" s="63">
-        <f>IF(OR(Pronostici!$R38="",Pronostici!$S38=""),"",Pronostici!$R38&amp;" a "&amp;Pronostici!$S38)</f>
         <v/>
       </c>
     </row>
@@ -11110,23 +10369,23 @@
         <v/>
       </c>
       <c r="D39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$F39&lt;&gt;"",Pronostici!$G39&lt;&gt;"",Pronostici!$F39=Partite!$G39,Pronostici!$G39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$P39)=1),Config!$D$9,Config!$D$6),IF(AND($J39&lt;&gt;"",$J39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$J39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$F39&lt;&gt;"",Pronostici!$G39&lt;&gt;"",Pronostici!$F39=Partite!$G39,Pronostici!$G39=Partite!$H39),Config!$D$6,IF(AND($J39&lt;&gt;"",$J39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$I39&lt;&gt;"",Pronostici!$J39&lt;&gt;"",Pronostici!$I39=Partite!$G39,Pronostici!$J39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$Q39)=1),Config!$D$9,Config!$D$6),IF(AND($K39&lt;&gt;"",$K39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$K39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$I39&lt;&gt;"",Pronostici!$J39&lt;&gt;"",Pronostici!$I39=Partite!$G39,Pronostici!$J39=Partite!$H39),Config!$D$6,IF(AND($K39&lt;&gt;"",$K39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$L39&lt;&gt;"",Pronostici!$M39&lt;&gt;"",Pronostici!$L39=Partite!$G39,Pronostici!$M39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$R39)=1),Config!$D$9,Config!$D$6),IF(AND($L39&lt;&gt;"",$L39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$L39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$L39&lt;&gt;"",Pronostici!$M39&lt;&gt;"",Pronostici!$L39=Partite!$G39,Pronostici!$M39=Partite!$H39),Config!$D$6,IF(AND($L39&lt;&gt;"",$L39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$O39&lt;&gt;"",Pronostici!$P39&lt;&gt;"",Pronostici!$O39=Partite!$G39,Pronostici!$P39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$S39)=1),Config!$D$9,Config!$D$6),IF(AND($M39&lt;&gt;"",$M39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$M39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$O39&lt;&gt;"",Pronostici!$P39&lt;&gt;"",Pronostici!$O39=Partite!$G39,Pronostici!$P39=Partite!$H39),Config!$D$6,IF(AND($M39&lt;&gt;"",$M39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$R39&lt;&gt;"",Pronostici!$S39&lt;&gt;"",Pronostici!$R39=Partite!$G39,Pronostici!$S39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$T39)=1),Config!$D$9,Config!$D$6),IF(AND($N39&lt;&gt;"",$N39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$N39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$R39&lt;&gt;"",Pronostici!$S39&lt;&gt;"",Pronostici!$R39=Partite!$G39,Pronostici!$S39=Partite!$H39),Config!$D$6,IF(AND($N39&lt;&gt;"",$N39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J39" s="63">
@@ -11147,26 +10406,6 @@
       </c>
       <c r="N39" s="63">
         <f>IF(Pronostici!$Q39&lt;&gt;"",UPPER(Pronostici!$Q39),IF(OR(Pronostici!$R39="",Pronostici!$S39=""),"",IF(Pronostici!$R39&gt;Pronostici!$S39,"1",IF(Pronostici!$R39=Pronostici!$S39,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P39" s="63">
-        <f>IF(OR(Pronostici!$F39="",Pronostici!$G39=""),"",Pronostici!$F39&amp;" a "&amp;Pronostici!$G39)</f>
-        <v/>
-      </c>
-      <c r="Q39" s="63">
-        <f>IF(OR(Pronostici!$I39="",Pronostici!$J39=""),"",Pronostici!$I39&amp;" a "&amp;Pronostici!$J39)</f>
-        <v/>
-      </c>
-      <c r="R39" s="63">
-        <f>IF(OR(Pronostici!$L39="",Pronostici!$M39=""),"",Pronostici!$L39&amp;" a "&amp;Pronostici!$M39)</f>
-        <v/>
-      </c>
-      <c r="S39" s="63">
-        <f>IF(OR(Pronostici!$O39="",Pronostici!$P39=""),"",Pronostici!$O39&amp;" a "&amp;Pronostici!$P39)</f>
-        <v/>
-      </c>
-      <c r="T39" s="63">
-        <f>IF(OR(Pronostici!$R39="",Pronostici!$S39=""),"",Pronostici!$R39&amp;" a "&amp;Pronostici!$S39)</f>
         <v/>
       </c>
     </row>
@@ -11184,23 +10423,23 @@
         <v/>
       </c>
       <c r="D40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$F40&lt;&gt;"",Pronostici!$G40&lt;&gt;"",Pronostici!$F40=Partite!$G40,Pronostici!$G40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$P40)=1),Config!$D$9,Config!$D$6),IF(AND($J40&lt;&gt;"",$J40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$J40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$F40&lt;&gt;"",Pronostici!$G40&lt;&gt;"",Pronostici!$F40=Partite!$G40,Pronostici!$G40=Partite!$H40),Config!$D$6,IF(AND($J40&lt;&gt;"",$J40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$I40&lt;&gt;"",Pronostici!$J40&lt;&gt;"",Pronostici!$I40=Partite!$G40,Pronostici!$J40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$Q40)=1),Config!$D$9,Config!$D$6),IF(AND($K40&lt;&gt;"",$K40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$K40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$I40&lt;&gt;"",Pronostici!$J40&lt;&gt;"",Pronostici!$I40=Partite!$G40,Pronostici!$J40=Partite!$H40),Config!$D$6,IF(AND($K40&lt;&gt;"",$K40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$L40&lt;&gt;"",Pronostici!$M40&lt;&gt;"",Pronostici!$L40=Partite!$G40,Pronostici!$M40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$R40)=1),Config!$D$9,Config!$D$6),IF(AND($L40&lt;&gt;"",$L40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$L40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$L40&lt;&gt;"",Pronostici!$M40&lt;&gt;"",Pronostici!$L40=Partite!$G40,Pronostici!$M40=Partite!$H40),Config!$D$6,IF(AND($L40&lt;&gt;"",$L40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$O40&lt;&gt;"",Pronostici!$P40&lt;&gt;"",Pronostici!$O40=Partite!$G40,Pronostici!$P40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$S40)=1),Config!$D$9,Config!$D$6),IF(AND($M40&lt;&gt;"",$M40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$M40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$O40&lt;&gt;"",Pronostici!$P40&lt;&gt;"",Pronostici!$O40=Partite!$G40,Pronostici!$P40=Partite!$H40),Config!$D$6,IF(AND($M40&lt;&gt;"",$M40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$R40&lt;&gt;"",Pronostici!$S40&lt;&gt;"",Pronostici!$R40=Partite!$G40,Pronostici!$S40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$T40)=1),Config!$D$9,Config!$D$6),IF(AND($N40&lt;&gt;"",$N40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$N40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$R40&lt;&gt;"",Pronostici!$S40&lt;&gt;"",Pronostici!$R40=Partite!$G40,Pronostici!$S40=Partite!$H40),Config!$D$6,IF(AND($N40&lt;&gt;"",$N40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J40" s="63">
@@ -11221,26 +10460,6 @@
       </c>
       <c r="N40" s="63">
         <f>IF(Pronostici!$Q40&lt;&gt;"",UPPER(Pronostici!$Q40),IF(OR(Pronostici!$R40="",Pronostici!$S40=""),"",IF(Pronostici!$R40&gt;Pronostici!$S40,"1",IF(Pronostici!$R40=Pronostici!$S40,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P40" s="63">
-        <f>IF(OR(Pronostici!$F40="",Pronostici!$G40=""),"",Pronostici!$F40&amp;" a "&amp;Pronostici!$G40)</f>
-        <v/>
-      </c>
-      <c r="Q40" s="63">
-        <f>IF(OR(Pronostici!$I40="",Pronostici!$J40=""),"",Pronostici!$I40&amp;" a "&amp;Pronostici!$J40)</f>
-        <v/>
-      </c>
-      <c r="R40" s="63">
-        <f>IF(OR(Pronostici!$L40="",Pronostici!$M40=""),"",Pronostici!$L40&amp;" a "&amp;Pronostici!$M40)</f>
-        <v/>
-      </c>
-      <c r="S40" s="63">
-        <f>IF(OR(Pronostici!$O40="",Pronostici!$P40=""),"",Pronostici!$O40&amp;" a "&amp;Pronostici!$P40)</f>
-        <v/>
-      </c>
-      <c r="T40" s="63">
-        <f>IF(OR(Pronostici!$R40="",Pronostici!$S40=""),"",Pronostici!$R40&amp;" a "&amp;Pronostici!$S40)</f>
         <v/>
       </c>
     </row>
@@ -11258,23 +10477,23 @@
         <v/>
       </c>
       <c r="D41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$F41&lt;&gt;"",Pronostici!$G41&lt;&gt;"",Pronostici!$F41=Partite!$G41,Pronostici!$G41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$P41)=1),Config!$D$9,Config!$D$6),IF(AND($J41&lt;&gt;"",$J41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$J41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$F41&lt;&gt;"",Pronostici!$G41&lt;&gt;"",Pronostici!$F41=Partite!$G41,Pronostici!$G41=Partite!$H41),Config!$D$6,IF(AND($J41&lt;&gt;"",$J41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$I41&lt;&gt;"",Pronostici!$J41&lt;&gt;"",Pronostici!$I41=Partite!$G41,Pronostici!$J41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$Q41)=1),Config!$D$9,Config!$D$6),IF(AND($K41&lt;&gt;"",$K41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$K41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$I41&lt;&gt;"",Pronostici!$J41&lt;&gt;"",Pronostici!$I41=Partite!$G41,Pronostici!$J41=Partite!$H41),Config!$D$6,IF(AND($K41&lt;&gt;"",$K41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$L41&lt;&gt;"",Pronostici!$M41&lt;&gt;"",Pronostici!$L41=Partite!$G41,Pronostici!$M41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$R41)=1),Config!$D$9,Config!$D$6),IF(AND($L41&lt;&gt;"",$L41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$L41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$L41&lt;&gt;"",Pronostici!$M41&lt;&gt;"",Pronostici!$L41=Partite!$G41,Pronostici!$M41=Partite!$H41),Config!$D$6,IF(AND($L41&lt;&gt;"",$L41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$O41&lt;&gt;"",Pronostici!$P41&lt;&gt;"",Pronostici!$O41=Partite!$G41,Pronostici!$P41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$S41)=1),Config!$D$9,Config!$D$6),IF(AND($M41&lt;&gt;"",$M41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$M41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$O41&lt;&gt;"",Pronostici!$P41&lt;&gt;"",Pronostici!$O41=Partite!$G41,Pronostici!$P41=Partite!$H41),Config!$D$6,IF(AND($M41&lt;&gt;"",$M41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$R41&lt;&gt;"",Pronostici!$S41&lt;&gt;"",Pronostici!$R41=Partite!$G41,Pronostici!$S41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$T41)=1),Config!$D$9,Config!$D$6),IF(AND($N41&lt;&gt;"",$N41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$N41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$R41&lt;&gt;"",Pronostici!$S41&lt;&gt;"",Pronostici!$R41=Partite!$G41,Pronostici!$S41=Partite!$H41),Config!$D$6,IF(AND($N41&lt;&gt;"",$N41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J41" s="63">
@@ -11295,26 +10514,6 @@
       </c>
       <c r="N41" s="63">
         <f>IF(Pronostici!$Q41&lt;&gt;"",UPPER(Pronostici!$Q41),IF(OR(Pronostici!$R41="",Pronostici!$S41=""),"",IF(Pronostici!$R41&gt;Pronostici!$S41,"1",IF(Pronostici!$R41=Pronostici!$S41,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P41" s="63">
-        <f>IF(OR(Pronostici!$F41="",Pronostici!$G41=""),"",Pronostici!$F41&amp;" a "&amp;Pronostici!$G41)</f>
-        <v/>
-      </c>
-      <c r="Q41" s="63">
-        <f>IF(OR(Pronostici!$I41="",Pronostici!$J41=""),"",Pronostici!$I41&amp;" a "&amp;Pronostici!$J41)</f>
-        <v/>
-      </c>
-      <c r="R41" s="63">
-        <f>IF(OR(Pronostici!$L41="",Pronostici!$M41=""),"",Pronostici!$L41&amp;" a "&amp;Pronostici!$M41)</f>
-        <v/>
-      </c>
-      <c r="S41" s="63">
-        <f>IF(OR(Pronostici!$O41="",Pronostici!$P41=""),"",Pronostici!$O41&amp;" a "&amp;Pronostici!$P41)</f>
-        <v/>
-      </c>
-      <c r="T41" s="63">
-        <f>IF(OR(Pronostici!$R41="",Pronostici!$S41=""),"",Pronostici!$R41&amp;" a "&amp;Pronostici!$S41)</f>
         <v/>
       </c>
     </row>
@@ -11332,23 +10531,23 @@
         <v/>
       </c>
       <c r="D42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$F42&lt;&gt;"",Pronostici!$G42&lt;&gt;"",Pronostici!$F42=Partite!$G42,Pronostici!$G42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$P42)=1),Config!$D$9,Config!$D$6),IF(AND($J42&lt;&gt;"",$J42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$J42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$F42&lt;&gt;"",Pronostici!$G42&lt;&gt;"",Pronostici!$F42=Partite!$G42,Pronostici!$G42=Partite!$H42),Config!$D$6,IF(AND($J42&lt;&gt;"",$J42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$I42&lt;&gt;"",Pronostici!$J42&lt;&gt;"",Pronostici!$I42=Partite!$G42,Pronostici!$J42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$Q42)=1),Config!$D$9,Config!$D$6),IF(AND($K42&lt;&gt;"",$K42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$K42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$I42&lt;&gt;"",Pronostici!$J42&lt;&gt;"",Pronostici!$I42=Partite!$G42,Pronostici!$J42=Partite!$H42),Config!$D$6,IF(AND($K42&lt;&gt;"",$K42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$L42&lt;&gt;"",Pronostici!$M42&lt;&gt;"",Pronostici!$L42=Partite!$G42,Pronostici!$M42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$R42)=1),Config!$D$9,Config!$D$6),IF(AND($L42&lt;&gt;"",$L42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$L42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$L42&lt;&gt;"",Pronostici!$M42&lt;&gt;"",Pronostici!$L42=Partite!$G42,Pronostici!$M42=Partite!$H42),Config!$D$6,IF(AND($L42&lt;&gt;"",$L42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$O42&lt;&gt;"",Pronostici!$P42&lt;&gt;"",Pronostici!$O42=Partite!$G42,Pronostici!$P42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$S42)=1),Config!$D$9,Config!$D$6),IF(AND($M42&lt;&gt;"",$M42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$M42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$O42&lt;&gt;"",Pronostici!$P42&lt;&gt;"",Pronostici!$O42=Partite!$G42,Pronostici!$P42=Partite!$H42),Config!$D$6,IF(AND($M42&lt;&gt;"",$M42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$R42&lt;&gt;"",Pronostici!$S42&lt;&gt;"",Pronostici!$R42=Partite!$G42,Pronostici!$S42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$T42)=1),Config!$D$9,Config!$D$6),IF(AND($N42&lt;&gt;"",$N42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$N42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$R42&lt;&gt;"",Pronostici!$S42&lt;&gt;"",Pronostici!$R42=Partite!$G42,Pronostici!$S42=Partite!$H42),Config!$D$6,IF(AND($N42&lt;&gt;"",$N42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J42" s="63">
@@ -11369,26 +10568,6 @@
       </c>
       <c r="N42" s="63">
         <f>IF(Pronostici!$Q42&lt;&gt;"",UPPER(Pronostici!$Q42),IF(OR(Pronostici!$R42="",Pronostici!$S42=""),"",IF(Pronostici!$R42&gt;Pronostici!$S42,"1",IF(Pronostici!$R42=Pronostici!$S42,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P42" s="63">
-        <f>IF(OR(Pronostici!$F42="",Pronostici!$G42=""),"",Pronostici!$F42&amp;" a "&amp;Pronostici!$G42)</f>
-        <v/>
-      </c>
-      <c r="Q42" s="63">
-        <f>IF(OR(Pronostici!$I42="",Pronostici!$J42=""),"",Pronostici!$I42&amp;" a "&amp;Pronostici!$J42)</f>
-        <v/>
-      </c>
-      <c r="R42" s="63">
-        <f>IF(OR(Pronostici!$L42="",Pronostici!$M42=""),"",Pronostici!$L42&amp;" a "&amp;Pronostici!$M42)</f>
-        <v/>
-      </c>
-      <c r="S42" s="63">
-        <f>IF(OR(Pronostici!$O42="",Pronostici!$P42=""),"",Pronostici!$O42&amp;" a "&amp;Pronostici!$P42)</f>
-        <v/>
-      </c>
-      <c r="T42" s="63">
-        <f>IF(OR(Pronostici!$R42="",Pronostici!$S42=""),"",Pronostici!$R42&amp;" a "&amp;Pronostici!$S42)</f>
         <v/>
       </c>
     </row>
@@ -11406,23 +10585,23 @@
         <v/>
       </c>
       <c r="D43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$F43&lt;&gt;"",Pronostici!$G43&lt;&gt;"",Pronostici!$F43=Partite!$G43,Pronostici!$G43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$P43)=1),Config!$D$9,Config!$D$6),IF(AND($J43&lt;&gt;"",$J43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$J43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$F43&lt;&gt;"",Pronostici!$G43&lt;&gt;"",Pronostici!$F43=Partite!$G43,Pronostici!$G43=Partite!$H43),Config!$D$6,IF(AND($J43&lt;&gt;"",$J43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$I43&lt;&gt;"",Pronostici!$J43&lt;&gt;"",Pronostici!$I43=Partite!$G43,Pronostici!$J43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$Q43)=1),Config!$D$9,Config!$D$6),IF(AND($K43&lt;&gt;"",$K43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$K43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$I43&lt;&gt;"",Pronostici!$J43&lt;&gt;"",Pronostici!$I43=Partite!$G43,Pronostici!$J43=Partite!$H43),Config!$D$6,IF(AND($K43&lt;&gt;"",$K43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$L43&lt;&gt;"",Pronostici!$M43&lt;&gt;"",Pronostici!$L43=Partite!$G43,Pronostici!$M43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$R43)=1),Config!$D$9,Config!$D$6),IF(AND($L43&lt;&gt;"",$L43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$L43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$L43&lt;&gt;"",Pronostici!$M43&lt;&gt;"",Pronostici!$L43=Partite!$G43,Pronostici!$M43=Partite!$H43),Config!$D$6,IF(AND($L43&lt;&gt;"",$L43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$O43&lt;&gt;"",Pronostici!$P43&lt;&gt;"",Pronostici!$O43=Partite!$G43,Pronostici!$P43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$S43)=1),Config!$D$9,Config!$D$6),IF(AND($M43&lt;&gt;"",$M43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$M43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$O43&lt;&gt;"",Pronostici!$P43&lt;&gt;"",Pronostici!$O43=Partite!$G43,Pronostici!$P43=Partite!$H43),Config!$D$6,IF(AND($M43&lt;&gt;"",$M43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$R43&lt;&gt;"",Pronostici!$S43&lt;&gt;"",Pronostici!$R43=Partite!$G43,Pronostici!$S43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$T43)=1),Config!$D$9,Config!$D$6),IF(AND($N43&lt;&gt;"",$N43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$N43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$R43&lt;&gt;"",Pronostici!$S43&lt;&gt;"",Pronostici!$R43=Partite!$G43,Pronostici!$S43=Partite!$H43),Config!$D$6,IF(AND($N43&lt;&gt;"",$N43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J43" s="63">
@@ -11443,26 +10622,6 @@
       </c>
       <c r="N43" s="63">
         <f>IF(Pronostici!$Q43&lt;&gt;"",UPPER(Pronostici!$Q43),IF(OR(Pronostici!$R43="",Pronostici!$S43=""),"",IF(Pronostici!$R43&gt;Pronostici!$S43,"1",IF(Pronostici!$R43=Pronostici!$S43,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P43" s="63">
-        <f>IF(OR(Pronostici!$F43="",Pronostici!$G43=""),"",Pronostici!$F43&amp;" a "&amp;Pronostici!$G43)</f>
-        <v/>
-      </c>
-      <c r="Q43" s="63">
-        <f>IF(OR(Pronostici!$I43="",Pronostici!$J43=""),"",Pronostici!$I43&amp;" a "&amp;Pronostici!$J43)</f>
-        <v/>
-      </c>
-      <c r="R43" s="63">
-        <f>IF(OR(Pronostici!$L43="",Pronostici!$M43=""),"",Pronostici!$L43&amp;" a "&amp;Pronostici!$M43)</f>
-        <v/>
-      </c>
-      <c r="S43" s="63">
-        <f>IF(OR(Pronostici!$O43="",Pronostici!$P43=""),"",Pronostici!$O43&amp;" a "&amp;Pronostici!$P43)</f>
-        <v/>
-      </c>
-      <c r="T43" s="63">
-        <f>IF(OR(Pronostici!$R43="",Pronostici!$S43=""),"",Pronostici!$R43&amp;" a "&amp;Pronostici!$S43)</f>
         <v/>
       </c>
     </row>
@@ -11480,23 +10639,23 @@
         <v/>
       </c>
       <c r="D44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$F44&lt;&gt;"",Pronostici!$G44&lt;&gt;"",Pronostici!$F44=Partite!$G44,Pronostici!$G44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$P44)=1),Config!$D$9,Config!$D$6),IF(AND($J44&lt;&gt;"",$J44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$J44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$F44&lt;&gt;"",Pronostici!$G44&lt;&gt;"",Pronostici!$F44=Partite!$G44,Pronostici!$G44=Partite!$H44),Config!$D$6,IF(AND($J44&lt;&gt;"",$J44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$I44&lt;&gt;"",Pronostici!$J44&lt;&gt;"",Pronostici!$I44=Partite!$G44,Pronostici!$J44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$Q44)=1),Config!$D$9,Config!$D$6),IF(AND($K44&lt;&gt;"",$K44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$K44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$I44&lt;&gt;"",Pronostici!$J44&lt;&gt;"",Pronostici!$I44=Partite!$G44,Pronostici!$J44=Partite!$H44),Config!$D$6,IF(AND($K44&lt;&gt;"",$K44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$L44&lt;&gt;"",Pronostici!$M44&lt;&gt;"",Pronostici!$L44=Partite!$G44,Pronostici!$M44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$R44)=1),Config!$D$9,Config!$D$6),IF(AND($L44&lt;&gt;"",$L44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$L44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$L44&lt;&gt;"",Pronostici!$M44&lt;&gt;"",Pronostici!$L44=Partite!$G44,Pronostici!$M44=Partite!$H44),Config!$D$6,IF(AND($L44&lt;&gt;"",$L44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$O44&lt;&gt;"",Pronostici!$P44&lt;&gt;"",Pronostici!$O44=Partite!$G44,Pronostici!$P44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$S44)=1),Config!$D$9,Config!$D$6),IF(AND($M44&lt;&gt;"",$M44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$M44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$O44&lt;&gt;"",Pronostici!$P44&lt;&gt;"",Pronostici!$O44=Partite!$G44,Pronostici!$P44=Partite!$H44),Config!$D$6,IF(AND($M44&lt;&gt;"",$M44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$R44&lt;&gt;"",Pronostici!$S44&lt;&gt;"",Pronostici!$R44=Partite!$G44,Pronostici!$S44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$T44)=1),Config!$D$9,Config!$D$6),IF(AND($N44&lt;&gt;"",$N44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$N44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$R44&lt;&gt;"",Pronostici!$S44&lt;&gt;"",Pronostici!$R44=Partite!$G44,Pronostici!$S44=Partite!$H44),Config!$D$6,IF(AND($N44&lt;&gt;"",$N44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J44" s="63">
@@ -11517,26 +10676,6 @@
       </c>
       <c r="N44" s="63">
         <f>IF(Pronostici!$Q44&lt;&gt;"",UPPER(Pronostici!$Q44),IF(OR(Pronostici!$R44="",Pronostici!$S44=""),"",IF(Pronostici!$R44&gt;Pronostici!$S44,"1",IF(Pronostici!$R44=Pronostici!$S44,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P44" s="63">
-        <f>IF(OR(Pronostici!$F44="",Pronostici!$G44=""),"",Pronostici!$F44&amp;" a "&amp;Pronostici!$G44)</f>
-        <v/>
-      </c>
-      <c r="Q44" s="63">
-        <f>IF(OR(Pronostici!$I44="",Pronostici!$J44=""),"",Pronostici!$I44&amp;" a "&amp;Pronostici!$J44)</f>
-        <v/>
-      </c>
-      <c r="R44" s="63">
-        <f>IF(OR(Pronostici!$L44="",Pronostici!$M44=""),"",Pronostici!$L44&amp;" a "&amp;Pronostici!$M44)</f>
-        <v/>
-      </c>
-      <c r="S44" s="63">
-        <f>IF(OR(Pronostici!$O44="",Pronostici!$P44=""),"",Pronostici!$O44&amp;" a "&amp;Pronostici!$P44)</f>
-        <v/>
-      </c>
-      <c r="T44" s="63">
-        <f>IF(OR(Pronostici!$R44="",Pronostici!$S44=""),"",Pronostici!$R44&amp;" a "&amp;Pronostici!$S44)</f>
         <v/>
       </c>
     </row>
@@ -11554,23 +10693,23 @@
         <v/>
       </c>
       <c r="D45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$F45&lt;&gt;"",Pronostici!$G45&lt;&gt;"",Pronostici!$F45=Partite!$G45,Pronostici!$G45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$P45)=1),Config!$D$9,Config!$D$6),IF(AND($J45&lt;&gt;"",$J45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$J45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$F45&lt;&gt;"",Pronostici!$G45&lt;&gt;"",Pronostici!$F45=Partite!$G45,Pronostici!$G45=Partite!$H45),Config!$D$6,IF(AND($J45&lt;&gt;"",$J45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$I45&lt;&gt;"",Pronostici!$J45&lt;&gt;"",Pronostici!$I45=Partite!$G45,Pronostici!$J45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$Q45)=1),Config!$D$9,Config!$D$6),IF(AND($K45&lt;&gt;"",$K45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$K45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$I45&lt;&gt;"",Pronostici!$J45&lt;&gt;"",Pronostici!$I45=Partite!$G45,Pronostici!$J45=Partite!$H45),Config!$D$6,IF(AND($K45&lt;&gt;"",$K45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$L45&lt;&gt;"",Pronostici!$M45&lt;&gt;"",Pronostici!$L45=Partite!$G45,Pronostici!$M45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$R45)=1),Config!$D$9,Config!$D$6),IF(AND($L45&lt;&gt;"",$L45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$L45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$L45&lt;&gt;"",Pronostici!$M45&lt;&gt;"",Pronostici!$L45=Partite!$G45,Pronostici!$M45=Partite!$H45),Config!$D$6,IF(AND($L45&lt;&gt;"",$L45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$O45&lt;&gt;"",Pronostici!$P45&lt;&gt;"",Pronostici!$O45=Partite!$G45,Pronostici!$P45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$S45)=1),Config!$D$9,Config!$D$6),IF(AND($M45&lt;&gt;"",$M45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$M45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$O45&lt;&gt;"",Pronostici!$P45&lt;&gt;"",Pronostici!$O45=Partite!$G45,Pronostici!$P45=Partite!$H45),Config!$D$6,IF(AND($M45&lt;&gt;"",$M45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$R45&lt;&gt;"",Pronostici!$S45&lt;&gt;"",Pronostici!$R45=Partite!$G45,Pronostici!$S45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$T45)=1),Config!$D$9,Config!$D$6),IF(AND($N45&lt;&gt;"",$N45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$N45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$R45&lt;&gt;"",Pronostici!$S45&lt;&gt;"",Pronostici!$R45=Partite!$G45,Pronostici!$S45=Partite!$H45),Config!$D$6,IF(AND($N45&lt;&gt;"",$N45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J45" s="63">
@@ -11591,26 +10730,6 @@
       </c>
       <c r="N45" s="63">
         <f>IF(Pronostici!$Q45&lt;&gt;"",UPPER(Pronostici!$Q45),IF(OR(Pronostici!$R45="",Pronostici!$S45=""),"",IF(Pronostici!$R45&gt;Pronostici!$S45,"1",IF(Pronostici!$R45=Pronostici!$S45,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P45" s="63">
-        <f>IF(OR(Pronostici!$F45="",Pronostici!$G45=""),"",Pronostici!$F45&amp;" a "&amp;Pronostici!$G45)</f>
-        <v/>
-      </c>
-      <c r="Q45" s="63">
-        <f>IF(OR(Pronostici!$I45="",Pronostici!$J45=""),"",Pronostici!$I45&amp;" a "&amp;Pronostici!$J45)</f>
-        <v/>
-      </c>
-      <c r="R45" s="63">
-        <f>IF(OR(Pronostici!$L45="",Pronostici!$M45=""),"",Pronostici!$L45&amp;" a "&amp;Pronostici!$M45)</f>
-        <v/>
-      </c>
-      <c r="S45" s="63">
-        <f>IF(OR(Pronostici!$O45="",Pronostici!$P45=""),"",Pronostici!$O45&amp;" a "&amp;Pronostici!$P45)</f>
-        <v/>
-      </c>
-      <c r="T45" s="63">
-        <f>IF(OR(Pronostici!$R45="",Pronostici!$S45=""),"",Pronostici!$R45&amp;" a "&amp;Pronostici!$S45)</f>
         <v/>
       </c>
     </row>
@@ -11628,23 +10747,23 @@
         <v/>
       </c>
       <c r="D46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$F46&lt;&gt;"",Pronostici!$G46&lt;&gt;"",Pronostici!$F46=Partite!$G46,Pronostici!$G46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$P46)=1),Config!$D$9,Config!$D$6),IF(AND($J46&lt;&gt;"",$J46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$J46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$F46&lt;&gt;"",Pronostici!$G46&lt;&gt;"",Pronostici!$F46=Partite!$G46,Pronostici!$G46=Partite!$H46),Config!$D$6,IF(AND($J46&lt;&gt;"",$J46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$I46&lt;&gt;"",Pronostici!$J46&lt;&gt;"",Pronostici!$I46=Partite!$G46,Pronostici!$J46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$Q46)=1),Config!$D$9,Config!$D$6),IF(AND($K46&lt;&gt;"",$K46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$K46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$I46&lt;&gt;"",Pronostici!$J46&lt;&gt;"",Pronostici!$I46=Partite!$G46,Pronostici!$J46=Partite!$H46),Config!$D$6,IF(AND($K46&lt;&gt;"",$K46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$L46&lt;&gt;"",Pronostici!$M46&lt;&gt;"",Pronostici!$L46=Partite!$G46,Pronostici!$M46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$R46)=1),Config!$D$9,Config!$D$6),IF(AND($L46&lt;&gt;"",$L46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$L46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$L46&lt;&gt;"",Pronostici!$M46&lt;&gt;"",Pronostici!$L46=Partite!$G46,Pronostici!$M46=Partite!$H46),Config!$D$6,IF(AND($L46&lt;&gt;"",$L46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$O46&lt;&gt;"",Pronostici!$P46&lt;&gt;"",Pronostici!$O46=Partite!$G46,Pronostici!$P46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$S46)=1),Config!$D$9,Config!$D$6),IF(AND($M46&lt;&gt;"",$M46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$M46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$O46&lt;&gt;"",Pronostici!$P46&lt;&gt;"",Pronostici!$O46=Partite!$G46,Pronostici!$P46=Partite!$H46),Config!$D$6,IF(AND($M46&lt;&gt;"",$M46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$R46&lt;&gt;"",Pronostici!$S46&lt;&gt;"",Pronostici!$R46=Partite!$G46,Pronostici!$S46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$T46)=1),Config!$D$9,Config!$D$6),IF(AND($N46&lt;&gt;"",$N46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$N46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$R46&lt;&gt;"",Pronostici!$S46&lt;&gt;"",Pronostici!$R46=Partite!$G46,Pronostici!$S46=Partite!$H46),Config!$D$6,IF(AND($N46&lt;&gt;"",$N46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J46" s="63">
@@ -11665,26 +10784,6 @@
       </c>
       <c r="N46" s="63">
         <f>IF(Pronostici!$Q46&lt;&gt;"",UPPER(Pronostici!$Q46),IF(OR(Pronostici!$R46="",Pronostici!$S46=""),"",IF(Pronostici!$R46&gt;Pronostici!$S46,"1",IF(Pronostici!$R46=Pronostici!$S46,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P46" s="63">
-        <f>IF(OR(Pronostici!$F46="",Pronostici!$G46=""),"",Pronostici!$F46&amp;" a "&amp;Pronostici!$G46)</f>
-        <v/>
-      </c>
-      <c r="Q46" s="63">
-        <f>IF(OR(Pronostici!$I46="",Pronostici!$J46=""),"",Pronostici!$I46&amp;" a "&amp;Pronostici!$J46)</f>
-        <v/>
-      </c>
-      <c r="R46" s="63">
-        <f>IF(OR(Pronostici!$L46="",Pronostici!$M46=""),"",Pronostici!$L46&amp;" a "&amp;Pronostici!$M46)</f>
-        <v/>
-      </c>
-      <c r="S46" s="63">
-        <f>IF(OR(Pronostici!$O46="",Pronostici!$P46=""),"",Pronostici!$O46&amp;" a "&amp;Pronostici!$P46)</f>
-        <v/>
-      </c>
-      <c r="T46" s="63">
-        <f>IF(OR(Pronostici!$R46="",Pronostici!$S46=""),"",Pronostici!$R46&amp;" a "&amp;Pronostici!$S46)</f>
         <v/>
       </c>
     </row>
@@ -11702,23 +10801,23 @@
         <v/>
       </c>
       <c r="D47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$F47&lt;&gt;"",Pronostici!$G47&lt;&gt;"",Pronostici!$F47=Partite!$G47,Pronostici!$G47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$P47)=1),Config!$D$9,Config!$D$6),IF(AND($J47&lt;&gt;"",$J47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$J47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$F47&lt;&gt;"",Pronostici!$G47&lt;&gt;"",Pronostici!$F47=Partite!$G47,Pronostici!$G47=Partite!$H47),Config!$D$6,IF(AND($J47&lt;&gt;"",$J47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$I47&lt;&gt;"",Pronostici!$J47&lt;&gt;"",Pronostici!$I47=Partite!$G47,Pronostici!$J47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$Q47)=1),Config!$D$9,Config!$D$6),IF(AND($K47&lt;&gt;"",$K47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$K47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$I47&lt;&gt;"",Pronostici!$J47&lt;&gt;"",Pronostici!$I47=Partite!$G47,Pronostici!$J47=Partite!$H47),Config!$D$6,IF(AND($K47&lt;&gt;"",$K47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$L47&lt;&gt;"",Pronostici!$M47&lt;&gt;"",Pronostici!$L47=Partite!$G47,Pronostici!$M47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$R47)=1),Config!$D$9,Config!$D$6),IF(AND($L47&lt;&gt;"",$L47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$L47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$L47&lt;&gt;"",Pronostici!$M47&lt;&gt;"",Pronostici!$L47=Partite!$G47,Pronostici!$M47=Partite!$H47),Config!$D$6,IF(AND($L47&lt;&gt;"",$L47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$O47&lt;&gt;"",Pronostici!$P47&lt;&gt;"",Pronostici!$O47=Partite!$G47,Pronostici!$P47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$S47)=1),Config!$D$9,Config!$D$6),IF(AND($M47&lt;&gt;"",$M47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$M47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$O47&lt;&gt;"",Pronostici!$P47&lt;&gt;"",Pronostici!$O47=Partite!$G47,Pronostici!$P47=Partite!$H47),Config!$D$6,IF(AND($M47&lt;&gt;"",$M47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$R47&lt;&gt;"",Pronostici!$S47&lt;&gt;"",Pronostici!$R47=Partite!$G47,Pronostici!$S47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$T47)=1),Config!$D$9,Config!$D$6),IF(AND($N47&lt;&gt;"",$N47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$N47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$R47&lt;&gt;"",Pronostici!$S47&lt;&gt;"",Pronostici!$R47=Partite!$G47,Pronostici!$S47=Partite!$H47),Config!$D$6,IF(AND($N47&lt;&gt;"",$N47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J47" s="63">
@@ -11739,26 +10838,6 @@
       </c>
       <c r="N47" s="63">
         <f>IF(Pronostici!$Q47&lt;&gt;"",UPPER(Pronostici!$Q47),IF(OR(Pronostici!$R47="",Pronostici!$S47=""),"",IF(Pronostici!$R47&gt;Pronostici!$S47,"1",IF(Pronostici!$R47=Pronostici!$S47,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P47" s="63">
-        <f>IF(OR(Pronostici!$F47="",Pronostici!$G47=""),"",Pronostici!$F47&amp;" a "&amp;Pronostici!$G47)</f>
-        <v/>
-      </c>
-      <c r="Q47" s="63">
-        <f>IF(OR(Pronostici!$I47="",Pronostici!$J47=""),"",Pronostici!$I47&amp;" a "&amp;Pronostici!$J47)</f>
-        <v/>
-      </c>
-      <c r="R47" s="63">
-        <f>IF(OR(Pronostici!$L47="",Pronostici!$M47=""),"",Pronostici!$L47&amp;" a "&amp;Pronostici!$M47)</f>
-        <v/>
-      </c>
-      <c r="S47" s="63">
-        <f>IF(OR(Pronostici!$O47="",Pronostici!$P47=""),"",Pronostici!$O47&amp;" a "&amp;Pronostici!$P47)</f>
-        <v/>
-      </c>
-      <c r="T47" s="63">
-        <f>IF(OR(Pronostici!$R47="",Pronostici!$S47=""),"",Pronostici!$R47&amp;" a "&amp;Pronostici!$S47)</f>
         <v/>
       </c>
     </row>
@@ -11776,23 +10855,23 @@
         <v/>
       </c>
       <c r="D48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$F48&lt;&gt;"",Pronostici!$G48&lt;&gt;"",Pronostici!$F48=Partite!$G48,Pronostici!$G48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$P48)=1),Config!$D$9,Config!$D$6),IF(AND($J48&lt;&gt;"",$J48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$J48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$F48&lt;&gt;"",Pronostici!$G48&lt;&gt;"",Pronostici!$F48=Partite!$G48,Pronostici!$G48=Partite!$H48),Config!$D$6,IF(AND($J48&lt;&gt;"",$J48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$I48&lt;&gt;"",Pronostici!$J48&lt;&gt;"",Pronostici!$I48=Partite!$G48,Pronostici!$J48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$Q48)=1),Config!$D$9,Config!$D$6),IF(AND($K48&lt;&gt;"",$K48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$K48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$I48&lt;&gt;"",Pronostici!$J48&lt;&gt;"",Pronostici!$I48=Partite!$G48,Pronostici!$J48=Partite!$H48),Config!$D$6,IF(AND($K48&lt;&gt;"",$K48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$L48&lt;&gt;"",Pronostici!$M48&lt;&gt;"",Pronostici!$L48=Partite!$G48,Pronostici!$M48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$R48)=1),Config!$D$9,Config!$D$6),IF(AND($L48&lt;&gt;"",$L48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$L48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$L48&lt;&gt;"",Pronostici!$M48&lt;&gt;"",Pronostici!$L48=Partite!$G48,Pronostici!$M48=Partite!$H48),Config!$D$6,IF(AND($L48&lt;&gt;"",$L48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$O48&lt;&gt;"",Pronostici!$P48&lt;&gt;"",Pronostici!$O48=Partite!$G48,Pronostici!$P48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$S48)=1),Config!$D$9,Config!$D$6),IF(AND($M48&lt;&gt;"",$M48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$M48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$O48&lt;&gt;"",Pronostici!$P48&lt;&gt;"",Pronostici!$O48=Partite!$G48,Pronostici!$P48=Partite!$H48),Config!$D$6,IF(AND($M48&lt;&gt;"",$M48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$R48&lt;&gt;"",Pronostici!$S48&lt;&gt;"",Pronostici!$R48=Partite!$G48,Pronostici!$S48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$T48)=1),Config!$D$9,Config!$D$6),IF(AND($N48&lt;&gt;"",$N48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$N48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$R48&lt;&gt;"",Pronostici!$S48&lt;&gt;"",Pronostici!$R48=Partite!$G48,Pronostici!$S48=Partite!$H48),Config!$D$6,IF(AND($N48&lt;&gt;"",$N48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J48" s="63">
@@ -11813,26 +10892,6 @@
       </c>
       <c r="N48" s="63">
         <f>IF(Pronostici!$Q48&lt;&gt;"",UPPER(Pronostici!$Q48),IF(OR(Pronostici!$R48="",Pronostici!$S48=""),"",IF(Pronostici!$R48&gt;Pronostici!$S48,"1",IF(Pronostici!$R48=Pronostici!$S48,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P48" s="63">
-        <f>IF(OR(Pronostici!$F48="",Pronostici!$G48=""),"",Pronostici!$F48&amp;" a "&amp;Pronostici!$G48)</f>
-        <v/>
-      </c>
-      <c r="Q48" s="63">
-        <f>IF(OR(Pronostici!$I48="",Pronostici!$J48=""),"",Pronostici!$I48&amp;" a "&amp;Pronostici!$J48)</f>
-        <v/>
-      </c>
-      <c r="R48" s="63">
-        <f>IF(OR(Pronostici!$L48="",Pronostici!$M48=""),"",Pronostici!$L48&amp;" a "&amp;Pronostici!$M48)</f>
-        <v/>
-      </c>
-      <c r="S48" s="63">
-        <f>IF(OR(Pronostici!$O48="",Pronostici!$P48=""),"",Pronostici!$O48&amp;" a "&amp;Pronostici!$P48)</f>
-        <v/>
-      </c>
-      <c r="T48" s="63">
-        <f>IF(OR(Pronostici!$R48="",Pronostici!$S48=""),"",Pronostici!$R48&amp;" a "&amp;Pronostici!$S48)</f>
         <v/>
       </c>
     </row>
@@ -11850,23 +10909,23 @@
         <v/>
       </c>
       <c r="D49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$F49&lt;&gt;"",Pronostici!$G49&lt;&gt;"",Pronostici!$F49=Partite!$G49,Pronostici!$G49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$P49)=1),Config!$D$9,Config!$D$6),IF(AND($J49&lt;&gt;"",$J49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$J49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$F49&lt;&gt;"",Pronostici!$G49&lt;&gt;"",Pronostici!$F49=Partite!$G49,Pronostici!$G49=Partite!$H49),Config!$D$6,IF(AND($J49&lt;&gt;"",$J49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$I49&lt;&gt;"",Pronostici!$J49&lt;&gt;"",Pronostici!$I49=Partite!$G49,Pronostici!$J49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$Q49)=1),Config!$D$9,Config!$D$6),IF(AND($K49&lt;&gt;"",$K49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$K49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$I49&lt;&gt;"",Pronostici!$J49&lt;&gt;"",Pronostici!$I49=Partite!$G49,Pronostici!$J49=Partite!$H49),Config!$D$6,IF(AND($K49&lt;&gt;"",$K49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$L49&lt;&gt;"",Pronostici!$M49&lt;&gt;"",Pronostici!$L49=Partite!$G49,Pronostici!$M49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$R49)=1),Config!$D$9,Config!$D$6),IF(AND($L49&lt;&gt;"",$L49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$L49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$L49&lt;&gt;"",Pronostici!$M49&lt;&gt;"",Pronostici!$L49=Partite!$G49,Pronostici!$M49=Partite!$H49),Config!$D$6,IF(AND($L49&lt;&gt;"",$L49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$O49&lt;&gt;"",Pronostici!$P49&lt;&gt;"",Pronostici!$O49=Partite!$G49,Pronostici!$P49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$S49)=1),Config!$D$9,Config!$D$6),IF(AND($M49&lt;&gt;"",$M49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$M49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$O49&lt;&gt;"",Pronostici!$P49&lt;&gt;"",Pronostici!$O49=Partite!$G49,Pronostici!$P49=Partite!$H49),Config!$D$6,IF(AND($M49&lt;&gt;"",$M49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$R49&lt;&gt;"",Pronostici!$S49&lt;&gt;"",Pronostici!$R49=Partite!$G49,Pronostici!$S49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$T49)=1),Config!$D$9,Config!$D$6),IF(AND($N49&lt;&gt;"",$N49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$N49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$R49&lt;&gt;"",Pronostici!$S49&lt;&gt;"",Pronostici!$R49=Partite!$G49,Pronostici!$S49=Partite!$H49),Config!$D$6,IF(AND($N49&lt;&gt;"",$N49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J49" s="63">
@@ -11887,26 +10946,6 @@
       </c>
       <c r="N49" s="63">
         <f>IF(Pronostici!$Q49&lt;&gt;"",UPPER(Pronostici!$Q49),IF(OR(Pronostici!$R49="",Pronostici!$S49=""),"",IF(Pronostici!$R49&gt;Pronostici!$S49,"1",IF(Pronostici!$R49=Pronostici!$S49,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P49" s="63">
-        <f>IF(OR(Pronostici!$F49="",Pronostici!$G49=""),"",Pronostici!$F49&amp;" a "&amp;Pronostici!$G49)</f>
-        <v/>
-      </c>
-      <c r="Q49" s="63">
-        <f>IF(OR(Pronostici!$I49="",Pronostici!$J49=""),"",Pronostici!$I49&amp;" a "&amp;Pronostici!$J49)</f>
-        <v/>
-      </c>
-      <c r="R49" s="63">
-        <f>IF(OR(Pronostici!$L49="",Pronostici!$M49=""),"",Pronostici!$L49&amp;" a "&amp;Pronostici!$M49)</f>
-        <v/>
-      </c>
-      <c r="S49" s="63">
-        <f>IF(OR(Pronostici!$O49="",Pronostici!$P49=""),"",Pronostici!$O49&amp;" a "&amp;Pronostici!$P49)</f>
-        <v/>
-      </c>
-      <c r="T49" s="63">
-        <f>IF(OR(Pronostici!$R49="",Pronostici!$S49=""),"",Pronostici!$R49&amp;" a "&amp;Pronostici!$S49)</f>
         <v/>
       </c>
     </row>
@@ -11924,23 +10963,23 @@
         <v/>
       </c>
       <c r="D50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$F50&lt;&gt;"",Pronostici!$G50&lt;&gt;"",Pronostici!$F50=Partite!$G50,Pronostici!$G50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$P50)=1),Config!$D$9,Config!$D$6),IF(AND($J50&lt;&gt;"",$J50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$J50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$F50&lt;&gt;"",Pronostici!$G50&lt;&gt;"",Pronostici!$F50=Partite!$G50,Pronostici!$G50=Partite!$H50),Config!$D$6,IF(AND($J50&lt;&gt;"",$J50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$I50&lt;&gt;"",Pronostici!$J50&lt;&gt;"",Pronostici!$I50=Partite!$G50,Pronostici!$J50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$Q50)=1),Config!$D$9,Config!$D$6),IF(AND($K50&lt;&gt;"",$K50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$K50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$I50&lt;&gt;"",Pronostici!$J50&lt;&gt;"",Pronostici!$I50=Partite!$G50,Pronostici!$J50=Partite!$H50),Config!$D$6,IF(AND($K50&lt;&gt;"",$K50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$L50&lt;&gt;"",Pronostici!$M50&lt;&gt;"",Pronostici!$L50=Partite!$G50,Pronostici!$M50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$R50)=1),Config!$D$9,Config!$D$6),IF(AND($L50&lt;&gt;"",$L50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$L50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$L50&lt;&gt;"",Pronostici!$M50&lt;&gt;"",Pronostici!$L50=Partite!$G50,Pronostici!$M50=Partite!$H50),Config!$D$6,IF(AND($L50&lt;&gt;"",$L50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$O50&lt;&gt;"",Pronostici!$P50&lt;&gt;"",Pronostici!$O50=Partite!$G50,Pronostici!$P50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$S50)=1),Config!$D$9,Config!$D$6),IF(AND($M50&lt;&gt;"",$M50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$M50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$O50&lt;&gt;"",Pronostici!$P50&lt;&gt;"",Pronostici!$O50=Partite!$G50,Pronostici!$P50=Partite!$H50),Config!$D$6,IF(AND($M50&lt;&gt;"",$M50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$R50&lt;&gt;"",Pronostici!$S50&lt;&gt;"",Pronostici!$R50=Partite!$G50,Pronostici!$S50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$T50)=1),Config!$D$9,Config!$D$6),IF(AND($N50&lt;&gt;"",$N50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$N50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$R50&lt;&gt;"",Pronostici!$S50&lt;&gt;"",Pronostici!$R50=Partite!$G50,Pronostici!$S50=Partite!$H50),Config!$D$6,IF(AND($N50&lt;&gt;"",$N50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J50" s="63">
@@ -11961,26 +11000,6 @@
       </c>
       <c r="N50" s="63">
         <f>IF(Pronostici!$Q50&lt;&gt;"",UPPER(Pronostici!$Q50),IF(OR(Pronostici!$R50="",Pronostici!$S50=""),"",IF(Pronostici!$R50&gt;Pronostici!$S50,"1",IF(Pronostici!$R50=Pronostici!$S50,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P50" s="63">
-        <f>IF(OR(Pronostici!$F50="",Pronostici!$G50=""),"",Pronostici!$F50&amp;" a "&amp;Pronostici!$G50)</f>
-        <v/>
-      </c>
-      <c r="Q50" s="63">
-        <f>IF(OR(Pronostici!$I50="",Pronostici!$J50=""),"",Pronostici!$I50&amp;" a "&amp;Pronostici!$J50)</f>
-        <v/>
-      </c>
-      <c r="R50" s="63">
-        <f>IF(OR(Pronostici!$L50="",Pronostici!$M50=""),"",Pronostici!$L50&amp;" a "&amp;Pronostici!$M50)</f>
-        <v/>
-      </c>
-      <c r="S50" s="63">
-        <f>IF(OR(Pronostici!$O50="",Pronostici!$P50=""),"",Pronostici!$O50&amp;" a "&amp;Pronostici!$P50)</f>
-        <v/>
-      </c>
-      <c r="T50" s="63">
-        <f>IF(OR(Pronostici!$R50="",Pronostici!$S50=""),"",Pronostici!$R50&amp;" a "&amp;Pronostici!$S50)</f>
         <v/>
       </c>
     </row>
@@ -11998,23 +11017,23 @@
         <v/>
       </c>
       <c r="D51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$F51&lt;&gt;"",Pronostici!$G51&lt;&gt;"",Pronostici!$F51=Partite!$G51,Pronostici!$G51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$P51)=1),Config!$D$9,Config!$D$6),IF(AND($J51&lt;&gt;"",$J51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$J51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$F51&lt;&gt;"",Pronostici!$G51&lt;&gt;"",Pronostici!$F51=Partite!$G51,Pronostici!$G51=Partite!$H51),Config!$D$6,IF(AND($J51&lt;&gt;"",$J51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$I51&lt;&gt;"",Pronostici!$J51&lt;&gt;"",Pronostici!$I51=Partite!$G51,Pronostici!$J51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$Q51)=1),Config!$D$9,Config!$D$6),IF(AND($K51&lt;&gt;"",$K51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$K51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$I51&lt;&gt;"",Pronostici!$J51&lt;&gt;"",Pronostici!$I51=Partite!$G51,Pronostici!$J51=Partite!$H51),Config!$D$6,IF(AND($K51&lt;&gt;"",$K51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$L51&lt;&gt;"",Pronostici!$M51&lt;&gt;"",Pronostici!$L51=Partite!$G51,Pronostici!$M51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$R51)=1),Config!$D$9,Config!$D$6),IF(AND($L51&lt;&gt;"",$L51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$L51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$L51&lt;&gt;"",Pronostici!$M51&lt;&gt;"",Pronostici!$L51=Partite!$G51,Pronostici!$M51=Partite!$H51),Config!$D$6,IF(AND($L51&lt;&gt;"",$L51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$O51&lt;&gt;"",Pronostici!$P51&lt;&gt;"",Pronostici!$O51=Partite!$G51,Pronostici!$P51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$S51)=1),Config!$D$9,Config!$D$6),IF(AND($M51&lt;&gt;"",$M51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$M51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$O51&lt;&gt;"",Pronostici!$P51&lt;&gt;"",Pronostici!$O51=Partite!$G51,Pronostici!$P51=Partite!$H51),Config!$D$6,IF(AND($M51&lt;&gt;"",$M51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$R51&lt;&gt;"",Pronostici!$S51&lt;&gt;"",Pronostici!$R51=Partite!$G51,Pronostici!$S51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$T51)=1),Config!$D$9,Config!$D$6),IF(AND($N51&lt;&gt;"",$N51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$N51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$R51&lt;&gt;"",Pronostici!$S51&lt;&gt;"",Pronostici!$R51=Partite!$G51,Pronostici!$S51=Partite!$H51),Config!$D$6,IF(AND($N51&lt;&gt;"",$N51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J51" s="63">
@@ -12035,26 +11054,6 @@
       </c>
       <c r="N51" s="63">
         <f>IF(Pronostici!$Q51&lt;&gt;"",UPPER(Pronostici!$Q51),IF(OR(Pronostici!$R51="",Pronostici!$S51=""),"",IF(Pronostici!$R51&gt;Pronostici!$S51,"1",IF(Pronostici!$R51=Pronostici!$S51,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P51" s="63">
-        <f>IF(OR(Pronostici!$F51="",Pronostici!$G51=""),"",Pronostici!$F51&amp;" a "&amp;Pronostici!$G51)</f>
-        <v/>
-      </c>
-      <c r="Q51" s="63">
-        <f>IF(OR(Pronostici!$I51="",Pronostici!$J51=""),"",Pronostici!$I51&amp;" a "&amp;Pronostici!$J51)</f>
-        <v/>
-      </c>
-      <c r="R51" s="63">
-        <f>IF(OR(Pronostici!$L51="",Pronostici!$M51=""),"",Pronostici!$L51&amp;" a "&amp;Pronostici!$M51)</f>
-        <v/>
-      </c>
-      <c r="S51" s="63">
-        <f>IF(OR(Pronostici!$O51="",Pronostici!$P51=""),"",Pronostici!$O51&amp;" a "&amp;Pronostici!$P51)</f>
-        <v/>
-      </c>
-      <c r="T51" s="63">
-        <f>IF(OR(Pronostici!$R51="",Pronostici!$S51=""),"",Pronostici!$R51&amp;" a "&amp;Pronostici!$S51)</f>
         <v/>
       </c>
     </row>
@@ -12072,23 +11071,23 @@
         <v/>
       </c>
       <c r="D52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$F52&lt;&gt;"",Pronostici!$G52&lt;&gt;"",Pronostici!$F52=Partite!$G52,Pronostici!$G52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$P52)=1),Config!$D$9,Config!$D$6),IF(AND($J52&lt;&gt;"",$J52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$J52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$F52&lt;&gt;"",Pronostici!$G52&lt;&gt;"",Pronostici!$F52=Partite!$G52,Pronostici!$G52=Partite!$H52),Config!$D$6,IF(AND($J52&lt;&gt;"",$J52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$I52&lt;&gt;"",Pronostici!$J52&lt;&gt;"",Pronostici!$I52=Partite!$G52,Pronostici!$J52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$Q52)=1),Config!$D$9,Config!$D$6),IF(AND($K52&lt;&gt;"",$K52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$K52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$I52&lt;&gt;"",Pronostici!$J52&lt;&gt;"",Pronostici!$I52=Partite!$G52,Pronostici!$J52=Partite!$H52),Config!$D$6,IF(AND($K52&lt;&gt;"",$K52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$L52&lt;&gt;"",Pronostici!$M52&lt;&gt;"",Pronostici!$L52=Partite!$G52,Pronostici!$M52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$R52)=1),Config!$D$9,Config!$D$6),IF(AND($L52&lt;&gt;"",$L52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$L52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$L52&lt;&gt;"",Pronostici!$M52&lt;&gt;"",Pronostici!$L52=Partite!$G52,Pronostici!$M52=Partite!$H52),Config!$D$6,IF(AND($L52&lt;&gt;"",$L52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$O52&lt;&gt;"",Pronostici!$P52&lt;&gt;"",Pronostici!$O52=Partite!$G52,Pronostici!$P52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$S52)=1),Config!$D$9,Config!$D$6),IF(AND($M52&lt;&gt;"",$M52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$M52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$O52&lt;&gt;"",Pronostici!$P52&lt;&gt;"",Pronostici!$O52=Partite!$G52,Pronostici!$P52=Partite!$H52),Config!$D$6,IF(AND($M52&lt;&gt;"",$M52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$R52&lt;&gt;"",Pronostici!$S52&lt;&gt;"",Pronostici!$R52=Partite!$G52,Pronostici!$S52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$T52)=1),Config!$D$9,Config!$D$6),IF(AND($N52&lt;&gt;"",$N52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$N52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$R52&lt;&gt;"",Pronostici!$S52&lt;&gt;"",Pronostici!$R52=Partite!$G52,Pronostici!$S52=Partite!$H52),Config!$D$6,IF(AND($N52&lt;&gt;"",$N52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J52" s="63">
@@ -12109,26 +11108,6 @@
       </c>
       <c r="N52" s="63">
         <f>IF(Pronostici!$Q52&lt;&gt;"",UPPER(Pronostici!$Q52),IF(OR(Pronostici!$R52="",Pronostici!$S52=""),"",IF(Pronostici!$R52&gt;Pronostici!$S52,"1",IF(Pronostici!$R52=Pronostici!$S52,"X","2"))))</f>
-        <v/>
-      </c>
-      <c r="P52" s="63">
-        <f>IF(OR(Pronostici!$F52="",Pronostici!$G52=""),"",Pronostici!$F52&amp;" a "&amp;Pronostici!$G52)</f>
-        <v/>
-      </c>
-      <c r="Q52" s="63">
-        <f>IF(OR(Pronostici!$I52="",Pronostici!$J52=""),"",Pronostici!$I52&amp;" a "&amp;Pronostici!$J52)</f>
-        <v/>
-      </c>
-      <c r="R52" s="63">
-        <f>IF(OR(Pronostici!$L52="",Pronostici!$M52=""),"",Pronostici!$L52&amp;" a "&amp;Pronostici!$M52)</f>
-        <v/>
-      </c>
-      <c r="S52" s="63">
-        <f>IF(OR(Pronostici!$O52="",Pronostici!$P52=""),"",Pronostici!$O52&amp;" a "&amp;Pronostici!$P52)</f>
-        <v/>
-      </c>
-      <c r="T52" s="63">
-        <f>IF(OR(Pronostici!$R52="",Pronostici!$S52=""),"",Pronostici!$R52&amp;" a "&amp;Pronostici!$S52)</f>
         <v/>
       </c>
     </row>
@@ -12140,45 +11119,40 @@
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>1</formula>
-      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E52">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>1</formula>
-      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F52">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
       <formula>1</formula>
-      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G52">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="1">
       <formula>1</formula>
-      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H52">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
       <formula>1</formula>
-      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12296,13 +11270,10 @@
           <t>Just Lele</t>
         </is>
       </c>
-      <c r="C9" s="47" t="inlineStr">
-        <is>
-          <t>CORAGGIO - risultato esatto, e nessun altro lo aveva scritto</t>
-        </is>
-      </c>
-      <c r="D9" s="96" t="n">
-        <v>6</v>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Il risultato esatto non si somma al segno. Non c'e' nient'altro: i punti non si moltiplicano mai.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -12311,21 +11282,6 @@
           <t>Lippi</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
-        <is>
-          <t>CORAGGIO - segno giusto, e nessun altro lo aveva scelto</t>
-        </is>
-      </c>
-      <c r="D10" s="96" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="C11" s="35" t="inlineStr">
-        <is>
-          <t>Il risultato esatto non si somma al segno. Gli ultimi due sono i punti coraggio: chi indovina da solo prende il doppio.</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="C13" s="36" t="inlineStr">
@@ -12366,16 +11322,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17">
-      <c r="C17" s="47" t="inlineStr">
-        <is>
-          <t>I punti coraggio valgono dalla giornata</t>
-        </is>
-      </c>
-      <c r="D17" s="71" t="n">
-        <v>5</v>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
@@ -12407,21 +11353,14 @@
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="102" t="inlineStr">
         <is>
-          <t>4.  Punti coraggio, dalla giornata 5: chi indovina da solo vale doppio, 2 il segno e 6 il risultato esatto.</t>
+          <t>4.  Parita' in classifica generale: passa avanti chi ha piu' risultati esatti.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="101" t="inlineStr">
         <is>
-          <t>5.  Parita' in classifica generale: passa avanti chi ha piu' risultati esatti.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="102" t="inlineStr">
-        <is>
-          <t>6.  Re della giornata = chi fa piu' punti in quella giornata (solo giornate complete).</t>
+          <t>5.  Re della giornata = chi fa piu' punti in quella giornata (solo giornate complete).</t>
         </is>
       </c>
     </row>
@@ -12554,11 +11493,11 @@
         <v>1</v>
       </c>
       <c r="E38" s="105" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F38" s="106" t="inlineStr">
         <is>
-          <t>risultato esatto, e nessun altro aveva scritto 2-1</t>
+          <t>risultato esatto: sul sito la casella e' oro, era l'unico</t>
         </is>
       </c>
     </row>
@@ -12584,7 +11523,7 @@
       </c>
       <c r="F39" s="106" t="inlineStr">
         <is>
-          <t>segno giusto, ma l'1 lo avevano in tre</t>
+          <t>solo il segno: casella bronzo</t>
         </is>
       </c>
     </row>
@@ -12606,7 +11545,7 @@
       </c>
       <c r="F40" s="106" t="inlineStr">
         <is>
-          <t>solo il segno, giusto ma in compagnia</t>
+          <t>solo il segno, senza punteggio: bronzo anche lui</t>
         </is>
       </c>
     </row>
@@ -12657,7 +11596,7 @@
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
         <is>
-          <t>Esempio dalla giornata 5 in poi. Se il segno giusto lo avesse scelto una persona sola, a lei varrebbe 2 punti invece di 1.</t>
+          <t>I colori delle caselle sul sito non cambiano i punti: oro e argento valgono gli stessi 3, e dicono solo se il risultato esatto lo aveva preso qualcun altro.</t>
         </is>
       </c>
     </row>
@@ -12676,14 +11615,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="C33:D33"/>
-    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="A25:D25"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 15:02
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -11497,7 +11497,7 @@
       </c>
       <c r="F38" s="106" t="inlineStr">
         <is>
-          <t>risultato esatto: sul sito la casella e' oro, era l'unico</t>
+          <t>risultato esatto: sul sito la casella e' argento</t>
         </is>
       </c>
     </row>
@@ -11596,7 +11596,7 @@
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
         <is>
-          <t>I colori delle caselle sul sito non cambiano i punti: oro e argento valgono gli stessi 3, e dicono solo se il risultato esatto lo aveva preso qualcun altro.</t>
+          <t>I colori delle caselle sul sito non cambiano i punti. Qui Berta e' argento e non oro perche' altri due erano sull'1: l'oro va a chi prende il risultato esatto quando nessun altro aveva nemmeno azzeccato il segno.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 17:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4314,8 +4314,12 @@
           <t>Genoa</t>
         </is>
       </c>
-      <c r="G40" s="71" t="n"/>
-      <c r="H40" s="71" t="n"/>
+      <c r="G40" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I40" s="76">
         <f>IF(OR($G40="",$H40=""),"",IF($G40&gt;$H40,"1",IF($G40=$H40,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 17:14
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4270,8 +4270,12 @@
           <t>Como</t>
         </is>
       </c>
-      <c r="G39" s="71" t="n"/>
-      <c r="H39" s="71" t="n"/>
+      <c r="G39" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I39" s="76">
         <f>IF(OR($G39="",$H39=""),"",IF($G39&gt;$H39,"1",IF($G39=$H39,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 20:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4366,8 +4366,12 @@
           <t>Atalanta</t>
         </is>
       </c>
-      <c r="G41" s="71" t="n"/>
-      <c r="H41" s="71" t="n"/>
+      <c r="G41" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I41" s="76">
         <f>IF(OR($G41="",$H41=""),"",IF($G41&gt;$H41,"1",IF($G41=$H41,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 20/09/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$37</f>
+              <f>'Classifica'!$A$33:$A$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$R$33:$R$37</f>
+              <f>'Classifica'!$R$33:$R$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -851,12 +851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$37</f>
+              <f>'Classifica'!$A$33:$A$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$S$33:$S$37</f>
+              <f>'Classifica'!$S$33:$S$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -888,12 +888,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$37</f>
+              <f>'Classifica'!$A$33:$A$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$T$33:$T$37</f>
+              <f>'Classifica'!$T$33:$T$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -925,12 +925,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$37</f>
+              <f>'Classifica'!$A$33:$A$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$U$33:$U$37</f>
+              <f>'Classifica'!$U$33:$U$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -962,12 +962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$37</f>
+              <f>'Classifica'!$A$33:$A$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$V$33:$V$37</f>
+              <f>'Classifica'!$V$33:$V$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1043,7 +1043,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9720000" cy="3420000"/>
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>COUNTIF($B$33:$B$37,"Completata")</f>
+        <f>COUNTIF($B$33:$B$38,"Completata")</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>COUNTIF($B$33:$B$37,"Completata")+COUNTIF($B$33:$B$37,"In corso")</f>
+        <f>COUNTIF($B$33:$B$38,"Completata")+COUNTIF($B$33:$B$38,"In corso")</f>
         <v/>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L7" s="13">
-        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$37="Completata")*$A$33:$A$37)))</f>
+        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$38="Completata")*$A$33:$A$38)))</f>
         <v/>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="L8" s="13">
-        <f>IF(SUMPRODUCT(MIN(($B$33:$B$37&lt;&gt;"Completata")*$A$33:$A$37+($B$33:$B$37="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$37&lt;&gt;"Completata")*$A$33:$A$37+($B$33:$B$37="Completata")*999)))</f>
+        <f>IF(SUMPRODUCT(MIN(($B$33:$B$38&lt;&gt;"Completata")*$A$33:$A$38+($B$33:$B$38="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$38&lt;&gt;"Completata")*$A$33:$A$38+($B$33:$B$38="Completata")*999)))</f>
         <v/>
       </c>
     </row>
@@ -1591,19 +1591,19 @@
         <v/>
       </c>
       <c r="C12" s="24">
-        <f>SUM(Punti!$D$3:$D$52)</f>
+        <f>SUM(Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$7)+COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$62,Config!$D$7)+COUNTIF(Punti!$D$3:$D$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>SUMPRODUCT(((Pronostici!$E$3:$E$52&lt;&gt;"")+(Pronostici!$F$3:$F$52&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$E$3:$E$62&lt;&gt;"")+(Pronostici!$F$3:$F$62&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>SUMPRODUCT(($C$33:$C$37=$H$33:$H$37)*($H$33:$H$37&gt;0)*($B$33:$B$37="Completata"))</f>
+        <f>SUMPRODUCT(($C$33:$C$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1625,19 +1625,19 @@
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>SUM(Punti!$E$3:$E$52)</f>
+        <f>SUM(Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$7)+COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$62,Config!$D$7)+COUNTIF(Punti!$E$3:$E$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
-        <f>SUMPRODUCT(((Pronostici!$H$3:$H$52&lt;&gt;"")+(Pronostici!$I$3:$I$52&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$H$3:$H$62&lt;&gt;"")+(Pronostici!$I$3:$I$62&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G13" s="31">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="H13" s="30">
-        <f>SUMPRODUCT(($D$33:$D$37=$H$33:$H$37)*($H$33:$H$37&gt;0)*($B$33:$B$37="Completata"))</f>
+        <f>SUMPRODUCT(($D$33:$D$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1659,19 @@
         <v/>
       </c>
       <c r="C14" s="24">
-        <f>SUM(Punti!$F$3:$F$52)</f>
+        <f>SUM(Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$7)+COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$62,Config!$D$7)+COUNTIF(Punti!$F$3:$F$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>SUMPRODUCT(((Pronostici!$K$3:$K$52&lt;&gt;"")+(Pronostici!$L$3:$L$52&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$K$3:$K$62&lt;&gt;"")+(Pronostici!$L$3:$L$62&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>SUMPRODUCT(($E$33:$E$37=$H$33:$H$37)*($H$33:$H$37&gt;0)*($B$33:$B$37="Completata"))</f>
+        <f>SUMPRODUCT(($E$33:$E$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1693,19 +1693,19 @@
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>SUM(Punti!$G$3:$G$52)</f>
+        <f>SUM(Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$7)+COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$62,Config!$D$7)+COUNTIF(Punti!$G$3:$G$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
-        <f>SUMPRODUCT(((Pronostici!$N$3:$N$52&lt;&gt;"")+(Pronostici!$O$3:$O$52&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$N$3:$N$62&lt;&gt;"")+(Pronostici!$O$3:$O$62&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G15" s="31">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="H15" s="30">
-        <f>SUMPRODUCT(($F$33:$F$37=$H$33:$H$37)*($H$33:$H$37&gt;0)*($B$33:$B$37="Completata"))</f>
+        <f>SUMPRODUCT(($F$33:$F$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1727,19 +1727,19 @@
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>SUM(Punti!$H$3:$H$52)</f>
+        <f>SUM(Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$7)+COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$62,Config!$D$7)+COUNTIF(Punti!$H$3:$H$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$62,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$52&lt;&gt;"")+(Pronostici!$R$3:$R$52&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$62&lt;&gt;"")+(Pronostici!$R$3:$R$62&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>SUMPRODUCT(($G$33:$G$37=$H$33:$H$37)*($H$33:$H$37&gt;0)*($B$33:$B$37="Completata"))</f>
+        <f>SUMPRODUCT(($G$33:$G$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         <v/>
       </c>
       <c r="C20" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$37,MATCH($L$7,$A$33:$A$37,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
         <v/>
       </c>
       <c r="D20" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$37,MATCH($L$7,$A$33:$A$37,0)),0)=IFERROR(INDEX($H$33:$H$37,MATCH($L$7,$A$33:$A$37,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E20" s="41" t="n"/>
       <c r="K20" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L20" s="43" t="n"/>
@@ -1826,7 +1826,7 @@
         <v/>
       </c>
       <c r="O20" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$52=$L$8)*(((Pronostici!$E$3:$E$52&lt;&gt;"")+(Pronostici!$F$3:$F$52&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$E$3:$E$62&lt;&gt;"")+(Pronostici!$F$3:$F$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1836,16 +1836,16 @@
         <v/>
       </c>
       <c r="C21" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$37,MATCH($L$7,$A$33:$A$37,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
         <v/>
       </c>
       <c r="D21" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$37,MATCH($L$7,$A$33:$A$37,0)),0)=IFERROR(INDEX($H$33:$H$37,MATCH($L$7,$A$33:$A$37,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E21" s="41" t="n"/>
       <c r="K21" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L21" s="47" t="n"/>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="O21" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$52=$L$8)*(((Pronostici!$H$3:$H$52&lt;&gt;"")+(Pronostici!$I$3:$I$52&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$H$3:$H$62&lt;&gt;"")+(Pronostici!$I$3:$I$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v/>
       </c>
       <c r="C22" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$37,MATCH($L$7,$A$33:$A$37,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
         <v/>
       </c>
       <c r="D22" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$37,MATCH($L$7,$A$33:$A$37,0)),0)=IFERROR(INDEX($H$33:$H$37,MATCH($L$7,$A$33:$A$37,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E22" s="41" t="n"/>
       <c r="K22" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L22" s="43" t="n"/>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="O22" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$52=$L$8)*(((Pronostici!$K$3:$K$52&lt;&gt;"")+(Pronostici!$L$3:$L$52&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$K$3:$K$62&lt;&gt;"")+(Pronostici!$L$3:$L$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1894,16 +1894,16 @@
         <v/>
       </c>
       <c r="C23" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$37,MATCH($L$7,$A$33:$A$37,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
         <v/>
       </c>
       <c r="D23" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$37,MATCH($L$7,$A$33:$A$37,0)),0)=IFERROR(INDEX($H$33:$H$37,MATCH($L$7,$A$33:$A$37,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E23" s="41" t="n"/>
       <c r="K23" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L23" s="47" t="n"/>
@@ -1913,7 +1913,7 @@
         <v/>
       </c>
       <c r="O23" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$52=$L$8)*(((Pronostici!$N$3:$N$52&lt;&gt;"")+(Pronostici!$O$3:$O$52&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$N$3:$N$62&lt;&gt;"")+(Pronostici!$O$3:$O$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1923,16 +1923,16 @@
         <v/>
       </c>
       <c r="C24" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$37,MATCH($L$7,$A$33:$A$37,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
         <v/>
       </c>
       <c r="D24" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$37,MATCH($L$7,$A$33:$A$37,0)),0)=IFERROR(INDEX($H$33:$H$37,MATCH($L$7,$A$33:$A$37,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E24" s="41" t="n"/>
       <c r="K24" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L24" s="43" t="n"/>
@@ -1942,13 +1942,13 @@
         <v/>
       </c>
       <c r="O24" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$52=$L$8)*(((Pronostici!$Q$3:$Q$52&lt;&gt;"")+(Pronostici!$R$3:$R$52&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$Q$3:$Q$62&lt;&gt;"")+(Pronostici!$R$3:$R$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L25" s="47" t="n"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="26">
       <c r="K26" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L26" s="43" t="n"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="27">
       <c r="K27" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L27" s="47" t="n"/>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="28">
       <c r="K28" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L28" s="43" t="n"/>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="29">
       <c r="K29" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$52,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$52,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$52,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$62,0)),"-")</f>
         <v/>
       </c>
       <c r="L29" s="47" t="n"/>
@@ -2070,27 +2070,27 @@
         <v>2</v>
       </c>
       <c r="B33" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$52,$A33,Partite!$E$3:$E$52,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$52,$A33,Partite!$K$3:$K$52,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$52,$A33,Partite!$K$3:$K$52,"Giocata")=COUNTIFS(Partite!$B$3:$B$52,$A33,Partite!$E$3:$E$52,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A33,Punti!$D$3:$D$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A33,Punti!$E$3:$E$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A33,Punti!$F$3:$F$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A33,Punti!$G$3:$G$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A33,Punti!$H$3:$H$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="H33" s="61">
@@ -2127,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="B34" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$52,$A34,Partite!$E$3:$E$52,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$52,$A34,Partite!$K$3:$K$52,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$52,$A34,Partite!$K$3:$K$52,"Giocata")=COUNTIFS(Partite!$B$3:$B$52,$A34,Partite!$E$3:$E$52,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A34,Punti!$D$3:$D$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A34,Punti!$E$3:$E$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A34,Punti!$F$3:$F$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A34,Punti!$G$3:$G$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A34,Punti!$H$3:$H$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="H34" s="61">
@@ -2184,27 +2184,27 @@
         <v>4</v>
       </c>
       <c r="B35" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$52,$A35,Partite!$E$3:$E$52,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$52,$A35,Partite!$K$3:$K$52,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$52,$A35,Partite!$K$3:$K$52,"Giocata")=COUNTIFS(Partite!$B$3:$B$52,$A35,Partite!$E$3:$E$52,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A35,Punti!$D$3:$D$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A35,Punti!$E$3:$E$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="E35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A35,Punti!$F$3:$F$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="F35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A35,Punti!$G$3:$G$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="G35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A35,Punti!$H$3:$H$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="H35" s="61">
@@ -2241,27 +2241,27 @@
         <v>5</v>
       </c>
       <c r="B36" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$52,$A36,Partite!$E$3:$E$52,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$52,$A36,Partite!$K$3:$K$52,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$52,$A36,Partite!$K$3:$K$52,"Giocata")=COUNTIFS(Partite!$B$3:$B$52,$A36,Partite!$E$3:$E$52,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A36,Punti!$D$3:$D$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A36,Punti!$E$3:$E$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A36,Punti!$F$3:$F$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A36,Punti!$G$3:$G$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$52,$A36,Punti!$H$3:$H$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="H36" s="61">
@@ -2298,27 +2298,27 @@
         <v>6</v>
       </c>
       <c r="B37" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$52,$A37,Partite!$E$3:$E$52,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$52,$A37,Partite!$K$3:$K$52,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$52,$A37,Partite!$K$3:$K$52,"Giocata")=COUNTIFS(Partite!$B$3:$B$52,$A37,Partite!$E$3:$E$52,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A37,Punti!$D$3:$D$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$D$3:$D$62)</f>
         <v/>
       </c>
       <c r="D37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A37,Punti!$E$3:$E$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$E$3:$E$62)</f>
         <v/>
       </c>
       <c r="E37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A37,Punti!$F$3:$F$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$F$3:$F$62)</f>
         <v/>
       </c>
       <c r="F37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A37,Punti!$G$3:$G$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$G$3:$G$62)</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$52,$A37,Punti!$H$3:$H$52)</f>
+        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$H$3:$H$62)</f>
         <v/>
       </c>
       <c r="H37" s="61">
@@ -2347,6 +2347,63 @@
       </c>
       <c r="V37" s="63">
         <f>V36+G37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" s="47">
+        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <v/>
+      </c>
+      <c r="C38" s="30">
+        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$D$3:$D$62)</f>
+        <v/>
+      </c>
+      <c r="D38" s="30">
+        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$E$3:$E$62)</f>
+        <v/>
+      </c>
+      <c r="E38" s="30">
+        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$F$3:$F$62)</f>
+        <v/>
+      </c>
+      <c r="F38" s="30">
+        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$G$3:$G$62)</f>
+        <v/>
+      </c>
+      <c r="G38" s="30">
+        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$H$3:$H$62)</f>
+        <v/>
+      </c>
+      <c r="H38" s="61">
+        <f>MAX($C38:$G38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="64">
+        <f>IF($H38&lt;=0,"-",INDEX($C$32:$G$32,MATCH($H38,$C38:$G38,0))&amp;IF(COUNTIF($C38:$G38,$H38)&gt;1," (a pari)","")&amp;IF($B38="Completata",""," - in corso"))</f>
+        <v/>
+      </c>
+      <c r="R38" s="63">
+        <f>R37+C38</f>
+        <v/>
+      </c>
+      <c r="S38" s="63">
+        <f>S37+D38</f>
+        <v/>
+      </c>
+      <c r="T38" s="63">
+        <f>T37+E38</f>
+        <v/>
+      </c>
+      <c r="U38" s="63">
+        <f>U37+F38</f>
+        <v/>
+      </c>
+      <c r="V38" s="63">
+        <f>V37+G38</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2450,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:G37">
+  <conditionalFormatting sqref="C33:G38">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2415,7 +2472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4414,8 +4471,12 @@
           <t>Lecce</t>
         </is>
       </c>
-      <c r="G42" s="71" t="n"/>
-      <c r="H42" s="71" t="n"/>
+      <c r="G42" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I42" s="76">
         <f>IF(OR($G42="",$H42=""),"",IF($G42&gt;$H42,"1",IF($G42=$H42,"X","2")))</f>
         <v/>
@@ -4869,14 +4930,454 @@
         <v/>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="74" t="inlineStr">
+        <is>
+          <t>G07-01</t>
+        </is>
+      </c>
+      <c r="B53" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C53" s="30" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E53" s="75" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="F53" s="75" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="G53" s="71" t="n"/>
+      <c r="H53" s="71" t="n"/>
+      <c r="I53" s="76">
+        <f>IF(OR($G53="",$H53=""),"",IF($G53&gt;$H53,"1",IF($G53=$H53,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J53" s="30">
+        <f>IF(OR($G53="",$H53=""),"",$G53&amp;"-"&amp;$H53)</f>
+        <v/>
+      </c>
+      <c r="K53" s="77">
+        <f>IF($E53="","Calendario da inserire",IF(OR($G53="",$H53=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="74" t="inlineStr">
+        <is>
+          <t>G07-02</t>
+        </is>
+      </c>
+      <c r="B54" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C54" s="30" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="D54" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E54" s="75" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="F54" s="75" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="G54" s="71" t="n"/>
+      <c r="H54" s="71" t="n"/>
+      <c r="I54" s="76">
+        <f>IF(OR($G54="",$H54=""),"",IF($G54&gt;$H54,"1",IF($G54=$H54,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J54" s="30">
+        <f>IF(OR($G54="",$H54=""),"",$G54&amp;"-"&amp;$H54)</f>
+        <v/>
+      </c>
+      <c r="K54" s="77">
+        <f>IF($E54="","Calendario da inserire",IF(OR($G54="",$H54=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="74" t="inlineStr">
+        <is>
+          <t>G07-03</t>
+        </is>
+      </c>
+      <c r="B55" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C55" s="30" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E55" s="75" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="F55" s="75" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="G55" s="71" t="n"/>
+      <c r="H55" s="71" t="n"/>
+      <c r="I55" s="76">
+        <f>IF(OR($G55="",$H55=""),"",IF($G55&gt;$H55,"1",IF($G55=$H55,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J55" s="30">
+        <f>IF(OR($G55="",$H55=""),"",$G55&amp;"-"&amp;$H55)</f>
+        <v/>
+      </c>
+      <c r="K55" s="77">
+        <f>IF($E55="","Calendario da inserire",IF(OR($G55="",$H55=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="74" t="inlineStr">
+        <is>
+          <t>G07-04</t>
+        </is>
+      </c>
+      <c r="B56" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="D56" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E56" s="75" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="F56" s="75" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="G56" s="71" t="n"/>
+      <c r="H56" s="71" t="n"/>
+      <c r="I56" s="76">
+        <f>IF(OR($G56="",$H56=""),"",IF($G56&gt;$H56,"1",IF($G56=$H56,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J56" s="30">
+        <f>IF(OR($G56="",$H56=""),"",$G56&amp;"-"&amp;$H56)</f>
+        <v/>
+      </c>
+      <c r="K56" s="77">
+        <f>IF($E56="","Calendario da inserire",IF(OR($G56="",$H56=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="74" t="inlineStr">
+        <is>
+          <t>G07-05</t>
+        </is>
+      </c>
+      <c r="B57" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E57" s="75" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="F57" s="75" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="G57" s="71" t="n"/>
+      <c r="H57" s="71" t="n"/>
+      <c r="I57" s="76">
+        <f>IF(OR($G57="",$H57=""),"",IF($G57&gt;$H57,"1",IF($G57=$H57,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J57" s="30">
+        <f>IF(OR($G57="",$H57=""),"",$G57&amp;"-"&amp;$H57)</f>
+        <v/>
+      </c>
+      <c r="K57" s="77">
+        <f>IF($E57="","Calendario da inserire",IF(OR($G57="",$H57=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="74" t="inlineStr">
+        <is>
+          <t>G07-06</t>
+        </is>
+      </c>
+      <c r="B58" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E58" s="75" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="F58" s="75" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="G58" s="71" t="n"/>
+      <c r="H58" s="71" t="n"/>
+      <c r="I58" s="76">
+        <f>IF(OR($G58="",$H58=""),"",IF($G58&gt;$H58,"1",IF($G58=$H58,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J58" s="30">
+        <f>IF(OR($G58="",$H58=""),"",$G58&amp;"-"&amp;$H58)</f>
+        <v/>
+      </c>
+      <c r="K58" s="77">
+        <f>IF($E58="","Calendario da inserire",IF(OR($G58="",$H58=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="74" t="inlineStr">
+        <is>
+          <t>G07-07</t>
+        </is>
+      </c>
+      <c r="B59" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="D59" s="30" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E59" s="75" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="F59" s="75" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="G59" s="71" t="n"/>
+      <c r="H59" s="71" t="n"/>
+      <c r="I59" s="76">
+        <f>IF(OR($G59="",$H59=""),"",IF($G59&gt;$H59,"1",IF($G59=$H59,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J59" s="30">
+        <f>IF(OR($G59="",$H59=""),"",$G59&amp;"-"&amp;$H59)</f>
+        <v/>
+      </c>
+      <c r="K59" s="77">
+        <f>IF($E59="","Calendario da inserire",IF(OR($G59="",$H59=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="74" t="inlineStr">
+        <is>
+          <t>G07-08</t>
+        </is>
+      </c>
+      <c r="B60" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" s="30" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="D60" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E60" s="75" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="F60" s="75" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="G60" s="71" t="n"/>
+      <c r="H60" s="71" t="n"/>
+      <c r="I60" s="76">
+        <f>IF(OR($G60="",$H60=""),"",IF($G60&gt;$H60,"1",IF($G60=$H60,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J60" s="30">
+        <f>IF(OR($G60="",$H60=""),"",$G60&amp;"-"&amp;$H60)</f>
+        <v/>
+      </c>
+      <c r="K60" s="77">
+        <f>IF($E60="","Calendario da inserire",IF(OR($G60="",$H60=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="74" t="inlineStr">
+        <is>
+          <t>G07-09</t>
+        </is>
+      </c>
+      <c r="B61" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C61" s="30" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="D61" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E61" s="75" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="F61" s="75" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="G61" s="71" t="n"/>
+      <c r="H61" s="71" t="n"/>
+      <c r="I61" s="76">
+        <f>IF(OR($G61="",$H61=""),"",IF($G61&gt;$H61,"1",IF($G61=$H61,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J61" s="30">
+        <f>IF(OR($G61="",$H61=""),"",$G61&amp;"-"&amp;$H61)</f>
+        <v/>
+      </c>
+      <c r="K61" s="77">
+        <f>IF($E61="","Calendario da inserire",IF(OR($G61="",$H61=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="74" t="inlineStr">
+        <is>
+          <t>G07-10</t>
+        </is>
+      </c>
+      <c r="B62" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C62" s="30" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="D62" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E62" s="75" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="F62" s="75" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="G62" s="71" t="n"/>
+      <c r="H62" s="71" t="n"/>
+      <c r="I62" s="76">
+        <f>IF(OR($G62="",$H62=""),"",IF($G62&gt;$H62,"1",IF($G62=$H62,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J62" s="30">
+        <f>IF(OR($G62="",$H62=""),"",$G62&amp;"-"&amp;$H62)</f>
+        <v/>
+      </c>
+      <c r="K62" s="77">
+        <f>IF($E62="","Calendario da inserire",IF(OR($G62="",$H62=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K52"/>
+  <autoFilter ref="A2:K62"/>
   <mergeCells count="3">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K3:K52">
+  <conditionalFormatting sqref="K3:K62">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Giocata"</formula>
     </cfRule>
@@ -4892,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S52"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8303,8 +8804,338 @@
       <c r="R52" s="71" t="n"/>
       <c r="S52" s="71" t="n"/>
     </row>
+    <row r="53">
+      <c r="A53" s="74">
+        <f>Partite!$A53</f>
+        <v/>
+      </c>
+      <c r="B53" s="30">
+        <f>Partite!$B53</f>
+        <v/>
+      </c>
+      <c r="C53" s="75">
+        <f>IF(Partite!$E53="","",Partite!$E53)</f>
+        <v/>
+      </c>
+      <c r="D53" s="75">
+        <f>IF(Partite!$F53="","",Partite!$F53)</f>
+        <v/>
+      </c>
+      <c r="E53" s="71" t="n"/>
+      <c r="F53" s="71" t="n"/>
+      <c r="G53" s="71" t="n"/>
+      <c r="H53" s="71" t="n"/>
+      <c r="I53" s="71" t="n"/>
+      <c r="J53" s="71" t="n"/>
+      <c r="K53" s="71" t="n"/>
+      <c r="L53" s="71" t="n"/>
+      <c r="M53" s="71" t="n"/>
+      <c r="N53" s="71" t="n"/>
+      <c r="O53" s="71" t="n"/>
+      <c r="P53" s="71" t="n"/>
+      <c r="Q53" s="71" t="n"/>
+      <c r="R53" s="71" t="n"/>
+      <c r="S53" s="71" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="74">
+        <f>Partite!$A54</f>
+        <v/>
+      </c>
+      <c r="B54" s="30">
+        <f>Partite!$B54</f>
+        <v/>
+      </c>
+      <c r="C54" s="75">
+        <f>IF(Partite!$E54="","",Partite!$E54)</f>
+        <v/>
+      </c>
+      <c r="D54" s="75">
+        <f>IF(Partite!$F54="","",Partite!$F54)</f>
+        <v/>
+      </c>
+      <c r="E54" s="71" t="n"/>
+      <c r="F54" s="71" t="n"/>
+      <c r="G54" s="71" t="n"/>
+      <c r="H54" s="71" t="n"/>
+      <c r="I54" s="71" t="n"/>
+      <c r="J54" s="71" t="n"/>
+      <c r="K54" s="71" t="n"/>
+      <c r="L54" s="71" t="n"/>
+      <c r="M54" s="71" t="n"/>
+      <c r="N54" s="71" t="n"/>
+      <c r="O54" s="71" t="n"/>
+      <c r="P54" s="71" t="n"/>
+      <c r="Q54" s="71" t="n"/>
+      <c r="R54" s="71" t="n"/>
+      <c r="S54" s="71" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="74">
+        <f>Partite!$A55</f>
+        <v/>
+      </c>
+      <c r="B55" s="30">
+        <f>Partite!$B55</f>
+        <v/>
+      </c>
+      <c r="C55" s="75">
+        <f>IF(Partite!$E55="","",Partite!$E55)</f>
+        <v/>
+      </c>
+      <c r="D55" s="75">
+        <f>IF(Partite!$F55="","",Partite!$F55)</f>
+        <v/>
+      </c>
+      <c r="E55" s="71" t="n"/>
+      <c r="F55" s="71" t="n"/>
+      <c r="G55" s="71" t="n"/>
+      <c r="H55" s="71" t="n"/>
+      <c r="I55" s="71" t="n"/>
+      <c r="J55" s="71" t="n"/>
+      <c r="K55" s="71" t="n"/>
+      <c r="L55" s="71" t="n"/>
+      <c r="M55" s="71" t="n"/>
+      <c r="N55" s="71" t="n"/>
+      <c r="O55" s="71" t="n"/>
+      <c r="P55" s="71" t="n"/>
+      <c r="Q55" s="71" t="n"/>
+      <c r="R55" s="71" t="n"/>
+      <c r="S55" s="71" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="74">
+        <f>Partite!$A56</f>
+        <v/>
+      </c>
+      <c r="B56" s="30">
+        <f>Partite!$B56</f>
+        <v/>
+      </c>
+      <c r="C56" s="75">
+        <f>IF(Partite!$E56="","",Partite!$E56)</f>
+        <v/>
+      </c>
+      <c r="D56" s="75">
+        <f>IF(Partite!$F56="","",Partite!$F56)</f>
+        <v/>
+      </c>
+      <c r="E56" s="71" t="n"/>
+      <c r="F56" s="71" t="n"/>
+      <c r="G56" s="71" t="n"/>
+      <c r="H56" s="71" t="n"/>
+      <c r="I56" s="71" t="n"/>
+      <c r="J56" s="71" t="n"/>
+      <c r="K56" s="71" t="n"/>
+      <c r="L56" s="71" t="n"/>
+      <c r="M56" s="71" t="n"/>
+      <c r="N56" s="71" t="n"/>
+      <c r="O56" s="71" t="n"/>
+      <c r="P56" s="71" t="n"/>
+      <c r="Q56" s="71" t="n"/>
+      <c r="R56" s="71" t="n"/>
+      <c r="S56" s="71" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="74">
+        <f>Partite!$A57</f>
+        <v/>
+      </c>
+      <c r="B57" s="30">
+        <f>Partite!$B57</f>
+        <v/>
+      </c>
+      <c r="C57" s="75">
+        <f>IF(Partite!$E57="","",Partite!$E57)</f>
+        <v/>
+      </c>
+      <c r="D57" s="75">
+        <f>IF(Partite!$F57="","",Partite!$F57)</f>
+        <v/>
+      </c>
+      <c r="E57" s="71" t="n"/>
+      <c r="F57" s="71" t="n"/>
+      <c r="G57" s="71" t="n"/>
+      <c r="H57" s="71" t="n"/>
+      <c r="I57" s="71" t="n"/>
+      <c r="J57" s="71" t="n"/>
+      <c r="K57" s="71" t="n"/>
+      <c r="L57" s="71" t="n"/>
+      <c r="M57" s="71" t="n"/>
+      <c r="N57" s="71" t="n"/>
+      <c r="O57" s="71" t="n"/>
+      <c r="P57" s="71" t="n"/>
+      <c r="Q57" s="71" t="n"/>
+      <c r="R57" s="71" t="n"/>
+      <c r="S57" s="71" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="74">
+        <f>Partite!$A58</f>
+        <v/>
+      </c>
+      <c r="B58" s="30">
+        <f>Partite!$B58</f>
+        <v/>
+      </c>
+      <c r="C58" s="75">
+        <f>IF(Partite!$E58="","",Partite!$E58)</f>
+        <v/>
+      </c>
+      <c r="D58" s="75">
+        <f>IF(Partite!$F58="","",Partite!$F58)</f>
+        <v/>
+      </c>
+      <c r="E58" s="71" t="n"/>
+      <c r="F58" s="71" t="n"/>
+      <c r="G58" s="71" t="n"/>
+      <c r="H58" s="71" t="n"/>
+      <c r="I58" s="71" t="n"/>
+      <c r="J58" s="71" t="n"/>
+      <c r="K58" s="71" t="n"/>
+      <c r="L58" s="71" t="n"/>
+      <c r="M58" s="71" t="n"/>
+      <c r="N58" s="71" t="n"/>
+      <c r="O58" s="71" t="n"/>
+      <c r="P58" s="71" t="n"/>
+      <c r="Q58" s="71" t="n"/>
+      <c r="R58" s="71" t="n"/>
+      <c r="S58" s="71" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="74">
+        <f>Partite!$A59</f>
+        <v/>
+      </c>
+      <c r="B59" s="30">
+        <f>Partite!$B59</f>
+        <v/>
+      </c>
+      <c r="C59" s="75">
+        <f>IF(Partite!$E59="","",Partite!$E59)</f>
+        <v/>
+      </c>
+      <c r="D59" s="75">
+        <f>IF(Partite!$F59="","",Partite!$F59)</f>
+        <v/>
+      </c>
+      <c r="E59" s="71" t="n"/>
+      <c r="F59" s="71" t="n"/>
+      <c r="G59" s="71" t="n"/>
+      <c r="H59" s="71" t="n"/>
+      <c r="I59" s="71" t="n"/>
+      <c r="J59" s="71" t="n"/>
+      <c r="K59" s="71" t="n"/>
+      <c r="L59" s="71" t="n"/>
+      <c r="M59" s="71" t="n"/>
+      <c r="N59" s="71" t="n"/>
+      <c r="O59" s="71" t="n"/>
+      <c r="P59" s="71" t="n"/>
+      <c r="Q59" s="71" t="n"/>
+      <c r="R59" s="71" t="n"/>
+      <c r="S59" s="71" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="74">
+        <f>Partite!$A60</f>
+        <v/>
+      </c>
+      <c r="B60" s="30">
+        <f>Partite!$B60</f>
+        <v/>
+      </c>
+      <c r="C60" s="75">
+        <f>IF(Partite!$E60="","",Partite!$E60)</f>
+        <v/>
+      </c>
+      <c r="D60" s="75">
+        <f>IF(Partite!$F60="","",Partite!$F60)</f>
+        <v/>
+      </c>
+      <c r="E60" s="71" t="n"/>
+      <c r="F60" s="71" t="n"/>
+      <c r="G60" s="71" t="n"/>
+      <c r="H60" s="71" t="n"/>
+      <c r="I60" s="71" t="n"/>
+      <c r="J60" s="71" t="n"/>
+      <c r="K60" s="71" t="n"/>
+      <c r="L60" s="71" t="n"/>
+      <c r="M60" s="71" t="n"/>
+      <c r="N60" s="71" t="n"/>
+      <c r="O60" s="71" t="n"/>
+      <c r="P60" s="71" t="n"/>
+      <c r="Q60" s="71" t="n"/>
+      <c r="R60" s="71" t="n"/>
+      <c r="S60" s="71" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="74">
+        <f>Partite!$A61</f>
+        <v/>
+      </c>
+      <c r="B61" s="30">
+        <f>Partite!$B61</f>
+        <v/>
+      </c>
+      <c r="C61" s="75">
+        <f>IF(Partite!$E61="","",Partite!$E61)</f>
+        <v/>
+      </c>
+      <c r="D61" s="75">
+        <f>IF(Partite!$F61="","",Partite!$F61)</f>
+        <v/>
+      </c>
+      <c r="E61" s="71" t="n"/>
+      <c r="F61" s="71" t="n"/>
+      <c r="G61" s="71" t="n"/>
+      <c r="H61" s="71" t="n"/>
+      <c r="I61" s="71" t="n"/>
+      <c r="J61" s="71" t="n"/>
+      <c r="K61" s="71" t="n"/>
+      <c r="L61" s="71" t="n"/>
+      <c r="M61" s="71" t="n"/>
+      <c r="N61" s="71" t="n"/>
+      <c r="O61" s="71" t="n"/>
+      <c r="P61" s="71" t="n"/>
+      <c r="Q61" s="71" t="n"/>
+      <c r="R61" s="71" t="n"/>
+      <c r="S61" s="71" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="74">
+        <f>Partite!$A62</f>
+        <v/>
+      </c>
+      <c r="B62" s="30">
+        <f>Partite!$B62</f>
+        <v/>
+      </c>
+      <c r="C62" s="75">
+        <f>IF(Partite!$E62="","",Partite!$E62)</f>
+        <v/>
+      </c>
+      <c r="D62" s="75">
+        <f>IF(Partite!$F62="","",Partite!$F62)</f>
+        <v/>
+      </c>
+      <c r="E62" s="71" t="n"/>
+      <c r="F62" s="71" t="n"/>
+      <c r="G62" s="71" t="n"/>
+      <c r="H62" s="71" t="n"/>
+      <c r="I62" s="71" t="n"/>
+      <c r="J62" s="71" t="n"/>
+      <c r="K62" s="71" t="n"/>
+      <c r="L62" s="71" t="n"/>
+      <c r="M62" s="71" t="n"/>
+      <c r="N62" s="71" t="n"/>
+      <c r="O62" s="71" t="n"/>
+      <c r="P62" s="71" t="n"/>
+      <c r="Q62" s="71" t="n"/>
+      <c r="R62" s="71" t="n"/>
+      <c r="S62" s="71" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:D52"/>
+  <autoFilter ref="A2:D62"/>
   <mergeCells count="6">
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A1:D1"/>
@@ -8314,7 +9145,7 @@
     <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
       <formula1>"1,X,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8329,7 +9160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11123,11 +11954,551 @@
         <v/>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="74">
+        <f>Partite!$A53</f>
+        <v/>
+      </c>
+      <c r="B53" s="30">
+        <f>Partite!$B53</f>
+        <v/>
+      </c>
+      <c r="C53" s="47">
+        <f>IF(Partite!$E53="","",Partite!$E53&amp;"  -  "&amp;Partite!$F53)</f>
+        <v/>
+      </c>
+      <c r="D53" s="27">
+        <f>IF(Partite!$K53&lt;&gt;"Giocata","",IF(AND(Pronostici!$F53&lt;&gt;"",Pronostici!$G53&lt;&gt;"",Pronostici!$F53=Partite!$G53,Pronostici!$G53=Partite!$H53),Config!$D$6,IF(AND($J53&lt;&gt;"",$J53=Partite!$I53),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E53" s="27">
+        <f>IF(Partite!$K53&lt;&gt;"Giocata","",IF(AND(Pronostici!$I53&lt;&gt;"",Pronostici!$J53&lt;&gt;"",Pronostici!$I53=Partite!$G53,Pronostici!$J53=Partite!$H53),Config!$D$6,IF(AND($K53&lt;&gt;"",$K53=Partite!$I53),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F53" s="27">
+        <f>IF(Partite!$K53&lt;&gt;"Giocata","",IF(AND(Pronostici!$L53&lt;&gt;"",Pronostici!$M53&lt;&gt;"",Pronostici!$L53=Partite!$G53,Pronostici!$M53=Partite!$H53),Config!$D$6,IF(AND($L53&lt;&gt;"",$L53=Partite!$I53),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G53" s="27">
+        <f>IF(Partite!$K53&lt;&gt;"Giocata","",IF(AND(Pronostici!$O53&lt;&gt;"",Pronostici!$P53&lt;&gt;"",Pronostici!$O53=Partite!$G53,Pronostici!$P53=Partite!$H53),Config!$D$6,IF(AND($M53&lt;&gt;"",$M53=Partite!$I53),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H53" s="27">
+        <f>IF(Partite!$K53&lt;&gt;"Giocata","",IF(AND(Pronostici!$R53&lt;&gt;"",Pronostici!$S53&lt;&gt;"",Pronostici!$R53=Partite!$G53,Pronostici!$S53=Partite!$H53),Config!$D$6,IF(AND($N53&lt;&gt;"",$N53=Partite!$I53),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J53" s="63">
+        <f>IF(Pronostici!$E53&lt;&gt;"",UPPER(Pronostici!$E53),IF(OR(Pronostici!$F53="",Pronostici!$G53=""),"",IF(Pronostici!$F53&gt;Pronostici!$G53,"1",IF(Pronostici!$F53=Pronostici!$G53,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K53" s="63">
+        <f>IF(Pronostici!$H53&lt;&gt;"",UPPER(Pronostici!$H53),IF(OR(Pronostici!$I53="",Pronostici!$J53=""),"",IF(Pronostici!$I53&gt;Pronostici!$J53,"1",IF(Pronostici!$I53=Pronostici!$J53,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L53" s="63">
+        <f>IF(Pronostici!$K53&lt;&gt;"",UPPER(Pronostici!$K53),IF(OR(Pronostici!$L53="",Pronostici!$M53=""),"",IF(Pronostici!$L53&gt;Pronostici!$M53,"1",IF(Pronostici!$L53=Pronostici!$M53,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M53" s="63">
+        <f>IF(Pronostici!$N53&lt;&gt;"",UPPER(Pronostici!$N53),IF(OR(Pronostici!$O53="",Pronostici!$P53=""),"",IF(Pronostici!$O53&gt;Pronostici!$P53,"1",IF(Pronostici!$O53=Pronostici!$P53,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N53" s="63">
+        <f>IF(Pronostici!$Q53&lt;&gt;"",UPPER(Pronostici!$Q53),IF(OR(Pronostici!$R53="",Pronostici!$S53=""),"",IF(Pronostici!$R53&gt;Pronostici!$S53,"1",IF(Pronostici!$R53=Pronostici!$S53,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="74">
+        <f>Partite!$A54</f>
+        <v/>
+      </c>
+      <c r="B54" s="30">
+        <f>Partite!$B54</f>
+        <v/>
+      </c>
+      <c r="C54" s="47">
+        <f>IF(Partite!$E54="","",Partite!$E54&amp;"  -  "&amp;Partite!$F54)</f>
+        <v/>
+      </c>
+      <c r="D54" s="27">
+        <f>IF(Partite!$K54&lt;&gt;"Giocata","",IF(AND(Pronostici!$F54&lt;&gt;"",Pronostici!$G54&lt;&gt;"",Pronostici!$F54=Partite!$G54,Pronostici!$G54=Partite!$H54),Config!$D$6,IF(AND($J54&lt;&gt;"",$J54=Partite!$I54),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E54" s="27">
+        <f>IF(Partite!$K54&lt;&gt;"Giocata","",IF(AND(Pronostici!$I54&lt;&gt;"",Pronostici!$J54&lt;&gt;"",Pronostici!$I54=Partite!$G54,Pronostici!$J54=Partite!$H54),Config!$D$6,IF(AND($K54&lt;&gt;"",$K54=Partite!$I54),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F54" s="27">
+        <f>IF(Partite!$K54&lt;&gt;"Giocata","",IF(AND(Pronostici!$L54&lt;&gt;"",Pronostici!$M54&lt;&gt;"",Pronostici!$L54=Partite!$G54,Pronostici!$M54=Partite!$H54),Config!$D$6,IF(AND($L54&lt;&gt;"",$L54=Partite!$I54),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G54" s="27">
+        <f>IF(Partite!$K54&lt;&gt;"Giocata","",IF(AND(Pronostici!$O54&lt;&gt;"",Pronostici!$P54&lt;&gt;"",Pronostici!$O54=Partite!$G54,Pronostici!$P54=Partite!$H54),Config!$D$6,IF(AND($M54&lt;&gt;"",$M54=Partite!$I54),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H54" s="27">
+        <f>IF(Partite!$K54&lt;&gt;"Giocata","",IF(AND(Pronostici!$R54&lt;&gt;"",Pronostici!$S54&lt;&gt;"",Pronostici!$R54=Partite!$G54,Pronostici!$S54=Partite!$H54),Config!$D$6,IF(AND($N54&lt;&gt;"",$N54=Partite!$I54),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J54" s="63">
+        <f>IF(Pronostici!$E54&lt;&gt;"",UPPER(Pronostici!$E54),IF(OR(Pronostici!$F54="",Pronostici!$G54=""),"",IF(Pronostici!$F54&gt;Pronostici!$G54,"1",IF(Pronostici!$F54=Pronostici!$G54,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K54" s="63">
+        <f>IF(Pronostici!$H54&lt;&gt;"",UPPER(Pronostici!$H54),IF(OR(Pronostici!$I54="",Pronostici!$J54=""),"",IF(Pronostici!$I54&gt;Pronostici!$J54,"1",IF(Pronostici!$I54=Pronostici!$J54,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L54" s="63">
+        <f>IF(Pronostici!$K54&lt;&gt;"",UPPER(Pronostici!$K54),IF(OR(Pronostici!$L54="",Pronostici!$M54=""),"",IF(Pronostici!$L54&gt;Pronostici!$M54,"1",IF(Pronostici!$L54=Pronostici!$M54,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M54" s="63">
+        <f>IF(Pronostici!$N54&lt;&gt;"",UPPER(Pronostici!$N54),IF(OR(Pronostici!$O54="",Pronostici!$P54=""),"",IF(Pronostici!$O54&gt;Pronostici!$P54,"1",IF(Pronostici!$O54=Pronostici!$P54,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N54" s="63">
+        <f>IF(Pronostici!$Q54&lt;&gt;"",UPPER(Pronostici!$Q54),IF(OR(Pronostici!$R54="",Pronostici!$S54=""),"",IF(Pronostici!$R54&gt;Pronostici!$S54,"1",IF(Pronostici!$R54=Pronostici!$S54,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="74">
+        <f>Partite!$A55</f>
+        <v/>
+      </c>
+      <c r="B55" s="30">
+        <f>Partite!$B55</f>
+        <v/>
+      </c>
+      <c r="C55" s="47">
+        <f>IF(Partite!$E55="","",Partite!$E55&amp;"  -  "&amp;Partite!$F55)</f>
+        <v/>
+      </c>
+      <c r="D55" s="27">
+        <f>IF(Partite!$K55&lt;&gt;"Giocata","",IF(AND(Pronostici!$F55&lt;&gt;"",Pronostici!$G55&lt;&gt;"",Pronostici!$F55=Partite!$G55,Pronostici!$G55=Partite!$H55),Config!$D$6,IF(AND($J55&lt;&gt;"",$J55=Partite!$I55),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E55" s="27">
+        <f>IF(Partite!$K55&lt;&gt;"Giocata","",IF(AND(Pronostici!$I55&lt;&gt;"",Pronostici!$J55&lt;&gt;"",Pronostici!$I55=Partite!$G55,Pronostici!$J55=Partite!$H55),Config!$D$6,IF(AND($K55&lt;&gt;"",$K55=Partite!$I55),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F55" s="27">
+        <f>IF(Partite!$K55&lt;&gt;"Giocata","",IF(AND(Pronostici!$L55&lt;&gt;"",Pronostici!$M55&lt;&gt;"",Pronostici!$L55=Partite!$G55,Pronostici!$M55=Partite!$H55),Config!$D$6,IF(AND($L55&lt;&gt;"",$L55=Partite!$I55),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G55" s="27">
+        <f>IF(Partite!$K55&lt;&gt;"Giocata","",IF(AND(Pronostici!$O55&lt;&gt;"",Pronostici!$P55&lt;&gt;"",Pronostici!$O55=Partite!$G55,Pronostici!$P55=Partite!$H55),Config!$D$6,IF(AND($M55&lt;&gt;"",$M55=Partite!$I55),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H55" s="27">
+        <f>IF(Partite!$K55&lt;&gt;"Giocata","",IF(AND(Pronostici!$R55&lt;&gt;"",Pronostici!$S55&lt;&gt;"",Pronostici!$R55=Partite!$G55,Pronostici!$S55=Partite!$H55),Config!$D$6,IF(AND($N55&lt;&gt;"",$N55=Partite!$I55),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J55" s="63">
+        <f>IF(Pronostici!$E55&lt;&gt;"",UPPER(Pronostici!$E55),IF(OR(Pronostici!$F55="",Pronostici!$G55=""),"",IF(Pronostici!$F55&gt;Pronostici!$G55,"1",IF(Pronostici!$F55=Pronostici!$G55,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K55" s="63">
+        <f>IF(Pronostici!$H55&lt;&gt;"",UPPER(Pronostici!$H55),IF(OR(Pronostici!$I55="",Pronostici!$J55=""),"",IF(Pronostici!$I55&gt;Pronostici!$J55,"1",IF(Pronostici!$I55=Pronostici!$J55,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L55" s="63">
+        <f>IF(Pronostici!$K55&lt;&gt;"",UPPER(Pronostici!$K55),IF(OR(Pronostici!$L55="",Pronostici!$M55=""),"",IF(Pronostici!$L55&gt;Pronostici!$M55,"1",IF(Pronostici!$L55=Pronostici!$M55,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M55" s="63">
+        <f>IF(Pronostici!$N55&lt;&gt;"",UPPER(Pronostici!$N55),IF(OR(Pronostici!$O55="",Pronostici!$P55=""),"",IF(Pronostici!$O55&gt;Pronostici!$P55,"1",IF(Pronostici!$O55=Pronostici!$P55,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N55" s="63">
+        <f>IF(Pronostici!$Q55&lt;&gt;"",UPPER(Pronostici!$Q55),IF(OR(Pronostici!$R55="",Pronostici!$S55=""),"",IF(Pronostici!$R55&gt;Pronostici!$S55,"1",IF(Pronostici!$R55=Pronostici!$S55,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="74">
+        <f>Partite!$A56</f>
+        <v/>
+      </c>
+      <c r="B56" s="30">
+        <f>Partite!$B56</f>
+        <v/>
+      </c>
+      <c r="C56" s="47">
+        <f>IF(Partite!$E56="","",Partite!$E56&amp;"  -  "&amp;Partite!$F56)</f>
+        <v/>
+      </c>
+      <c r="D56" s="27">
+        <f>IF(Partite!$K56&lt;&gt;"Giocata","",IF(AND(Pronostici!$F56&lt;&gt;"",Pronostici!$G56&lt;&gt;"",Pronostici!$F56=Partite!$G56,Pronostici!$G56=Partite!$H56),Config!$D$6,IF(AND($J56&lt;&gt;"",$J56=Partite!$I56),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E56" s="27">
+        <f>IF(Partite!$K56&lt;&gt;"Giocata","",IF(AND(Pronostici!$I56&lt;&gt;"",Pronostici!$J56&lt;&gt;"",Pronostici!$I56=Partite!$G56,Pronostici!$J56=Partite!$H56),Config!$D$6,IF(AND($K56&lt;&gt;"",$K56=Partite!$I56),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F56" s="27">
+        <f>IF(Partite!$K56&lt;&gt;"Giocata","",IF(AND(Pronostici!$L56&lt;&gt;"",Pronostici!$M56&lt;&gt;"",Pronostici!$L56=Partite!$G56,Pronostici!$M56=Partite!$H56),Config!$D$6,IF(AND($L56&lt;&gt;"",$L56=Partite!$I56),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G56" s="27">
+        <f>IF(Partite!$K56&lt;&gt;"Giocata","",IF(AND(Pronostici!$O56&lt;&gt;"",Pronostici!$P56&lt;&gt;"",Pronostici!$O56=Partite!$G56,Pronostici!$P56=Partite!$H56),Config!$D$6,IF(AND($M56&lt;&gt;"",$M56=Partite!$I56),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H56" s="27">
+        <f>IF(Partite!$K56&lt;&gt;"Giocata","",IF(AND(Pronostici!$R56&lt;&gt;"",Pronostici!$S56&lt;&gt;"",Pronostici!$R56=Partite!$G56,Pronostici!$S56=Partite!$H56),Config!$D$6,IF(AND($N56&lt;&gt;"",$N56=Partite!$I56),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J56" s="63">
+        <f>IF(Pronostici!$E56&lt;&gt;"",UPPER(Pronostici!$E56),IF(OR(Pronostici!$F56="",Pronostici!$G56=""),"",IF(Pronostici!$F56&gt;Pronostici!$G56,"1",IF(Pronostici!$F56=Pronostici!$G56,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K56" s="63">
+        <f>IF(Pronostici!$H56&lt;&gt;"",UPPER(Pronostici!$H56),IF(OR(Pronostici!$I56="",Pronostici!$J56=""),"",IF(Pronostici!$I56&gt;Pronostici!$J56,"1",IF(Pronostici!$I56=Pronostici!$J56,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L56" s="63">
+        <f>IF(Pronostici!$K56&lt;&gt;"",UPPER(Pronostici!$K56),IF(OR(Pronostici!$L56="",Pronostici!$M56=""),"",IF(Pronostici!$L56&gt;Pronostici!$M56,"1",IF(Pronostici!$L56=Pronostici!$M56,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M56" s="63">
+        <f>IF(Pronostici!$N56&lt;&gt;"",UPPER(Pronostici!$N56),IF(OR(Pronostici!$O56="",Pronostici!$P56=""),"",IF(Pronostici!$O56&gt;Pronostici!$P56,"1",IF(Pronostici!$O56=Pronostici!$P56,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N56" s="63">
+        <f>IF(Pronostici!$Q56&lt;&gt;"",UPPER(Pronostici!$Q56),IF(OR(Pronostici!$R56="",Pronostici!$S56=""),"",IF(Pronostici!$R56&gt;Pronostici!$S56,"1",IF(Pronostici!$R56=Pronostici!$S56,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="74">
+        <f>Partite!$A57</f>
+        <v/>
+      </c>
+      <c r="B57" s="30">
+        <f>Partite!$B57</f>
+        <v/>
+      </c>
+      <c r="C57" s="47">
+        <f>IF(Partite!$E57="","",Partite!$E57&amp;"  -  "&amp;Partite!$F57)</f>
+        <v/>
+      </c>
+      <c r="D57" s="27">
+        <f>IF(Partite!$K57&lt;&gt;"Giocata","",IF(AND(Pronostici!$F57&lt;&gt;"",Pronostici!$G57&lt;&gt;"",Pronostici!$F57=Partite!$G57,Pronostici!$G57=Partite!$H57),Config!$D$6,IF(AND($J57&lt;&gt;"",$J57=Partite!$I57),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E57" s="27">
+        <f>IF(Partite!$K57&lt;&gt;"Giocata","",IF(AND(Pronostici!$I57&lt;&gt;"",Pronostici!$J57&lt;&gt;"",Pronostici!$I57=Partite!$G57,Pronostici!$J57=Partite!$H57),Config!$D$6,IF(AND($K57&lt;&gt;"",$K57=Partite!$I57),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F57" s="27">
+        <f>IF(Partite!$K57&lt;&gt;"Giocata","",IF(AND(Pronostici!$L57&lt;&gt;"",Pronostici!$M57&lt;&gt;"",Pronostici!$L57=Partite!$G57,Pronostici!$M57=Partite!$H57),Config!$D$6,IF(AND($L57&lt;&gt;"",$L57=Partite!$I57),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G57" s="27">
+        <f>IF(Partite!$K57&lt;&gt;"Giocata","",IF(AND(Pronostici!$O57&lt;&gt;"",Pronostici!$P57&lt;&gt;"",Pronostici!$O57=Partite!$G57,Pronostici!$P57=Partite!$H57),Config!$D$6,IF(AND($M57&lt;&gt;"",$M57=Partite!$I57),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H57" s="27">
+        <f>IF(Partite!$K57&lt;&gt;"Giocata","",IF(AND(Pronostici!$R57&lt;&gt;"",Pronostici!$S57&lt;&gt;"",Pronostici!$R57=Partite!$G57,Pronostici!$S57=Partite!$H57),Config!$D$6,IF(AND($N57&lt;&gt;"",$N57=Partite!$I57),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J57" s="63">
+        <f>IF(Pronostici!$E57&lt;&gt;"",UPPER(Pronostici!$E57),IF(OR(Pronostici!$F57="",Pronostici!$G57=""),"",IF(Pronostici!$F57&gt;Pronostici!$G57,"1",IF(Pronostici!$F57=Pronostici!$G57,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K57" s="63">
+        <f>IF(Pronostici!$H57&lt;&gt;"",UPPER(Pronostici!$H57),IF(OR(Pronostici!$I57="",Pronostici!$J57=""),"",IF(Pronostici!$I57&gt;Pronostici!$J57,"1",IF(Pronostici!$I57=Pronostici!$J57,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L57" s="63">
+        <f>IF(Pronostici!$K57&lt;&gt;"",UPPER(Pronostici!$K57),IF(OR(Pronostici!$L57="",Pronostici!$M57=""),"",IF(Pronostici!$L57&gt;Pronostici!$M57,"1",IF(Pronostici!$L57=Pronostici!$M57,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M57" s="63">
+        <f>IF(Pronostici!$N57&lt;&gt;"",UPPER(Pronostici!$N57),IF(OR(Pronostici!$O57="",Pronostici!$P57=""),"",IF(Pronostici!$O57&gt;Pronostici!$P57,"1",IF(Pronostici!$O57=Pronostici!$P57,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N57" s="63">
+        <f>IF(Pronostici!$Q57&lt;&gt;"",UPPER(Pronostici!$Q57),IF(OR(Pronostici!$R57="",Pronostici!$S57=""),"",IF(Pronostici!$R57&gt;Pronostici!$S57,"1",IF(Pronostici!$R57=Pronostici!$S57,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="74">
+        <f>Partite!$A58</f>
+        <v/>
+      </c>
+      <c r="B58" s="30">
+        <f>Partite!$B58</f>
+        <v/>
+      </c>
+      <c r="C58" s="47">
+        <f>IF(Partite!$E58="","",Partite!$E58&amp;"  -  "&amp;Partite!$F58)</f>
+        <v/>
+      </c>
+      <c r="D58" s="27">
+        <f>IF(Partite!$K58&lt;&gt;"Giocata","",IF(AND(Pronostici!$F58&lt;&gt;"",Pronostici!$G58&lt;&gt;"",Pronostici!$F58=Partite!$G58,Pronostici!$G58=Partite!$H58),Config!$D$6,IF(AND($J58&lt;&gt;"",$J58=Partite!$I58),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E58" s="27">
+        <f>IF(Partite!$K58&lt;&gt;"Giocata","",IF(AND(Pronostici!$I58&lt;&gt;"",Pronostici!$J58&lt;&gt;"",Pronostici!$I58=Partite!$G58,Pronostici!$J58=Partite!$H58),Config!$D$6,IF(AND($K58&lt;&gt;"",$K58=Partite!$I58),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F58" s="27">
+        <f>IF(Partite!$K58&lt;&gt;"Giocata","",IF(AND(Pronostici!$L58&lt;&gt;"",Pronostici!$M58&lt;&gt;"",Pronostici!$L58=Partite!$G58,Pronostici!$M58=Partite!$H58),Config!$D$6,IF(AND($L58&lt;&gt;"",$L58=Partite!$I58),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G58" s="27">
+        <f>IF(Partite!$K58&lt;&gt;"Giocata","",IF(AND(Pronostici!$O58&lt;&gt;"",Pronostici!$P58&lt;&gt;"",Pronostici!$O58=Partite!$G58,Pronostici!$P58=Partite!$H58),Config!$D$6,IF(AND($M58&lt;&gt;"",$M58=Partite!$I58),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H58" s="27">
+        <f>IF(Partite!$K58&lt;&gt;"Giocata","",IF(AND(Pronostici!$R58&lt;&gt;"",Pronostici!$S58&lt;&gt;"",Pronostici!$R58=Partite!$G58,Pronostici!$S58=Partite!$H58),Config!$D$6,IF(AND($N58&lt;&gt;"",$N58=Partite!$I58),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J58" s="63">
+        <f>IF(Pronostici!$E58&lt;&gt;"",UPPER(Pronostici!$E58),IF(OR(Pronostici!$F58="",Pronostici!$G58=""),"",IF(Pronostici!$F58&gt;Pronostici!$G58,"1",IF(Pronostici!$F58=Pronostici!$G58,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K58" s="63">
+        <f>IF(Pronostici!$H58&lt;&gt;"",UPPER(Pronostici!$H58),IF(OR(Pronostici!$I58="",Pronostici!$J58=""),"",IF(Pronostici!$I58&gt;Pronostici!$J58,"1",IF(Pronostici!$I58=Pronostici!$J58,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L58" s="63">
+        <f>IF(Pronostici!$K58&lt;&gt;"",UPPER(Pronostici!$K58),IF(OR(Pronostici!$L58="",Pronostici!$M58=""),"",IF(Pronostici!$L58&gt;Pronostici!$M58,"1",IF(Pronostici!$L58=Pronostici!$M58,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M58" s="63">
+        <f>IF(Pronostici!$N58&lt;&gt;"",UPPER(Pronostici!$N58),IF(OR(Pronostici!$O58="",Pronostici!$P58=""),"",IF(Pronostici!$O58&gt;Pronostici!$P58,"1",IF(Pronostici!$O58=Pronostici!$P58,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N58" s="63">
+        <f>IF(Pronostici!$Q58&lt;&gt;"",UPPER(Pronostici!$Q58),IF(OR(Pronostici!$R58="",Pronostici!$S58=""),"",IF(Pronostici!$R58&gt;Pronostici!$S58,"1",IF(Pronostici!$R58=Pronostici!$S58,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="74">
+        <f>Partite!$A59</f>
+        <v/>
+      </c>
+      <c r="B59" s="30">
+        <f>Partite!$B59</f>
+        <v/>
+      </c>
+      <c r="C59" s="47">
+        <f>IF(Partite!$E59="","",Partite!$E59&amp;"  -  "&amp;Partite!$F59)</f>
+        <v/>
+      </c>
+      <c r="D59" s="27">
+        <f>IF(Partite!$K59&lt;&gt;"Giocata","",IF(AND(Pronostici!$F59&lt;&gt;"",Pronostici!$G59&lt;&gt;"",Pronostici!$F59=Partite!$G59,Pronostici!$G59=Partite!$H59),Config!$D$6,IF(AND($J59&lt;&gt;"",$J59=Partite!$I59),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E59" s="27">
+        <f>IF(Partite!$K59&lt;&gt;"Giocata","",IF(AND(Pronostici!$I59&lt;&gt;"",Pronostici!$J59&lt;&gt;"",Pronostici!$I59=Partite!$G59,Pronostici!$J59=Partite!$H59),Config!$D$6,IF(AND($K59&lt;&gt;"",$K59=Partite!$I59),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F59" s="27">
+        <f>IF(Partite!$K59&lt;&gt;"Giocata","",IF(AND(Pronostici!$L59&lt;&gt;"",Pronostici!$M59&lt;&gt;"",Pronostici!$L59=Partite!$G59,Pronostici!$M59=Partite!$H59),Config!$D$6,IF(AND($L59&lt;&gt;"",$L59=Partite!$I59),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G59" s="27">
+        <f>IF(Partite!$K59&lt;&gt;"Giocata","",IF(AND(Pronostici!$O59&lt;&gt;"",Pronostici!$P59&lt;&gt;"",Pronostici!$O59=Partite!$G59,Pronostici!$P59=Partite!$H59),Config!$D$6,IF(AND($M59&lt;&gt;"",$M59=Partite!$I59),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H59" s="27">
+        <f>IF(Partite!$K59&lt;&gt;"Giocata","",IF(AND(Pronostici!$R59&lt;&gt;"",Pronostici!$S59&lt;&gt;"",Pronostici!$R59=Partite!$G59,Pronostici!$S59=Partite!$H59),Config!$D$6,IF(AND($N59&lt;&gt;"",$N59=Partite!$I59),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J59" s="63">
+        <f>IF(Pronostici!$E59&lt;&gt;"",UPPER(Pronostici!$E59),IF(OR(Pronostici!$F59="",Pronostici!$G59=""),"",IF(Pronostici!$F59&gt;Pronostici!$G59,"1",IF(Pronostici!$F59=Pronostici!$G59,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K59" s="63">
+        <f>IF(Pronostici!$H59&lt;&gt;"",UPPER(Pronostici!$H59),IF(OR(Pronostici!$I59="",Pronostici!$J59=""),"",IF(Pronostici!$I59&gt;Pronostici!$J59,"1",IF(Pronostici!$I59=Pronostici!$J59,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L59" s="63">
+        <f>IF(Pronostici!$K59&lt;&gt;"",UPPER(Pronostici!$K59),IF(OR(Pronostici!$L59="",Pronostici!$M59=""),"",IF(Pronostici!$L59&gt;Pronostici!$M59,"1",IF(Pronostici!$L59=Pronostici!$M59,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M59" s="63">
+        <f>IF(Pronostici!$N59&lt;&gt;"",UPPER(Pronostici!$N59),IF(OR(Pronostici!$O59="",Pronostici!$P59=""),"",IF(Pronostici!$O59&gt;Pronostici!$P59,"1",IF(Pronostici!$O59=Pronostici!$P59,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N59" s="63">
+        <f>IF(Pronostici!$Q59&lt;&gt;"",UPPER(Pronostici!$Q59),IF(OR(Pronostici!$R59="",Pronostici!$S59=""),"",IF(Pronostici!$R59&gt;Pronostici!$S59,"1",IF(Pronostici!$R59=Pronostici!$S59,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="74">
+        <f>Partite!$A60</f>
+        <v/>
+      </c>
+      <c r="B60" s="30">
+        <f>Partite!$B60</f>
+        <v/>
+      </c>
+      <c r="C60" s="47">
+        <f>IF(Partite!$E60="","",Partite!$E60&amp;"  -  "&amp;Partite!$F60)</f>
+        <v/>
+      </c>
+      <c r="D60" s="27">
+        <f>IF(Partite!$K60&lt;&gt;"Giocata","",IF(AND(Pronostici!$F60&lt;&gt;"",Pronostici!$G60&lt;&gt;"",Pronostici!$F60=Partite!$G60,Pronostici!$G60=Partite!$H60),Config!$D$6,IF(AND($J60&lt;&gt;"",$J60=Partite!$I60),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E60" s="27">
+        <f>IF(Partite!$K60&lt;&gt;"Giocata","",IF(AND(Pronostici!$I60&lt;&gt;"",Pronostici!$J60&lt;&gt;"",Pronostici!$I60=Partite!$G60,Pronostici!$J60=Partite!$H60),Config!$D$6,IF(AND($K60&lt;&gt;"",$K60=Partite!$I60),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F60" s="27">
+        <f>IF(Partite!$K60&lt;&gt;"Giocata","",IF(AND(Pronostici!$L60&lt;&gt;"",Pronostici!$M60&lt;&gt;"",Pronostici!$L60=Partite!$G60,Pronostici!$M60=Partite!$H60),Config!$D$6,IF(AND($L60&lt;&gt;"",$L60=Partite!$I60),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G60" s="27">
+        <f>IF(Partite!$K60&lt;&gt;"Giocata","",IF(AND(Pronostici!$O60&lt;&gt;"",Pronostici!$P60&lt;&gt;"",Pronostici!$O60=Partite!$G60,Pronostici!$P60=Partite!$H60),Config!$D$6,IF(AND($M60&lt;&gt;"",$M60=Partite!$I60),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H60" s="27">
+        <f>IF(Partite!$K60&lt;&gt;"Giocata","",IF(AND(Pronostici!$R60&lt;&gt;"",Pronostici!$S60&lt;&gt;"",Pronostici!$R60=Partite!$G60,Pronostici!$S60=Partite!$H60),Config!$D$6,IF(AND($N60&lt;&gt;"",$N60=Partite!$I60),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J60" s="63">
+        <f>IF(Pronostici!$E60&lt;&gt;"",UPPER(Pronostici!$E60),IF(OR(Pronostici!$F60="",Pronostici!$G60=""),"",IF(Pronostici!$F60&gt;Pronostici!$G60,"1",IF(Pronostici!$F60=Pronostici!$G60,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K60" s="63">
+        <f>IF(Pronostici!$H60&lt;&gt;"",UPPER(Pronostici!$H60),IF(OR(Pronostici!$I60="",Pronostici!$J60=""),"",IF(Pronostici!$I60&gt;Pronostici!$J60,"1",IF(Pronostici!$I60=Pronostici!$J60,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L60" s="63">
+        <f>IF(Pronostici!$K60&lt;&gt;"",UPPER(Pronostici!$K60),IF(OR(Pronostici!$L60="",Pronostici!$M60=""),"",IF(Pronostici!$L60&gt;Pronostici!$M60,"1",IF(Pronostici!$L60=Pronostici!$M60,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M60" s="63">
+        <f>IF(Pronostici!$N60&lt;&gt;"",UPPER(Pronostici!$N60),IF(OR(Pronostici!$O60="",Pronostici!$P60=""),"",IF(Pronostici!$O60&gt;Pronostici!$P60,"1",IF(Pronostici!$O60=Pronostici!$P60,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N60" s="63">
+        <f>IF(Pronostici!$Q60&lt;&gt;"",UPPER(Pronostici!$Q60),IF(OR(Pronostici!$R60="",Pronostici!$S60=""),"",IF(Pronostici!$R60&gt;Pronostici!$S60,"1",IF(Pronostici!$R60=Pronostici!$S60,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="74">
+        <f>Partite!$A61</f>
+        <v/>
+      </c>
+      <c r="B61" s="30">
+        <f>Partite!$B61</f>
+        <v/>
+      </c>
+      <c r="C61" s="47">
+        <f>IF(Partite!$E61="","",Partite!$E61&amp;"  -  "&amp;Partite!$F61)</f>
+        <v/>
+      </c>
+      <c r="D61" s="27">
+        <f>IF(Partite!$K61&lt;&gt;"Giocata","",IF(AND(Pronostici!$F61&lt;&gt;"",Pronostici!$G61&lt;&gt;"",Pronostici!$F61=Partite!$G61,Pronostici!$G61=Partite!$H61),Config!$D$6,IF(AND($J61&lt;&gt;"",$J61=Partite!$I61),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E61" s="27">
+        <f>IF(Partite!$K61&lt;&gt;"Giocata","",IF(AND(Pronostici!$I61&lt;&gt;"",Pronostici!$J61&lt;&gt;"",Pronostici!$I61=Partite!$G61,Pronostici!$J61=Partite!$H61),Config!$D$6,IF(AND($K61&lt;&gt;"",$K61=Partite!$I61),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F61" s="27">
+        <f>IF(Partite!$K61&lt;&gt;"Giocata","",IF(AND(Pronostici!$L61&lt;&gt;"",Pronostici!$M61&lt;&gt;"",Pronostici!$L61=Partite!$G61,Pronostici!$M61=Partite!$H61),Config!$D$6,IF(AND($L61&lt;&gt;"",$L61=Partite!$I61),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G61" s="27">
+        <f>IF(Partite!$K61&lt;&gt;"Giocata","",IF(AND(Pronostici!$O61&lt;&gt;"",Pronostici!$P61&lt;&gt;"",Pronostici!$O61=Partite!$G61,Pronostici!$P61=Partite!$H61),Config!$D$6,IF(AND($M61&lt;&gt;"",$M61=Partite!$I61),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H61" s="27">
+        <f>IF(Partite!$K61&lt;&gt;"Giocata","",IF(AND(Pronostici!$R61&lt;&gt;"",Pronostici!$S61&lt;&gt;"",Pronostici!$R61=Partite!$G61,Pronostici!$S61=Partite!$H61),Config!$D$6,IF(AND($N61&lt;&gt;"",$N61=Partite!$I61),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J61" s="63">
+        <f>IF(Pronostici!$E61&lt;&gt;"",UPPER(Pronostici!$E61),IF(OR(Pronostici!$F61="",Pronostici!$G61=""),"",IF(Pronostici!$F61&gt;Pronostici!$G61,"1",IF(Pronostici!$F61=Pronostici!$G61,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K61" s="63">
+        <f>IF(Pronostici!$H61&lt;&gt;"",UPPER(Pronostici!$H61),IF(OR(Pronostici!$I61="",Pronostici!$J61=""),"",IF(Pronostici!$I61&gt;Pronostici!$J61,"1",IF(Pronostici!$I61=Pronostici!$J61,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L61" s="63">
+        <f>IF(Pronostici!$K61&lt;&gt;"",UPPER(Pronostici!$K61),IF(OR(Pronostici!$L61="",Pronostici!$M61=""),"",IF(Pronostici!$L61&gt;Pronostici!$M61,"1",IF(Pronostici!$L61=Pronostici!$M61,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M61" s="63">
+        <f>IF(Pronostici!$N61&lt;&gt;"",UPPER(Pronostici!$N61),IF(OR(Pronostici!$O61="",Pronostici!$P61=""),"",IF(Pronostici!$O61&gt;Pronostici!$P61,"1",IF(Pronostici!$O61=Pronostici!$P61,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N61" s="63">
+        <f>IF(Pronostici!$Q61&lt;&gt;"",UPPER(Pronostici!$Q61),IF(OR(Pronostici!$R61="",Pronostici!$S61=""),"",IF(Pronostici!$R61&gt;Pronostici!$S61,"1",IF(Pronostici!$R61=Pronostici!$S61,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="74">
+        <f>Partite!$A62</f>
+        <v/>
+      </c>
+      <c r="B62" s="30">
+        <f>Partite!$B62</f>
+        <v/>
+      </c>
+      <c r="C62" s="47">
+        <f>IF(Partite!$E62="","",Partite!$E62&amp;"  -  "&amp;Partite!$F62)</f>
+        <v/>
+      </c>
+      <c r="D62" s="27">
+        <f>IF(Partite!$K62&lt;&gt;"Giocata","",IF(AND(Pronostici!$F62&lt;&gt;"",Pronostici!$G62&lt;&gt;"",Pronostici!$F62=Partite!$G62,Pronostici!$G62=Partite!$H62),Config!$D$6,IF(AND($J62&lt;&gt;"",$J62=Partite!$I62),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E62" s="27">
+        <f>IF(Partite!$K62&lt;&gt;"Giocata","",IF(AND(Pronostici!$I62&lt;&gt;"",Pronostici!$J62&lt;&gt;"",Pronostici!$I62=Partite!$G62,Pronostici!$J62=Partite!$H62),Config!$D$6,IF(AND($K62&lt;&gt;"",$K62=Partite!$I62),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F62" s="27">
+        <f>IF(Partite!$K62&lt;&gt;"Giocata","",IF(AND(Pronostici!$L62&lt;&gt;"",Pronostici!$M62&lt;&gt;"",Pronostici!$L62=Partite!$G62,Pronostici!$M62=Partite!$H62),Config!$D$6,IF(AND($L62&lt;&gt;"",$L62=Partite!$I62),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G62" s="27">
+        <f>IF(Partite!$K62&lt;&gt;"Giocata","",IF(AND(Pronostici!$O62&lt;&gt;"",Pronostici!$P62&lt;&gt;"",Pronostici!$O62=Partite!$G62,Pronostici!$P62=Partite!$H62),Config!$D$6,IF(AND($M62&lt;&gt;"",$M62=Partite!$I62),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H62" s="27">
+        <f>IF(Partite!$K62&lt;&gt;"Giocata","",IF(AND(Pronostici!$R62&lt;&gt;"",Pronostici!$S62&lt;&gt;"",Pronostici!$R62=Partite!$G62,Pronostici!$S62=Partite!$H62),Config!$D$6,IF(AND($N62&lt;&gt;"",$N62=Partite!$I62),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J62" s="63">
+        <f>IF(Pronostici!$E62&lt;&gt;"",UPPER(Pronostici!$E62),IF(OR(Pronostici!$F62="",Pronostici!$G62=""),"",IF(Pronostici!$F62&gt;Pronostici!$G62,"1",IF(Pronostici!$F62=Pronostici!$G62,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K62" s="63">
+        <f>IF(Pronostici!$H62&lt;&gt;"",UPPER(Pronostici!$H62),IF(OR(Pronostici!$I62="",Pronostici!$J62=""),"",IF(Pronostici!$I62&gt;Pronostici!$J62,"1",IF(Pronostici!$I62=Pronostici!$J62,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L62" s="63">
+        <f>IF(Pronostici!$K62&lt;&gt;"",UPPER(Pronostici!$K62),IF(OR(Pronostici!$L62="",Pronostici!$M62=""),"",IF(Pronostici!$L62&gt;Pronostici!$M62,"1",IF(Pronostici!$L62=Pronostici!$M62,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M62" s="63">
+        <f>IF(Pronostici!$N62&lt;&gt;"",UPPER(Pronostici!$N62),IF(OR(Pronostici!$O62="",Pronostici!$P62=""),"",IF(Pronostici!$O62&gt;Pronostici!$P62,"1",IF(Pronostici!$O62=Pronostici!$P62,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N62" s="63">
+        <f>IF(Pronostici!$Q62&lt;&gt;"",UPPER(Pronostici!$Q62),IF(OR(Pronostici!$R62="",Pronostici!$S62=""),"",IF(Pronostici!$R62&gt;Pronostici!$S62,"1",IF(Pronostici!$R62=Pronostici!$S62,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D52">
+  <conditionalFormatting sqref="D3:D62">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -11135,7 +12506,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E52">
+  <conditionalFormatting sqref="E3:E62">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -11143,7 +12514,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F52">
+  <conditionalFormatting sqref="F3:F62">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -11151,7 +12522,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G52">
+  <conditionalFormatting sqref="G3:G62">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -11159,7 +12530,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H52">
+  <conditionalFormatting sqref="H3:H62">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento automatico del 10/10/2026 alle 15:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -8491,21 +8491,61 @@
         <f>IF(Partite!$F43="","",Partite!$F43)</f>
         <v/>
       </c>
-      <c r="E43" s="71" t="n"/>
-      <c r="F43" s="71" t="n"/>
-      <c r="G43" s="71" t="n"/>
-      <c r="H43" s="71" t="n"/>
-      <c r="I43" s="71" t="n"/>
-      <c r="J43" s="71" t="n"/>
-      <c r="K43" s="71" t="n"/>
-      <c r="L43" s="71" t="n"/>
-      <c r="M43" s="71" t="n"/>
-      <c r="N43" s="71" t="n"/>
-      <c r="O43" s="71" t="n"/>
-      <c r="P43" s="71" t="n"/>
-      <c r="Q43" s="71" t="n"/>
-      <c r="R43" s="71" t="n"/>
-      <c r="S43" s="71" t="n"/>
+      <c r="E43" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I43" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J43" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L43" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M43" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O43" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P43" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S43" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="69">
@@ -8524,21 +8564,61 @@
         <f>IF(Partite!$F44="","",Partite!$F44)</f>
         <v/>
       </c>
-      <c r="E44" s="71" t="n"/>
-      <c r="F44" s="71" t="n"/>
-      <c r="G44" s="71" t="n"/>
-      <c r="H44" s="71" t="n"/>
-      <c r="I44" s="71" t="n"/>
-      <c r="J44" s="71" t="n"/>
-      <c r="K44" s="71" t="n"/>
-      <c r="L44" s="71" t="n"/>
-      <c r="M44" s="71" t="n"/>
-      <c r="N44" s="71" t="n"/>
-      <c r="O44" s="71" t="n"/>
-      <c r="P44" s="71" t="n"/>
-      <c r="Q44" s="71" t="n"/>
-      <c r="R44" s="71" t="n"/>
-      <c r="S44" s="71" t="n"/>
+      <c r="E44" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F44" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I44" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K44" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L44" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N44" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O44" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R44" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="69">
@@ -8557,21 +8637,61 @@
         <f>IF(Partite!$F45="","",Partite!$F45)</f>
         <v/>
       </c>
-      <c r="E45" s="71" t="n"/>
-      <c r="F45" s="71" t="n"/>
-      <c r="G45" s="71" t="n"/>
-      <c r="H45" s="71" t="n"/>
-      <c r="I45" s="71" t="n"/>
-      <c r="J45" s="71" t="n"/>
-      <c r="K45" s="71" t="n"/>
-      <c r="L45" s="71" t="n"/>
-      <c r="M45" s="71" t="n"/>
-      <c r="N45" s="71" t="n"/>
-      <c r="O45" s="71" t="n"/>
-      <c r="P45" s="71" t="n"/>
-      <c r="Q45" s="71" t="n"/>
-      <c r="R45" s="71" t="n"/>
-      <c r="S45" s="71" t="n"/>
+      <c r="E45" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F45" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I45" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K45" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L45" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O45" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P45" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q45" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R45" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S45" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="69">
@@ -8590,21 +8710,61 @@
         <f>IF(Partite!$F46="","",Partite!$F46)</f>
         <v/>
       </c>
-      <c r="E46" s="71" t="n"/>
-      <c r="F46" s="71" t="n"/>
-      <c r="G46" s="71" t="n"/>
-      <c r="H46" s="71" t="n"/>
-      <c r="I46" s="71" t="n"/>
-      <c r="J46" s="71" t="n"/>
-      <c r="K46" s="71" t="n"/>
-      <c r="L46" s="71" t="n"/>
-      <c r="M46" s="71" t="n"/>
-      <c r="N46" s="71" t="n"/>
-      <c r="O46" s="71" t="n"/>
-      <c r="P46" s="71" t="n"/>
-      <c r="Q46" s="71" t="n"/>
-      <c r="R46" s="71" t="n"/>
-      <c r="S46" s="71" t="n"/>
+      <c r="E46" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F46" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I46" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L46" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M46" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N46" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O46" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R46" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S46" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="69">
@@ -8623,21 +8783,61 @@
         <f>IF(Partite!$F47="","",Partite!$F47)</f>
         <v/>
       </c>
-      <c r="E47" s="71" t="n"/>
-      <c r="F47" s="71" t="n"/>
-      <c r="G47" s="71" t="n"/>
-      <c r="H47" s="71" t="n"/>
-      <c r="I47" s="71" t="n"/>
-      <c r="J47" s="71" t="n"/>
-      <c r="K47" s="71" t="n"/>
-      <c r="L47" s="71" t="n"/>
-      <c r="M47" s="71" t="n"/>
-      <c r="N47" s="71" t="n"/>
-      <c r="O47" s="71" t="n"/>
-      <c r="P47" s="71" t="n"/>
-      <c r="Q47" s="71" t="n"/>
-      <c r="R47" s="71" t="n"/>
-      <c r="S47" s="71" t="n"/>
+      <c r="E47" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F47" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I47" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L47" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M47" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O47" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P47" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S47" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="69">
@@ -8656,21 +8856,61 @@
         <f>IF(Partite!$F48="","",Partite!$F48)</f>
         <v/>
       </c>
-      <c r="E48" s="71" t="n"/>
-      <c r="F48" s="71" t="n"/>
-      <c r="G48" s="71" t="n"/>
-      <c r="H48" s="71" t="n"/>
-      <c r="I48" s="71" t="n"/>
-      <c r="J48" s="71" t="n"/>
-      <c r="K48" s="71" t="n"/>
-      <c r="L48" s="71" t="n"/>
-      <c r="M48" s="71" t="n"/>
-      <c r="N48" s="71" t="n"/>
-      <c r="O48" s="71" t="n"/>
-      <c r="P48" s="71" t="n"/>
-      <c r="Q48" s="71" t="n"/>
-      <c r="R48" s="71" t="n"/>
-      <c r="S48" s="71" t="n"/>
+      <c r="E48" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F48" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I48" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J48" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L48" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M48" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O48" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P48" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S48" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="69">
@@ -8689,21 +8929,61 @@
         <f>IF(Partite!$F49="","",Partite!$F49)</f>
         <v/>
       </c>
-      <c r="E49" s="71" t="n"/>
-      <c r="F49" s="71" t="n"/>
-      <c r="G49" s="71" t="n"/>
-      <c r="H49" s="71" t="n"/>
-      <c r="I49" s="71" t="n"/>
-      <c r="J49" s="71" t="n"/>
-      <c r="K49" s="71" t="n"/>
-      <c r="L49" s="71" t="n"/>
-      <c r="M49" s="71" t="n"/>
-      <c r="N49" s="71" t="n"/>
-      <c r="O49" s="71" t="n"/>
-      <c r="P49" s="71" t="n"/>
-      <c r="Q49" s="71" t="n"/>
-      <c r="R49" s="71" t="n"/>
-      <c r="S49" s="71" t="n"/>
+      <c r="E49" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F49" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I49" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L49" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O49" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P49" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q49" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R49" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="69">
@@ -8722,21 +9002,61 @@
         <f>IF(Partite!$F50="","",Partite!$F50)</f>
         <v/>
       </c>
-      <c r="E50" s="71" t="n"/>
-      <c r="F50" s="71" t="n"/>
-      <c r="G50" s="71" t="n"/>
-      <c r="H50" s="71" t="n"/>
-      <c r="I50" s="71" t="n"/>
-      <c r="J50" s="71" t="n"/>
-      <c r="K50" s="71" t="n"/>
-      <c r="L50" s="71" t="n"/>
-      <c r="M50" s="71" t="n"/>
-      <c r="N50" s="71" t="n"/>
-      <c r="O50" s="71" t="n"/>
-      <c r="P50" s="71" t="n"/>
-      <c r="Q50" s="71" t="n"/>
-      <c r="R50" s="71" t="n"/>
-      <c r="S50" s="71" t="n"/>
+      <c r="E50" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F50" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I50" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L50" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M50" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O50" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q50" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S50" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="69">
@@ -8755,21 +9075,61 @@
         <f>IF(Partite!$F51="","",Partite!$F51)</f>
         <v/>
       </c>
-      <c r="E51" s="71" t="n"/>
-      <c r="F51" s="71" t="n"/>
-      <c r="G51" s="71" t="n"/>
-      <c r="H51" s="71" t="n"/>
-      <c r="I51" s="71" t="n"/>
-      <c r="J51" s="71" t="n"/>
-      <c r="K51" s="71" t="n"/>
-      <c r="L51" s="71" t="n"/>
-      <c r="M51" s="71" t="n"/>
-      <c r="N51" s="71" t="n"/>
-      <c r="O51" s="71" t="n"/>
-      <c r="P51" s="71" t="n"/>
-      <c r="Q51" s="71" t="n"/>
-      <c r="R51" s="71" t="n"/>
-      <c r="S51" s="71" t="n"/>
+      <c r="E51" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F51" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I51" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L51" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M51" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N51" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O51" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q51" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="S51" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="69">
@@ -8788,21 +9148,61 @@
         <f>IF(Partite!$F52="","",Partite!$F52)</f>
         <v/>
       </c>
-      <c r="E52" s="71" t="n"/>
-      <c r="F52" s="71" t="n"/>
-      <c r="G52" s="71" t="n"/>
-      <c r="H52" s="71" t="n"/>
-      <c r="I52" s="71" t="n"/>
-      <c r="J52" s="71" t="n"/>
-      <c r="K52" s="71" t="n"/>
-      <c r="L52" s="71" t="n"/>
-      <c r="M52" s="71" t="n"/>
-      <c r="N52" s="71" t="n"/>
-      <c r="O52" s="71" t="n"/>
-      <c r="P52" s="71" t="n"/>
-      <c r="Q52" s="71" t="n"/>
-      <c r="R52" s="71" t="n"/>
-      <c r="S52" s="71" t="n"/>
+      <c r="E52" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F52" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H52" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I52" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K52" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N52" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P52" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q52" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="74">

</xml_diff>

<commit_message>
Aggiornamento automatico del 10/10/2026 alle 17:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4651,8 +4651,12 @@
           <t>Fiorentina</t>
         </is>
       </c>
-      <c r="G46" s="71" t="n"/>
-      <c r="H46" s="71" t="n"/>
+      <c r="G46" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I46" s="72">
         <f>IF(OR($G46="",$H46=""),"",IF($G46&gt;$H46,"1",IF($G46=$H46,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 10/10/2026 alle 20:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4699,8 +4699,12 @@
           <t>Parma</t>
         </is>
       </c>
-      <c r="G47" s="71" t="n"/>
-      <c r="H47" s="71" t="n"/>
+      <c r="G47" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I47" s="72">
         <f>IF(OR($G47="",$H47=""),"",IF($G47&gt;$H47,"1",IF($G47=$H47,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 10/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4835,8 +4835,12 @@
           <t>Frosinone</t>
         </is>
       </c>
-      <c r="G50" s="71" t="n"/>
-      <c r="H50" s="71" t="n"/>
+      <c r="G50" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H50" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I50" s="72">
         <f>IF(OR($G50="",$H50=""),"",IF($G50&gt;$H50,"1",IF($G50=$H50,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/10/2026 alle 14:39
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4607,8 +4607,12 @@
           <t>Roma</t>
         </is>
       </c>
-      <c r="G45" s="71" t="n"/>
-      <c r="H45" s="71" t="n"/>
+      <c r="G45" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I45" s="72">
         <f>IF(OR($G45="",$H45=""),"",IF($G45&gt;$H45,"1",IF($G45=$H45,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/10/2026 alle 17:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4751,8 +4751,12 @@
           <t>Monza</t>
         </is>
       </c>
-      <c r="G48" s="71" t="n"/>
-      <c r="H48" s="71" t="n"/>
+      <c r="G48" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H48" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I48" s="72">
         <f>IF(OR($G48="",$H48=""),"",IF($G48&gt;$H48,"1",IF($G48=$H48,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/10/2026 alle 17:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4799,8 +4799,12 @@
           <t>Bologna</t>
         </is>
       </c>
-      <c r="G49" s="71" t="n"/>
-      <c r="H49" s="71" t="n"/>
+      <c r="G49" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I49" s="72">
         <f>IF(OR($G49="",$H49=""),"",IF($G49&gt;$H49,"1",IF($G49=$H49,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/10/2026 alle 20:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4895,8 +4895,12 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="G51" s="71" t="n"/>
-      <c r="H51" s="71" t="n"/>
+      <c r="G51" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I51" s="72">
         <f>IF(OR($G51="",$H51=""),"",IF($G51&gt;$H51,"1",IF($G51=$H51,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4563,8 +4563,12 @@
           <t>Juventus</t>
         </is>
       </c>
-      <c r="G44" s="71" t="n"/>
-      <c r="H44" s="71" t="n"/>
+      <c r="G44" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I44" s="72">
         <f>IF(OR($G44="",$H44=""),"",IF($G44&gt;$H44,"1",IF($G44=$H44,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 12/10/2026 alle 20:29
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -4519,8 +4519,12 @@
           <t>Venezia</t>
         </is>
       </c>
-      <c r="G43" s="71" t="n"/>
-      <c r="H43" s="71" t="n"/>
+      <c r="G43" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I43" s="72">
         <f>IF(OR($G43="",$H43=""),"",IF($G43&gt;$H43,"1",IF($G43=$H43,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 12/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$62</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$38</f>
+              <f>'Classifica'!$A$33:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$R$33:$R$38</f>
+              <f>'Classifica'!$R$33:$R$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -851,12 +851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$38</f>
+              <f>'Classifica'!$A$33:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$S$33:$S$38</f>
+              <f>'Classifica'!$S$33:$S$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -888,12 +888,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$38</f>
+              <f>'Classifica'!$A$33:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$T$33:$T$38</f>
+              <f>'Classifica'!$T$33:$T$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -925,12 +925,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$38</f>
+              <f>'Classifica'!$A$33:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$U$33:$U$38</f>
+              <f>'Classifica'!$U$33:$U$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -962,12 +962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$38</f>
+              <f>'Classifica'!$A$33:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$V$33:$V$38</f>
+              <f>'Classifica'!$V$33:$V$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1043,7 +1043,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>41</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9720000" cy="3420000"/>
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V38"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>COUNTIF($B$33:$B$38,"Completata")</f>
+        <f>COUNTIF($B$33:$B$39,"Completata")</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>COUNTIF($B$33:$B$38,"Completata")+COUNTIF($B$33:$B$38,"In corso")</f>
+        <f>COUNTIF($B$33:$B$39,"Completata")+COUNTIF($B$33:$B$39,"In corso")</f>
         <v/>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L7" s="13">
-        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$38="Completata")*$A$33:$A$38)))</f>
+        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$39="Completata")*$A$33:$A$39)))</f>
         <v/>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="L8" s="13">
-        <f>IF(SUMPRODUCT(MIN(($B$33:$B$38&lt;&gt;"Completata")*$A$33:$A$38+($B$33:$B$38="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$38&lt;&gt;"Completata")*$A$33:$A$38+($B$33:$B$38="Completata")*999)))</f>
+        <f>IF(SUMPRODUCT(MIN(($B$33:$B$39&lt;&gt;"Completata")*$A$33:$A$39+($B$33:$B$39="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$39&lt;&gt;"Completata")*$A$33:$A$39+($B$33:$B$39="Completata")*999)))</f>
         <v/>
       </c>
     </row>
@@ -1591,19 +1591,19 @@
         <v/>
       </c>
       <c r="C12" s="24">
-        <f>SUM(Punti!$D$3:$D$62)</f>
+        <f>SUM(Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$62,Config!$D$7)+COUNTIF(Punti!$D$3:$D$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$72,Config!$D$7)+COUNTIF(Punti!$D$3:$D$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>SUMPRODUCT(((Pronostici!$E$3:$E$62&lt;&gt;"")+(Pronostici!$F$3:$F$62&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$E$3:$E$72&lt;&gt;"")+(Pronostici!$F$3:$F$72&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>SUMPRODUCT(($C$33:$C$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
+        <f>SUMPRODUCT(($C$33:$C$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1625,19 +1625,19 @@
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>SUM(Punti!$E$3:$E$62)</f>
+        <f>SUM(Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$62,Config!$D$7)+COUNTIF(Punti!$E$3:$E$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$72,Config!$D$7)+COUNTIF(Punti!$E$3:$E$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
-        <f>SUMPRODUCT(((Pronostici!$H$3:$H$62&lt;&gt;"")+(Pronostici!$I$3:$I$62&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$H$3:$H$72&lt;&gt;"")+(Pronostici!$I$3:$I$72&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G13" s="31">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="H13" s="30">
-        <f>SUMPRODUCT(($D$33:$D$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
+        <f>SUMPRODUCT(($D$33:$D$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1659,19 @@
         <v/>
       </c>
       <c r="C14" s="24">
-        <f>SUM(Punti!$F$3:$F$62)</f>
+        <f>SUM(Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$62,Config!$D$7)+COUNTIF(Punti!$F$3:$F$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$72,Config!$D$7)+COUNTIF(Punti!$F$3:$F$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>SUMPRODUCT(((Pronostici!$K$3:$K$62&lt;&gt;"")+(Pronostici!$L$3:$L$62&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$K$3:$K$72&lt;&gt;"")+(Pronostici!$L$3:$L$72&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>SUMPRODUCT(($E$33:$E$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
+        <f>SUMPRODUCT(($E$33:$E$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1693,19 +1693,19 @@
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>SUM(Punti!$G$3:$G$62)</f>
+        <f>SUM(Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$62,Config!$D$7)+COUNTIF(Punti!$G$3:$G$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$72,Config!$D$7)+COUNTIF(Punti!$G$3:$G$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
-        <f>SUMPRODUCT(((Pronostici!$N$3:$N$62&lt;&gt;"")+(Pronostici!$O$3:$O$62&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$N$3:$N$72&lt;&gt;"")+(Pronostici!$O$3:$O$72&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G15" s="31">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="H15" s="30">
-        <f>SUMPRODUCT(($F$33:$F$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
+        <f>SUMPRODUCT(($F$33:$F$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1727,19 +1727,19 @@
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>SUM(Punti!$H$3:$H$62)</f>
+        <f>SUM(Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$62,Config!$D$7)+COUNTIF(Punti!$H$3:$H$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$72,Config!$D$7)+COUNTIF(Punti!$H$3:$H$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$62,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$72,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$62&lt;&gt;"")+(Pronostici!$R$3:$R$62&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$72&lt;&gt;"")+(Pronostici!$R$3:$R$72&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>SUMPRODUCT(($G$33:$G$38=$H$33:$H$38)*($H$33:$H$38&gt;0)*($B$33:$B$38="Completata"))</f>
+        <f>SUMPRODUCT(($G$33:$G$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         <v/>
       </c>
       <c r="C20" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
         <v/>
       </c>
       <c r="D20" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E20" s="41" t="n"/>
       <c r="K20" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L20" s="43" t="n"/>
@@ -1826,7 +1826,7 @@
         <v/>
       </c>
       <c r="O20" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$E$3:$E$62&lt;&gt;"")+(Pronostici!$F$3:$F$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$E$3:$E$72&lt;&gt;"")+(Pronostici!$F$3:$F$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1836,16 +1836,16 @@
         <v/>
       </c>
       <c r="C21" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
         <v/>
       </c>
       <c r="D21" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E21" s="41" t="n"/>
       <c r="K21" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L21" s="47" t="n"/>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="O21" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$H$3:$H$62&lt;&gt;"")+(Pronostici!$I$3:$I$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$H$3:$H$72&lt;&gt;"")+(Pronostici!$I$3:$I$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v/>
       </c>
       <c r="C22" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
         <v/>
       </c>
       <c r="D22" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E22" s="41" t="n"/>
       <c r="K22" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L22" s="43" t="n"/>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="O22" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$K$3:$K$62&lt;&gt;"")+(Pronostici!$L$3:$L$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$K$3:$K$72&lt;&gt;"")+(Pronostici!$L$3:$L$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1894,16 +1894,16 @@
         <v/>
       </c>
       <c r="C23" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
         <v/>
       </c>
       <c r="D23" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E23" s="41" t="n"/>
       <c r="K23" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L23" s="47" t="n"/>
@@ -1913,7 +1913,7 @@
         <v/>
       </c>
       <c r="O23" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$N$3:$N$62&lt;&gt;"")+(Pronostici!$O$3:$O$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$N$3:$N$72&lt;&gt;"")+(Pronostici!$O$3:$O$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1923,16 +1923,16 @@
         <v/>
       </c>
       <c r="C24" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$38,MATCH($L$7,$A$33:$A$38,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
         <v/>
       </c>
       <c r="D24" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$38,MATCH($L$7,$A$33:$A$38,0)),0)=IFERROR(INDEX($H$33:$H$38,MATCH($L$7,$A$33:$A$38,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E24" s="41" t="n"/>
       <c r="K24" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L24" s="43" t="n"/>
@@ -1942,13 +1942,13 @@
         <v/>
       </c>
       <c r="O24" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$62=$L$8)*(((Pronostici!$Q$3:$Q$62&lt;&gt;"")+(Pronostici!$R$3:$R$62&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$Q$3:$Q$72&lt;&gt;"")+(Pronostici!$R$3:$R$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L25" s="47" t="n"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="26">
       <c r="K26" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L26" s="43" t="n"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="27">
       <c r="K27" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L27" s="47" t="n"/>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="28">
       <c r="K28" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L28" s="43" t="n"/>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="29">
       <c r="K29" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$62,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$62,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$62,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$72,0)),"-")</f>
         <v/>
       </c>
       <c r="L29" s="47" t="n"/>
@@ -2070,27 +2070,27 @@
         <v>2</v>
       </c>
       <c r="B33" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A33,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A33,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H33" s="61">
@@ -2127,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="B34" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A34,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A34,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H34" s="61">
@@ -2184,27 +2184,27 @@
         <v>4</v>
       </c>
       <c r="B35" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A35,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A35,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H35" s="61">
@@ -2241,27 +2241,27 @@
         <v>5</v>
       </c>
       <c r="B36" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A36,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A36,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H36" s="61">
@@ -2298,27 +2298,27 @@
         <v>6</v>
       </c>
       <c r="B37" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A37,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$62,$A37,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H37" s="61">
@@ -2355,27 +2355,27 @@
         <v>7</v>
       </c>
       <c r="B38" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$E$3:$E$62,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$K$3:$K$62,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$K$3:$K$62,"Giocata")=COUNTIFS(Partite!$B$3:$B$62,$A38,Partite!$E$3:$E$62,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$D$3:$D$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$D$3:$D$72)</f>
         <v/>
       </c>
       <c r="D38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$E$3:$E$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$E$3:$E$72)</f>
         <v/>
       </c>
       <c r="E38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$F$3:$F$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$F$3:$F$72)</f>
         <v/>
       </c>
       <c r="F38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$G$3:$G$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$G$3:$G$72)</f>
         <v/>
       </c>
       <c r="G38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$62,$A38,Punti!$H$3:$H$62)</f>
+        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$H$3:$H$72)</f>
         <v/>
       </c>
       <c r="H38" s="61">
@@ -2404,6 +2404,63 @@
       </c>
       <c r="V38" s="63">
         <f>V37+G38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B39" s="43">
+        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <v/>
+      </c>
+      <c r="C39" s="25">
+        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$D$3:$D$72)</f>
+        <v/>
+      </c>
+      <c r="D39" s="25">
+        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$E$3:$E$72)</f>
+        <v/>
+      </c>
+      <c r="E39" s="25">
+        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$F$3:$F$72)</f>
+        <v/>
+      </c>
+      <c r="F39" s="25">
+        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$G$3:$G$72)</f>
+        <v/>
+      </c>
+      <c r="G39" s="25">
+        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$H$3:$H$72)</f>
+        <v/>
+      </c>
+      <c r="H39" s="61">
+        <f>MAX($C39:$G39)</f>
+        <v/>
+      </c>
+      <c r="I39" s="62">
+        <f>IF($H39&lt;=0,"-",INDEX($C$32:$G$32,MATCH($H39,$C39:$G39,0))&amp;IF(COUNTIF($C39:$G39,$H39)&gt;1," (a pari)","")&amp;IF($B39="Completata",""," - in corso"))</f>
+        <v/>
+      </c>
+      <c r="R39" s="63">
+        <f>R38+C39</f>
+        <v/>
+      </c>
+      <c r="S39" s="63">
+        <f>S38+D39</f>
+        <v/>
+      </c>
+      <c r="T39" s="63">
+        <f>T38+E39</f>
+        <v/>
+      </c>
+      <c r="U39" s="63">
+        <f>U38+F39</f>
+        <v/>
+      </c>
+      <c r="V39" s="63">
+        <f>V38+G39</f>
         <v/>
       </c>
     </row>
@@ -2450,7 +2507,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:G38">
+  <conditionalFormatting sqref="C33:G39">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2472,7 +2529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4951,8 +5008,12 @@
           <t>Udinese</t>
         </is>
       </c>
-      <c r="G52" s="71" t="n"/>
-      <c r="H52" s="71" t="n"/>
+      <c r="G52" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H52" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I52" s="72">
         <f>IF(OR($G52="",$H52=""),"",IF($G52&gt;$H52,"1",IF($G52=$H52,"X","2")))</f>
         <v/>
@@ -5406,14 +5467,454 @@
         <v/>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="69" t="inlineStr">
+        <is>
+          <t>G08-01</t>
+        </is>
+      </c>
+      <c r="B63" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C63" s="25" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E63" s="70" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="F63" s="70" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="G63" s="71" t="n"/>
+      <c r="H63" s="71" t="n"/>
+      <c r="I63" s="72">
+        <f>IF(OR($G63="",$H63=""),"",IF($G63&gt;$H63,"1",IF($G63=$H63,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J63" s="25">
+        <f>IF(OR($G63="",$H63=""),"",$G63&amp;"-"&amp;$H63)</f>
+        <v/>
+      </c>
+      <c r="K63" s="73">
+        <f>IF($E63="","Calendario da inserire",IF(OR($G63="",$H63=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="69" t="inlineStr">
+        <is>
+          <t>G08-02</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E64" s="70" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="F64" s="70" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="G64" s="71" t="n"/>
+      <c r="H64" s="71" t="n"/>
+      <c r="I64" s="72">
+        <f>IF(OR($G64="",$H64=""),"",IF($G64&gt;$H64,"1",IF($G64=$H64,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J64" s="25">
+        <f>IF(OR($G64="",$H64=""),"",$G64&amp;"-"&amp;$H64)</f>
+        <v/>
+      </c>
+      <c r="K64" s="73">
+        <f>IF($E64="","Calendario da inserire",IF(OR($G64="",$H64=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="69" t="inlineStr">
+        <is>
+          <t>G08-03</t>
+        </is>
+      </c>
+      <c r="B65" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="D65" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E65" s="70" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="F65" s="70" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="G65" s="71" t="n"/>
+      <c r="H65" s="71" t="n"/>
+      <c r="I65" s="72">
+        <f>IF(OR($G65="",$H65=""),"",IF($G65&gt;$H65,"1",IF($G65=$H65,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J65" s="25">
+        <f>IF(OR($G65="",$H65=""),"",$G65&amp;"-"&amp;$H65)</f>
+        <v/>
+      </c>
+      <c r="K65" s="73">
+        <f>IF($E65="","Calendario da inserire",IF(OR($G65="",$H65=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="69" t="inlineStr">
+        <is>
+          <t>G08-04</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E66" s="70" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="F66" s="70" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="G66" s="71" t="n"/>
+      <c r="H66" s="71" t="n"/>
+      <c r="I66" s="72">
+        <f>IF(OR($G66="",$H66=""),"",IF($G66&gt;$H66,"1",IF($G66=$H66,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J66" s="25">
+        <f>IF(OR($G66="",$H66=""),"",$G66&amp;"-"&amp;$H66)</f>
+        <v/>
+      </c>
+      <c r="K66" s="73">
+        <f>IF($E66="","Calendario da inserire",IF(OR($G66="",$H66=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="69" t="inlineStr">
+        <is>
+          <t>G08-05</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C67" s="25" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="D67" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E67" s="70" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="F67" s="70" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="G67" s="71" t="n"/>
+      <c r="H67" s="71" t="n"/>
+      <c r="I67" s="72">
+        <f>IF(OR($G67="",$H67=""),"",IF($G67&gt;$H67,"1",IF($G67=$H67,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J67" s="25">
+        <f>IF(OR($G67="",$H67=""),"",$G67&amp;"-"&amp;$H67)</f>
+        <v/>
+      </c>
+      <c r="K67" s="73">
+        <f>IF($E67="","Calendario da inserire",IF(OR($G67="",$H67=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="69" t="inlineStr">
+        <is>
+          <t>G08-06</t>
+        </is>
+      </c>
+      <c r="B68" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C68" s="25" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="D68" s="25" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E68" s="70" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="F68" s="70" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="G68" s="71" t="n"/>
+      <c r="H68" s="71" t="n"/>
+      <c r="I68" s="72">
+        <f>IF(OR($G68="",$H68=""),"",IF($G68&gt;$H68,"1",IF($G68=$H68,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J68" s="25">
+        <f>IF(OR($G68="",$H68=""),"",$G68&amp;"-"&amp;$H68)</f>
+        <v/>
+      </c>
+      <c r="K68" s="73">
+        <f>IF($E68="","Calendario da inserire",IF(OR($G68="",$H68=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="69" t="inlineStr">
+        <is>
+          <t>G08-07</t>
+        </is>
+      </c>
+      <c r="B69" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C69" s="25" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E69" s="70" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="F69" s="70" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="G69" s="71" t="n"/>
+      <c r="H69" s="71" t="n"/>
+      <c r="I69" s="72">
+        <f>IF(OR($G69="",$H69=""),"",IF($G69&gt;$H69,"1",IF($G69=$H69,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J69" s="25">
+        <f>IF(OR($G69="",$H69=""),"",$G69&amp;"-"&amp;$H69)</f>
+        <v/>
+      </c>
+      <c r="K69" s="73">
+        <f>IF($E69="","Calendario da inserire",IF(OR($G69="",$H69=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="69" t="inlineStr">
+        <is>
+          <t>G08-08</t>
+        </is>
+      </c>
+      <c r="B70" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C70" s="25" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="D70" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E70" s="70" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="F70" s="70" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="G70" s="71" t="n"/>
+      <c r="H70" s="71" t="n"/>
+      <c r="I70" s="72">
+        <f>IF(OR($G70="",$H70=""),"",IF($G70&gt;$H70,"1",IF($G70=$H70,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J70" s="25">
+        <f>IF(OR($G70="",$H70=""),"",$G70&amp;"-"&amp;$H70)</f>
+        <v/>
+      </c>
+      <c r="K70" s="73">
+        <f>IF($E70="","Calendario da inserire",IF(OR($G70="",$H70=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="69" t="inlineStr">
+        <is>
+          <t>G08-09</t>
+        </is>
+      </c>
+      <c r="B71" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C71" s="25" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="D71" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E71" s="70" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="F71" s="70" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="G71" s="71" t="n"/>
+      <c r="H71" s="71" t="n"/>
+      <c r="I71" s="72">
+        <f>IF(OR($G71="",$H71=""),"",IF($G71&gt;$H71,"1",IF($G71=$H71,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J71" s="25">
+        <f>IF(OR($G71="",$H71=""),"",$G71&amp;"-"&amp;$H71)</f>
+        <v/>
+      </c>
+      <c r="K71" s="73">
+        <f>IF($E71="","Calendario da inserire",IF(OR($G71="",$H71=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="69" t="inlineStr">
+        <is>
+          <t>G08-10</t>
+        </is>
+      </c>
+      <c r="B72" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C72" s="25" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="D72" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E72" s="70" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="F72" s="70" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="G72" s="71" t="n"/>
+      <c r="H72" s="71" t="n"/>
+      <c r="I72" s="72">
+        <f>IF(OR($G72="",$H72=""),"",IF($G72&gt;$H72,"1",IF($G72=$H72,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J72" s="25">
+        <f>IF(OR($G72="",$H72=""),"",$G72&amp;"-"&amp;$H72)</f>
+        <v/>
+      </c>
+      <c r="K72" s="73">
+        <f>IF($E72="","Calendario da inserire",IF(OR($G72="",$H72=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K62"/>
+  <autoFilter ref="A2:K72"/>
   <mergeCells count="3">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K3:K62">
+  <conditionalFormatting sqref="K3:K72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Giocata"</formula>
     </cfRule>
@@ -5429,7 +5930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9570,8 +10071,338 @@
       <c r="R62" s="71" t="n"/>
       <c r="S62" s="71" t="n"/>
     </row>
+    <row r="63">
+      <c r="A63" s="69">
+        <f>Partite!$A63</f>
+        <v/>
+      </c>
+      <c r="B63" s="25">
+        <f>Partite!$B63</f>
+        <v/>
+      </c>
+      <c r="C63" s="70">
+        <f>IF(Partite!$E63="","",Partite!$E63)</f>
+        <v/>
+      </c>
+      <c r="D63" s="70">
+        <f>IF(Partite!$F63="","",Partite!$F63)</f>
+        <v/>
+      </c>
+      <c r="E63" s="71" t="n"/>
+      <c r="F63" s="71" t="n"/>
+      <c r="G63" s="71" t="n"/>
+      <c r="H63" s="71" t="n"/>
+      <c r="I63" s="71" t="n"/>
+      <c r="J63" s="71" t="n"/>
+      <c r="K63" s="71" t="n"/>
+      <c r="L63" s="71" t="n"/>
+      <c r="M63" s="71" t="n"/>
+      <c r="N63" s="71" t="n"/>
+      <c r="O63" s="71" t="n"/>
+      <c r="P63" s="71" t="n"/>
+      <c r="Q63" s="71" t="n"/>
+      <c r="R63" s="71" t="n"/>
+      <c r="S63" s="71" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="69">
+        <f>Partite!$A64</f>
+        <v/>
+      </c>
+      <c r="B64" s="25">
+        <f>Partite!$B64</f>
+        <v/>
+      </c>
+      <c r="C64" s="70">
+        <f>IF(Partite!$E64="","",Partite!$E64)</f>
+        <v/>
+      </c>
+      <c r="D64" s="70">
+        <f>IF(Partite!$F64="","",Partite!$F64)</f>
+        <v/>
+      </c>
+      <c r="E64" s="71" t="n"/>
+      <c r="F64" s="71" t="n"/>
+      <c r="G64" s="71" t="n"/>
+      <c r="H64" s="71" t="n"/>
+      <c r="I64" s="71" t="n"/>
+      <c r="J64" s="71" t="n"/>
+      <c r="K64" s="71" t="n"/>
+      <c r="L64" s="71" t="n"/>
+      <c r="M64" s="71" t="n"/>
+      <c r="N64" s="71" t="n"/>
+      <c r="O64" s="71" t="n"/>
+      <c r="P64" s="71" t="n"/>
+      <c r="Q64" s="71" t="n"/>
+      <c r="R64" s="71" t="n"/>
+      <c r="S64" s="71" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="69">
+        <f>Partite!$A65</f>
+        <v/>
+      </c>
+      <c r="B65" s="25">
+        <f>Partite!$B65</f>
+        <v/>
+      </c>
+      <c r="C65" s="70">
+        <f>IF(Partite!$E65="","",Partite!$E65)</f>
+        <v/>
+      </c>
+      <c r="D65" s="70">
+        <f>IF(Partite!$F65="","",Partite!$F65)</f>
+        <v/>
+      </c>
+      <c r="E65" s="71" t="n"/>
+      <c r="F65" s="71" t="n"/>
+      <c r="G65" s="71" t="n"/>
+      <c r="H65" s="71" t="n"/>
+      <c r="I65" s="71" t="n"/>
+      <c r="J65" s="71" t="n"/>
+      <c r="K65" s="71" t="n"/>
+      <c r="L65" s="71" t="n"/>
+      <c r="M65" s="71" t="n"/>
+      <c r="N65" s="71" t="n"/>
+      <c r="O65" s="71" t="n"/>
+      <c r="P65" s="71" t="n"/>
+      <c r="Q65" s="71" t="n"/>
+      <c r="R65" s="71" t="n"/>
+      <c r="S65" s="71" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="69">
+        <f>Partite!$A66</f>
+        <v/>
+      </c>
+      <c r="B66" s="25">
+        <f>Partite!$B66</f>
+        <v/>
+      </c>
+      <c r="C66" s="70">
+        <f>IF(Partite!$E66="","",Partite!$E66)</f>
+        <v/>
+      </c>
+      <c r="D66" s="70">
+        <f>IF(Partite!$F66="","",Partite!$F66)</f>
+        <v/>
+      </c>
+      <c r="E66" s="71" t="n"/>
+      <c r="F66" s="71" t="n"/>
+      <c r="G66" s="71" t="n"/>
+      <c r="H66" s="71" t="n"/>
+      <c r="I66" s="71" t="n"/>
+      <c r="J66" s="71" t="n"/>
+      <c r="K66" s="71" t="n"/>
+      <c r="L66" s="71" t="n"/>
+      <c r="M66" s="71" t="n"/>
+      <c r="N66" s="71" t="n"/>
+      <c r="O66" s="71" t="n"/>
+      <c r="P66" s="71" t="n"/>
+      <c r="Q66" s="71" t="n"/>
+      <c r="R66" s="71" t="n"/>
+      <c r="S66" s="71" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="69">
+        <f>Partite!$A67</f>
+        <v/>
+      </c>
+      <c r="B67" s="25">
+        <f>Partite!$B67</f>
+        <v/>
+      </c>
+      <c r="C67" s="70">
+        <f>IF(Partite!$E67="","",Partite!$E67)</f>
+        <v/>
+      </c>
+      <c r="D67" s="70">
+        <f>IF(Partite!$F67="","",Partite!$F67)</f>
+        <v/>
+      </c>
+      <c r="E67" s="71" t="n"/>
+      <c r="F67" s="71" t="n"/>
+      <c r="G67" s="71" t="n"/>
+      <c r="H67" s="71" t="n"/>
+      <c r="I67" s="71" t="n"/>
+      <c r="J67" s="71" t="n"/>
+      <c r="K67" s="71" t="n"/>
+      <c r="L67" s="71" t="n"/>
+      <c r="M67" s="71" t="n"/>
+      <c r="N67" s="71" t="n"/>
+      <c r="O67" s="71" t="n"/>
+      <c r="P67" s="71" t="n"/>
+      <c r="Q67" s="71" t="n"/>
+      <c r="R67" s="71" t="n"/>
+      <c r="S67" s="71" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="69">
+        <f>Partite!$A68</f>
+        <v/>
+      </c>
+      <c r="B68" s="25">
+        <f>Partite!$B68</f>
+        <v/>
+      </c>
+      <c r="C68" s="70">
+        <f>IF(Partite!$E68="","",Partite!$E68)</f>
+        <v/>
+      </c>
+      <c r="D68" s="70">
+        <f>IF(Partite!$F68="","",Partite!$F68)</f>
+        <v/>
+      </c>
+      <c r="E68" s="71" t="n"/>
+      <c r="F68" s="71" t="n"/>
+      <c r="G68" s="71" t="n"/>
+      <c r="H68" s="71" t="n"/>
+      <c r="I68" s="71" t="n"/>
+      <c r="J68" s="71" t="n"/>
+      <c r="K68" s="71" t="n"/>
+      <c r="L68" s="71" t="n"/>
+      <c r="M68" s="71" t="n"/>
+      <c r="N68" s="71" t="n"/>
+      <c r="O68" s="71" t="n"/>
+      <c r="P68" s="71" t="n"/>
+      <c r="Q68" s="71" t="n"/>
+      <c r="R68" s="71" t="n"/>
+      <c r="S68" s="71" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="69">
+        <f>Partite!$A69</f>
+        <v/>
+      </c>
+      <c r="B69" s="25">
+        <f>Partite!$B69</f>
+        <v/>
+      </c>
+      <c r="C69" s="70">
+        <f>IF(Partite!$E69="","",Partite!$E69)</f>
+        <v/>
+      </c>
+      <c r="D69" s="70">
+        <f>IF(Partite!$F69="","",Partite!$F69)</f>
+        <v/>
+      </c>
+      <c r="E69" s="71" t="n"/>
+      <c r="F69" s="71" t="n"/>
+      <c r="G69" s="71" t="n"/>
+      <c r="H69" s="71" t="n"/>
+      <c r="I69" s="71" t="n"/>
+      <c r="J69" s="71" t="n"/>
+      <c r="K69" s="71" t="n"/>
+      <c r="L69" s="71" t="n"/>
+      <c r="M69" s="71" t="n"/>
+      <c r="N69" s="71" t="n"/>
+      <c r="O69" s="71" t="n"/>
+      <c r="P69" s="71" t="n"/>
+      <c r="Q69" s="71" t="n"/>
+      <c r="R69" s="71" t="n"/>
+      <c r="S69" s="71" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="69">
+        <f>Partite!$A70</f>
+        <v/>
+      </c>
+      <c r="B70" s="25">
+        <f>Partite!$B70</f>
+        <v/>
+      </c>
+      <c r="C70" s="70">
+        <f>IF(Partite!$E70="","",Partite!$E70)</f>
+        <v/>
+      </c>
+      <c r="D70" s="70">
+        <f>IF(Partite!$F70="","",Partite!$F70)</f>
+        <v/>
+      </c>
+      <c r="E70" s="71" t="n"/>
+      <c r="F70" s="71" t="n"/>
+      <c r="G70" s="71" t="n"/>
+      <c r="H70" s="71" t="n"/>
+      <c r="I70" s="71" t="n"/>
+      <c r="J70" s="71" t="n"/>
+      <c r="K70" s="71" t="n"/>
+      <c r="L70" s="71" t="n"/>
+      <c r="M70" s="71" t="n"/>
+      <c r="N70" s="71" t="n"/>
+      <c r="O70" s="71" t="n"/>
+      <c r="P70" s="71" t="n"/>
+      <c r="Q70" s="71" t="n"/>
+      <c r="R70" s="71" t="n"/>
+      <c r="S70" s="71" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="69">
+        <f>Partite!$A71</f>
+        <v/>
+      </c>
+      <c r="B71" s="25">
+        <f>Partite!$B71</f>
+        <v/>
+      </c>
+      <c r="C71" s="70">
+        <f>IF(Partite!$E71="","",Partite!$E71)</f>
+        <v/>
+      </c>
+      <c r="D71" s="70">
+        <f>IF(Partite!$F71="","",Partite!$F71)</f>
+        <v/>
+      </c>
+      <c r="E71" s="71" t="n"/>
+      <c r="F71" s="71" t="n"/>
+      <c r="G71" s="71" t="n"/>
+      <c r="H71" s="71" t="n"/>
+      <c r="I71" s="71" t="n"/>
+      <c r="J71" s="71" t="n"/>
+      <c r="K71" s="71" t="n"/>
+      <c r="L71" s="71" t="n"/>
+      <c r="M71" s="71" t="n"/>
+      <c r="N71" s="71" t="n"/>
+      <c r="O71" s="71" t="n"/>
+      <c r="P71" s="71" t="n"/>
+      <c r="Q71" s="71" t="n"/>
+      <c r="R71" s="71" t="n"/>
+      <c r="S71" s="71" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="69">
+        <f>Partite!$A72</f>
+        <v/>
+      </c>
+      <c r="B72" s="25">
+        <f>Partite!$B72</f>
+        <v/>
+      </c>
+      <c r="C72" s="70">
+        <f>IF(Partite!$E72="","",Partite!$E72)</f>
+        <v/>
+      </c>
+      <c r="D72" s="70">
+        <f>IF(Partite!$F72="","",Partite!$F72)</f>
+        <v/>
+      </c>
+      <c r="E72" s="71" t="n"/>
+      <c r="F72" s="71" t="n"/>
+      <c r="G72" s="71" t="n"/>
+      <c r="H72" s="71" t="n"/>
+      <c r="I72" s="71" t="n"/>
+      <c r="J72" s="71" t="n"/>
+      <c r="K72" s="71" t="n"/>
+      <c r="L72" s="71" t="n"/>
+      <c r="M72" s="71" t="n"/>
+      <c r="N72" s="71" t="n"/>
+      <c r="O72" s="71" t="n"/>
+      <c r="P72" s="71" t="n"/>
+      <c r="Q72" s="71" t="n"/>
+      <c r="R72" s="71" t="n"/>
+      <c r="S72" s="71" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:D62"/>
+  <autoFilter ref="A2:D72"/>
   <mergeCells count="6">
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A1:D1"/>
@@ -9581,7 +10412,7 @@
     <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
       <formula1>"1,X,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9596,7 +10427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12930,11 +13761,551 @@
         <v/>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="69">
+        <f>Partite!$A63</f>
+        <v/>
+      </c>
+      <c r="B63" s="25">
+        <f>Partite!$B63</f>
+        <v/>
+      </c>
+      <c r="C63" s="43">
+        <f>IF(Partite!$E63="","",Partite!$E63&amp;"  -  "&amp;Partite!$F63)</f>
+        <v/>
+      </c>
+      <c r="D63" s="22">
+        <f>IF(Partite!$K63&lt;&gt;"Giocata","",IF(AND(Pronostici!$F63&lt;&gt;"",Pronostici!$G63&lt;&gt;"",Pronostici!$F63=Partite!$G63,Pronostici!$G63=Partite!$H63),Config!$D$6,IF(AND($J63&lt;&gt;"",$J63=Partite!$I63),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E63" s="22">
+        <f>IF(Partite!$K63&lt;&gt;"Giocata","",IF(AND(Pronostici!$I63&lt;&gt;"",Pronostici!$J63&lt;&gt;"",Pronostici!$I63=Partite!$G63,Pronostici!$J63=Partite!$H63),Config!$D$6,IF(AND($K63&lt;&gt;"",$K63=Partite!$I63),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F63" s="22">
+        <f>IF(Partite!$K63&lt;&gt;"Giocata","",IF(AND(Pronostici!$L63&lt;&gt;"",Pronostici!$M63&lt;&gt;"",Pronostici!$L63=Partite!$G63,Pronostici!$M63=Partite!$H63),Config!$D$6,IF(AND($L63&lt;&gt;"",$L63=Partite!$I63),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G63" s="22">
+        <f>IF(Partite!$K63&lt;&gt;"Giocata","",IF(AND(Pronostici!$O63&lt;&gt;"",Pronostici!$P63&lt;&gt;"",Pronostici!$O63=Partite!$G63,Pronostici!$P63=Partite!$H63),Config!$D$6,IF(AND($M63&lt;&gt;"",$M63=Partite!$I63),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H63" s="22">
+        <f>IF(Partite!$K63&lt;&gt;"Giocata","",IF(AND(Pronostici!$R63&lt;&gt;"",Pronostici!$S63&lt;&gt;"",Pronostici!$R63=Partite!$G63,Pronostici!$S63=Partite!$H63),Config!$D$6,IF(AND($N63&lt;&gt;"",$N63=Partite!$I63),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J63" s="63">
+        <f>IF(Pronostici!$E63&lt;&gt;"",UPPER(Pronostici!$E63),IF(OR(Pronostici!$F63="",Pronostici!$G63=""),"",IF(Pronostici!$F63&gt;Pronostici!$G63,"1",IF(Pronostici!$F63=Pronostici!$G63,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K63" s="63">
+        <f>IF(Pronostici!$H63&lt;&gt;"",UPPER(Pronostici!$H63),IF(OR(Pronostici!$I63="",Pronostici!$J63=""),"",IF(Pronostici!$I63&gt;Pronostici!$J63,"1",IF(Pronostici!$I63=Pronostici!$J63,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L63" s="63">
+        <f>IF(Pronostici!$K63&lt;&gt;"",UPPER(Pronostici!$K63),IF(OR(Pronostici!$L63="",Pronostici!$M63=""),"",IF(Pronostici!$L63&gt;Pronostici!$M63,"1",IF(Pronostici!$L63=Pronostici!$M63,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M63" s="63">
+        <f>IF(Pronostici!$N63&lt;&gt;"",UPPER(Pronostici!$N63),IF(OR(Pronostici!$O63="",Pronostici!$P63=""),"",IF(Pronostici!$O63&gt;Pronostici!$P63,"1",IF(Pronostici!$O63=Pronostici!$P63,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N63" s="63">
+        <f>IF(Pronostici!$Q63&lt;&gt;"",UPPER(Pronostici!$Q63),IF(OR(Pronostici!$R63="",Pronostici!$S63=""),"",IF(Pronostici!$R63&gt;Pronostici!$S63,"1",IF(Pronostici!$R63=Pronostici!$S63,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="69">
+        <f>Partite!$A64</f>
+        <v/>
+      </c>
+      <c r="B64" s="25">
+        <f>Partite!$B64</f>
+        <v/>
+      </c>
+      <c r="C64" s="43">
+        <f>IF(Partite!$E64="","",Partite!$E64&amp;"  -  "&amp;Partite!$F64)</f>
+        <v/>
+      </c>
+      <c r="D64" s="22">
+        <f>IF(Partite!$K64&lt;&gt;"Giocata","",IF(AND(Pronostici!$F64&lt;&gt;"",Pronostici!$G64&lt;&gt;"",Pronostici!$F64=Partite!$G64,Pronostici!$G64=Partite!$H64),Config!$D$6,IF(AND($J64&lt;&gt;"",$J64=Partite!$I64),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E64" s="22">
+        <f>IF(Partite!$K64&lt;&gt;"Giocata","",IF(AND(Pronostici!$I64&lt;&gt;"",Pronostici!$J64&lt;&gt;"",Pronostici!$I64=Partite!$G64,Pronostici!$J64=Partite!$H64),Config!$D$6,IF(AND($K64&lt;&gt;"",$K64=Partite!$I64),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F64" s="22">
+        <f>IF(Partite!$K64&lt;&gt;"Giocata","",IF(AND(Pronostici!$L64&lt;&gt;"",Pronostici!$M64&lt;&gt;"",Pronostici!$L64=Partite!$G64,Pronostici!$M64=Partite!$H64),Config!$D$6,IF(AND($L64&lt;&gt;"",$L64=Partite!$I64),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G64" s="22">
+        <f>IF(Partite!$K64&lt;&gt;"Giocata","",IF(AND(Pronostici!$O64&lt;&gt;"",Pronostici!$P64&lt;&gt;"",Pronostici!$O64=Partite!$G64,Pronostici!$P64=Partite!$H64),Config!$D$6,IF(AND($M64&lt;&gt;"",$M64=Partite!$I64),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H64" s="22">
+        <f>IF(Partite!$K64&lt;&gt;"Giocata","",IF(AND(Pronostici!$R64&lt;&gt;"",Pronostici!$S64&lt;&gt;"",Pronostici!$R64=Partite!$G64,Pronostici!$S64=Partite!$H64),Config!$D$6,IF(AND($N64&lt;&gt;"",$N64=Partite!$I64),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J64" s="63">
+        <f>IF(Pronostici!$E64&lt;&gt;"",UPPER(Pronostici!$E64),IF(OR(Pronostici!$F64="",Pronostici!$G64=""),"",IF(Pronostici!$F64&gt;Pronostici!$G64,"1",IF(Pronostici!$F64=Pronostici!$G64,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K64" s="63">
+        <f>IF(Pronostici!$H64&lt;&gt;"",UPPER(Pronostici!$H64),IF(OR(Pronostici!$I64="",Pronostici!$J64=""),"",IF(Pronostici!$I64&gt;Pronostici!$J64,"1",IF(Pronostici!$I64=Pronostici!$J64,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L64" s="63">
+        <f>IF(Pronostici!$K64&lt;&gt;"",UPPER(Pronostici!$K64),IF(OR(Pronostici!$L64="",Pronostici!$M64=""),"",IF(Pronostici!$L64&gt;Pronostici!$M64,"1",IF(Pronostici!$L64=Pronostici!$M64,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M64" s="63">
+        <f>IF(Pronostici!$N64&lt;&gt;"",UPPER(Pronostici!$N64),IF(OR(Pronostici!$O64="",Pronostici!$P64=""),"",IF(Pronostici!$O64&gt;Pronostici!$P64,"1",IF(Pronostici!$O64=Pronostici!$P64,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N64" s="63">
+        <f>IF(Pronostici!$Q64&lt;&gt;"",UPPER(Pronostici!$Q64),IF(OR(Pronostici!$R64="",Pronostici!$S64=""),"",IF(Pronostici!$R64&gt;Pronostici!$S64,"1",IF(Pronostici!$R64=Pronostici!$S64,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="69">
+        <f>Partite!$A65</f>
+        <v/>
+      </c>
+      <c r="B65" s="25">
+        <f>Partite!$B65</f>
+        <v/>
+      </c>
+      <c r="C65" s="43">
+        <f>IF(Partite!$E65="","",Partite!$E65&amp;"  -  "&amp;Partite!$F65)</f>
+        <v/>
+      </c>
+      <c r="D65" s="22">
+        <f>IF(Partite!$K65&lt;&gt;"Giocata","",IF(AND(Pronostici!$F65&lt;&gt;"",Pronostici!$G65&lt;&gt;"",Pronostici!$F65=Partite!$G65,Pronostici!$G65=Partite!$H65),Config!$D$6,IF(AND($J65&lt;&gt;"",$J65=Partite!$I65),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E65" s="22">
+        <f>IF(Partite!$K65&lt;&gt;"Giocata","",IF(AND(Pronostici!$I65&lt;&gt;"",Pronostici!$J65&lt;&gt;"",Pronostici!$I65=Partite!$G65,Pronostici!$J65=Partite!$H65),Config!$D$6,IF(AND($K65&lt;&gt;"",$K65=Partite!$I65),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F65" s="22">
+        <f>IF(Partite!$K65&lt;&gt;"Giocata","",IF(AND(Pronostici!$L65&lt;&gt;"",Pronostici!$M65&lt;&gt;"",Pronostici!$L65=Partite!$G65,Pronostici!$M65=Partite!$H65),Config!$D$6,IF(AND($L65&lt;&gt;"",$L65=Partite!$I65),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G65" s="22">
+        <f>IF(Partite!$K65&lt;&gt;"Giocata","",IF(AND(Pronostici!$O65&lt;&gt;"",Pronostici!$P65&lt;&gt;"",Pronostici!$O65=Partite!$G65,Pronostici!$P65=Partite!$H65),Config!$D$6,IF(AND($M65&lt;&gt;"",$M65=Partite!$I65),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H65" s="22">
+        <f>IF(Partite!$K65&lt;&gt;"Giocata","",IF(AND(Pronostici!$R65&lt;&gt;"",Pronostici!$S65&lt;&gt;"",Pronostici!$R65=Partite!$G65,Pronostici!$S65=Partite!$H65),Config!$D$6,IF(AND($N65&lt;&gt;"",$N65=Partite!$I65),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J65" s="63">
+        <f>IF(Pronostici!$E65&lt;&gt;"",UPPER(Pronostici!$E65),IF(OR(Pronostici!$F65="",Pronostici!$G65=""),"",IF(Pronostici!$F65&gt;Pronostici!$G65,"1",IF(Pronostici!$F65=Pronostici!$G65,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K65" s="63">
+        <f>IF(Pronostici!$H65&lt;&gt;"",UPPER(Pronostici!$H65),IF(OR(Pronostici!$I65="",Pronostici!$J65=""),"",IF(Pronostici!$I65&gt;Pronostici!$J65,"1",IF(Pronostici!$I65=Pronostici!$J65,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L65" s="63">
+        <f>IF(Pronostici!$K65&lt;&gt;"",UPPER(Pronostici!$K65),IF(OR(Pronostici!$L65="",Pronostici!$M65=""),"",IF(Pronostici!$L65&gt;Pronostici!$M65,"1",IF(Pronostici!$L65=Pronostici!$M65,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M65" s="63">
+        <f>IF(Pronostici!$N65&lt;&gt;"",UPPER(Pronostici!$N65),IF(OR(Pronostici!$O65="",Pronostici!$P65=""),"",IF(Pronostici!$O65&gt;Pronostici!$P65,"1",IF(Pronostici!$O65=Pronostici!$P65,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N65" s="63">
+        <f>IF(Pronostici!$Q65&lt;&gt;"",UPPER(Pronostici!$Q65),IF(OR(Pronostici!$R65="",Pronostici!$S65=""),"",IF(Pronostici!$R65&gt;Pronostici!$S65,"1",IF(Pronostici!$R65=Pronostici!$S65,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="69">
+        <f>Partite!$A66</f>
+        <v/>
+      </c>
+      <c r="B66" s="25">
+        <f>Partite!$B66</f>
+        <v/>
+      </c>
+      <c r="C66" s="43">
+        <f>IF(Partite!$E66="","",Partite!$E66&amp;"  -  "&amp;Partite!$F66)</f>
+        <v/>
+      </c>
+      <c r="D66" s="22">
+        <f>IF(Partite!$K66&lt;&gt;"Giocata","",IF(AND(Pronostici!$F66&lt;&gt;"",Pronostici!$G66&lt;&gt;"",Pronostici!$F66=Partite!$G66,Pronostici!$G66=Partite!$H66),Config!$D$6,IF(AND($J66&lt;&gt;"",$J66=Partite!$I66),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E66" s="22">
+        <f>IF(Partite!$K66&lt;&gt;"Giocata","",IF(AND(Pronostici!$I66&lt;&gt;"",Pronostici!$J66&lt;&gt;"",Pronostici!$I66=Partite!$G66,Pronostici!$J66=Partite!$H66),Config!$D$6,IF(AND($K66&lt;&gt;"",$K66=Partite!$I66),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F66" s="22">
+        <f>IF(Partite!$K66&lt;&gt;"Giocata","",IF(AND(Pronostici!$L66&lt;&gt;"",Pronostici!$M66&lt;&gt;"",Pronostici!$L66=Partite!$G66,Pronostici!$M66=Partite!$H66),Config!$D$6,IF(AND($L66&lt;&gt;"",$L66=Partite!$I66),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G66" s="22">
+        <f>IF(Partite!$K66&lt;&gt;"Giocata","",IF(AND(Pronostici!$O66&lt;&gt;"",Pronostici!$P66&lt;&gt;"",Pronostici!$O66=Partite!$G66,Pronostici!$P66=Partite!$H66),Config!$D$6,IF(AND($M66&lt;&gt;"",$M66=Partite!$I66),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H66" s="22">
+        <f>IF(Partite!$K66&lt;&gt;"Giocata","",IF(AND(Pronostici!$R66&lt;&gt;"",Pronostici!$S66&lt;&gt;"",Pronostici!$R66=Partite!$G66,Pronostici!$S66=Partite!$H66),Config!$D$6,IF(AND($N66&lt;&gt;"",$N66=Partite!$I66),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J66" s="63">
+        <f>IF(Pronostici!$E66&lt;&gt;"",UPPER(Pronostici!$E66),IF(OR(Pronostici!$F66="",Pronostici!$G66=""),"",IF(Pronostici!$F66&gt;Pronostici!$G66,"1",IF(Pronostici!$F66=Pronostici!$G66,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K66" s="63">
+        <f>IF(Pronostici!$H66&lt;&gt;"",UPPER(Pronostici!$H66),IF(OR(Pronostici!$I66="",Pronostici!$J66=""),"",IF(Pronostici!$I66&gt;Pronostici!$J66,"1",IF(Pronostici!$I66=Pronostici!$J66,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L66" s="63">
+        <f>IF(Pronostici!$K66&lt;&gt;"",UPPER(Pronostici!$K66),IF(OR(Pronostici!$L66="",Pronostici!$M66=""),"",IF(Pronostici!$L66&gt;Pronostici!$M66,"1",IF(Pronostici!$L66=Pronostici!$M66,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M66" s="63">
+        <f>IF(Pronostici!$N66&lt;&gt;"",UPPER(Pronostici!$N66),IF(OR(Pronostici!$O66="",Pronostici!$P66=""),"",IF(Pronostici!$O66&gt;Pronostici!$P66,"1",IF(Pronostici!$O66=Pronostici!$P66,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N66" s="63">
+        <f>IF(Pronostici!$Q66&lt;&gt;"",UPPER(Pronostici!$Q66),IF(OR(Pronostici!$R66="",Pronostici!$S66=""),"",IF(Pronostici!$R66&gt;Pronostici!$S66,"1",IF(Pronostici!$R66=Pronostici!$S66,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="69">
+        <f>Partite!$A67</f>
+        <v/>
+      </c>
+      <c r="B67" s="25">
+        <f>Partite!$B67</f>
+        <v/>
+      </c>
+      <c r="C67" s="43">
+        <f>IF(Partite!$E67="","",Partite!$E67&amp;"  -  "&amp;Partite!$F67)</f>
+        <v/>
+      </c>
+      <c r="D67" s="22">
+        <f>IF(Partite!$K67&lt;&gt;"Giocata","",IF(AND(Pronostici!$F67&lt;&gt;"",Pronostici!$G67&lt;&gt;"",Pronostici!$F67=Partite!$G67,Pronostici!$G67=Partite!$H67),Config!$D$6,IF(AND($J67&lt;&gt;"",$J67=Partite!$I67),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E67" s="22">
+        <f>IF(Partite!$K67&lt;&gt;"Giocata","",IF(AND(Pronostici!$I67&lt;&gt;"",Pronostici!$J67&lt;&gt;"",Pronostici!$I67=Partite!$G67,Pronostici!$J67=Partite!$H67),Config!$D$6,IF(AND($K67&lt;&gt;"",$K67=Partite!$I67),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F67" s="22">
+        <f>IF(Partite!$K67&lt;&gt;"Giocata","",IF(AND(Pronostici!$L67&lt;&gt;"",Pronostici!$M67&lt;&gt;"",Pronostici!$L67=Partite!$G67,Pronostici!$M67=Partite!$H67),Config!$D$6,IF(AND($L67&lt;&gt;"",$L67=Partite!$I67),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G67" s="22">
+        <f>IF(Partite!$K67&lt;&gt;"Giocata","",IF(AND(Pronostici!$O67&lt;&gt;"",Pronostici!$P67&lt;&gt;"",Pronostici!$O67=Partite!$G67,Pronostici!$P67=Partite!$H67),Config!$D$6,IF(AND($M67&lt;&gt;"",$M67=Partite!$I67),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H67" s="22">
+        <f>IF(Partite!$K67&lt;&gt;"Giocata","",IF(AND(Pronostici!$R67&lt;&gt;"",Pronostici!$S67&lt;&gt;"",Pronostici!$R67=Partite!$G67,Pronostici!$S67=Partite!$H67),Config!$D$6,IF(AND($N67&lt;&gt;"",$N67=Partite!$I67),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J67" s="63">
+        <f>IF(Pronostici!$E67&lt;&gt;"",UPPER(Pronostici!$E67),IF(OR(Pronostici!$F67="",Pronostici!$G67=""),"",IF(Pronostici!$F67&gt;Pronostici!$G67,"1",IF(Pronostici!$F67=Pronostici!$G67,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K67" s="63">
+        <f>IF(Pronostici!$H67&lt;&gt;"",UPPER(Pronostici!$H67),IF(OR(Pronostici!$I67="",Pronostici!$J67=""),"",IF(Pronostici!$I67&gt;Pronostici!$J67,"1",IF(Pronostici!$I67=Pronostici!$J67,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L67" s="63">
+        <f>IF(Pronostici!$K67&lt;&gt;"",UPPER(Pronostici!$K67),IF(OR(Pronostici!$L67="",Pronostici!$M67=""),"",IF(Pronostici!$L67&gt;Pronostici!$M67,"1",IF(Pronostici!$L67=Pronostici!$M67,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M67" s="63">
+        <f>IF(Pronostici!$N67&lt;&gt;"",UPPER(Pronostici!$N67),IF(OR(Pronostici!$O67="",Pronostici!$P67=""),"",IF(Pronostici!$O67&gt;Pronostici!$P67,"1",IF(Pronostici!$O67=Pronostici!$P67,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N67" s="63">
+        <f>IF(Pronostici!$Q67&lt;&gt;"",UPPER(Pronostici!$Q67),IF(OR(Pronostici!$R67="",Pronostici!$S67=""),"",IF(Pronostici!$R67&gt;Pronostici!$S67,"1",IF(Pronostici!$R67=Pronostici!$S67,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="69">
+        <f>Partite!$A68</f>
+        <v/>
+      </c>
+      <c r="B68" s="25">
+        <f>Partite!$B68</f>
+        <v/>
+      </c>
+      <c r="C68" s="43">
+        <f>IF(Partite!$E68="","",Partite!$E68&amp;"  -  "&amp;Partite!$F68)</f>
+        <v/>
+      </c>
+      <c r="D68" s="22">
+        <f>IF(Partite!$K68&lt;&gt;"Giocata","",IF(AND(Pronostici!$F68&lt;&gt;"",Pronostici!$G68&lt;&gt;"",Pronostici!$F68=Partite!$G68,Pronostici!$G68=Partite!$H68),Config!$D$6,IF(AND($J68&lt;&gt;"",$J68=Partite!$I68),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E68" s="22">
+        <f>IF(Partite!$K68&lt;&gt;"Giocata","",IF(AND(Pronostici!$I68&lt;&gt;"",Pronostici!$J68&lt;&gt;"",Pronostici!$I68=Partite!$G68,Pronostici!$J68=Partite!$H68),Config!$D$6,IF(AND($K68&lt;&gt;"",$K68=Partite!$I68),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F68" s="22">
+        <f>IF(Partite!$K68&lt;&gt;"Giocata","",IF(AND(Pronostici!$L68&lt;&gt;"",Pronostici!$M68&lt;&gt;"",Pronostici!$L68=Partite!$G68,Pronostici!$M68=Partite!$H68),Config!$D$6,IF(AND($L68&lt;&gt;"",$L68=Partite!$I68),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G68" s="22">
+        <f>IF(Partite!$K68&lt;&gt;"Giocata","",IF(AND(Pronostici!$O68&lt;&gt;"",Pronostici!$P68&lt;&gt;"",Pronostici!$O68=Partite!$G68,Pronostici!$P68=Partite!$H68),Config!$D$6,IF(AND($M68&lt;&gt;"",$M68=Partite!$I68),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H68" s="22">
+        <f>IF(Partite!$K68&lt;&gt;"Giocata","",IF(AND(Pronostici!$R68&lt;&gt;"",Pronostici!$S68&lt;&gt;"",Pronostici!$R68=Partite!$G68,Pronostici!$S68=Partite!$H68),Config!$D$6,IF(AND($N68&lt;&gt;"",$N68=Partite!$I68),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J68" s="63">
+        <f>IF(Pronostici!$E68&lt;&gt;"",UPPER(Pronostici!$E68),IF(OR(Pronostici!$F68="",Pronostici!$G68=""),"",IF(Pronostici!$F68&gt;Pronostici!$G68,"1",IF(Pronostici!$F68=Pronostici!$G68,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K68" s="63">
+        <f>IF(Pronostici!$H68&lt;&gt;"",UPPER(Pronostici!$H68),IF(OR(Pronostici!$I68="",Pronostici!$J68=""),"",IF(Pronostici!$I68&gt;Pronostici!$J68,"1",IF(Pronostici!$I68=Pronostici!$J68,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L68" s="63">
+        <f>IF(Pronostici!$K68&lt;&gt;"",UPPER(Pronostici!$K68),IF(OR(Pronostici!$L68="",Pronostici!$M68=""),"",IF(Pronostici!$L68&gt;Pronostici!$M68,"1",IF(Pronostici!$L68=Pronostici!$M68,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M68" s="63">
+        <f>IF(Pronostici!$N68&lt;&gt;"",UPPER(Pronostici!$N68),IF(OR(Pronostici!$O68="",Pronostici!$P68=""),"",IF(Pronostici!$O68&gt;Pronostici!$P68,"1",IF(Pronostici!$O68=Pronostici!$P68,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N68" s="63">
+        <f>IF(Pronostici!$Q68&lt;&gt;"",UPPER(Pronostici!$Q68),IF(OR(Pronostici!$R68="",Pronostici!$S68=""),"",IF(Pronostici!$R68&gt;Pronostici!$S68,"1",IF(Pronostici!$R68=Pronostici!$S68,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="69">
+        <f>Partite!$A69</f>
+        <v/>
+      </c>
+      <c r="B69" s="25">
+        <f>Partite!$B69</f>
+        <v/>
+      </c>
+      <c r="C69" s="43">
+        <f>IF(Partite!$E69="","",Partite!$E69&amp;"  -  "&amp;Partite!$F69)</f>
+        <v/>
+      </c>
+      <c r="D69" s="22">
+        <f>IF(Partite!$K69&lt;&gt;"Giocata","",IF(AND(Pronostici!$F69&lt;&gt;"",Pronostici!$G69&lt;&gt;"",Pronostici!$F69=Partite!$G69,Pronostici!$G69=Partite!$H69),Config!$D$6,IF(AND($J69&lt;&gt;"",$J69=Partite!$I69),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E69" s="22">
+        <f>IF(Partite!$K69&lt;&gt;"Giocata","",IF(AND(Pronostici!$I69&lt;&gt;"",Pronostici!$J69&lt;&gt;"",Pronostici!$I69=Partite!$G69,Pronostici!$J69=Partite!$H69),Config!$D$6,IF(AND($K69&lt;&gt;"",$K69=Partite!$I69),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F69" s="22">
+        <f>IF(Partite!$K69&lt;&gt;"Giocata","",IF(AND(Pronostici!$L69&lt;&gt;"",Pronostici!$M69&lt;&gt;"",Pronostici!$L69=Partite!$G69,Pronostici!$M69=Partite!$H69),Config!$D$6,IF(AND($L69&lt;&gt;"",$L69=Partite!$I69),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G69" s="22">
+        <f>IF(Partite!$K69&lt;&gt;"Giocata","",IF(AND(Pronostici!$O69&lt;&gt;"",Pronostici!$P69&lt;&gt;"",Pronostici!$O69=Partite!$G69,Pronostici!$P69=Partite!$H69),Config!$D$6,IF(AND($M69&lt;&gt;"",$M69=Partite!$I69),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H69" s="22">
+        <f>IF(Partite!$K69&lt;&gt;"Giocata","",IF(AND(Pronostici!$R69&lt;&gt;"",Pronostici!$S69&lt;&gt;"",Pronostici!$R69=Partite!$G69,Pronostici!$S69=Partite!$H69),Config!$D$6,IF(AND($N69&lt;&gt;"",$N69=Partite!$I69),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J69" s="63">
+        <f>IF(Pronostici!$E69&lt;&gt;"",UPPER(Pronostici!$E69),IF(OR(Pronostici!$F69="",Pronostici!$G69=""),"",IF(Pronostici!$F69&gt;Pronostici!$G69,"1",IF(Pronostici!$F69=Pronostici!$G69,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K69" s="63">
+        <f>IF(Pronostici!$H69&lt;&gt;"",UPPER(Pronostici!$H69),IF(OR(Pronostici!$I69="",Pronostici!$J69=""),"",IF(Pronostici!$I69&gt;Pronostici!$J69,"1",IF(Pronostici!$I69=Pronostici!$J69,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L69" s="63">
+        <f>IF(Pronostici!$K69&lt;&gt;"",UPPER(Pronostici!$K69),IF(OR(Pronostici!$L69="",Pronostici!$M69=""),"",IF(Pronostici!$L69&gt;Pronostici!$M69,"1",IF(Pronostici!$L69=Pronostici!$M69,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M69" s="63">
+        <f>IF(Pronostici!$N69&lt;&gt;"",UPPER(Pronostici!$N69),IF(OR(Pronostici!$O69="",Pronostici!$P69=""),"",IF(Pronostici!$O69&gt;Pronostici!$P69,"1",IF(Pronostici!$O69=Pronostici!$P69,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N69" s="63">
+        <f>IF(Pronostici!$Q69&lt;&gt;"",UPPER(Pronostici!$Q69),IF(OR(Pronostici!$R69="",Pronostici!$S69=""),"",IF(Pronostici!$R69&gt;Pronostici!$S69,"1",IF(Pronostici!$R69=Pronostici!$S69,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="69">
+        <f>Partite!$A70</f>
+        <v/>
+      </c>
+      <c r="B70" s="25">
+        <f>Partite!$B70</f>
+        <v/>
+      </c>
+      <c r="C70" s="43">
+        <f>IF(Partite!$E70="","",Partite!$E70&amp;"  -  "&amp;Partite!$F70)</f>
+        <v/>
+      </c>
+      <c r="D70" s="22">
+        <f>IF(Partite!$K70&lt;&gt;"Giocata","",IF(AND(Pronostici!$F70&lt;&gt;"",Pronostici!$G70&lt;&gt;"",Pronostici!$F70=Partite!$G70,Pronostici!$G70=Partite!$H70),Config!$D$6,IF(AND($J70&lt;&gt;"",$J70=Partite!$I70),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E70" s="22">
+        <f>IF(Partite!$K70&lt;&gt;"Giocata","",IF(AND(Pronostici!$I70&lt;&gt;"",Pronostici!$J70&lt;&gt;"",Pronostici!$I70=Partite!$G70,Pronostici!$J70=Partite!$H70),Config!$D$6,IF(AND($K70&lt;&gt;"",$K70=Partite!$I70),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F70" s="22">
+        <f>IF(Partite!$K70&lt;&gt;"Giocata","",IF(AND(Pronostici!$L70&lt;&gt;"",Pronostici!$M70&lt;&gt;"",Pronostici!$L70=Partite!$G70,Pronostici!$M70=Partite!$H70),Config!$D$6,IF(AND($L70&lt;&gt;"",$L70=Partite!$I70),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G70" s="22">
+        <f>IF(Partite!$K70&lt;&gt;"Giocata","",IF(AND(Pronostici!$O70&lt;&gt;"",Pronostici!$P70&lt;&gt;"",Pronostici!$O70=Partite!$G70,Pronostici!$P70=Partite!$H70),Config!$D$6,IF(AND($M70&lt;&gt;"",$M70=Partite!$I70),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H70" s="22">
+        <f>IF(Partite!$K70&lt;&gt;"Giocata","",IF(AND(Pronostici!$R70&lt;&gt;"",Pronostici!$S70&lt;&gt;"",Pronostici!$R70=Partite!$G70,Pronostici!$S70=Partite!$H70),Config!$D$6,IF(AND($N70&lt;&gt;"",$N70=Partite!$I70),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J70" s="63">
+        <f>IF(Pronostici!$E70&lt;&gt;"",UPPER(Pronostici!$E70),IF(OR(Pronostici!$F70="",Pronostici!$G70=""),"",IF(Pronostici!$F70&gt;Pronostici!$G70,"1",IF(Pronostici!$F70=Pronostici!$G70,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K70" s="63">
+        <f>IF(Pronostici!$H70&lt;&gt;"",UPPER(Pronostici!$H70),IF(OR(Pronostici!$I70="",Pronostici!$J70=""),"",IF(Pronostici!$I70&gt;Pronostici!$J70,"1",IF(Pronostici!$I70=Pronostici!$J70,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L70" s="63">
+        <f>IF(Pronostici!$K70&lt;&gt;"",UPPER(Pronostici!$K70),IF(OR(Pronostici!$L70="",Pronostici!$M70=""),"",IF(Pronostici!$L70&gt;Pronostici!$M70,"1",IF(Pronostici!$L70=Pronostici!$M70,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M70" s="63">
+        <f>IF(Pronostici!$N70&lt;&gt;"",UPPER(Pronostici!$N70),IF(OR(Pronostici!$O70="",Pronostici!$P70=""),"",IF(Pronostici!$O70&gt;Pronostici!$P70,"1",IF(Pronostici!$O70=Pronostici!$P70,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N70" s="63">
+        <f>IF(Pronostici!$Q70&lt;&gt;"",UPPER(Pronostici!$Q70),IF(OR(Pronostici!$R70="",Pronostici!$S70=""),"",IF(Pronostici!$R70&gt;Pronostici!$S70,"1",IF(Pronostici!$R70=Pronostici!$S70,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="69">
+        <f>Partite!$A71</f>
+        <v/>
+      </c>
+      <c r="B71" s="25">
+        <f>Partite!$B71</f>
+        <v/>
+      </c>
+      <c r="C71" s="43">
+        <f>IF(Partite!$E71="","",Partite!$E71&amp;"  -  "&amp;Partite!$F71)</f>
+        <v/>
+      </c>
+      <c r="D71" s="22">
+        <f>IF(Partite!$K71&lt;&gt;"Giocata","",IF(AND(Pronostici!$F71&lt;&gt;"",Pronostici!$G71&lt;&gt;"",Pronostici!$F71=Partite!$G71,Pronostici!$G71=Partite!$H71),Config!$D$6,IF(AND($J71&lt;&gt;"",$J71=Partite!$I71),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E71" s="22">
+        <f>IF(Partite!$K71&lt;&gt;"Giocata","",IF(AND(Pronostici!$I71&lt;&gt;"",Pronostici!$J71&lt;&gt;"",Pronostici!$I71=Partite!$G71,Pronostici!$J71=Partite!$H71),Config!$D$6,IF(AND($K71&lt;&gt;"",$K71=Partite!$I71),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F71" s="22">
+        <f>IF(Partite!$K71&lt;&gt;"Giocata","",IF(AND(Pronostici!$L71&lt;&gt;"",Pronostici!$M71&lt;&gt;"",Pronostici!$L71=Partite!$G71,Pronostici!$M71=Partite!$H71),Config!$D$6,IF(AND($L71&lt;&gt;"",$L71=Partite!$I71),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G71" s="22">
+        <f>IF(Partite!$K71&lt;&gt;"Giocata","",IF(AND(Pronostici!$O71&lt;&gt;"",Pronostici!$P71&lt;&gt;"",Pronostici!$O71=Partite!$G71,Pronostici!$P71=Partite!$H71),Config!$D$6,IF(AND($M71&lt;&gt;"",$M71=Partite!$I71),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H71" s="22">
+        <f>IF(Partite!$K71&lt;&gt;"Giocata","",IF(AND(Pronostici!$R71&lt;&gt;"",Pronostici!$S71&lt;&gt;"",Pronostici!$R71=Partite!$G71,Pronostici!$S71=Partite!$H71),Config!$D$6,IF(AND($N71&lt;&gt;"",$N71=Partite!$I71),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J71" s="63">
+        <f>IF(Pronostici!$E71&lt;&gt;"",UPPER(Pronostici!$E71),IF(OR(Pronostici!$F71="",Pronostici!$G71=""),"",IF(Pronostici!$F71&gt;Pronostici!$G71,"1",IF(Pronostici!$F71=Pronostici!$G71,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K71" s="63">
+        <f>IF(Pronostici!$H71&lt;&gt;"",UPPER(Pronostici!$H71),IF(OR(Pronostici!$I71="",Pronostici!$J71=""),"",IF(Pronostici!$I71&gt;Pronostici!$J71,"1",IF(Pronostici!$I71=Pronostici!$J71,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L71" s="63">
+        <f>IF(Pronostici!$K71&lt;&gt;"",UPPER(Pronostici!$K71),IF(OR(Pronostici!$L71="",Pronostici!$M71=""),"",IF(Pronostici!$L71&gt;Pronostici!$M71,"1",IF(Pronostici!$L71=Pronostici!$M71,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M71" s="63">
+        <f>IF(Pronostici!$N71&lt;&gt;"",UPPER(Pronostici!$N71),IF(OR(Pronostici!$O71="",Pronostici!$P71=""),"",IF(Pronostici!$O71&gt;Pronostici!$P71,"1",IF(Pronostici!$O71=Pronostici!$P71,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N71" s="63">
+        <f>IF(Pronostici!$Q71&lt;&gt;"",UPPER(Pronostici!$Q71),IF(OR(Pronostici!$R71="",Pronostici!$S71=""),"",IF(Pronostici!$R71&gt;Pronostici!$S71,"1",IF(Pronostici!$R71=Pronostici!$S71,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="69">
+        <f>Partite!$A72</f>
+        <v/>
+      </c>
+      <c r="B72" s="25">
+        <f>Partite!$B72</f>
+        <v/>
+      </c>
+      <c r="C72" s="43">
+        <f>IF(Partite!$E72="","",Partite!$E72&amp;"  -  "&amp;Partite!$F72)</f>
+        <v/>
+      </c>
+      <c r="D72" s="22">
+        <f>IF(Partite!$K72&lt;&gt;"Giocata","",IF(AND(Pronostici!$F72&lt;&gt;"",Pronostici!$G72&lt;&gt;"",Pronostici!$F72=Partite!$G72,Pronostici!$G72=Partite!$H72),Config!$D$6,IF(AND($J72&lt;&gt;"",$J72=Partite!$I72),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E72" s="22">
+        <f>IF(Partite!$K72&lt;&gt;"Giocata","",IF(AND(Pronostici!$I72&lt;&gt;"",Pronostici!$J72&lt;&gt;"",Pronostici!$I72=Partite!$G72,Pronostici!$J72=Partite!$H72),Config!$D$6,IF(AND($K72&lt;&gt;"",$K72=Partite!$I72),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F72" s="22">
+        <f>IF(Partite!$K72&lt;&gt;"Giocata","",IF(AND(Pronostici!$L72&lt;&gt;"",Pronostici!$M72&lt;&gt;"",Pronostici!$L72=Partite!$G72,Pronostici!$M72=Partite!$H72),Config!$D$6,IF(AND($L72&lt;&gt;"",$L72=Partite!$I72),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G72" s="22">
+        <f>IF(Partite!$K72&lt;&gt;"Giocata","",IF(AND(Pronostici!$O72&lt;&gt;"",Pronostici!$P72&lt;&gt;"",Pronostici!$O72=Partite!$G72,Pronostici!$P72=Partite!$H72),Config!$D$6,IF(AND($M72&lt;&gt;"",$M72=Partite!$I72),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H72" s="22">
+        <f>IF(Partite!$K72&lt;&gt;"Giocata","",IF(AND(Pronostici!$R72&lt;&gt;"",Pronostici!$S72&lt;&gt;"",Pronostici!$R72=Partite!$G72,Pronostici!$S72=Partite!$H72),Config!$D$6,IF(AND($N72&lt;&gt;"",$N72=Partite!$I72),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J72" s="63">
+        <f>IF(Pronostici!$E72&lt;&gt;"",UPPER(Pronostici!$E72),IF(OR(Pronostici!$F72="",Pronostici!$G72=""),"",IF(Pronostici!$F72&gt;Pronostici!$G72,"1",IF(Pronostici!$F72=Pronostici!$G72,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K72" s="63">
+        <f>IF(Pronostici!$H72&lt;&gt;"",UPPER(Pronostici!$H72),IF(OR(Pronostici!$I72="",Pronostici!$J72=""),"",IF(Pronostici!$I72&gt;Pronostici!$J72,"1",IF(Pronostici!$I72=Pronostici!$J72,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L72" s="63">
+        <f>IF(Pronostici!$K72&lt;&gt;"",UPPER(Pronostici!$K72),IF(OR(Pronostici!$L72="",Pronostici!$M72=""),"",IF(Pronostici!$L72&gt;Pronostici!$M72,"1",IF(Pronostici!$L72=Pronostici!$M72,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M72" s="63">
+        <f>IF(Pronostici!$N72&lt;&gt;"",UPPER(Pronostici!$N72),IF(OR(Pronostici!$O72="",Pronostici!$P72=""),"",IF(Pronostici!$O72&gt;Pronostici!$P72,"1",IF(Pronostici!$O72=Pronostici!$P72,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N72" s="63">
+        <f>IF(Pronostici!$Q72&lt;&gt;"",UPPER(Pronostici!$Q72),IF(OR(Pronostici!$R72="",Pronostici!$S72=""),"",IF(Pronostici!$R72&gt;Pronostici!$S72,"1",IF(Pronostici!$R72=Pronostici!$S72,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D62">
+  <conditionalFormatting sqref="D3:D72">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -12942,7 +14313,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E62">
+  <conditionalFormatting sqref="E3:E72">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -12950,7 +14321,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F62">
+  <conditionalFormatting sqref="F3:F72">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -12958,7 +14329,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G62">
+  <conditionalFormatting sqref="G3:G72">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -12966,7 +14337,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H62">
+  <conditionalFormatting sqref="H3:H72">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento automatico del 16/10/2026 alle 20:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -9758,21 +9758,61 @@
         <f>IF(Partite!$F53="","",Partite!$F53)</f>
         <v/>
       </c>
-      <c r="E53" s="71" t="n"/>
-      <c r="F53" s="71" t="n"/>
-      <c r="G53" s="71" t="n"/>
-      <c r="H53" s="71" t="n"/>
-      <c r="I53" s="71" t="n"/>
-      <c r="J53" s="71" t="n"/>
-      <c r="K53" s="71" t="n"/>
-      <c r="L53" s="71" t="n"/>
-      <c r="M53" s="71" t="n"/>
-      <c r="N53" s="71" t="n"/>
-      <c r="O53" s="71" t="n"/>
-      <c r="P53" s="71" t="n"/>
-      <c r="Q53" s="71" t="n"/>
-      <c r="R53" s="71" t="n"/>
-      <c r="S53" s="71" t="n"/>
+      <c r="E53" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F53" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H53" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I53" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K53" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L53" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M53" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O53" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P53" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q53" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R53" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S53" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="74">
@@ -9791,21 +9831,61 @@
         <f>IF(Partite!$F54="","",Partite!$F54)</f>
         <v/>
       </c>
-      <c r="E54" s="71" t="n"/>
-      <c r="F54" s="71" t="n"/>
-      <c r="G54" s="71" t="n"/>
-      <c r="H54" s="71" t="n"/>
-      <c r="I54" s="71" t="n"/>
-      <c r="J54" s="71" t="n"/>
-      <c r="K54" s="71" t="n"/>
-      <c r="L54" s="71" t="n"/>
-      <c r="M54" s="71" t="n"/>
-      <c r="N54" s="71" t="n"/>
-      <c r="O54" s="71" t="n"/>
-      <c r="P54" s="71" t="n"/>
-      <c r="Q54" s="71" t="n"/>
-      <c r="R54" s="71" t="n"/>
-      <c r="S54" s="71" t="n"/>
+      <c r="E54" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F54" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I54" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J54" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L54" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O54" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q54" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R54" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="74">
@@ -9824,21 +9904,61 @@
         <f>IF(Partite!$F55="","",Partite!$F55)</f>
         <v/>
       </c>
-      <c r="E55" s="71" t="n"/>
-      <c r="F55" s="71" t="n"/>
-      <c r="G55" s="71" t="n"/>
-      <c r="H55" s="71" t="n"/>
-      <c r="I55" s="71" t="n"/>
-      <c r="J55" s="71" t="n"/>
-      <c r="K55" s="71" t="n"/>
-      <c r="L55" s="71" t="n"/>
-      <c r="M55" s="71" t="n"/>
-      <c r="N55" s="71" t="n"/>
-      <c r="O55" s="71" t="n"/>
-      <c r="P55" s="71" t="n"/>
-      <c r="Q55" s="71" t="n"/>
-      <c r="R55" s="71" t="n"/>
-      <c r="S55" s="71" t="n"/>
+      <c r="E55" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F55" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I55" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L55" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N55" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O55" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P55" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q55" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R55" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="74">
@@ -9857,21 +9977,61 @@
         <f>IF(Partite!$F56="","",Partite!$F56)</f>
         <v/>
       </c>
-      <c r="E56" s="71" t="n"/>
-      <c r="F56" s="71" t="n"/>
-      <c r="G56" s="71" t="n"/>
-      <c r="H56" s="71" t="n"/>
-      <c r="I56" s="71" t="n"/>
-      <c r="J56" s="71" t="n"/>
-      <c r="K56" s="71" t="n"/>
-      <c r="L56" s="71" t="n"/>
-      <c r="M56" s="71" t="n"/>
-      <c r="N56" s="71" t="n"/>
-      <c r="O56" s="71" t="n"/>
-      <c r="P56" s="71" t="n"/>
-      <c r="Q56" s="71" t="n"/>
-      <c r="R56" s="71" t="n"/>
-      <c r="S56" s="71" t="n"/>
+      <c r="E56" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F56" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I56" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J56" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L56" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M56" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O56" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P56" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R56" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="S56" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="74">
@@ -9890,21 +10050,61 @@
         <f>IF(Partite!$F57="","",Partite!$F57)</f>
         <v/>
       </c>
-      <c r="E57" s="71" t="n"/>
-      <c r="F57" s="71" t="n"/>
-      <c r="G57" s="71" t="n"/>
-      <c r="H57" s="71" t="n"/>
-      <c r="I57" s="71" t="n"/>
-      <c r="J57" s="71" t="n"/>
-      <c r="K57" s="71" t="n"/>
-      <c r="L57" s="71" t="n"/>
-      <c r="M57" s="71" t="n"/>
-      <c r="N57" s="71" t="n"/>
-      <c r="O57" s="71" t="n"/>
-      <c r="P57" s="71" t="n"/>
-      <c r="Q57" s="71" t="n"/>
-      <c r="R57" s="71" t="n"/>
-      <c r="S57" s="71" t="n"/>
+      <c r="E57" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F57" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G57" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I57" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J57" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L57" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O57" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P57" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R57" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S57" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="74">
@@ -9923,21 +10123,61 @@
         <f>IF(Partite!$F58="","",Partite!$F58)</f>
         <v/>
       </c>
-      <c r="E58" s="71" t="n"/>
-      <c r="F58" s="71" t="n"/>
-      <c r="G58" s="71" t="n"/>
-      <c r="H58" s="71" t="n"/>
-      <c r="I58" s="71" t="n"/>
-      <c r="J58" s="71" t="n"/>
-      <c r="K58" s="71" t="n"/>
-      <c r="L58" s="71" t="n"/>
-      <c r="M58" s="71" t="n"/>
-      <c r="N58" s="71" t="n"/>
-      <c r="O58" s="71" t="n"/>
-      <c r="P58" s="71" t="n"/>
-      <c r="Q58" s="71" t="n"/>
-      <c r="R58" s="71" t="n"/>
-      <c r="S58" s="71" t="n"/>
+      <c r="E58" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q58" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R58" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S58" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="74">
@@ -9956,21 +10196,61 @@
         <f>IF(Partite!$F59="","",Partite!$F59)</f>
         <v/>
       </c>
-      <c r="E59" s="71" t="n"/>
-      <c r="F59" s="71" t="n"/>
-      <c r="G59" s="71" t="n"/>
-      <c r="H59" s="71" t="n"/>
-      <c r="I59" s="71" t="n"/>
-      <c r="J59" s="71" t="n"/>
-      <c r="K59" s="71" t="n"/>
-      <c r="L59" s="71" t="n"/>
-      <c r="M59" s="71" t="n"/>
-      <c r="N59" s="71" t="n"/>
-      <c r="O59" s="71" t="n"/>
-      <c r="P59" s="71" t="n"/>
-      <c r="Q59" s="71" t="n"/>
-      <c r="R59" s="71" t="n"/>
-      <c r="S59" s="71" t="n"/>
+      <c r="E59" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F59" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I59" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O59" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q59" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R59" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S59" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="74">
@@ -9989,21 +10269,61 @@
         <f>IF(Partite!$F60="","",Partite!$F60)</f>
         <v/>
       </c>
-      <c r="E60" s="71" t="n"/>
-      <c r="F60" s="71" t="n"/>
-      <c r="G60" s="71" t="n"/>
-      <c r="H60" s="71" t="n"/>
-      <c r="I60" s="71" t="n"/>
-      <c r="J60" s="71" t="n"/>
-      <c r="K60" s="71" t="n"/>
-      <c r="L60" s="71" t="n"/>
-      <c r="M60" s="71" t="n"/>
-      <c r="N60" s="71" t="n"/>
-      <c r="O60" s="71" t="n"/>
-      <c r="P60" s="71" t="n"/>
-      <c r="Q60" s="71" t="n"/>
-      <c r="R60" s="71" t="n"/>
-      <c r="S60" s="71" t="n"/>
+      <c r="E60" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F60" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N60" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P60" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R60" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S60" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="74">
@@ -10022,21 +10342,61 @@
         <f>IF(Partite!$F61="","",Partite!$F61)</f>
         <v/>
       </c>
-      <c r="E61" s="71" t="n"/>
-      <c r="F61" s="71" t="n"/>
-      <c r="G61" s="71" t="n"/>
-      <c r="H61" s="71" t="n"/>
-      <c r="I61" s="71" t="n"/>
-      <c r="J61" s="71" t="n"/>
-      <c r="K61" s="71" t="n"/>
-      <c r="L61" s="71" t="n"/>
-      <c r="M61" s="71" t="n"/>
-      <c r="N61" s="71" t="n"/>
-      <c r="O61" s="71" t="n"/>
-      <c r="P61" s="71" t="n"/>
-      <c r="Q61" s="71" t="n"/>
-      <c r="R61" s="71" t="n"/>
-      <c r="S61" s="71" t="n"/>
+      <c r="E61" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F61" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I61" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K61" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L61" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M61" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N61" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O61" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P61" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q61" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R61" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S61" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="74">
@@ -10055,21 +10415,61 @@
         <f>IF(Partite!$F62="","",Partite!$F62)</f>
         <v/>
       </c>
-      <c r="E62" s="71" t="n"/>
-      <c r="F62" s="71" t="n"/>
-      <c r="G62" s="71" t="n"/>
-      <c r="H62" s="71" t="n"/>
-      <c r="I62" s="71" t="n"/>
-      <c r="J62" s="71" t="n"/>
-      <c r="K62" s="71" t="n"/>
-      <c r="L62" s="71" t="n"/>
-      <c r="M62" s="71" t="n"/>
-      <c r="N62" s="71" t="n"/>
-      <c r="O62" s="71" t="n"/>
-      <c r="P62" s="71" t="n"/>
-      <c r="Q62" s="71" t="n"/>
-      <c r="R62" s="71" t="n"/>
-      <c r="S62" s="71" t="n"/>
+      <c r="E62" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I62" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N62" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q62" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S62" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="69">

</xml_diff>

<commit_message>
Aggiornamento automatico del 16/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5056,8 +5056,12 @@
           <t>Sassuolo</t>
         </is>
       </c>
-      <c r="G53" s="71" t="n"/>
-      <c r="H53" s="71" t="n"/>
+      <c r="G53" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I53" s="76">
         <f>IF(OR($G53="",$H53=""),"",IF($G53&gt;$H53,"1",IF($G53=$H53,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 17/10/2026 alle 17:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5104,8 +5104,12 @@
           <t>Napoli</t>
         </is>
       </c>
-      <c r="G54" s="71" t="n"/>
-      <c r="H54" s="71" t="n"/>
+      <c r="G54" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I54" s="76">
         <f>IF(OR($G54="",$H54=""),"",IF($G54&gt;$H54,"1",IF($G54=$H54,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 17/10/2026 alle 20:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5152,8 +5152,12 @@
           <t>Inter</t>
         </is>
       </c>
-      <c r="G55" s="71" t="n"/>
-      <c r="H55" s="71" t="n"/>
+      <c r="G55" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I55" s="76">
         <f>IF(OR($G55="",$H55=""),"",IF($G55&gt;$H55,"1",IF($G55=$H55,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 17/10/2026 alle 22:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5200,8 +5200,12 @@
           <t>Genoa</t>
         </is>
       </c>
-      <c r="G56" s="71" t="n"/>
-      <c r="H56" s="71" t="n"/>
+      <c r="G56" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I56" s="76">
         <f>IF(OR($G56="",$H56=""),"",IF($G56&gt;$H56,"1",IF($G56=$H56,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/10/2026 alle 14:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5248,8 +5248,12 @@
           <t>Lecce</t>
         </is>
       </c>
-      <c r="G57" s="71" t="n"/>
-      <c r="H57" s="71" t="n"/>
+      <c r="G57" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I57" s="76">
         <f>IF(OR($G57="",$H57=""),"",IF($G57&gt;$H57,"1",IF($G57=$H57,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/10/2026 alle 17:14
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5296,8 +5296,12 @@
           <t>Como</t>
         </is>
       </c>
-      <c r="G58" s="71" t="n"/>
-      <c r="H58" s="71" t="n"/>
+      <c r="G58" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I58" s="76">
         <f>IF(OR($G58="",$H58=""),"",IF($G58&gt;$H58,"1",IF($G58=$H58,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/10/2026 alle 20:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5344,8 +5344,12 @@
           <t>Atalanta</t>
         </is>
       </c>
-      <c r="G59" s="71" t="n"/>
-      <c r="H59" s="71" t="n"/>
+      <c r="G59" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H59" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I59" s="76">
         <f>IF(OR($G59="",$H59=""),"",IF($G59&gt;$H59,"1",IF($G59=$H59,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 18/10/2026 alle 22:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5392,8 +5392,12 @@
           <t>Lazio</t>
         </is>
       </c>
-      <c r="G60" s="71" t="n"/>
-      <c r="H60" s="71" t="n"/>
+      <c r="G60" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I60" s="76">
         <f>IF(OR($G60="",$H60=""),"",IF($G60&gt;$H60,"1",IF($G60=$H60,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 19/10/2026 alle 20:29
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5440,8 +5440,12 @@
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="G61" s="71" t="n"/>
-      <c r="H61" s="71" t="n"/>
+      <c r="G61" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H61" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I61" s="76">
         <f>IF(OR($G61="",$H61=""),"",IF($G61&gt;$H61,"1",IF($G61=$H61,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 19/10/2026 alle 22:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$39</f>
+              <f>'Classifica'!$A$33:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$R$33:$R$39</f>
+              <f>'Classifica'!$R$33:$R$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -851,12 +851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$39</f>
+              <f>'Classifica'!$A$33:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$S$33:$S$39</f>
+              <f>'Classifica'!$S$33:$S$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -888,12 +888,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$39</f>
+              <f>'Classifica'!$A$33:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$T$33:$T$39</f>
+              <f>'Classifica'!$T$33:$T$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -925,12 +925,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$39</f>
+              <f>'Classifica'!$A$33:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$U$33:$U$39</f>
+              <f>'Classifica'!$U$33:$U$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -962,12 +962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$39</f>
+              <f>'Classifica'!$A$33:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$V$33:$V$39</f>
+              <f>'Classifica'!$V$33:$V$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1043,7 +1043,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>41</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9720000" cy="3420000"/>
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>COUNTIF($B$33:$B$39,"Completata")</f>
+        <f>COUNTIF($B$33:$B$40,"Completata")</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>COUNTIF($B$33:$B$39,"Completata")+COUNTIF($B$33:$B$39,"In corso")</f>
+        <f>COUNTIF($B$33:$B$40,"Completata")+COUNTIF($B$33:$B$40,"In corso")</f>
         <v/>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L7" s="13">
-        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$39="Completata")*$A$33:$A$39)))</f>
+        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$40="Completata")*$A$33:$A$40)))</f>
         <v/>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="L8" s="13">
-        <f>IF(SUMPRODUCT(MIN(($B$33:$B$39&lt;&gt;"Completata")*$A$33:$A$39+($B$33:$B$39="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$39&lt;&gt;"Completata")*$A$33:$A$39+($B$33:$B$39="Completata")*999)))</f>
+        <f>IF(SUMPRODUCT(MIN(($B$33:$B$40&lt;&gt;"Completata")*$A$33:$A$40+($B$33:$B$40="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$40&lt;&gt;"Completata")*$A$33:$A$40+($B$33:$B$40="Completata")*999)))</f>
         <v/>
       </c>
     </row>
@@ -1591,19 +1591,19 @@
         <v/>
       </c>
       <c r="C12" s="24">
-        <f>SUM(Punti!$D$3:$D$72)</f>
+        <f>SUM(Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$72,Config!$D$7)+COUNTIF(Punti!$D$3:$D$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$82,Config!$D$7)+COUNTIF(Punti!$D$3:$D$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>SUMPRODUCT(((Pronostici!$E$3:$E$72&lt;&gt;"")+(Pronostici!$F$3:$F$72&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$E$3:$E$82&lt;&gt;"")+(Pronostici!$F$3:$F$82&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>SUMPRODUCT(($C$33:$C$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
+        <f>SUMPRODUCT(($C$33:$C$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1625,19 +1625,19 @@
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>SUM(Punti!$E$3:$E$72)</f>
+        <f>SUM(Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$72,Config!$D$7)+COUNTIF(Punti!$E$3:$E$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$82,Config!$D$7)+COUNTIF(Punti!$E$3:$E$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
-        <f>SUMPRODUCT(((Pronostici!$H$3:$H$72&lt;&gt;"")+(Pronostici!$I$3:$I$72&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$H$3:$H$82&lt;&gt;"")+(Pronostici!$I$3:$I$82&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G13" s="31">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="H13" s="30">
-        <f>SUMPRODUCT(($D$33:$D$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
+        <f>SUMPRODUCT(($D$33:$D$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1659,19 @@
         <v/>
       </c>
       <c r="C14" s="24">
-        <f>SUM(Punti!$F$3:$F$72)</f>
+        <f>SUM(Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$72,Config!$D$7)+COUNTIF(Punti!$F$3:$F$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$82,Config!$D$7)+COUNTIF(Punti!$F$3:$F$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>SUMPRODUCT(((Pronostici!$K$3:$K$72&lt;&gt;"")+(Pronostici!$L$3:$L$72&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$K$3:$K$82&lt;&gt;"")+(Pronostici!$L$3:$L$82&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>SUMPRODUCT(($E$33:$E$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
+        <f>SUMPRODUCT(($E$33:$E$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1693,19 +1693,19 @@
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>SUM(Punti!$G$3:$G$72)</f>
+        <f>SUM(Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$72,Config!$D$7)+COUNTIF(Punti!$G$3:$G$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$82,Config!$D$7)+COUNTIF(Punti!$G$3:$G$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
-        <f>SUMPRODUCT(((Pronostici!$N$3:$N$72&lt;&gt;"")+(Pronostici!$O$3:$O$72&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$N$3:$N$82&lt;&gt;"")+(Pronostici!$O$3:$O$82&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G15" s="31">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="H15" s="30">
-        <f>SUMPRODUCT(($F$33:$F$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
+        <f>SUMPRODUCT(($F$33:$F$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1727,19 +1727,19 @@
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>SUM(Punti!$H$3:$H$72)</f>
+        <f>SUM(Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$72,Config!$D$7)+COUNTIF(Punti!$H$3:$H$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$82,Config!$D$7)+COUNTIF(Punti!$H$3:$H$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$72,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$82,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$72&lt;&gt;"")+(Pronostici!$R$3:$R$72&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$82&lt;&gt;"")+(Pronostici!$R$3:$R$82&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>SUMPRODUCT(($G$33:$G$39=$H$33:$H$39)*($H$33:$H$39&gt;0)*($B$33:$B$39="Completata"))</f>
+        <f>SUMPRODUCT(($G$33:$G$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         <v/>
       </c>
       <c r="C20" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
         <v/>
       </c>
       <c r="D20" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E20" s="41" t="n"/>
       <c r="K20" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L20" s="43" t="n"/>
@@ -1826,7 +1826,7 @@
         <v/>
       </c>
       <c r="O20" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$E$3:$E$72&lt;&gt;"")+(Pronostici!$F$3:$F$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$E$3:$E$82&lt;&gt;"")+(Pronostici!$F$3:$F$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1836,16 +1836,16 @@
         <v/>
       </c>
       <c r="C21" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
         <v/>
       </c>
       <c r="D21" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E21" s="41" t="n"/>
       <c r="K21" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L21" s="47" t="n"/>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="O21" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$H$3:$H$72&lt;&gt;"")+(Pronostici!$I$3:$I$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$H$3:$H$82&lt;&gt;"")+(Pronostici!$I$3:$I$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v/>
       </c>
       <c r="C22" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
         <v/>
       </c>
       <c r="D22" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E22" s="41" t="n"/>
       <c r="K22" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L22" s="43" t="n"/>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="O22" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$K$3:$K$72&lt;&gt;"")+(Pronostici!$L$3:$L$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$K$3:$K$82&lt;&gt;"")+(Pronostici!$L$3:$L$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1894,16 +1894,16 @@
         <v/>
       </c>
       <c r="C23" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
         <v/>
       </c>
       <c r="D23" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E23" s="41" t="n"/>
       <c r="K23" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L23" s="47" t="n"/>
@@ -1913,7 +1913,7 @@
         <v/>
       </c>
       <c r="O23" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$N$3:$N$72&lt;&gt;"")+(Pronostici!$O$3:$O$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$N$3:$N$82&lt;&gt;"")+(Pronostici!$O$3:$O$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1923,16 +1923,16 @@
         <v/>
       </c>
       <c r="C24" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$39,MATCH($L$7,$A$33:$A$39,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
         <v/>
       </c>
       <c r="D24" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$39,MATCH($L$7,$A$33:$A$39,0)),0)=IFERROR(INDEX($H$33:$H$39,MATCH($L$7,$A$33:$A$39,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E24" s="41" t="n"/>
       <c r="K24" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L24" s="43" t="n"/>
@@ -1942,13 +1942,13 @@
         <v/>
       </c>
       <c r="O24" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$72=$L$8)*(((Pronostici!$Q$3:$Q$72&lt;&gt;"")+(Pronostici!$R$3:$R$72&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$Q$3:$Q$82&lt;&gt;"")+(Pronostici!$R$3:$R$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L25" s="47" t="n"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="26">
       <c r="K26" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L26" s="43" t="n"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="27">
       <c r="K27" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L27" s="47" t="n"/>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="28">
       <c r="K28" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L28" s="43" t="n"/>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="29">
       <c r="K29" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$72,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$72,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$72,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$82,0)),"-")</f>
         <v/>
       </c>
       <c r="L29" s="47" t="n"/>
@@ -2070,27 +2070,27 @@
         <v>2</v>
       </c>
       <c r="B33" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A33,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A33,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H33" s="61">
@@ -2127,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="B34" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A34,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A34,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H34" s="61">
@@ -2184,27 +2184,27 @@
         <v>4</v>
       </c>
       <c r="B35" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A35,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A35,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H35" s="61">
@@ -2241,27 +2241,27 @@
         <v>5</v>
       </c>
       <c r="B36" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A36,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A36,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H36" s="61">
@@ -2298,27 +2298,27 @@
         <v>6</v>
       </c>
       <c r="B37" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A37,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A37,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H37" s="61">
@@ -2355,27 +2355,27 @@
         <v>7</v>
       </c>
       <c r="B38" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A38,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$72,$A38,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H38" s="61">
@@ -2412,27 +2412,27 @@
         <v>8</v>
       </c>
       <c r="B39" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$E$3:$E$72,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$K$3:$K$72,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$K$3:$K$72,"Giocata")=COUNTIFS(Partite!$B$3:$B$72,$A39,Partite!$E$3:$E$72,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$D$3:$D$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$D$3:$D$82)</f>
         <v/>
       </c>
       <c r="D39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$E$3:$E$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$E$3:$E$82)</f>
         <v/>
       </c>
       <c r="E39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$F$3:$F$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$F$3:$F$82)</f>
         <v/>
       </c>
       <c r="F39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$G$3:$G$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$G$3:$G$82)</f>
         <v/>
       </c>
       <c r="G39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$72,$A39,Punti!$H$3:$H$72)</f>
+        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$H$3:$H$82)</f>
         <v/>
       </c>
       <c r="H39" s="61">
@@ -2461,6 +2461,63 @@
       </c>
       <c r="V39" s="63">
         <f>V38+G39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" s="47">
+        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <v/>
+      </c>
+      <c r="C40" s="30">
+        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$D$3:$D$82)</f>
+        <v/>
+      </c>
+      <c r="D40" s="30">
+        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$E$3:$E$82)</f>
+        <v/>
+      </c>
+      <c r="E40" s="30">
+        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$F$3:$F$82)</f>
+        <v/>
+      </c>
+      <c r="F40" s="30">
+        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$G$3:$G$82)</f>
+        <v/>
+      </c>
+      <c r="G40" s="30">
+        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$H$3:$H$82)</f>
+        <v/>
+      </c>
+      <c r="H40" s="61">
+        <f>MAX($C40:$G40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="64">
+        <f>IF($H40&lt;=0,"-",INDEX($C$32:$G$32,MATCH($H40,$C40:$G40,0))&amp;IF(COUNTIF($C40:$G40,$H40)&gt;1," (a pari)","")&amp;IF($B40="Completata",""," - in corso"))</f>
+        <v/>
+      </c>
+      <c r="R40" s="63">
+        <f>R39+C40</f>
+        <v/>
+      </c>
+      <c r="S40" s="63">
+        <f>S39+D40</f>
+        <v/>
+      </c>
+      <c r="T40" s="63">
+        <f>T39+E40</f>
+        <v/>
+      </c>
+      <c r="U40" s="63">
+        <f>U39+F40</f>
+        <v/>
+      </c>
+      <c r="V40" s="63">
+        <f>V39+G40</f>
         <v/>
       </c>
     </row>
@@ -2507,7 +2564,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:G39">
+  <conditionalFormatting sqref="C33:G40">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2529,7 +2586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5488,8 +5545,12 @@
           <t>Torino</t>
         </is>
       </c>
-      <c r="G62" s="71" t="n"/>
-      <c r="H62" s="71" t="n"/>
+      <c r="G62" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I62" s="76">
         <f>IF(OR($G62="",$H62=""),"",IF($G62&gt;$H62,"1",IF($G62=$H62,"X","2")))</f>
         <v/>
@@ -5943,14 +6004,454 @@
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="74" t="inlineStr">
+        <is>
+          <t>G09-01</t>
+        </is>
+      </c>
+      <c r="B73" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="D73" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E73" s="75" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="F73" s="75" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="G73" s="71" t="n"/>
+      <c r="H73" s="71" t="n"/>
+      <c r="I73" s="76">
+        <f>IF(OR($G73="",$H73=""),"",IF($G73&gt;$H73,"1",IF($G73=$H73,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J73" s="30">
+        <f>IF(OR($G73="",$H73=""),"",$G73&amp;"-"&amp;$H73)</f>
+        <v/>
+      </c>
+      <c r="K73" s="77">
+        <f>IF($E73="","Calendario da inserire",IF(OR($G73="",$H73=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="74" t="inlineStr">
+        <is>
+          <t>G09-02</t>
+        </is>
+      </c>
+      <c r="B74" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E74" s="75" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="F74" s="75" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="G74" s="71" t="n"/>
+      <c r="H74" s="71" t="n"/>
+      <c r="I74" s="76">
+        <f>IF(OR($G74="",$H74=""),"",IF($G74&gt;$H74,"1",IF($G74=$H74,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J74" s="30">
+        <f>IF(OR($G74="",$H74=""),"",$G74&amp;"-"&amp;$H74)</f>
+        <v/>
+      </c>
+      <c r="K74" s="77">
+        <f>IF($E74="","Calendario da inserire",IF(OR($G74="",$H74=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="74" t="inlineStr">
+        <is>
+          <t>G09-03</t>
+        </is>
+      </c>
+      <c r="B75" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="D75" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E75" s="75" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="F75" s="75" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="G75" s="71" t="n"/>
+      <c r="H75" s="71" t="n"/>
+      <c r="I75" s="76">
+        <f>IF(OR($G75="",$H75=""),"",IF($G75&gt;$H75,"1",IF($G75=$H75,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J75" s="30">
+        <f>IF(OR($G75="",$H75=""),"",$G75&amp;"-"&amp;$H75)</f>
+        <v/>
+      </c>
+      <c r="K75" s="77">
+        <f>IF($E75="","Calendario da inserire",IF(OR($G75="",$H75=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="74" t="inlineStr">
+        <is>
+          <t>G09-04</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E76" s="75" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="F76" s="75" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="G76" s="71" t="n"/>
+      <c r="H76" s="71" t="n"/>
+      <c r="I76" s="76">
+        <f>IF(OR($G76="",$H76=""),"",IF($G76&gt;$H76,"1",IF($G76=$H76,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J76" s="30">
+        <f>IF(OR($G76="",$H76=""),"",$G76&amp;"-"&amp;$H76)</f>
+        <v/>
+      </c>
+      <c r="K76" s="77">
+        <f>IF($E76="","Calendario da inserire",IF(OR($G76="",$H76=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="74" t="inlineStr">
+        <is>
+          <t>G09-05</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E77" s="75" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="F77" s="75" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="G77" s="71" t="n"/>
+      <c r="H77" s="71" t="n"/>
+      <c r="I77" s="76">
+        <f>IF(OR($G77="",$H77=""),"",IF($G77&gt;$H77,"1",IF($G77=$H77,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J77" s="30">
+        <f>IF(OR($G77="",$H77=""),"",$G77&amp;"-"&amp;$H77)</f>
+        <v/>
+      </c>
+      <c r="K77" s="77">
+        <f>IF($E77="","Calendario da inserire",IF(OR($G77="",$H77=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="74" t="inlineStr">
+        <is>
+          <t>G09-06</t>
+        </is>
+      </c>
+      <c r="B78" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E78" s="75" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="F78" s="75" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="G78" s="71" t="n"/>
+      <c r="H78" s="71" t="n"/>
+      <c r="I78" s="76">
+        <f>IF(OR($G78="",$H78=""),"",IF($G78&gt;$H78,"1",IF($G78=$H78,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J78" s="30">
+        <f>IF(OR($G78="",$H78=""),"",$G78&amp;"-"&amp;$H78)</f>
+        <v/>
+      </c>
+      <c r="K78" s="77">
+        <f>IF($E78="","Calendario da inserire",IF(OR($G78="",$H78=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="74" t="inlineStr">
+        <is>
+          <t>G09-07</t>
+        </is>
+      </c>
+      <c r="B79" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C79" s="30" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D79" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E79" s="75" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="F79" s="75" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="G79" s="71" t="n"/>
+      <c r="H79" s="71" t="n"/>
+      <c r="I79" s="76">
+        <f>IF(OR($G79="",$H79=""),"",IF($G79&gt;$H79,"1",IF($G79=$H79,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J79" s="30">
+        <f>IF(OR($G79="",$H79=""),"",$G79&amp;"-"&amp;$H79)</f>
+        <v/>
+      </c>
+      <c r="K79" s="77">
+        <f>IF($E79="","Calendario da inserire",IF(OR($G79="",$H79=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="74" t="inlineStr">
+        <is>
+          <t>G09-08</t>
+        </is>
+      </c>
+      <c r="B80" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C80" s="30" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D80" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E80" s="75" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="F80" s="75" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="G80" s="71" t="n"/>
+      <c r="H80" s="71" t="n"/>
+      <c r="I80" s="76">
+        <f>IF(OR($G80="",$H80=""),"",IF($G80&gt;$H80,"1",IF($G80=$H80,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J80" s="30">
+        <f>IF(OR($G80="",$H80=""),"",$G80&amp;"-"&amp;$H80)</f>
+        <v/>
+      </c>
+      <c r="K80" s="77">
+        <f>IF($E80="","Calendario da inserire",IF(OR($G80="",$H80=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="74" t="inlineStr">
+        <is>
+          <t>G09-09</t>
+        </is>
+      </c>
+      <c r="B81" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C81" s="30" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="D81" s="30" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E81" s="75" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="F81" s="75" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="G81" s="71" t="n"/>
+      <c r="H81" s="71" t="n"/>
+      <c r="I81" s="76">
+        <f>IF(OR($G81="",$H81=""),"",IF($G81&gt;$H81,"1",IF($G81=$H81,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J81" s="30">
+        <f>IF(OR($G81="",$H81=""),"",$G81&amp;"-"&amp;$H81)</f>
+        <v/>
+      </c>
+      <c r="K81" s="77">
+        <f>IF($E81="","Calendario da inserire",IF(OR($G81="",$H81=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="74" t="inlineStr">
+        <is>
+          <t>G09-10</t>
+        </is>
+      </c>
+      <c r="B82" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C82" s="30" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="D82" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E82" s="75" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="F82" s="75" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="G82" s="71" t="n"/>
+      <c r="H82" s="71" t="n"/>
+      <c r="I82" s="76">
+        <f>IF(OR($G82="",$H82=""),"",IF($G82&gt;$H82,"1",IF($G82=$H82,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J82" s="30">
+        <f>IF(OR($G82="",$H82=""),"",$G82&amp;"-"&amp;$H82)</f>
+        <v/>
+      </c>
+      <c r="K82" s="77">
+        <f>IF($E82="","Calendario da inserire",IF(OR($G82="",$H82=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K72"/>
+  <autoFilter ref="A2:K82"/>
   <mergeCells count="3">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K3:K72">
+  <conditionalFormatting sqref="K3:K82">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Giocata"</formula>
     </cfRule>
@@ -5966,7 +6467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S72"/>
+  <dimension ref="A1:S82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10837,8 +11338,338 @@
       <c r="R72" s="71" t="n"/>
       <c r="S72" s="71" t="n"/>
     </row>
+    <row r="73">
+      <c r="A73" s="74">
+        <f>Partite!$A73</f>
+        <v/>
+      </c>
+      <c r="B73" s="30">
+        <f>Partite!$B73</f>
+        <v/>
+      </c>
+      <c r="C73" s="75">
+        <f>IF(Partite!$E73="","",Partite!$E73)</f>
+        <v/>
+      </c>
+      <c r="D73" s="75">
+        <f>IF(Partite!$F73="","",Partite!$F73)</f>
+        <v/>
+      </c>
+      <c r="E73" s="71" t="n"/>
+      <c r="F73" s="71" t="n"/>
+      <c r="G73" s="71" t="n"/>
+      <c r="H73" s="71" t="n"/>
+      <c r="I73" s="71" t="n"/>
+      <c r="J73" s="71" t="n"/>
+      <c r="K73" s="71" t="n"/>
+      <c r="L73" s="71" t="n"/>
+      <c r="M73" s="71" t="n"/>
+      <c r="N73" s="71" t="n"/>
+      <c r="O73" s="71" t="n"/>
+      <c r="P73" s="71" t="n"/>
+      <c r="Q73" s="71" t="n"/>
+      <c r="R73" s="71" t="n"/>
+      <c r="S73" s="71" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="74">
+        <f>Partite!$A74</f>
+        <v/>
+      </c>
+      <c r="B74" s="30">
+        <f>Partite!$B74</f>
+        <v/>
+      </c>
+      <c r="C74" s="75">
+        <f>IF(Partite!$E74="","",Partite!$E74)</f>
+        <v/>
+      </c>
+      <c r="D74" s="75">
+        <f>IF(Partite!$F74="","",Partite!$F74)</f>
+        <v/>
+      </c>
+      <c r="E74" s="71" t="n"/>
+      <c r="F74" s="71" t="n"/>
+      <c r="G74" s="71" t="n"/>
+      <c r="H74" s="71" t="n"/>
+      <c r="I74" s="71" t="n"/>
+      <c r="J74" s="71" t="n"/>
+      <c r="K74" s="71" t="n"/>
+      <c r="L74" s="71" t="n"/>
+      <c r="M74" s="71" t="n"/>
+      <c r="N74" s="71" t="n"/>
+      <c r="O74" s="71" t="n"/>
+      <c r="P74" s="71" t="n"/>
+      <c r="Q74" s="71" t="n"/>
+      <c r="R74" s="71" t="n"/>
+      <c r="S74" s="71" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="74">
+        <f>Partite!$A75</f>
+        <v/>
+      </c>
+      <c r="B75" s="30">
+        <f>Partite!$B75</f>
+        <v/>
+      </c>
+      <c r="C75" s="75">
+        <f>IF(Partite!$E75="","",Partite!$E75)</f>
+        <v/>
+      </c>
+      <c r="D75" s="75">
+        <f>IF(Partite!$F75="","",Partite!$F75)</f>
+        <v/>
+      </c>
+      <c r="E75" s="71" t="n"/>
+      <c r="F75" s="71" t="n"/>
+      <c r="G75" s="71" t="n"/>
+      <c r="H75" s="71" t="n"/>
+      <c r="I75" s="71" t="n"/>
+      <c r="J75" s="71" t="n"/>
+      <c r="K75" s="71" t="n"/>
+      <c r="L75" s="71" t="n"/>
+      <c r="M75" s="71" t="n"/>
+      <c r="N75" s="71" t="n"/>
+      <c r="O75" s="71" t="n"/>
+      <c r="P75" s="71" t="n"/>
+      <c r="Q75" s="71" t="n"/>
+      <c r="R75" s="71" t="n"/>
+      <c r="S75" s="71" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="74">
+        <f>Partite!$A76</f>
+        <v/>
+      </c>
+      <c r="B76" s="30">
+        <f>Partite!$B76</f>
+        <v/>
+      </c>
+      <c r="C76" s="75">
+        <f>IF(Partite!$E76="","",Partite!$E76)</f>
+        <v/>
+      </c>
+      <c r="D76" s="75">
+        <f>IF(Partite!$F76="","",Partite!$F76)</f>
+        <v/>
+      </c>
+      <c r="E76" s="71" t="n"/>
+      <c r="F76" s="71" t="n"/>
+      <c r="G76" s="71" t="n"/>
+      <c r="H76" s="71" t="n"/>
+      <c r="I76" s="71" t="n"/>
+      <c r="J76" s="71" t="n"/>
+      <c r="K76" s="71" t="n"/>
+      <c r="L76" s="71" t="n"/>
+      <c r="M76" s="71" t="n"/>
+      <c r="N76" s="71" t="n"/>
+      <c r="O76" s="71" t="n"/>
+      <c r="P76" s="71" t="n"/>
+      <c r="Q76" s="71" t="n"/>
+      <c r="R76" s="71" t="n"/>
+      <c r="S76" s="71" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="74">
+        <f>Partite!$A77</f>
+        <v/>
+      </c>
+      <c r="B77" s="30">
+        <f>Partite!$B77</f>
+        <v/>
+      </c>
+      <c r="C77" s="75">
+        <f>IF(Partite!$E77="","",Partite!$E77)</f>
+        <v/>
+      </c>
+      <c r="D77" s="75">
+        <f>IF(Partite!$F77="","",Partite!$F77)</f>
+        <v/>
+      </c>
+      <c r="E77" s="71" t="n"/>
+      <c r="F77" s="71" t="n"/>
+      <c r="G77" s="71" t="n"/>
+      <c r="H77" s="71" t="n"/>
+      <c r="I77" s="71" t="n"/>
+      <c r="J77" s="71" t="n"/>
+      <c r="K77" s="71" t="n"/>
+      <c r="L77" s="71" t="n"/>
+      <c r="M77" s="71" t="n"/>
+      <c r="N77" s="71" t="n"/>
+      <c r="O77" s="71" t="n"/>
+      <c r="P77" s="71" t="n"/>
+      <c r="Q77" s="71" t="n"/>
+      <c r="R77" s="71" t="n"/>
+      <c r="S77" s="71" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="74">
+        <f>Partite!$A78</f>
+        <v/>
+      </c>
+      <c r="B78" s="30">
+        <f>Partite!$B78</f>
+        <v/>
+      </c>
+      <c r="C78" s="75">
+        <f>IF(Partite!$E78="","",Partite!$E78)</f>
+        <v/>
+      </c>
+      <c r="D78" s="75">
+        <f>IF(Partite!$F78="","",Partite!$F78)</f>
+        <v/>
+      </c>
+      <c r="E78" s="71" t="n"/>
+      <c r="F78" s="71" t="n"/>
+      <c r="G78" s="71" t="n"/>
+      <c r="H78" s="71" t="n"/>
+      <c r="I78" s="71" t="n"/>
+      <c r="J78" s="71" t="n"/>
+      <c r="K78" s="71" t="n"/>
+      <c r="L78" s="71" t="n"/>
+      <c r="M78" s="71" t="n"/>
+      <c r="N78" s="71" t="n"/>
+      <c r="O78" s="71" t="n"/>
+      <c r="P78" s="71" t="n"/>
+      <c r="Q78" s="71" t="n"/>
+      <c r="R78" s="71" t="n"/>
+      <c r="S78" s="71" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="74">
+        <f>Partite!$A79</f>
+        <v/>
+      </c>
+      <c r="B79" s="30">
+        <f>Partite!$B79</f>
+        <v/>
+      </c>
+      <c r="C79" s="75">
+        <f>IF(Partite!$E79="","",Partite!$E79)</f>
+        <v/>
+      </c>
+      <c r="D79" s="75">
+        <f>IF(Partite!$F79="","",Partite!$F79)</f>
+        <v/>
+      </c>
+      <c r="E79" s="71" t="n"/>
+      <c r="F79" s="71" t="n"/>
+      <c r="G79" s="71" t="n"/>
+      <c r="H79" s="71" t="n"/>
+      <c r="I79" s="71" t="n"/>
+      <c r="J79" s="71" t="n"/>
+      <c r="K79" s="71" t="n"/>
+      <c r="L79" s="71" t="n"/>
+      <c r="M79" s="71" t="n"/>
+      <c r="N79" s="71" t="n"/>
+      <c r="O79" s="71" t="n"/>
+      <c r="P79" s="71" t="n"/>
+      <c r="Q79" s="71" t="n"/>
+      <c r="R79" s="71" t="n"/>
+      <c r="S79" s="71" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="74">
+        <f>Partite!$A80</f>
+        <v/>
+      </c>
+      <c r="B80" s="30">
+        <f>Partite!$B80</f>
+        <v/>
+      </c>
+      <c r="C80" s="75">
+        <f>IF(Partite!$E80="","",Partite!$E80)</f>
+        <v/>
+      </c>
+      <c r="D80" s="75">
+        <f>IF(Partite!$F80="","",Partite!$F80)</f>
+        <v/>
+      </c>
+      <c r="E80" s="71" t="n"/>
+      <c r="F80" s="71" t="n"/>
+      <c r="G80" s="71" t="n"/>
+      <c r="H80" s="71" t="n"/>
+      <c r="I80" s="71" t="n"/>
+      <c r="J80" s="71" t="n"/>
+      <c r="K80" s="71" t="n"/>
+      <c r="L80" s="71" t="n"/>
+      <c r="M80" s="71" t="n"/>
+      <c r="N80" s="71" t="n"/>
+      <c r="O80" s="71" t="n"/>
+      <c r="P80" s="71" t="n"/>
+      <c r="Q80" s="71" t="n"/>
+      <c r="R80" s="71" t="n"/>
+      <c r="S80" s="71" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="74">
+        <f>Partite!$A81</f>
+        <v/>
+      </c>
+      <c r="B81" s="30">
+        <f>Partite!$B81</f>
+        <v/>
+      </c>
+      <c r="C81" s="75">
+        <f>IF(Partite!$E81="","",Partite!$E81)</f>
+        <v/>
+      </c>
+      <c r="D81" s="75">
+        <f>IF(Partite!$F81="","",Partite!$F81)</f>
+        <v/>
+      </c>
+      <c r="E81" s="71" t="n"/>
+      <c r="F81" s="71" t="n"/>
+      <c r="G81" s="71" t="n"/>
+      <c r="H81" s="71" t="n"/>
+      <c r="I81" s="71" t="n"/>
+      <c r="J81" s="71" t="n"/>
+      <c r="K81" s="71" t="n"/>
+      <c r="L81" s="71" t="n"/>
+      <c r="M81" s="71" t="n"/>
+      <c r="N81" s="71" t="n"/>
+      <c r="O81" s="71" t="n"/>
+      <c r="P81" s="71" t="n"/>
+      <c r="Q81" s="71" t="n"/>
+      <c r="R81" s="71" t="n"/>
+      <c r="S81" s="71" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="74">
+        <f>Partite!$A82</f>
+        <v/>
+      </c>
+      <c r="B82" s="30">
+        <f>Partite!$B82</f>
+        <v/>
+      </c>
+      <c r="C82" s="75">
+        <f>IF(Partite!$E82="","",Partite!$E82)</f>
+        <v/>
+      </c>
+      <c r="D82" s="75">
+        <f>IF(Partite!$F82="","",Partite!$F82)</f>
+        <v/>
+      </c>
+      <c r="E82" s="71" t="n"/>
+      <c r="F82" s="71" t="n"/>
+      <c r="G82" s="71" t="n"/>
+      <c r="H82" s="71" t="n"/>
+      <c r="I82" s="71" t="n"/>
+      <c r="J82" s="71" t="n"/>
+      <c r="K82" s="71" t="n"/>
+      <c r="L82" s="71" t="n"/>
+      <c r="M82" s="71" t="n"/>
+      <c r="N82" s="71" t="n"/>
+      <c r="O82" s="71" t="n"/>
+      <c r="P82" s="71" t="n"/>
+      <c r="Q82" s="71" t="n"/>
+      <c r="R82" s="71" t="n"/>
+      <c r="S82" s="71" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:D72"/>
+  <autoFilter ref="A2:D82"/>
   <mergeCells count="6">
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A1:D1"/>
@@ -10848,7 +11679,7 @@
     <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
       <formula1>"1,X,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10863,7 +11694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14737,11 +15568,551 @@
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="74">
+        <f>Partite!$A73</f>
+        <v/>
+      </c>
+      <c r="B73" s="30">
+        <f>Partite!$B73</f>
+        <v/>
+      </c>
+      <c r="C73" s="47">
+        <f>IF(Partite!$E73="","",Partite!$E73&amp;"  -  "&amp;Partite!$F73)</f>
+        <v/>
+      </c>
+      <c r="D73" s="27">
+        <f>IF(Partite!$K73&lt;&gt;"Giocata","",IF(AND(Pronostici!$F73&lt;&gt;"",Pronostici!$G73&lt;&gt;"",Pronostici!$F73=Partite!$G73,Pronostici!$G73=Partite!$H73),Config!$D$6,IF(AND($J73&lt;&gt;"",$J73=Partite!$I73),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E73" s="27">
+        <f>IF(Partite!$K73&lt;&gt;"Giocata","",IF(AND(Pronostici!$I73&lt;&gt;"",Pronostici!$J73&lt;&gt;"",Pronostici!$I73=Partite!$G73,Pronostici!$J73=Partite!$H73),Config!$D$6,IF(AND($K73&lt;&gt;"",$K73=Partite!$I73),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F73" s="27">
+        <f>IF(Partite!$K73&lt;&gt;"Giocata","",IF(AND(Pronostici!$L73&lt;&gt;"",Pronostici!$M73&lt;&gt;"",Pronostici!$L73=Partite!$G73,Pronostici!$M73=Partite!$H73),Config!$D$6,IF(AND($L73&lt;&gt;"",$L73=Partite!$I73),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G73" s="27">
+        <f>IF(Partite!$K73&lt;&gt;"Giocata","",IF(AND(Pronostici!$O73&lt;&gt;"",Pronostici!$P73&lt;&gt;"",Pronostici!$O73=Partite!$G73,Pronostici!$P73=Partite!$H73),Config!$D$6,IF(AND($M73&lt;&gt;"",$M73=Partite!$I73),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H73" s="27">
+        <f>IF(Partite!$K73&lt;&gt;"Giocata","",IF(AND(Pronostici!$R73&lt;&gt;"",Pronostici!$S73&lt;&gt;"",Pronostici!$R73=Partite!$G73,Pronostici!$S73=Partite!$H73),Config!$D$6,IF(AND($N73&lt;&gt;"",$N73=Partite!$I73),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J73" s="63">
+        <f>IF(Pronostici!$E73&lt;&gt;"",UPPER(Pronostici!$E73),IF(OR(Pronostici!$F73="",Pronostici!$G73=""),"",IF(Pronostici!$F73&gt;Pronostici!$G73,"1",IF(Pronostici!$F73=Pronostici!$G73,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K73" s="63">
+        <f>IF(Pronostici!$H73&lt;&gt;"",UPPER(Pronostici!$H73),IF(OR(Pronostici!$I73="",Pronostici!$J73=""),"",IF(Pronostici!$I73&gt;Pronostici!$J73,"1",IF(Pronostici!$I73=Pronostici!$J73,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L73" s="63">
+        <f>IF(Pronostici!$K73&lt;&gt;"",UPPER(Pronostici!$K73),IF(OR(Pronostici!$L73="",Pronostici!$M73=""),"",IF(Pronostici!$L73&gt;Pronostici!$M73,"1",IF(Pronostici!$L73=Pronostici!$M73,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M73" s="63">
+        <f>IF(Pronostici!$N73&lt;&gt;"",UPPER(Pronostici!$N73),IF(OR(Pronostici!$O73="",Pronostici!$P73=""),"",IF(Pronostici!$O73&gt;Pronostici!$P73,"1",IF(Pronostici!$O73=Pronostici!$P73,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N73" s="63">
+        <f>IF(Pronostici!$Q73&lt;&gt;"",UPPER(Pronostici!$Q73),IF(OR(Pronostici!$R73="",Pronostici!$S73=""),"",IF(Pronostici!$R73&gt;Pronostici!$S73,"1",IF(Pronostici!$R73=Pronostici!$S73,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="74">
+        <f>Partite!$A74</f>
+        <v/>
+      </c>
+      <c r="B74" s="30">
+        <f>Partite!$B74</f>
+        <v/>
+      </c>
+      <c r="C74" s="47">
+        <f>IF(Partite!$E74="","",Partite!$E74&amp;"  -  "&amp;Partite!$F74)</f>
+        <v/>
+      </c>
+      <c r="D74" s="27">
+        <f>IF(Partite!$K74&lt;&gt;"Giocata","",IF(AND(Pronostici!$F74&lt;&gt;"",Pronostici!$G74&lt;&gt;"",Pronostici!$F74=Partite!$G74,Pronostici!$G74=Partite!$H74),Config!$D$6,IF(AND($J74&lt;&gt;"",$J74=Partite!$I74),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E74" s="27">
+        <f>IF(Partite!$K74&lt;&gt;"Giocata","",IF(AND(Pronostici!$I74&lt;&gt;"",Pronostici!$J74&lt;&gt;"",Pronostici!$I74=Partite!$G74,Pronostici!$J74=Partite!$H74),Config!$D$6,IF(AND($K74&lt;&gt;"",$K74=Partite!$I74),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F74" s="27">
+        <f>IF(Partite!$K74&lt;&gt;"Giocata","",IF(AND(Pronostici!$L74&lt;&gt;"",Pronostici!$M74&lt;&gt;"",Pronostici!$L74=Partite!$G74,Pronostici!$M74=Partite!$H74),Config!$D$6,IF(AND($L74&lt;&gt;"",$L74=Partite!$I74),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G74" s="27">
+        <f>IF(Partite!$K74&lt;&gt;"Giocata","",IF(AND(Pronostici!$O74&lt;&gt;"",Pronostici!$P74&lt;&gt;"",Pronostici!$O74=Partite!$G74,Pronostici!$P74=Partite!$H74),Config!$D$6,IF(AND($M74&lt;&gt;"",$M74=Partite!$I74),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H74" s="27">
+        <f>IF(Partite!$K74&lt;&gt;"Giocata","",IF(AND(Pronostici!$R74&lt;&gt;"",Pronostici!$S74&lt;&gt;"",Pronostici!$R74=Partite!$G74,Pronostici!$S74=Partite!$H74),Config!$D$6,IF(AND($N74&lt;&gt;"",$N74=Partite!$I74),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J74" s="63">
+        <f>IF(Pronostici!$E74&lt;&gt;"",UPPER(Pronostici!$E74),IF(OR(Pronostici!$F74="",Pronostici!$G74=""),"",IF(Pronostici!$F74&gt;Pronostici!$G74,"1",IF(Pronostici!$F74=Pronostici!$G74,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K74" s="63">
+        <f>IF(Pronostici!$H74&lt;&gt;"",UPPER(Pronostici!$H74),IF(OR(Pronostici!$I74="",Pronostici!$J74=""),"",IF(Pronostici!$I74&gt;Pronostici!$J74,"1",IF(Pronostici!$I74=Pronostici!$J74,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L74" s="63">
+        <f>IF(Pronostici!$K74&lt;&gt;"",UPPER(Pronostici!$K74),IF(OR(Pronostici!$L74="",Pronostici!$M74=""),"",IF(Pronostici!$L74&gt;Pronostici!$M74,"1",IF(Pronostici!$L74=Pronostici!$M74,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M74" s="63">
+        <f>IF(Pronostici!$N74&lt;&gt;"",UPPER(Pronostici!$N74),IF(OR(Pronostici!$O74="",Pronostici!$P74=""),"",IF(Pronostici!$O74&gt;Pronostici!$P74,"1",IF(Pronostici!$O74=Pronostici!$P74,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N74" s="63">
+        <f>IF(Pronostici!$Q74&lt;&gt;"",UPPER(Pronostici!$Q74),IF(OR(Pronostici!$R74="",Pronostici!$S74=""),"",IF(Pronostici!$R74&gt;Pronostici!$S74,"1",IF(Pronostici!$R74=Pronostici!$S74,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="74">
+        <f>Partite!$A75</f>
+        <v/>
+      </c>
+      <c r="B75" s="30">
+        <f>Partite!$B75</f>
+        <v/>
+      </c>
+      <c r="C75" s="47">
+        <f>IF(Partite!$E75="","",Partite!$E75&amp;"  -  "&amp;Partite!$F75)</f>
+        <v/>
+      </c>
+      <c r="D75" s="27">
+        <f>IF(Partite!$K75&lt;&gt;"Giocata","",IF(AND(Pronostici!$F75&lt;&gt;"",Pronostici!$G75&lt;&gt;"",Pronostici!$F75=Partite!$G75,Pronostici!$G75=Partite!$H75),Config!$D$6,IF(AND($J75&lt;&gt;"",$J75=Partite!$I75),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E75" s="27">
+        <f>IF(Partite!$K75&lt;&gt;"Giocata","",IF(AND(Pronostici!$I75&lt;&gt;"",Pronostici!$J75&lt;&gt;"",Pronostici!$I75=Partite!$G75,Pronostici!$J75=Partite!$H75),Config!$D$6,IF(AND($K75&lt;&gt;"",$K75=Partite!$I75),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F75" s="27">
+        <f>IF(Partite!$K75&lt;&gt;"Giocata","",IF(AND(Pronostici!$L75&lt;&gt;"",Pronostici!$M75&lt;&gt;"",Pronostici!$L75=Partite!$G75,Pronostici!$M75=Partite!$H75),Config!$D$6,IF(AND($L75&lt;&gt;"",$L75=Partite!$I75),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G75" s="27">
+        <f>IF(Partite!$K75&lt;&gt;"Giocata","",IF(AND(Pronostici!$O75&lt;&gt;"",Pronostici!$P75&lt;&gt;"",Pronostici!$O75=Partite!$G75,Pronostici!$P75=Partite!$H75),Config!$D$6,IF(AND($M75&lt;&gt;"",$M75=Partite!$I75),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H75" s="27">
+        <f>IF(Partite!$K75&lt;&gt;"Giocata","",IF(AND(Pronostici!$R75&lt;&gt;"",Pronostici!$S75&lt;&gt;"",Pronostici!$R75=Partite!$G75,Pronostici!$S75=Partite!$H75),Config!$D$6,IF(AND($N75&lt;&gt;"",$N75=Partite!$I75),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J75" s="63">
+        <f>IF(Pronostici!$E75&lt;&gt;"",UPPER(Pronostici!$E75),IF(OR(Pronostici!$F75="",Pronostici!$G75=""),"",IF(Pronostici!$F75&gt;Pronostici!$G75,"1",IF(Pronostici!$F75=Pronostici!$G75,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K75" s="63">
+        <f>IF(Pronostici!$H75&lt;&gt;"",UPPER(Pronostici!$H75),IF(OR(Pronostici!$I75="",Pronostici!$J75=""),"",IF(Pronostici!$I75&gt;Pronostici!$J75,"1",IF(Pronostici!$I75=Pronostici!$J75,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L75" s="63">
+        <f>IF(Pronostici!$K75&lt;&gt;"",UPPER(Pronostici!$K75),IF(OR(Pronostici!$L75="",Pronostici!$M75=""),"",IF(Pronostici!$L75&gt;Pronostici!$M75,"1",IF(Pronostici!$L75=Pronostici!$M75,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M75" s="63">
+        <f>IF(Pronostici!$N75&lt;&gt;"",UPPER(Pronostici!$N75),IF(OR(Pronostici!$O75="",Pronostici!$P75=""),"",IF(Pronostici!$O75&gt;Pronostici!$P75,"1",IF(Pronostici!$O75=Pronostici!$P75,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N75" s="63">
+        <f>IF(Pronostici!$Q75&lt;&gt;"",UPPER(Pronostici!$Q75),IF(OR(Pronostici!$R75="",Pronostici!$S75=""),"",IF(Pronostici!$R75&gt;Pronostici!$S75,"1",IF(Pronostici!$R75=Pronostici!$S75,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="74">
+        <f>Partite!$A76</f>
+        <v/>
+      </c>
+      <c r="B76" s="30">
+        <f>Partite!$B76</f>
+        <v/>
+      </c>
+      <c r="C76" s="47">
+        <f>IF(Partite!$E76="","",Partite!$E76&amp;"  -  "&amp;Partite!$F76)</f>
+        <v/>
+      </c>
+      <c r="D76" s="27">
+        <f>IF(Partite!$K76&lt;&gt;"Giocata","",IF(AND(Pronostici!$F76&lt;&gt;"",Pronostici!$G76&lt;&gt;"",Pronostici!$F76=Partite!$G76,Pronostici!$G76=Partite!$H76),Config!$D$6,IF(AND($J76&lt;&gt;"",$J76=Partite!$I76),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E76" s="27">
+        <f>IF(Partite!$K76&lt;&gt;"Giocata","",IF(AND(Pronostici!$I76&lt;&gt;"",Pronostici!$J76&lt;&gt;"",Pronostici!$I76=Partite!$G76,Pronostici!$J76=Partite!$H76),Config!$D$6,IF(AND($K76&lt;&gt;"",$K76=Partite!$I76),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F76" s="27">
+        <f>IF(Partite!$K76&lt;&gt;"Giocata","",IF(AND(Pronostici!$L76&lt;&gt;"",Pronostici!$M76&lt;&gt;"",Pronostici!$L76=Partite!$G76,Pronostici!$M76=Partite!$H76),Config!$D$6,IF(AND($L76&lt;&gt;"",$L76=Partite!$I76),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G76" s="27">
+        <f>IF(Partite!$K76&lt;&gt;"Giocata","",IF(AND(Pronostici!$O76&lt;&gt;"",Pronostici!$P76&lt;&gt;"",Pronostici!$O76=Partite!$G76,Pronostici!$P76=Partite!$H76),Config!$D$6,IF(AND($M76&lt;&gt;"",$M76=Partite!$I76),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H76" s="27">
+        <f>IF(Partite!$K76&lt;&gt;"Giocata","",IF(AND(Pronostici!$R76&lt;&gt;"",Pronostici!$S76&lt;&gt;"",Pronostici!$R76=Partite!$G76,Pronostici!$S76=Partite!$H76),Config!$D$6,IF(AND($N76&lt;&gt;"",$N76=Partite!$I76),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J76" s="63">
+        <f>IF(Pronostici!$E76&lt;&gt;"",UPPER(Pronostici!$E76),IF(OR(Pronostici!$F76="",Pronostici!$G76=""),"",IF(Pronostici!$F76&gt;Pronostici!$G76,"1",IF(Pronostici!$F76=Pronostici!$G76,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K76" s="63">
+        <f>IF(Pronostici!$H76&lt;&gt;"",UPPER(Pronostici!$H76),IF(OR(Pronostici!$I76="",Pronostici!$J76=""),"",IF(Pronostici!$I76&gt;Pronostici!$J76,"1",IF(Pronostici!$I76=Pronostici!$J76,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L76" s="63">
+        <f>IF(Pronostici!$K76&lt;&gt;"",UPPER(Pronostici!$K76),IF(OR(Pronostici!$L76="",Pronostici!$M76=""),"",IF(Pronostici!$L76&gt;Pronostici!$M76,"1",IF(Pronostici!$L76=Pronostici!$M76,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M76" s="63">
+        <f>IF(Pronostici!$N76&lt;&gt;"",UPPER(Pronostici!$N76),IF(OR(Pronostici!$O76="",Pronostici!$P76=""),"",IF(Pronostici!$O76&gt;Pronostici!$P76,"1",IF(Pronostici!$O76=Pronostici!$P76,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N76" s="63">
+        <f>IF(Pronostici!$Q76&lt;&gt;"",UPPER(Pronostici!$Q76),IF(OR(Pronostici!$R76="",Pronostici!$S76=""),"",IF(Pronostici!$R76&gt;Pronostici!$S76,"1",IF(Pronostici!$R76=Pronostici!$S76,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="74">
+        <f>Partite!$A77</f>
+        <v/>
+      </c>
+      <c r="B77" s="30">
+        <f>Partite!$B77</f>
+        <v/>
+      </c>
+      <c r="C77" s="47">
+        <f>IF(Partite!$E77="","",Partite!$E77&amp;"  -  "&amp;Partite!$F77)</f>
+        <v/>
+      </c>
+      <c r="D77" s="27">
+        <f>IF(Partite!$K77&lt;&gt;"Giocata","",IF(AND(Pronostici!$F77&lt;&gt;"",Pronostici!$G77&lt;&gt;"",Pronostici!$F77=Partite!$G77,Pronostici!$G77=Partite!$H77),Config!$D$6,IF(AND($J77&lt;&gt;"",$J77=Partite!$I77),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E77" s="27">
+        <f>IF(Partite!$K77&lt;&gt;"Giocata","",IF(AND(Pronostici!$I77&lt;&gt;"",Pronostici!$J77&lt;&gt;"",Pronostici!$I77=Partite!$G77,Pronostici!$J77=Partite!$H77),Config!$D$6,IF(AND($K77&lt;&gt;"",$K77=Partite!$I77),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F77" s="27">
+        <f>IF(Partite!$K77&lt;&gt;"Giocata","",IF(AND(Pronostici!$L77&lt;&gt;"",Pronostici!$M77&lt;&gt;"",Pronostici!$L77=Partite!$G77,Pronostici!$M77=Partite!$H77),Config!$D$6,IF(AND($L77&lt;&gt;"",$L77=Partite!$I77),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G77" s="27">
+        <f>IF(Partite!$K77&lt;&gt;"Giocata","",IF(AND(Pronostici!$O77&lt;&gt;"",Pronostici!$P77&lt;&gt;"",Pronostici!$O77=Partite!$G77,Pronostici!$P77=Partite!$H77),Config!$D$6,IF(AND($M77&lt;&gt;"",$M77=Partite!$I77),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H77" s="27">
+        <f>IF(Partite!$K77&lt;&gt;"Giocata","",IF(AND(Pronostici!$R77&lt;&gt;"",Pronostici!$S77&lt;&gt;"",Pronostici!$R77=Partite!$G77,Pronostici!$S77=Partite!$H77),Config!$D$6,IF(AND($N77&lt;&gt;"",$N77=Partite!$I77),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J77" s="63">
+        <f>IF(Pronostici!$E77&lt;&gt;"",UPPER(Pronostici!$E77),IF(OR(Pronostici!$F77="",Pronostici!$G77=""),"",IF(Pronostici!$F77&gt;Pronostici!$G77,"1",IF(Pronostici!$F77=Pronostici!$G77,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K77" s="63">
+        <f>IF(Pronostici!$H77&lt;&gt;"",UPPER(Pronostici!$H77),IF(OR(Pronostici!$I77="",Pronostici!$J77=""),"",IF(Pronostici!$I77&gt;Pronostici!$J77,"1",IF(Pronostici!$I77=Pronostici!$J77,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L77" s="63">
+        <f>IF(Pronostici!$K77&lt;&gt;"",UPPER(Pronostici!$K77),IF(OR(Pronostici!$L77="",Pronostici!$M77=""),"",IF(Pronostici!$L77&gt;Pronostici!$M77,"1",IF(Pronostici!$L77=Pronostici!$M77,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M77" s="63">
+        <f>IF(Pronostici!$N77&lt;&gt;"",UPPER(Pronostici!$N77),IF(OR(Pronostici!$O77="",Pronostici!$P77=""),"",IF(Pronostici!$O77&gt;Pronostici!$P77,"1",IF(Pronostici!$O77=Pronostici!$P77,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N77" s="63">
+        <f>IF(Pronostici!$Q77&lt;&gt;"",UPPER(Pronostici!$Q77),IF(OR(Pronostici!$R77="",Pronostici!$S77=""),"",IF(Pronostici!$R77&gt;Pronostici!$S77,"1",IF(Pronostici!$R77=Pronostici!$S77,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="74">
+        <f>Partite!$A78</f>
+        <v/>
+      </c>
+      <c r="B78" s="30">
+        <f>Partite!$B78</f>
+        <v/>
+      </c>
+      <c r="C78" s="47">
+        <f>IF(Partite!$E78="","",Partite!$E78&amp;"  -  "&amp;Partite!$F78)</f>
+        <v/>
+      </c>
+      <c r="D78" s="27">
+        <f>IF(Partite!$K78&lt;&gt;"Giocata","",IF(AND(Pronostici!$F78&lt;&gt;"",Pronostici!$G78&lt;&gt;"",Pronostici!$F78=Partite!$G78,Pronostici!$G78=Partite!$H78),Config!$D$6,IF(AND($J78&lt;&gt;"",$J78=Partite!$I78),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E78" s="27">
+        <f>IF(Partite!$K78&lt;&gt;"Giocata","",IF(AND(Pronostici!$I78&lt;&gt;"",Pronostici!$J78&lt;&gt;"",Pronostici!$I78=Partite!$G78,Pronostici!$J78=Partite!$H78),Config!$D$6,IF(AND($K78&lt;&gt;"",$K78=Partite!$I78),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F78" s="27">
+        <f>IF(Partite!$K78&lt;&gt;"Giocata","",IF(AND(Pronostici!$L78&lt;&gt;"",Pronostici!$M78&lt;&gt;"",Pronostici!$L78=Partite!$G78,Pronostici!$M78=Partite!$H78),Config!$D$6,IF(AND($L78&lt;&gt;"",$L78=Partite!$I78),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G78" s="27">
+        <f>IF(Partite!$K78&lt;&gt;"Giocata","",IF(AND(Pronostici!$O78&lt;&gt;"",Pronostici!$P78&lt;&gt;"",Pronostici!$O78=Partite!$G78,Pronostici!$P78=Partite!$H78),Config!$D$6,IF(AND($M78&lt;&gt;"",$M78=Partite!$I78),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H78" s="27">
+        <f>IF(Partite!$K78&lt;&gt;"Giocata","",IF(AND(Pronostici!$R78&lt;&gt;"",Pronostici!$S78&lt;&gt;"",Pronostici!$R78=Partite!$G78,Pronostici!$S78=Partite!$H78),Config!$D$6,IF(AND($N78&lt;&gt;"",$N78=Partite!$I78),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J78" s="63">
+        <f>IF(Pronostici!$E78&lt;&gt;"",UPPER(Pronostici!$E78),IF(OR(Pronostici!$F78="",Pronostici!$G78=""),"",IF(Pronostici!$F78&gt;Pronostici!$G78,"1",IF(Pronostici!$F78=Pronostici!$G78,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K78" s="63">
+        <f>IF(Pronostici!$H78&lt;&gt;"",UPPER(Pronostici!$H78),IF(OR(Pronostici!$I78="",Pronostici!$J78=""),"",IF(Pronostici!$I78&gt;Pronostici!$J78,"1",IF(Pronostici!$I78=Pronostici!$J78,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L78" s="63">
+        <f>IF(Pronostici!$K78&lt;&gt;"",UPPER(Pronostici!$K78),IF(OR(Pronostici!$L78="",Pronostici!$M78=""),"",IF(Pronostici!$L78&gt;Pronostici!$M78,"1",IF(Pronostici!$L78=Pronostici!$M78,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M78" s="63">
+        <f>IF(Pronostici!$N78&lt;&gt;"",UPPER(Pronostici!$N78),IF(OR(Pronostici!$O78="",Pronostici!$P78=""),"",IF(Pronostici!$O78&gt;Pronostici!$P78,"1",IF(Pronostici!$O78=Pronostici!$P78,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N78" s="63">
+        <f>IF(Pronostici!$Q78&lt;&gt;"",UPPER(Pronostici!$Q78),IF(OR(Pronostici!$R78="",Pronostici!$S78=""),"",IF(Pronostici!$R78&gt;Pronostici!$S78,"1",IF(Pronostici!$R78=Pronostici!$S78,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="74">
+        <f>Partite!$A79</f>
+        <v/>
+      </c>
+      <c r="B79" s="30">
+        <f>Partite!$B79</f>
+        <v/>
+      </c>
+      <c r="C79" s="47">
+        <f>IF(Partite!$E79="","",Partite!$E79&amp;"  -  "&amp;Partite!$F79)</f>
+        <v/>
+      </c>
+      <c r="D79" s="27">
+        <f>IF(Partite!$K79&lt;&gt;"Giocata","",IF(AND(Pronostici!$F79&lt;&gt;"",Pronostici!$G79&lt;&gt;"",Pronostici!$F79=Partite!$G79,Pronostici!$G79=Partite!$H79),Config!$D$6,IF(AND($J79&lt;&gt;"",$J79=Partite!$I79),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E79" s="27">
+        <f>IF(Partite!$K79&lt;&gt;"Giocata","",IF(AND(Pronostici!$I79&lt;&gt;"",Pronostici!$J79&lt;&gt;"",Pronostici!$I79=Partite!$G79,Pronostici!$J79=Partite!$H79),Config!$D$6,IF(AND($K79&lt;&gt;"",$K79=Partite!$I79),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F79" s="27">
+        <f>IF(Partite!$K79&lt;&gt;"Giocata","",IF(AND(Pronostici!$L79&lt;&gt;"",Pronostici!$M79&lt;&gt;"",Pronostici!$L79=Partite!$G79,Pronostici!$M79=Partite!$H79),Config!$D$6,IF(AND($L79&lt;&gt;"",$L79=Partite!$I79),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G79" s="27">
+        <f>IF(Partite!$K79&lt;&gt;"Giocata","",IF(AND(Pronostici!$O79&lt;&gt;"",Pronostici!$P79&lt;&gt;"",Pronostici!$O79=Partite!$G79,Pronostici!$P79=Partite!$H79),Config!$D$6,IF(AND($M79&lt;&gt;"",$M79=Partite!$I79),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H79" s="27">
+        <f>IF(Partite!$K79&lt;&gt;"Giocata","",IF(AND(Pronostici!$R79&lt;&gt;"",Pronostici!$S79&lt;&gt;"",Pronostici!$R79=Partite!$G79,Pronostici!$S79=Partite!$H79),Config!$D$6,IF(AND($N79&lt;&gt;"",$N79=Partite!$I79),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J79" s="63">
+        <f>IF(Pronostici!$E79&lt;&gt;"",UPPER(Pronostici!$E79),IF(OR(Pronostici!$F79="",Pronostici!$G79=""),"",IF(Pronostici!$F79&gt;Pronostici!$G79,"1",IF(Pronostici!$F79=Pronostici!$G79,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K79" s="63">
+        <f>IF(Pronostici!$H79&lt;&gt;"",UPPER(Pronostici!$H79),IF(OR(Pronostici!$I79="",Pronostici!$J79=""),"",IF(Pronostici!$I79&gt;Pronostici!$J79,"1",IF(Pronostici!$I79=Pronostici!$J79,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L79" s="63">
+        <f>IF(Pronostici!$K79&lt;&gt;"",UPPER(Pronostici!$K79),IF(OR(Pronostici!$L79="",Pronostici!$M79=""),"",IF(Pronostici!$L79&gt;Pronostici!$M79,"1",IF(Pronostici!$L79=Pronostici!$M79,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M79" s="63">
+        <f>IF(Pronostici!$N79&lt;&gt;"",UPPER(Pronostici!$N79),IF(OR(Pronostici!$O79="",Pronostici!$P79=""),"",IF(Pronostici!$O79&gt;Pronostici!$P79,"1",IF(Pronostici!$O79=Pronostici!$P79,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N79" s="63">
+        <f>IF(Pronostici!$Q79&lt;&gt;"",UPPER(Pronostici!$Q79),IF(OR(Pronostici!$R79="",Pronostici!$S79=""),"",IF(Pronostici!$R79&gt;Pronostici!$S79,"1",IF(Pronostici!$R79=Pronostici!$S79,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="74">
+        <f>Partite!$A80</f>
+        <v/>
+      </c>
+      <c r="B80" s="30">
+        <f>Partite!$B80</f>
+        <v/>
+      </c>
+      <c r="C80" s="47">
+        <f>IF(Partite!$E80="","",Partite!$E80&amp;"  -  "&amp;Partite!$F80)</f>
+        <v/>
+      </c>
+      <c r="D80" s="27">
+        <f>IF(Partite!$K80&lt;&gt;"Giocata","",IF(AND(Pronostici!$F80&lt;&gt;"",Pronostici!$G80&lt;&gt;"",Pronostici!$F80=Partite!$G80,Pronostici!$G80=Partite!$H80),Config!$D$6,IF(AND($J80&lt;&gt;"",$J80=Partite!$I80),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E80" s="27">
+        <f>IF(Partite!$K80&lt;&gt;"Giocata","",IF(AND(Pronostici!$I80&lt;&gt;"",Pronostici!$J80&lt;&gt;"",Pronostici!$I80=Partite!$G80,Pronostici!$J80=Partite!$H80),Config!$D$6,IF(AND($K80&lt;&gt;"",$K80=Partite!$I80),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F80" s="27">
+        <f>IF(Partite!$K80&lt;&gt;"Giocata","",IF(AND(Pronostici!$L80&lt;&gt;"",Pronostici!$M80&lt;&gt;"",Pronostici!$L80=Partite!$G80,Pronostici!$M80=Partite!$H80),Config!$D$6,IF(AND($L80&lt;&gt;"",$L80=Partite!$I80),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G80" s="27">
+        <f>IF(Partite!$K80&lt;&gt;"Giocata","",IF(AND(Pronostici!$O80&lt;&gt;"",Pronostici!$P80&lt;&gt;"",Pronostici!$O80=Partite!$G80,Pronostici!$P80=Partite!$H80),Config!$D$6,IF(AND($M80&lt;&gt;"",$M80=Partite!$I80),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H80" s="27">
+        <f>IF(Partite!$K80&lt;&gt;"Giocata","",IF(AND(Pronostici!$R80&lt;&gt;"",Pronostici!$S80&lt;&gt;"",Pronostici!$R80=Partite!$G80,Pronostici!$S80=Partite!$H80),Config!$D$6,IF(AND($N80&lt;&gt;"",$N80=Partite!$I80),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J80" s="63">
+        <f>IF(Pronostici!$E80&lt;&gt;"",UPPER(Pronostici!$E80),IF(OR(Pronostici!$F80="",Pronostici!$G80=""),"",IF(Pronostici!$F80&gt;Pronostici!$G80,"1",IF(Pronostici!$F80=Pronostici!$G80,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K80" s="63">
+        <f>IF(Pronostici!$H80&lt;&gt;"",UPPER(Pronostici!$H80),IF(OR(Pronostici!$I80="",Pronostici!$J80=""),"",IF(Pronostici!$I80&gt;Pronostici!$J80,"1",IF(Pronostici!$I80=Pronostici!$J80,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L80" s="63">
+        <f>IF(Pronostici!$K80&lt;&gt;"",UPPER(Pronostici!$K80),IF(OR(Pronostici!$L80="",Pronostici!$M80=""),"",IF(Pronostici!$L80&gt;Pronostici!$M80,"1",IF(Pronostici!$L80=Pronostici!$M80,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M80" s="63">
+        <f>IF(Pronostici!$N80&lt;&gt;"",UPPER(Pronostici!$N80),IF(OR(Pronostici!$O80="",Pronostici!$P80=""),"",IF(Pronostici!$O80&gt;Pronostici!$P80,"1",IF(Pronostici!$O80=Pronostici!$P80,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N80" s="63">
+        <f>IF(Pronostici!$Q80&lt;&gt;"",UPPER(Pronostici!$Q80),IF(OR(Pronostici!$R80="",Pronostici!$S80=""),"",IF(Pronostici!$R80&gt;Pronostici!$S80,"1",IF(Pronostici!$R80=Pronostici!$S80,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="74">
+        <f>Partite!$A81</f>
+        <v/>
+      </c>
+      <c r="B81" s="30">
+        <f>Partite!$B81</f>
+        <v/>
+      </c>
+      <c r="C81" s="47">
+        <f>IF(Partite!$E81="","",Partite!$E81&amp;"  -  "&amp;Partite!$F81)</f>
+        <v/>
+      </c>
+      <c r="D81" s="27">
+        <f>IF(Partite!$K81&lt;&gt;"Giocata","",IF(AND(Pronostici!$F81&lt;&gt;"",Pronostici!$G81&lt;&gt;"",Pronostici!$F81=Partite!$G81,Pronostici!$G81=Partite!$H81),Config!$D$6,IF(AND($J81&lt;&gt;"",$J81=Partite!$I81),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E81" s="27">
+        <f>IF(Partite!$K81&lt;&gt;"Giocata","",IF(AND(Pronostici!$I81&lt;&gt;"",Pronostici!$J81&lt;&gt;"",Pronostici!$I81=Partite!$G81,Pronostici!$J81=Partite!$H81),Config!$D$6,IF(AND($K81&lt;&gt;"",$K81=Partite!$I81),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F81" s="27">
+        <f>IF(Partite!$K81&lt;&gt;"Giocata","",IF(AND(Pronostici!$L81&lt;&gt;"",Pronostici!$M81&lt;&gt;"",Pronostici!$L81=Partite!$G81,Pronostici!$M81=Partite!$H81),Config!$D$6,IF(AND($L81&lt;&gt;"",$L81=Partite!$I81),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G81" s="27">
+        <f>IF(Partite!$K81&lt;&gt;"Giocata","",IF(AND(Pronostici!$O81&lt;&gt;"",Pronostici!$P81&lt;&gt;"",Pronostici!$O81=Partite!$G81,Pronostici!$P81=Partite!$H81),Config!$D$6,IF(AND($M81&lt;&gt;"",$M81=Partite!$I81),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H81" s="27">
+        <f>IF(Partite!$K81&lt;&gt;"Giocata","",IF(AND(Pronostici!$R81&lt;&gt;"",Pronostici!$S81&lt;&gt;"",Pronostici!$R81=Partite!$G81,Pronostici!$S81=Partite!$H81),Config!$D$6,IF(AND($N81&lt;&gt;"",$N81=Partite!$I81),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J81" s="63">
+        <f>IF(Pronostici!$E81&lt;&gt;"",UPPER(Pronostici!$E81),IF(OR(Pronostici!$F81="",Pronostici!$G81=""),"",IF(Pronostici!$F81&gt;Pronostici!$G81,"1",IF(Pronostici!$F81=Pronostici!$G81,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K81" s="63">
+        <f>IF(Pronostici!$H81&lt;&gt;"",UPPER(Pronostici!$H81),IF(OR(Pronostici!$I81="",Pronostici!$J81=""),"",IF(Pronostici!$I81&gt;Pronostici!$J81,"1",IF(Pronostici!$I81=Pronostici!$J81,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L81" s="63">
+        <f>IF(Pronostici!$K81&lt;&gt;"",UPPER(Pronostici!$K81),IF(OR(Pronostici!$L81="",Pronostici!$M81=""),"",IF(Pronostici!$L81&gt;Pronostici!$M81,"1",IF(Pronostici!$L81=Pronostici!$M81,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M81" s="63">
+        <f>IF(Pronostici!$N81&lt;&gt;"",UPPER(Pronostici!$N81),IF(OR(Pronostici!$O81="",Pronostici!$P81=""),"",IF(Pronostici!$O81&gt;Pronostici!$P81,"1",IF(Pronostici!$O81=Pronostici!$P81,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N81" s="63">
+        <f>IF(Pronostici!$Q81&lt;&gt;"",UPPER(Pronostici!$Q81),IF(OR(Pronostici!$R81="",Pronostici!$S81=""),"",IF(Pronostici!$R81&gt;Pronostici!$S81,"1",IF(Pronostici!$R81=Pronostici!$S81,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="74">
+        <f>Partite!$A82</f>
+        <v/>
+      </c>
+      <c r="B82" s="30">
+        <f>Partite!$B82</f>
+        <v/>
+      </c>
+      <c r="C82" s="47">
+        <f>IF(Partite!$E82="","",Partite!$E82&amp;"  -  "&amp;Partite!$F82)</f>
+        <v/>
+      </c>
+      <c r="D82" s="27">
+        <f>IF(Partite!$K82&lt;&gt;"Giocata","",IF(AND(Pronostici!$F82&lt;&gt;"",Pronostici!$G82&lt;&gt;"",Pronostici!$F82=Partite!$G82,Pronostici!$G82=Partite!$H82),Config!$D$6,IF(AND($J82&lt;&gt;"",$J82=Partite!$I82),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E82" s="27">
+        <f>IF(Partite!$K82&lt;&gt;"Giocata","",IF(AND(Pronostici!$I82&lt;&gt;"",Pronostici!$J82&lt;&gt;"",Pronostici!$I82=Partite!$G82,Pronostici!$J82=Partite!$H82),Config!$D$6,IF(AND($K82&lt;&gt;"",$K82=Partite!$I82),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F82" s="27">
+        <f>IF(Partite!$K82&lt;&gt;"Giocata","",IF(AND(Pronostici!$L82&lt;&gt;"",Pronostici!$M82&lt;&gt;"",Pronostici!$L82=Partite!$G82,Pronostici!$M82=Partite!$H82),Config!$D$6,IF(AND($L82&lt;&gt;"",$L82=Partite!$I82),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G82" s="27">
+        <f>IF(Partite!$K82&lt;&gt;"Giocata","",IF(AND(Pronostici!$O82&lt;&gt;"",Pronostici!$P82&lt;&gt;"",Pronostici!$O82=Partite!$G82,Pronostici!$P82=Partite!$H82),Config!$D$6,IF(AND($M82&lt;&gt;"",$M82=Partite!$I82),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H82" s="27">
+        <f>IF(Partite!$K82&lt;&gt;"Giocata","",IF(AND(Pronostici!$R82&lt;&gt;"",Pronostici!$S82&lt;&gt;"",Pronostici!$R82=Partite!$G82,Pronostici!$S82=Partite!$H82),Config!$D$6,IF(AND($N82&lt;&gt;"",$N82=Partite!$I82),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J82" s="63">
+        <f>IF(Pronostici!$E82&lt;&gt;"",UPPER(Pronostici!$E82),IF(OR(Pronostici!$F82="",Pronostici!$G82=""),"",IF(Pronostici!$F82&gt;Pronostici!$G82,"1",IF(Pronostici!$F82=Pronostici!$G82,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K82" s="63">
+        <f>IF(Pronostici!$H82&lt;&gt;"",UPPER(Pronostici!$H82),IF(OR(Pronostici!$I82="",Pronostici!$J82=""),"",IF(Pronostici!$I82&gt;Pronostici!$J82,"1",IF(Pronostici!$I82=Pronostici!$J82,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L82" s="63">
+        <f>IF(Pronostici!$K82&lt;&gt;"",UPPER(Pronostici!$K82),IF(OR(Pronostici!$L82="",Pronostici!$M82=""),"",IF(Pronostici!$L82&gt;Pronostici!$M82,"1",IF(Pronostici!$L82=Pronostici!$M82,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M82" s="63">
+        <f>IF(Pronostici!$N82&lt;&gt;"",UPPER(Pronostici!$N82),IF(OR(Pronostici!$O82="",Pronostici!$P82=""),"",IF(Pronostici!$O82&gt;Pronostici!$P82,"1",IF(Pronostici!$O82=Pronostici!$P82,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N82" s="63">
+        <f>IF(Pronostici!$Q82&lt;&gt;"",UPPER(Pronostici!$Q82),IF(OR(Pronostici!$R82="",Pronostici!$S82=""),"",IF(Pronostici!$R82&gt;Pronostici!$S82,"1",IF(Pronostici!$R82=Pronostici!$S82,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D72">
+  <conditionalFormatting sqref="D3:D82">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -14749,7 +16120,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E72">
+  <conditionalFormatting sqref="E3:E82">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -14757,7 +16128,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F72">
+  <conditionalFormatting sqref="F3:F82">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -14765,7 +16136,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G72">
+  <conditionalFormatting sqref="G3:G82">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -14773,7 +16144,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H72">
+  <conditionalFormatting sqref="H3:H82">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento automatico del 23/10/2026 alle 20:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -11025,21 +11025,61 @@
         <f>IF(Partite!$F63="","",Partite!$F63)</f>
         <v/>
       </c>
-      <c r="E63" s="71" t="n"/>
-      <c r="F63" s="71" t="n"/>
-      <c r="G63" s="71" t="n"/>
-      <c r="H63" s="71" t="n"/>
-      <c r="I63" s="71" t="n"/>
-      <c r="J63" s="71" t="n"/>
-      <c r="K63" s="71" t="n"/>
-      <c r="L63" s="71" t="n"/>
-      <c r="M63" s="71" t="n"/>
-      <c r="N63" s="71" t="n"/>
-      <c r="O63" s="71" t="n"/>
-      <c r="P63" s="71" t="n"/>
-      <c r="Q63" s="71" t="n"/>
-      <c r="R63" s="71" t="n"/>
-      <c r="S63" s="71" t="n"/>
+      <c r="E63" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F63" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G63" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I63" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J63" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L63" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M63" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N63" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O63" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P63" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q63" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R63" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S63" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="69">
@@ -11058,21 +11098,61 @@
         <f>IF(Partite!$F64="","",Partite!$F64)</f>
         <v/>
       </c>
-      <c r="E64" s="71" t="n"/>
-      <c r="F64" s="71" t="n"/>
-      <c r="G64" s="71" t="n"/>
-      <c r="H64" s="71" t="n"/>
-      <c r="I64" s="71" t="n"/>
-      <c r="J64" s="71" t="n"/>
-      <c r="K64" s="71" t="n"/>
-      <c r="L64" s="71" t="n"/>
-      <c r="M64" s="71" t="n"/>
-      <c r="N64" s="71" t="n"/>
-      <c r="O64" s="71" t="n"/>
-      <c r="P64" s="71" t="n"/>
-      <c r="Q64" s="71" t="n"/>
-      <c r="R64" s="71" t="n"/>
-      <c r="S64" s="71" t="n"/>
+      <c r="E64" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F64" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I64" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L64" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M64" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N64" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O64" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P64" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q64" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R64" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="69">
@@ -11091,21 +11171,61 @@
         <f>IF(Partite!$F65="","",Partite!$F65)</f>
         <v/>
       </c>
-      <c r="E65" s="71" t="n"/>
-      <c r="F65" s="71" t="n"/>
-      <c r="G65" s="71" t="n"/>
-      <c r="H65" s="71" t="n"/>
-      <c r="I65" s="71" t="n"/>
-      <c r="J65" s="71" t="n"/>
-      <c r="K65" s="71" t="n"/>
-      <c r="L65" s="71" t="n"/>
-      <c r="M65" s="71" t="n"/>
-      <c r="N65" s="71" t="n"/>
-      <c r="O65" s="71" t="n"/>
-      <c r="P65" s="71" t="n"/>
-      <c r="Q65" s="71" t="n"/>
-      <c r="R65" s="71" t="n"/>
-      <c r="S65" s="71" t="n"/>
+      <c r="E65" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F65" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G65" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I65" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J65" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L65" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M65" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N65" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O65" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P65" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q65" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R65" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="S65" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="69">
@@ -11124,21 +11244,61 @@
         <f>IF(Partite!$F66="","",Partite!$F66)</f>
         <v/>
       </c>
-      <c r="E66" s="71" t="n"/>
-      <c r="F66" s="71" t="n"/>
-      <c r="G66" s="71" t="n"/>
-      <c r="H66" s="71" t="n"/>
-      <c r="I66" s="71" t="n"/>
-      <c r="J66" s="71" t="n"/>
-      <c r="K66" s="71" t="n"/>
-      <c r="L66" s="71" t="n"/>
-      <c r="M66" s="71" t="n"/>
-      <c r="N66" s="71" t="n"/>
-      <c r="O66" s="71" t="n"/>
-      <c r="P66" s="71" t="n"/>
-      <c r="Q66" s="71" t="n"/>
-      <c r="R66" s="71" t="n"/>
-      <c r="S66" s="71" t="n"/>
+      <c r="E66" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F66" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G66" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I66" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L66" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M66" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N66" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O66" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P66" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q66" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R66" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S66" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="69">
@@ -11157,21 +11317,61 @@
         <f>IF(Partite!$F67="","",Partite!$F67)</f>
         <v/>
       </c>
-      <c r="E67" s="71" t="n"/>
-      <c r="F67" s="71" t="n"/>
-      <c r="G67" s="71" t="n"/>
-      <c r="H67" s="71" t="n"/>
-      <c r="I67" s="71" t="n"/>
-      <c r="J67" s="71" t="n"/>
-      <c r="K67" s="71" t="n"/>
-      <c r="L67" s="71" t="n"/>
-      <c r="M67" s="71" t="n"/>
-      <c r="N67" s="71" t="n"/>
-      <c r="O67" s="71" t="n"/>
-      <c r="P67" s="71" t="n"/>
-      <c r="Q67" s="71" t="n"/>
-      <c r="R67" s="71" t="n"/>
-      <c r="S67" s="71" t="n"/>
+      <c r="E67" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F67" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I67" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J67" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L67" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M67" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N67" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O67" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P67" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R67" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S67" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="69">
@@ -11190,21 +11390,61 @@
         <f>IF(Partite!$F68="","",Partite!$F68)</f>
         <v/>
       </c>
-      <c r="E68" s="71" t="n"/>
-      <c r="F68" s="71" t="n"/>
-      <c r="G68" s="71" t="n"/>
-      <c r="H68" s="71" t="n"/>
-      <c r="I68" s="71" t="n"/>
-      <c r="J68" s="71" t="n"/>
-      <c r="K68" s="71" t="n"/>
-      <c r="L68" s="71" t="n"/>
-      <c r="M68" s="71" t="n"/>
-      <c r="N68" s="71" t="n"/>
-      <c r="O68" s="71" t="n"/>
-      <c r="P68" s="71" t="n"/>
-      <c r="Q68" s="71" t="n"/>
-      <c r="R68" s="71" t="n"/>
-      <c r="S68" s="71" t="n"/>
+      <c r="E68" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F68" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G68" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I68" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J68" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L68" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M68" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O68" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P68" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R68" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S68" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="69">
@@ -11223,21 +11463,61 @@
         <f>IF(Partite!$F69="","",Partite!$F69)</f>
         <v/>
       </c>
-      <c r="E69" s="71" t="n"/>
-      <c r="F69" s="71" t="n"/>
-      <c r="G69" s="71" t="n"/>
-      <c r="H69" s="71" t="n"/>
-      <c r="I69" s="71" t="n"/>
-      <c r="J69" s="71" t="n"/>
-      <c r="K69" s="71" t="n"/>
-      <c r="L69" s="71" t="n"/>
-      <c r="M69" s="71" t="n"/>
-      <c r="N69" s="71" t="n"/>
-      <c r="O69" s="71" t="n"/>
-      <c r="P69" s="71" t="n"/>
-      <c r="Q69" s="71" t="n"/>
-      <c r="R69" s="71" t="n"/>
-      <c r="S69" s="71" t="n"/>
+      <c r="E69" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F69" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I69" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K69" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M69" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N69" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q69" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R69" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S69" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="69">
@@ -11256,21 +11536,61 @@
         <f>IF(Partite!$F70="","",Partite!$F70)</f>
         <v/>
       </c>
-      <c r="E70" s="71" t="n"/>
-      <c r="F70" s="71" t="n"/>
-      <c r="G70" s="71" t="n"/>
-      <c r="H70" s="71" t="n"/>
-      <c r="I70" s="71" t="n"/>
-      <c r="J70" s="71" t="n"/>
-      <c r="K70" s="71" t="n"/>
-      <c r="L70" s="71" t="n"/>
-      <c r="M70" s="71" t="n"/>
-      <c r="N70" s="71" t="n"/>
-      <c r="O70" s="71" t="n"/>
-      <c r="P70" s="71" t="n"/>
-      <c r="Q70" s="71" t="n"/>
-      <c r="R70" s="71" t="n"/>
-      <c r="S70" s="71" t="n"/>
+      <c r="E70" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K70" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L70" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M70" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S70" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="69">
@@ -11289,21 +11609,61 @@
         <f>IF(Partite!$F71="","",Partite!$F71)</f>
         <v/>
       </c>
-      <c r="E71" s="71" t="n"/>
-      <c r="F71" s="71" t="n"/>
-      <c r="G71" s="71" t="n"/>
-      <c r="H71" s="71" t="n"/>
-      <c r="I71" s="71" t="n"/>
-      <c r="J71" s="71" t="n"/>
-      <c r="K71" s="71" t="n"/>
-      <c r="L71" s="71" t="n"/>
-      <c r="M71" s="71" t="n"/>
-      <c r="N71" s="71" t="n"/>
-      <c r="O71" s="71" t="n"/>
-      <c r="P71" s="71" t="n"/>
-      <c r="Q71" s="71" t="n"/>
-      <c r="R71" s="71" t="n"/>
-      <c r="S71" s="71" t="n"/>
+      <c r="E71" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H71" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K71" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N71" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q71" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="69">
@@ -11322,21 +11682,61 @@
         <f>IF(Partite!$F72="","",Partite!$F72)</f>
         <v/>
       </c>
-      <c r="E72" s="71" t="n"/>
-      <c r="F72" s="71" t="n"/>
-      <c r="G72" s="71" t="n"/>
-      <c r="H72" s="71" t="n"/>
-      <c r="I72" s="71" t="n"/>
-      <c r="J72" s="71" t="n"/>
-      <c r="K72" s="71" t="n"/>
-      <c r="L72" s="71" t="n"/>
-      <c r="M72" s="71" t="n"/>
-      <c r="N72" s="71" t="n"/>
-      <c r="O72" s="71" t="n"/>
-      <c r="P72" s="71" t="n"/>
-      <c r="Q72" s="71" t="n"/>
-      <c r="R72" s="71" t="n"/>
-      <c r="S72" s="71" t="n"/>
+      <c r="E72" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F72" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I72" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J72" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L72" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N72" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O72" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q72" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R72" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S72" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="74">

</xml_diff>

<commit_message>
Aggiornamento automatico del 23/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5593,8 +5593,12 @@
           <t>Monza</t>
         </is>
       </c>
-      <c r="G63" s="71" t="n"/>
-      <c r="H63" s="71" t="n"/>
+      <c r="G63" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H63" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I63" s="72">
         <f>IF(OR($G63="",$H63=""),"",IF($G63&gt;$H63,"1",IF($G63=$H63,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 24/10/2026 alle 17:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5641,8 +5641,12 @@
           <t>Bologna</t>
         </is>
       </c>
-      <c r="G64" s="71" t="n"/>
-      <c r="H64" s="71" t="n"/>
+      <c r="G64" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I64" s="72">
         <f>IF(OR($G64="",$H64=""),"",IF($G64&gt;$H64,"1",IF($G64=$H64,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 24/10/2026 alle 20:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5689,8 +5689,12 @@
           <t>Sassuolo</t>
         </is>
       </c>
-      <c r="G65" s="71" t="n"/>
-      <c r="H65" s="71" t="n"/>
+      <c r="G65" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I65" s="72">
         <f>IF(OR($G65="",$H65=""),"",IF($G65&gt;$H65,"1",IF($G65=$H65,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 24/10/2026 alle 23:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5781,8 +5781,12 @@
           <t>Parma</t>
         </is>
       </c>
-      <c r="G67" s="71" t="n"/>
-      <c r="H67" s="71" t="n"/>
+      <c r="G67" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H67" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I67" s="72">
         <f>IF(OR($G67="",$H67=""),"",IF($G67&gt;$H67,"1",IF($G67=$H67,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 25/10/2026 alle 09:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5737,8 +5737,12 @@
           <t>Roma</t>
         </is>
       </c>
-      <c r="G66" s="71" t="n"/>
-      <c r="H66" s="71" t="n"/>
+      <c r="G66" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H66" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I66" s="72">
         <f>IF(OR($G66="",$H66=""),"",IF($G66&gt;$H66,"1",IF($G66=$H66,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 25/10/2026 alle 14:39
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5833,8 +5833,12 @@
           <t>Fiorentina</t>
         </is>
       </c>
-      <c r="G68" s="71" t="n"/>
-      <c r="H68" s="71" t="n"/>
+      <c r="G68" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I68" s="72">
         <f>IF(OR($G68="",$H68=""),"",IF($G68&gt;$H68,"1",IF($G68=$H68,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 25/10/2026 alle 17:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5881,8 +5881,12 @@
           <t>Frosinone</t>
         </is>
       </c>
-      <c r="G69" s="71" t="n"/>
-      <c r="H69" s="71" t="n"/>
+      <c r="G69" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H69" s="71" t="n">
+        <v>4</v>
+      </c>
       <c r="I69" s="72">
         <f>IF(OR($G69="",$H69=""),"",IF($G69&gt;$H69,"1",IF($G69=$H69,"X","2")))</f>
         <v/>
@@ -5925,8 +5929,12 @@
           <t>Venezia</t>
         </is>
       </c>
-      <c r="G70" s="71" t="n"/>
-      <c r="H70" s="71" t="n"/>
+      <c r="G70" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I70" s="72">
         <f>IF(OR($G70="",$H70=""),"",IF($G70&gt;$H70,"1",IF($G70=$H70,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 25/10/2026 alle 20:09
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -5977,8 +5977,12 @@
           <t>Juventus</t>
         </is>
       </c>
-      <c r="G71" s="71" t="n"/>
-      <c r="H71" s="71" t="n"/>
+      <c r="G71" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I71" s="72">
         <f>IF(OR($G71="",$H71=""),"",IF($G71&gt;$H71,"1",IF($G71=$H71,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 25/10/2026 alle 22:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$82</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$40</f>
+              <f>'Classifica'!$A$33:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$R$33:$R$40</f>
+              <f>'Classifica'!$R$33:$R$41</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -851,12 +851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$40</f>
+              <f>'Classifica'!$A$33:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$S$33:$S$40</f>
+              <f>'Classifica'!$S$33:$S$41</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -888,12 +888,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$40</f>
+              <f>'Classifica'!$A$33:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$T$33:$T$40</f>
+              <f>'Classifica'!$T$33:$T$41</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -925,12 +925,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$40</f>
+              <f>'Classifica'!$A$33:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$U$33:$U$40</f>
+              <f>'Classifica'!$U$33:$U$41</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -962,12 +962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$40</f>
+              <f>'Classifica'!$A$33:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$V$33:$V$40</f>
+              <f>'Classifica'!$V$33:$V$41</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1043,7 +1043,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>42</row>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9720000" cy="3420000"/>
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V40"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>COUNTIF($B$33:$B$40,"Completata")</f>
+        <f>COUNTIF($B$33:$B$41,"Completata")</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>COUNTIF($B$33:$B$40,"Completata")+COUNTIF($B$33:$B$40,"In corso")</f>
+        <f>COUNTIF($B$33:$B$41,"Completata")+COUNTIF($B$33:$B$41,"In corso")</f>
         <v/>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L7" s="13">
-        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$40="Completata")*$A$33:$A$40)))</f>
+        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$41="Completata")*$A$33:$A$41)))</f>
         <v/>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="L8" s="13">
-        <f>IF(SUMPRODUCT(MIN(($B$33:$B$40&lt;&gt;"Completata")*$A$33:$A$40+($B$33:$B$40="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$40&lt;&gt;"Completata")*$A$33:$A$40+($B$33:$B$40="Completata")*999)))</f>
+        <f>IF(SUMPRODUCT(MIN(($B$33:$B$41&lt;&gt;"Completata")*$A$33:$A$41+($B$33:$B$41="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$41&lt;&gt;"Completata")*$A$33:$A$41+($B$33:$B$41="Completata")*999)))</f>
         <v/>
       </c>
     </row>
@@ -1591,19 +1591,19 @@
         <v/>
       </c>
       <c r="C12" s="24">
-        <f>SUM(Punti!$D$3:$D$82)</f>
+        <f>SUM(Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$82,Config!$D$7)+COUNTIF(Punti!$D$3:$D$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$92,Config!$D$7)+COUNTIF(Punti!$D$3:$D$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>SUMPRODUCT(((Pronostici!$E$3:$E$82&lt;&gt;"")+(Pronostici!$F$3:$F$82&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$E$3:$E$92&lt;&gt;"")+(Pronostici!$F$3:$F$92&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>SUMPRODUCT(($C$33:$C$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
+        <f>SUMPRODUCT(($C$33:$C$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1625,19 +1625,19 @@
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>SUM(Punti!$E$3:$E$82)</f>
+        <f>SUM(Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$82,Config!$D$7)+COUNTIF(Punti!$E$3:$E$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$92,Config!$D$7)+COUNTIF(Punti!$E$3:$E$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
-        <f>SUMPRODUCT(((Pronostici!$H$3:$H$82&lt;&gt;"")+(Pronostici!$I$3:$I$82&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$H$3:$H$92&lt;&gt;"")+(Pronostici!$I$3:$I$92&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G13" s="31">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="H13" s="30">
-        <f>SUMPRODUCT(($D$33:$D$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
+        <f>SUMPRODUCT(($D$33:$D$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1659,19 @@
         <v/>
       </c>
       <c r="C14" s="24">
-        <f>SUM(Punti!$F$3:$F$82)</f>
+        <f>SUM(Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$82,Config!$D$7)+COUNTIF(Punti!$F$3:$F$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$92,Config!$D$7)+COUNTIF(Punti!$F$3:$F$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>SUMPRODUCT(((Pronostici!$K$3:$K$82&lt;&gt;"")+(Pronostici!$L$3:$L$82&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$K$3:$K$92&lt;&gt;"")+(Pronostici!$L$3:$L$92&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>SUMPRODUCT(($E$33:$E$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
+        <f>SUMPRODUCT(($E$33:$E$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1693,19 +1693,19 @@
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>SUM(Punti!$G$3:$G$82)</f>
+        <f>SUM(Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$82,Config!$D$7)+COUNTIF(Punti!$G$3:$G$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$92,Config!$D$7)+COUNTIF(Punti!$G$3:$G$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
-        <f>SUMPRODUCT(((Pronostici!$N$3:$N$82&lt;&gt;"")+(Pronostici!$O$3:$O$82&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$N$3:$N$92&lt;&gt;"")+(Pronostici!$O$3:$O$92&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G15" s="31">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="H15" s="30">
-        <f>SUMPRODUCT(($F$33:$F$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
+        <f>SUMPRODUCT(($F$33:$F$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1727,19 +1727,19 @@
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>SUM(Punti!$H$3:$H$82)</f>
+        <f>SUM(Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$82,Config!$D$7)+COUNTIF(Punti!$H$3:$H$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$92,Config!$D$7)+COUNTIF(Punti!$H$3:$H$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$82,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$92,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$82&lt;&gt;"")+(Pronostici!$R$3:$R$82&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$92&lt;&gt;"")+(Pronostici!$R$3:$R$92&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>SUMPRODUCT(($G$33:$G$40=$H$33:$H$40)*($H$33:$H$40&gt;0)*($B$33:$B$40="Completata"))</f>
+        <f>SUMPRODUCT(($G$33:$G$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         <v/>
       </c>
       <c r="C20" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
         <v/>
       </c>
       <c r="D20" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E20" s="41" t="n"/>
       <c r="K20" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L20" s="43" t="n"/>
@@ -1826,7 +1826,7 @@
         <v/>
       </c>
       <c r="O20" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$E$3:$E$82&lt;&gt;"")+(Pronostici!$F$3:$F$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$E$3:$E$92&lt;&gt;"")+(Pronostici!$F$3:$F$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1836,16 +1836,16 @@
         <v/>
       </c>
       <c r="C21" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
         <v/>
       </c>
       <c r="D21" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E21" s="41" t="n"/>
       <c r="K21" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L21" s="47" t="n"/>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="O21" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$H$3:$H$82&lt;&gt;"")+(Pronostici!$I$3:$I$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$H$3:$H$92&lt;&gt;"")+(Pronostici!$I$3:$I$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v/>
       </c>
       <c r="C22" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
         <v/>
       </c>
       <c r="D22" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E22" s="41" t="n"/>
       <c r="K22" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L22" s="43" t="n"/>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="O22" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$K$3:$K$82&lt;&gt;"")+(Pronostici!$L$3:$L$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$K$3:$K$92&lt;&gt;"")+(Pronostici!$L$3:$L$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1894,16 +1894,16 @@
         <v/>
       </c>
       <c r="C23" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
         <v/>
       </c>
       <c r="D23" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E23" s="41" t="n"/>
       <c r="K23" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L23" s="47" t="n"/>
@@ -1913,7 +1913,7 @@
         <v/>
       </c>
       <c r="O23" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$N$3:$N$82&lt;&gt;"")+(Pronostici!$O$3:$O$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$N$3:$N$92&lt;&gt;"")+(Pronostici!$O$3:$O$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1923,16 +1923,16 @@
         <v/>
       </c>
       <c r="C24" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$40,MATCH($L$7,$A$33:$A$40,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
         <v/>
       </c>
       <c r="D24" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$40,MATCH($L$7,$A$33:$A$40,0)),0)=IFERROR(INDEX($H$33:$H$40,MATCH($L$7,$A$33:$A$40,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E24" s="41" t="n"/>
       <c r="K24" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L24" s="43" t="n"/>
@@ -1942,13 +1942,13 @@
         <v/>
       </c>
       <c r="O24" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$82=$L$8)*(((Pronostici!$Q$3:$Q$82&lt;&gt;"")+(Pronostici!$R$3:$R$82&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$Q$3:$Q$92&lt;&gt;"")+(Pronostici!$R$3:$R$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L25" s="47" t="n"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="26">
       <c r="K26" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L26" s="43" t="n"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="27">
       <c r="K27" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L27" s="47" t="n"/>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="28">
       <c r="K28" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L28" s="43" t="n"/>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="29">
       <c r="K29" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$82,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$82,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$82,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$92,0)),"-")</f>
         <v/>
       </c>
       <c r="L29" s="47" t="n"/>
@@ -2070,27 +2070,27 @@
         <v>2</v>
       </c>
       <c r="B33" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A33,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A33,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H33" s="61">
@@ -2127,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="B34" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A34,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A34,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H34" s="61">
@@ -2184,27 +2184,27 @@
         <v>4</v>
       </c>
       <c r="B35" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A35,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A35,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H35" s="61">
@@ -2241,27 +2241,27 @@
         <v>5</v>
       </c>
       <c r="B36" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A36,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A36,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H36" s="61">
@@ -2298,27 +2298,27 @@
         <v>6</v>
       </c>
       <c r="B37" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A37,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A37,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H37" s="61">
@@ -2355,27 +2355,27 @@
         <v>7</v>
       </c>
       <c r="B38" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A38,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A38,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H38" s="61">
@@ -2412,27 +2412,27 @@
         <v>8</v>
       </c>
       <c r="B39" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A39,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$82,$A39,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H39" s="61">
@@ -2469,27 +2469,27 @@
         <v>9</v>
       </c>
       <c r="B40" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$E$3:$E$82,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$K$3:$K$82,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$K$3:$K$82,"Giocata")=COUNTIFS(Partite!$B$3:$B$82,$A40,Partite!$E$3:$E$82,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$D$3:$D$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$D$3:$D$92)</f>
         <v/>
       </c>
       <c r="D40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$E$3:$E$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$E$3:$E$92)</f>
         <v/>
       </c>
       <c r="E40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$F$3:$F$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$F$3:$F$92)</f>
         <v/>
       </c>
       <c r="F40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$G$3:$G$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$G$3:$G$92)</f>
         <v/>
       </c>
       <c r="G40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$82,$A40,Punti!$H$3:$H$82)</f>
+        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$H$3:$H$92)</f>
         <v/>
       </c>
       <c r="H40" s="61">
@@ -2518,6 +2518,63 @@
       </c>
       <c r="V40" s="63">
         <f>V39+G40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="B41" s="43">
+        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <v/>
+      </c>
+      <c r="C41" s="25">
+        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$D$3:$D$92)</f>
+        <v/>
+      </c>
+      <c r="D41" s="25">
+        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$E$3:$E$92)</f>
+        <v/>
+      </c>
+      <c r="E41" s="25">
+        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$F$3:$F$92)</f>
+        <v/>
+      </c>
+      <c r="F41" s="25">
+        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$G$3:$G$92)</f>
+        <v/>
+      </c>
+      <c r="G41" s="25">
+        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$H$3:$H$92)</f>
+        <v/>
+      </c>
+      <c r="H41" s="61">
+        <f>MAX($C41:$G41)</f>
+        <v/>
+      </c>
+      <c r="I41" s="62">
+        <f>IF($H41&lt;=0,"-",INDEX($C$32:$G$32,MATCH($H41,$C41:$G41,0))&amp;IF(COUNTIF($C41:$G41,$H41)&gt;1," (a pari)","")&amp;IF($B41="Completata",""," - in corso"))</f>
+        <v/>
+      </c>
+      <c r="R41" s="63">
+        <f>R40+C41</f>
+        <v/>
+      </c>
+      <c r="S41" s="63">
+        <f>S40+D41</f>
+        <v/>
+      </c>
+      <c r="T41" s="63">
+        <f>T40+E41</f>
+        <v/>
+      </c>
+      <c r="U41" s="63">
+        <f>U40+F41</f>
+        <v/>
+      </c>
+      <c r="V41" s="63">
+        <f>V40+G41</f>
         <v/>
       </c>
     </row>
@@ -2564,7 +2621,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:G40">
+  <conditionalFormatting sqref="C33:G41">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2586,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6025,8 +6082,12 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="G72" s="71" t="n"/>
-      <c r="H72" s="71" t="n"/>
+      <c r="G72" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I72" s="72">
         <f>IF(OR($G72="",$H72=""),"",IF($G72&gt;$H72,"1",IF($G72=$H72,"X","2")))</f>
         <v/>
@@ -6480,14 +6541,454 @@
         <v/>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="69" t="inlineStr">
+        <is>
+          <t>G10-01</t>
+        </is>
+      </c>
+      <c r="B83" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C83" s="25" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="D83" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E83" s="70" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="F83" s="70" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="G83" s="71" t="n"/>
+      <c r="H83" s="71" t="n"/>
+      <c r="I83" s="72">
+        <f>IF(OR($G83="",$H83=""),"",IF($G83&gt;$H83,"1",IF($G83=$H83,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J83" s="25">
+        <f>IF(OR($G83="",$H83=""),"",$G83&amp;"-"&amp;$H83)</f>
+        <v/>
+      </c>
+      <c r="K83" s="73">
+        <f>IF($E83="","Calendario da inserire",IF(OR($G83="",$H83=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="69" t="inlineStr">
+        <is>
+          <t>G10-02</t>
+        </is>
+      </c>
+      <c r="B84" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C84" s="25" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="D84" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E84" s="70" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="F84" s="70" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="G84" s="71" t="n"/>
+      <c r="H84" s="71" t="n"/>
+      <c r="I84" s="72">
+        <f>IF(OR($G84="",$H84=""),"",IF($G84&gt;$H84,"1",IF($G84=$H84,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J84" s="25">
+        <f>IF(OR($G84="",$H84=""),"",$G84&amp;"-"&amp;$H84)</f>
+        <v/>
+      </c>
+      <c r="K84" s="73">
+        <f>IF($E84="","Calendario da inserire",IF(OR($G84="",$H84=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="69" t="inlineStr">
+        <is>
+          <t>G10-03</t>
+        </is>
+      </c>
+      <c r="B85" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C85" s="25" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="D85" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E85" s="70" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="F85" s="70" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="G85" s="71" t="n"/>
+      <c r="H85" s="71" t="n"/>
+      <c r="I85" s="72">
+        <f>IF(OR($G85="",$H85=""),"",IF($G85&gt;$H85,"1",IF($G85=$H85,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J85" s="25">
+        <f>IF(OR($G85="",$H85=""),"",$G85&amp;"-"&amp;$H85)</f>
+        <v/>
+      </c>
+      <c r="K85" s="73">
+        <f>IF($E85="","Calendario da inserire",IF(OR($G85="",$H85=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="69" t="inlineStr">
+        <is>
+          <t>G10-04</t>
+        </is>
+      </c>
+      <c r="B86" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C86" s="25" t="inlineStr">
+        <is>
+          <t>01/11/2026</t>
+        </is>
+      </c>
+      <c r="D86" s="25" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E86" s="70" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="F86" s="70" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="G86" s="71" t="n"/>
+      <c r="H86" s="71" t="n"/>
+      <c r="I86" s="72">
+        <f>IF(OR($G86="",$H86=""),"",IF($G86&gt;$H86,"1",IF($G86=$H86,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J86" s="25">
+        <f>IF(OR($G86="",$H86=""),"",$G86&amp;"-"&amp;$H86)</f>
+        <v/>
+      </c>
+      <c r="K86" s="73">
+        <f>IF($E86="","Calendario da inserire",IF(OR($G86="",$H86=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="69" t="inlineStr">
+        <is>
+          <t>G10-05</t>
+        </is>
+      </c>
+      <c r="B87" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t>01/11/2026</t>
+        </is>
+      </c>
+      <c r="D87" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E87" s="70" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="F87" s="70" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="G87" s="71" t="n"/>
+      <c r="H87" s="71" t="n"/>
+      <c r="I87" s="72">
+        <f>IF(OR($G87="",$H87=""),"",IF($G87&gt;$H87,"1",IF($G87=$H87,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J87" s="25">
+        <f>IF(OR($G87="",$H87=""),"",$G87&amp;"-"&amp;$H87)</f>
+        <v/>
+      </c>
+      <c r="K87" s="73">
+        <f>IF($E87="","Calendario da inserire",IF(OR($G87="",$H87=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="69" t="inlineStr">
+        <is>
+          <t>G10-06</t>
+        </is>
+      </c>
+      <c r="B88" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C88" s="25" t="inlineStr">
+        <is>
+          <t>01/11/2026</t>
+        </is>
+      </c>
+      <c r="D88" s="25" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E88" s="70" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="F88" s="70" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="G88" s="71" t="n"/>
+      <c r="H88" s="71" t="n"/>
+      <c r="I88" s="72">
+        <f>IF(OR($G88="",$H88=""),"",IF($G88&gt;$H88,"1",IF($G88=$H88,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J88" s="25">
+        <f>IF(OR($G88="",$H88=""),"",$G88&amp;"-"&amp;$H88)</f>
+        <v/>
+      </c>
+      <c r="K88" s="73">
+        <f>IF($E88="","Calendario da inserire",IF(OR($G88="",$H88=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="69" t="inlineStr">
+        <is>
+          <t>G10-07</t>
+        </is>
+      </c>
+      <c r="B89" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C89" s="25" t="inlineStr">
+        <is>
+          <t>01/11/2026</t>
+        </is>
+      </c>
+      <c r="D89" s="25" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E89" s="70" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="F89" s="70" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="G89" s="71" t="n"/>
+      <c r="H89" s="71" t="n"/>
+      <c r="I89" s="72">
+        <f>IF(OR($G89="",$H89=""),"",IF($G89&gt;$H89,"1",IF($G89=$H89,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J89" s="25">
+        <f>IF(OR($G89="",$H89=""),"",$G89&amp;"-"&amp;$H89)</f>
+        <v/>
+      </c>
+      <c r="K89" s="73">
+        <f>IF($E89="","Calendario da inserire",IF(OR($G89="",$H89=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="69" t="inlineStr">
+        <is>
+          <t>G10-08</t>
+        </is>
+      </c>
+      <c r="B90" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C90" s="25" t="inlineStr">
+        <is>
+          <t>01/11/2026</t>
+        </is>
+      </c>
+      <c r="D90" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E90" s="70" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="F90" s="70" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="G90" s="71" t="n"/>
+      <c r="H90" s="71" t="n"/>
+      <c r="I90" s="72">
+        <f>IF(OR($G90="",$H90=""),"",IF($G90&gt;$H90,"1",IF($G90=$H90,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J90" s="25">
+        <f>IF(OR($G90="",$H90=""),"",$G90&amp;"-"&amp;$H90)</f>
+        <v/>
+      </c>
+      <c r="K90" s="73">
+        <f>IF($E90="","Calendario da inserire",IF(OR($G90="",$H90=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="69" t="inlineStr">
+        <is>
+          <t>G10-09</t>
+        </is>
+      </c>
+      <c r="B91" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C91" s="25" t="inlineStr">
+        <is>
+          <t>02/11/2026</t>
+        </is>
+      </c>
+      <c r="D91" s="25" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E91" s="70" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="F91" s="70" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="G91" s="71" t="n"/>
+      <c r="H91" s="71" t="n"/>
+      <c r="I91" s="72">
+        <f>IF(OR($G91="",$H91=""),"",IF($G91&gt;$H91,"1",IF($G91=$H91,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J91" s="25">
+        <f>IF(OR($G91="",$H91=""),"",$G91&amp;"-"&amp;$H91)</f>
+        <v/>
+      </c>
+      <c r="K91" s="73">
+        <f>IF($E91="","Calendario da inserire",IF(OR($G91="",$H91=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="69" t="inlineStr">
+        <is>
+          <t>G10-10</t>
+        </is>
+      </c>
+      <c r="B92" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C92" s="25" t="inlineStr">
+        <is>
+          <t>02/11/2026</t>
+        </is>
+      </c>
+      <c r="D92" s="25" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E92" s="70" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="F92" s="70" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="G92" s="71" t="n"/>
+      <c r="H92" s="71" t="n"/>
+      <c r="I92" s="72">
+        <f>IF(OR($G92="",$H92=""),"",IF($G92&gt;$H92,"1",IF($G92=$H92,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J92" s="25">
+        <f>IF(OR($G92="",$H92=""),"",$G92&amp;"-"&amp;$H92)</f>
+        <v/>
+      </c>
+      <c r="K92" s="73">
+        <f>IF($E92="","Calendario da inserire",IF(OR($G92="",$H92=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K82"/>
+  <autoFilter ref="A2:K92"/>
   <mergeCells count="3">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K3:K82">
+  <conditionalFormatting sqref="K3:K92">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Giocata"</formula>
     </cfRule>
@@ -6503,7 +7004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S82"/>
+  <dimension ref="A1:S92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12104,8 +12605,338 @@
       <c r="R82" s="71" t="n"/>
       <c r="S82" s="71" t="n"/>
     </row>
+    <row r="83">
+      <c r="A83" s="69">
+        <f>Partite!$A83</f>
+        <v/>
+      </c>
+      <c r="B83" s="25">
+        <f>Partite!$B83</f>
+        <v/>
+      </c>
+      <c r="C83" s="70">
+        <f>IF(Partite!$E83="","",Partite!$E83)</f>
+        <v/>
+      </c>
+      <c r="D83" s="70">
+        <f>IF(Partite!$F83="","",Partite!$F83)</f>
+        <v/>
+      </c>
+      <c r="E83" s="71" t="n"/>
+      <c r="F83" s="71" t="n"/>
+      <c r="G83" s="71" t="n"/>
+      <c r="H83" s="71" t="n"/>
+      <c r="I83" s="71" t="n"/>
+      <c r="J83" s="71" t="n"/>
+      <c r="K83" s="71" t="n"/>
+      <c r="L83" s="71" t="n"/>
+      <c r="M83" s="71" t="n"/>
+      <c r="N83" s="71" t="n"/>
+      <c r="O83" s="71" t="n"/>
+      <c r="P83" s="71" t="n"/>
+      <c r="Q83" s="71" t="n"/>
+      <c r="R83" s="71" t="n"/>
+      <c r="S83" s="71" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="69">
+        <f>Partite!$A84</f>
+        <v/>
+      </c>
+      <c r="B84" s="25">
+        <f>Partite!$B84</f>
+        <v/>
+      </c>
+      <c r="C84" s="70">
+        <f>IF(Partite!$E84="","",Partite!$E84)</f>
+        <v/>
+      </c>
+      <c r="D84" s="70">
+        <f>IF(Partite!$F84="","",Partite!$F84)</f>
+        <v/>
+      </c>
+      <c r="E84" s="71" t="n"/>
+      <c r="F84" s="71" t="n"/>
+      <c r="G84" s="71" t="n"/>
+      <c r="H84" s="71" t="n"/>
+      <c r="I84" s="71" t="n"/>
+      <c r="J84" s="71" t="n"/>
+      <c r="K84" s="71" t="n"/>
+      <c r="L84" s="71" t="n"/>
+      <c r="M84" s="71" t="n"/>
+      <c r="N84" s="71" t="n"/>
+      <c r="O84" s="71" t="n"/>
+      <c r="P84" s="71" t="n"/>
+      <c r="Q84" s="71" t="n"/>
+      <c r="R84" s="71" t="n"/>
+      <c r="S84" s="71" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="69">
+        <f>Partite!$A85</f>
+        <v/>
+      </c>
+      <c r="B85" s="25">
+        <f>Partite!$B85</f>
+        <v/>
+      </c>
+      <c r="C85" s="70">
+        <f>IF(Partite!$E85="","",Partite!$E85)</f>
+        <v/>
+      </c>
+      <c r="D85" s="70">
+        <f>IF(Partite!$F85="","",Partite!$F85)</f>
+        <v/>
+      </c>
+      <c r="E85" s="71" t="n"/>
+      <c r="F85" s="71" t="n"/>
+      <c r="G85" s="71" t="n"/>
+      <c r="H85" s="71" t="n"/>
+      <c r="I85" s="71" t="n"/>
+      <c r="J85" s="71" t="n"/>
+      <c r="K85" s="71" t="n"/>
+      <c r="L85" s="71" t="n"/>
+      <c r="M85" s="71" t="n"/>
+      <c r="N85" s="71" t="n"/>
+      <c r="O85" s="71" t="n"/>
+      <c r="P85" s="71" t="n"/>
+      <c r="Q85" s="71" t="n"/>
+      <c r="R85" s="71" t="n"/>
+      <c r="S85" s="71" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="69">
+        <f>Partite!$A86</f>
+        <v/>
+      </c>
+      <c r="B86" s="25">
+        <f>Partite!$B86</f>
+        <v/>
+      </c>
+      <c r="C86" s="70">
+        <f>IF(Partite!$E86="","",Partite!$E86)</f>
+        <v/>
+      </c>
+      <c r="D86" s="70">
+        <f>IF(Partite!$F86="","",Partite!$F86)</f>
+        <v/>
+      </c>
+      <c r="E86" s="71" t="n"/>
+      <c r="F86" s="71" t="n"/>
+      <c r="G86" s="71" t="n"/>
+      <c r="H86" s="71" t="n"/>
+      <c r="I86" s="71" t="n"/>
+      <c r="J86" s="71" t="n"/>
+      <c r="K86" s="71" t="n"/>
+      <c r="L86" s="71" t="n"/>
+      <c r="M86" s="71" t="n"/>
+      <c r="N86" s="71" t="n"/>
+      <c r="O86" s="71" t="n"/>
+      <c r="P86" s="71" t="n"/>
+      <c r="Q86" s="71" t="n"/>
+      <c r="R86" s="71" t="n"/>
+      <c r="S86" s="71" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="69">
+        <f>Partite!$A87</f>
+        <v/>
+      </c>
+      <c r="B87" s="25">
+        <f>Partite!$B87</f>
+        <v/>
+      </c>
+      <c r="C87" s="70">
+        <f>IF(Partite!$E87="","",Partite!$E87)</f>
+        <v/>
+      </c>
+      <c r="D87" s="70">
+        <f>IF(Partite!$F87="","",Partite!$F87)</f>
+        <v/>
+      </c>
+      <c r="E87" s="71" t="n"/>
+      <c r="F87" s="71" t="n"/>
+      <c r="G87" s="71" t="n"/>
+      <c r="H87" s="71" t="n"/>
+      <c r="I87" s="71" t="n"/>
+      <c r="J87" s="71" t="n"/>
+      <c r="K87" s="71" t="n"/>
+      <c r="L87" s="71" t="n"/>
+      <c r="M87" s="71" t="n"/>
+      <c r="N87" s="71" t="n"/>
+      <c r="O87" s="71" t="n"/>
+      <c r="P87" s="71" t="n"/>
+      <c r="Q87" s="71" t="n"/>
+      <c r="R87" s="71" t="n"/>
+      <c r="S87" s="71" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="69">
+        <f>Partite!$A88</f>
+        <v/>
+      </c>
+      <c r="B88" s="25">
+        <f>Partite!$B88</f>
+        <v/>
+      </c>
+      <c r="C88" s="70">
+        <f>IF(Partite!$E88="","",Partite!$E88)</f>
+        <v/>
+      </c>
+      <c r="D88" s="70">
+        <f>IF(Partite!$F88="","",Partite!$F88)</f>
+        <v/>
+      </c>
+      <c r="E88" s="71" t="n"/>
+      <c r="F88" s="71" t="n"/>
+      <c r="G88" s="71" t="n"/>
+      <c r="H88" s="71" t="n"/>
+      <c r="I88" s="71" t="n"/>
+      <c r="J88" s="71" t="n"/>
+      <c r="K88" s="71" t="n"/>
+      <c r="L88" s="71" t="n"/>
+      <c r="M88" s="71" t="n"/>
+      <c r="N88" s="71" t="n"/>
+      <c r="O88" s="71" t="n"/>
+      <c r="P88" s="71" t="n"/>
+      <c r="Q88" s="71" t="n"/>
+      <c r="R88" s="71" t="n"/>
+      <c r="S88" s="71" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="69">
+        <f>Partite!$A89</f>
+        <v/>
+      </c>
+      <c r="B89" s="25">
+        <f>Partite!$B89</f>
+        <v/>
+      </c>
+      <c r="C89" s="70">
+        <f>IF(Partite!$E89="","",Partite!$E89)</f>
+        <v/>
+      </c>
+      <c r="D89" s="70">
+        <f>IF(Partite!$F89="","",Partite!$F89)</f>
+        <v/>
+      </c>
+      <c r="E89" s="71" t="n"/>
+      <c r="F89" s="71" t="n"/>
+      <c r="G89" s="71" t="n"/>
+      <c r="H89" s="71" t="n"/>
+      <c r="I89" s="71" t="n"/>
+      <c r="J89" s="71" t="n"/>
+      <c r="K89" s="71" t="n"/>
+      <c r="L89" s="71" t="n"/>
+      <c r="M89" s="71" t="n"/>
+      <c r="N89" s="71" t="n"/>
+      <c r="O89" s="71" t="n"/>
+      <c r="P89" s="71" t="n"/>
+      <c r="Q89" s="71" t="n"/>
+      <c r="R89" s="71" t="n"/>
+      <c r="S89" s="71" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="69">
+        <f>Partite!$A90</f>
+        <v/>
+      </c>
+      <c r="B90" s="25">
+        <f>Partite!$B90</f>
+        <v/>
+      </c>
+      <c r="C90" s="70">
+        <f>IF(Partite!$E90="","",Partite!$E90)</f>
+        <v/>
+      </c>
+      <c r="D90" s="70">
+        <f>IF(Partite!$F90="","",Partite!$F90)</f>
+        <v/>
+      </c>
+      <c r="E90" s="71" t="n"/>
+      <c r="F90" s="71" t="n"/>
+      <c r="G90" s="71" t="n"/>
+      <c r="H90" s="71" t="n"/>
+      <c r="I90" s="71" t="n"/>
+      <c r="J90" s="71" t="n"/>
+      <c r="K90" s="71" t="n"/>
+      <c r="L90" s="71" t="n"/>
+      <c r="M90" s="71" t="n"/>
+      <c r="N90" s="71" t="n"/>
+      <c r="O90" s="71" t="n"/>
+      <c r="P90" s="71" t="n"/>
+      <c r="Q90" s="71" t="n"/>
+      <c r="R90" s="71" t="n"/>
+      <c r="S90" s="71" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="69">
+        <f>Partite!$A91</f>
+        <v/>
+      </c>
+      <c r="B91" s="25">
+        <f>Partite!$B91</f>
+        <v/>
+      </c>
+      <c r="C91" s="70">
+        <f>IF(Partite!$E91="","",Partite!$E91)</f>
+        <v/>
+      </c>
+      <c r="D91" s="70">
+        <f>IF(Partite!$F91="","",Partite!$F91)</f>
+        <v/>
+      </c>
+      <c r="E91" s="71" t="n"/>
+      <c r="F91" s="71" t="n"/>
+      <c r="G91" s="71" t="n"/>
+      <c r="H91" s="71" t="n"/>
+      <c r="I91" s="71" t="n"/>
+      <c r="J91" s="71" t="n"/>
+      <c r="K91" s="71" t="n"/>
+      <c r="L91" s="71" t="n"/>
+      <c r="M91" s="71" t="n"/>
+      <c r="N91" s="71" t="n"/>
+      <c r="O91" s="71" t="n"/>
+      <c r="P91" s="71" t="n"/>
+      <c r="Q91" s="71" t="n"/>
+      <c r="R91" s="71" t="n"/>
+      <c r="S91" s="71" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="69">
+        <f>Partite!$A92</f>
+        <v/>
+      </c>
+      <c r="B92" s="25">
+        <f>Partite!$B92</f>
+        <v/>
+      </c>
+      <c r="C92" s="70">
+        <f>IF(Partite!$E92="","",Partite!$E92)</f>
+        <v/>
+      </c>
+      <c r="D92" s="70">
+        <f>IF(Partite!$F92="","",Partite!$F92)</f>
+        <v/>
+      </c>
+      <c r="E92" s="71" t="n"/>
+      <c r="F92" s="71" t="n"/>
+      <c r="G92" s="71" t="n"/>
+      <c r="H92" s="71" t="n"/>
+      <c r="I92" s="71" t="n"/>
+      <c r="J92" s="71" t="n"/>
+      <c r="K92" s="71" t="n"/>
+      <c r="L92" s="71" t="n"/>
+      <c r="M92" s="71" t="n"/>
+      <c r="N92" s="71" t="n"/>
+      <c r="O92" s="71" t="n"/>
+      <c r="P92" s="71" t="n"/>
+      <c r="Q92" s="71" t="n"/>
+      <c r="R92" s="71" t="n"/>
+      <c r="S92" s="71" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:D82"/>
+  <autoFilter ref="A2:D92"/>
   <mergeCells count="6">
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A1:D1"/>
@@ -12115,7 +12946,7 @@
     <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 K92 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 N83 N84 N85 N86 N87 N88 N89 N90 N91 N92 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82 Q83 Q84 Q85 Q86 Q87 Q88 Q89 Q90 Q91 Q92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
       <formula1>"1,X,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12130,7 +12961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N82"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16544,11 +17375,551 @@
         <v/>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="69">
+        <f>Partite!$A83</f>
+        <v/>
+      </c>
+      <c r="B83" s="25">
+        <f>Partite!$B83</f>
+        <v/>
+      </c>
+      <c r="C83" s="43">
+        <f>IF(Partite!$E83="","",Partite!$E83&amp;"  -  "&amp;Partite!$F83)</f>
+        <v/>
+      </c>
+      <c r="D83" s="22">
+        <f>IF(Partite!$K83&lt;&gt;"Giocata","",IF(AND(Pronostici!$F83&lt;&gt;"",Pronostici!$G83&lt;&gt;"",Pronostici!$F83=Partite!$G83,Pronostici!$G83=Partite!$H83),Config!$D$6,IF(AND($J83&lt;&gt;"",$J83=Partite!$I83),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E83" s="22">
+        <f>IF(Partite!$K83&lt;&gt;"Giocata","",IF(AND(Pronostici!$I83&lt;&gt;"",Pronostici!$J83&lt;&gt;"",Pronostici!$I83=Partite!$G83,Pronostici!$J83=Partite!$H83),Config!$D$6,IF(AND($K83&lt;&gt;"",$K83=Partite!$I83),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F83" s="22">
+        <f>IF(Partite!$K83&lt;&gt;"Giocata","",IF(AND(Pronostici!$L83&lt;&gt;"",Pronostici!$M83&lt;&gt;"",Pronostici!$L83=Partite!$G83,Pronostici!$M83=Partite!$H83),Config!$D$6,IF(AND($L83&lt;&gt;"",$L83=Partite!$I83),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G83" s="22">
+        <f>IF(Partite!$K83&lt;&gt;"Giocata","",IF(AND(Pronostici!$O83&lt;&gt;"",Pronostici!$P83&lt;&gt;"",Pronostici!$O83=Partite!$G83,Pronostici!$P83=Partite!$H83),Config!$D$6,IF(AND($M83&lt;&gt;"",$M83=Partite!$I83),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H83" s="22">
+        <f>IF(Partite!$K83&lt;&gt;"Giocata","",IF(AND(Pronostici!$R83&lt;&gt;"",Pronostici!$S83&lt;&gt;"",Pronostici!$R83=Partite!$G83,Pronostici!$S83=Partite!$H83),Config!$D$6,IF(AND($N83&lt;&gt;"",$N83=Partite!$I83),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J83" s="63">
+        <f>IF(Pronostici!$E83&lt;&gt;"",UPPER(Pronostici!$E83),IF(OR(Pronostici!$F83="",Pronostici!$G83=""),"",IF(Pronostici!$F83&gt;Pronostici!$G83,"1",IF(Pronostici!$F83=Pronostici!$G83,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K83" s="63">
+        <f>IF(Pronostici!$H83&lt;&gt;"",UPPER(Pronostici!$H83),IF(OR(Pronostici!$I83="",Pronostici!$J83=""),"",IF(Pronostici!$I83&gt;Pronostici!$J83,"1",IF(Pronostici!$I83=Pronostici!$J83,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L83" s="63">
+        <f>IF(Pronostici!$K83&lt;&gt;"",UPPER(Pronostici!$K83),IF(OR(Pronostici!$L83="",Pronostici!$M83=""),"",IF(Pronostici!$L83&gt;Pronostici!$M83,"1",IF(Pronostici!$L83=Pronostici!$M83,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M83" s="63">
+        <f>IF(Pronostici!$N83&lt;&gt;"",UPPER(Pronostici!$N83),IF(OR(Pronostici!$O83="",Pronostici!$P83=""),"",IF(Pronostici!$O83&gt;Pronostici!$P83,"1",IF(Pronostici!$O83=Pronostici!$P83,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N83" s="63">
+        <f>IF(Pronostici!$Q83&lt;&gt;"",UPPER(Pronostici!$Q83),IF(OR(Pronostici!$R83="",Pronostici!$S83=""),"",IF(Pronostici!$R83&gt;Pronostici!$S83,"1",IF(Pronostici!$R83=Pronostici!$S83,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="69">
+        <f>Partite!$A84</f>
+        <v/>
+      </c>
+      <c r="B84" s="25">
+        <f>Partite!$B84</f>
+        <v/>
+      </c>
+      <c r="C84" s="43">
+        <f>IF(Partite!$E84="","",Partite!$E84&amp;"  -  "&amp;Partite!$F84)</f>
+        <v/>
+      </c>
+      <c r="D84" s="22">
+        <f>IF(Partite!$K84&lt;&gt;"Giocata","",IF(AND(Pronostici!$F84&lt;&gt;"",Pronostici!$G84&lt;&gt;"",Pronostici!$F84=Partite!$G84,Pronostici!$G84=Partite!$H84),Config!$D$6,IF(AND($J84&lt;&gt;"",$J84=Partite!$I84),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E84" s="22">
+        <f>IF(Partite!$K84&lt;&gt;"Giocata","",IF(AND(Pronostici!$I84&lt;&gt;"",Pronostici!$J84&lt;&gt;"",Pronostici!$I84=Partite!$G84,Pronostici!$J84=Partite!$H84),Config!$D$6,IF(AND($K84&lt;&gt;"",$K84=Partite!$I84),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F84" s="22">
+        <f>IF(Partite!$K84&lt;&gt;"Giocata","",IF(AND(Pronostici!$L84&lt;&gt;"",Pronostici!$M84&lt;&gt;"",Pronostici!$L84=Partite!$G84,Pronostici!$M84=Partite!$H84),Config!$D$6,IF(AND($L84&lt;&gt;"",$L84=Partite!$I84),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G84" s="22">
+        <f>IF(Partite!$K84&lt;&gt;"Giocata","",IF(AND(Pronostici!$O84&lt;&gt;"",Pronostici!$P84&lt;&gt;"",Pronostici!$O84=Partite!$G84,Pronostici!$P84=Partite!$H84),Config!$D$6,IF(AND($M84&lt;&gt;"",$M84=Partite!$I84),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H84" s="22">
+        <f>IF(Partite!$K84&lt;&gt;"Giocata","",IF(AND(Pronostici!$R84&lt;&gt;"",Pronostici!$S84&lt;&gt;"",Pronostici!$R84=Partite!$G84,Pronostici!$S84=Partite!$H84),Config!$D$6,IF(AND($N84&lt;&gt;"",$N84=Partite!$I84),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J84" s="63">
+        <f>IF(Pronostici!$E84&lt;&gt;"",UPPER(Pronostici!$E84),IF(OR(Pronostici!$F84="",Pronostici!$G84=""),"",IF(Pronostici!$F84&gt;Pronostici!$G84,"1",IF(Pronostici!$F84=Pronostici!$G84,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K84" s="63">
+        <f>IF(Pronostici!$H84&lt;&gt;"",UPPER(Pronostici!$H84),IF(OR(Pronostici!$I84="",Pronostici!$J84=""),"",IF(Pronostici!$I84&gt;Pronostici!$J84,"1",IF(Pronostici!$I84=Pronostici!$J84,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L84" s="63">
+        <f>IF(Pronostici!$K84&lt;&gt;"",UPPER(Pronostici!$K84),IF(OR(Pronostici!$L84="",Pronostici!$M84=""),"",IF(Pronostici!$L84&gt;Pronostici!$M84,"1",IF(Pronostici!$L84=Pronostici!$M84,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M84" s="63">
+        <f>IF(Pronostici!$N84&lt;&gt;"",UPPER(Pronostici!$N84),IF(OR(Pronostici!$O84="",Pronostici!$P84=""),"",IF(Pronostici!$O84&gt;Pronostici!$P84,"1",IF(Pronostici!$O84=Pronostici!$P84,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N84" s="63">
+        <f>IF(Pronostici!$Q84&lt;&gt;"",UPPER(Pronostici!$Q84),IF(OR(Pronostici!$R84="",Pronostici!$S84=""),"",IF(Pronostici!$R84&gt;Pronostici!$S84,"1",IF(Pronostici!$R84=Pronostici!$S84,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="69">
+        <f>Partite!$A85</f>
+        <v/>
+      </c>
+      <c r="B85" s="25">
+        <f>Partite!$B85</f>
+        <v/>
+      </c>
+      <c r="C85" s="43">
+        <f>IF(Partite!$E85="","",Partite!$E85&amp;"  -  "&amp;Partite!$F85)</f>
+        <v/>
+      </c>
+      <c r="D85" s="22">
+        <f>IF(Partite!$K85&lt;&gt;"Giocata","",IF(AND(Pronostici!$F85&lt;&gt;"",Pronostici!$G85&lt;&gt;"",Pronostici!$F85=Partite!$G85,Pronostici!$G85=Partite!$H85),Config!$D$6,IF(AND($J85&lt;&gt;"",$J85=Partite!$I85),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E85" s="22">
+        <f>IF(Partite!$K85&lt;&gt;"Giocata","",IF(AND(Pronostici!$I85&lt;&gt;"",Pronostici!$J85&lt;&gt;"",Pronostici!$I85=Partite!$G85,Pronostici!$J85=Partite!$H85),Config!$D$6,IF(AND($K85&lt;&gt;"",$K85=Partite!$I85),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F85" s="22">
+        <f>IF(Partite!$K85&lt;&gt;"Giocata","",IF(AND(Pronostici!$L85&lt;&gt;"",Pronostici!$M85&lt;&gt;"",Pronostici!$L85=Partite!$G85,Pronostici!$M85=Partite!$H85),Config!$D$6,IF(AND($L85&lt;&gt;"",$L85=Partite!$I85),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G85" s="22">
+        <f>IF(Partite!$K85&lt;&gt;"Giocata","",IF(AND(Pronostici!$O85&lt;&gt;"",Pronostici!$P85&lt;&gt;"",Pronostici!$O85=Partite!$G85,Pronostici!$P85=Partite!$H85),Config!$D$6,IF(AND($M85&lt;&gt;"",$M85=Partite!$I85),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H85" s="22">
+        <f>IF(Partite!$K85&lt;&gt;"Giocata","",IF(AND(Pronostici!$R85&lt;&gt;"",Pronostici!$S85&lt;&gt;"",Pronostici!$R85=Partite!$G85,Pronostici!$S85=Partite!$H85),Config!$D$6,IF(AND($N85&lt;&gt;"",$N85=Partite!$I85),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J85" s="63">
+        <f>IF(Pronostici!$E85&lt;&gt;"",UPPER(Pronostici!$E85),IF(OR(Pronostici!$F85="",Pronostici!$G85=""),"",IF(Pronostici!$F85&gt;Pronostici!$G85,"1",IF(Pronostici!$F85=Pronostici!$G85,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K85" s="63">
+        <f>IF(Pronostici!$H85&lt;&gt;"",UPPER(Pronostici!$H85),IF(OR(Pronostici!$I85="",Pronostici!$J85=""),"",IF(Pronostici!$I85&gt;Pronostici!$J85,"1",IF(Pronostici!$I85=Pronostici!$J85,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L85" s="63">
+        <f>IF(Pronostici!$K85&lt;&gt;"",UPPER(Pronostici!$K85),IF(OR(Pronostici!$L85="",Pronostici!$M85=""),"",IF(Pronostici!$L85&gt;Pronostici!$M85,"1",IF(Pronostici!$L85=Pronostici!$M85,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M85" s="63">
+        <f>IF(Pronostici!$N85&lt;&gt;"",UPPER(Pronostici!$N85),IF(OR(Pronostici!$O85="",Pronostici!$P85=""),"",IF(Pronostici!$O85&gt;Pronostici!$P85,"1",IF(Pronostici!$O85=Pronostici!$P85,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N85" s="63">
+        <f>IF(Pronostici!$Q85&lt;&gt;"",UPPER(Pronostici!$Q85),IF(OR(Pronostici!$R85="",Pronostici!$S85=""),"",IF(Pronostici!$R85&gt;Pronostici!$S85,"1",IF(Pronostici!$R85=Pronostici!$S85,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="69">
+        <f>Partite!$A86</f>
+        <v/>
+      </c>
+      <c r="B86" s="25">
+        <f>Partite!$B86</f>
+        <v/>
+      </c>
+      <c r="C86" s="43">
+        <f>IF(Partite!$E86="","",Partite!$E86&amp;"  -  "&amp;Partite!$F86)</f>
+        <v/>
+      </c>
+      <c r="D86" s="22">
+        <f>IF(Partite!$K86&lt;&gt;"Giocata","",IF(AND(Pronostici!$F86&lt;&gt;"",Pronostici!$G86&lt;&gt;"",Pronostici!$F86=Partite!$G86,Pronostici!$G86=Partite!$H86),Config!$D$6,IF(AND($J86&lt;&gt;"",$J86=Partite!$I86),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E86" s="22">
+        <f>IF(Partite!$K86&lt;&gt;"Giocata","",IF(AND(Pronostici!$I86&lt;&gt;"",Pronostici!$J86&lt;&gt;"",Pronostici!$I86=Partite!$G86,Pronostici!$J86=Partite!$H86),Config!$D$6,IF(AND($K86&lt;&gt;"",$K86=Partite!$I86),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F86" s="22">
+        <f>IF(Partite!$K86&lt;&gt;"Giocata","",IF(AND(Pronostici!$L86&lt;&gt;"",Pronostici!$M86&lt;&gt;"",Pronostici!$L86=Partite!$G86,Pronostici!$M86=Partite!$H86),Config!$D$6,IF(AND($L86&lt;&gt;"",$L86=Partite!$I86),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G86" s="22">
+        <f>IF(Partite!$K86&lt;&gt;"Giocata","",IF(AND(Pronostici!$O86&lt;&gt;"",Pronostici!$P86&lt;&gt;"",Pronostici!$O86=Partite!$G86,Pronostici!$P86=Partite!$H86),Config!$D$6,IF(AND($M86&lt;&gt;"",$M86=Partite!$I86),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H86" s="22">
+        <f>IF(Partite!$K86&lt;&gt;"Giocata","",IF(AND(Pronostici!$R86&lt;&gt;"",Pronostici!$S86&lt;&gt;"",Pronostici!$R86=Partite!$G86,Pronostici!$S86=Partite!$H86),Config!$D$6,IF(AND($N86&lt;&gt;"",$N86=Partite!$I86),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J86" s="63">
+        <f>IF(Pronostici!$E86&lt;&gt;"",UPPER(Pronostici!$E86),IF(OR(Pronostici!$F86="",Pronostici!$G86=""),"",IF(Pronostici!$F86&gt;Pronostici!$G86,"1",IF(Pronostici!$F86=Pronostici!$G86,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K86" s="63">
+        <f>IF(Pronostici!$H86&lt;&gt;"",UPPER(Pronostici!$H86),IF(OR(Pronostici!$I86="",Pronostici!$J86=""),"",IF(Pronostici!$I86&gt;Pronostici!$J86,"1",IF(Pronostici!$I86=Pronostici!$J86,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L86" s="63">
+        <f>IF(Pronostici!$K86&lt;&gt;"",UPPER(Pronostici!$K86),IF(OR(Pronostici!$L86="",Pronostici!$M86=""),"",IF(Pronostici!$L86&gt;Pronostici!$M86,"1",IF(Pronostici!$L86=Pronostici!$M86,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M86" s="63">
+        <f>IF(Pronostici!$N86&lt;&gt;"",UPPER(Pronostici!$N86),IF(OR(Pronostici!$O86="",Pronostici!$P86=""),"",IF(Pronostici!$O86&gt;Pronostici!$P86,"1",IF(Pronostici!$O86=Pronostici!$P86,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N86" s="63">
+        <f>IF(Pronostici!$Q86&lt;&gt;"",UPPER(Pronostici!$Q86),IF(OR(Pronostici!$R86="",Pronostici!$S86=""),"",IF(Pronostici!$R86&gt;Pronostici!$S86,"1",IF(Pronostici!$R86=Pronostici!$S86,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="69">
+        <f>Partite!$A87</f>
+        <v/>
+      </c>
+      <c r="B87" s="25">
+        <f>Partite!$B87</f>
+        <v/>
+      </c>
+      <c r="C87" s="43">
+        <f>IF(Partite!$E87="","",Partite!$E87&amp;"  -  "&amp;Partite!$F87)</f>
+        <v/>
+      </c>
+      <c r="D87" s="22">
+        <f>IF(Partite!$K87&lt;&gt;"Giocata","",IF(AND(Pronostici!$F87&lt;&gt;"",Pronostici!$G87&lt;&gt;"",Pronostici!$F87=Partite!$G87,Pronostici!$G87=Partite!$H87),Config!$D$6,IF(AND($J87&lt;&gt;"",$J87=Partite!$I87),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E87" s="22">
+        <f>IF(Partite!$K87&lt;&gt;"Giocata","",IF(AND(Pronostici!$I87&lt;&gt;"",Pronostici!$J87&lt;&gt;"",Pronostici!$I87=Partite!$G87,Pronostici!$J87=Partite!$H87),Config!$D$6,IF(AND($K87&lt;&gt;"",$K87=Partite!$I87),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F87" s="22">
+        <f>IF(Partite!$K87&lt;&gt;"Giocata","",IF(AND(Pronostici!$L87&lt;&gt;"",Pronostici!$M87&lt;&gt;"",Pronostici!$L87=Partite!$G87,Pronostici!$M87=Partite!$H87),Config!$D$6,IF(AND($L87&lt;&gt;"",$L87=Partite!$I87),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G87" s="22">
+        <f>IF(Partite!$K87&lt;&gt;"Giocata","",IF(AND(Pronostici!$O87&lt;&gt;"",Pronostici!$P87&lt;&gt;"",Pronostici!$O87=Partite!$G87,Pronostici!$P87=Partite!$H87),Config!$D$6,IF(AND($M87&lt;&gt;"",$M87=Partite!$I87),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H87" s="22">
+        <f>IF(Partite!$K87&lt;&gt;"Giocata","",IF(AND(Pronostici!$R87&lt;&gt;"",Pronostici!$S87&lt;&gt;"",Pronostici!$R87=Partite!$G87,Pronostici!$S87=Partite!$H87),Config!$D$6,IF(AND($N87&lt;&gt;"",$N87=Partite!$I87),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J87" s="63">
+        <f>IF(Pronostici!$E87&lt;&gt;"",UPPER(Pronostici!$E87),IF(OR(Pronostici!$F87="",Pronostici!$G87=""),"",IF(Pronostici!$F87&gt;Pronostici!$G87,"1",IF(Pronostici!$F87=Pronostici!$G87,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K87" s="63">
+        <f>IF(Pronostici!$H87&lt;&gt;"",UPPER(Pronostici!$H87),IF(OR(Pronostici!$I87="",Pronostici!$J87=""),"",IF(Pronostici!$I87&gt;Pronostici!$J87,"1",IF(Pronostici!$I87=Pronostici!$J87,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L87" s="63">
+        <f>IF(Pronostici!$K87&lt;&gt;"",UPPER(Pronostici!$K87),IF(OR(Pronostici!$L87="",Pronostici!$M87=""),"",IF(Pronostici!$L87&gt;Pronostici!$M87,"1",IF(Pronostici!$L87=Pronostici!$M87,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M87" s="63">
+        <f>IF(Pronostici!$N87&lt;&gt;"",UPPER(Pronostici!$N87),IF(OR(Pronostici!$O87="",Pronostici!$P87=""),"",IF(Pronostici!$O87&gt;Pronostici!$P87,"1",IF(Pronostici!$O87=Pronostici!$P87,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N87" s="63">
+        <f>IF(Pronostici!$Q87&lt;&gt;"",UPPER(Pronostici!$Q87),IF(OR(Pronostici!$R87="",Pronostici!$S87=""),"",IF(Pronostici!$R87&gt;Pronostici!$S87,"1",IF(Pronostici!$R87=Pronostici!$S87,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="69">
+        <f>Partite!$A88</f>
+        <v/>
+      </c>
+      <c r="B88" s="25">
+        <f>Partite!$B88</f>
+        <v/>
+      </c>
+      <c r="C88" s="43">
+        <f>IF(Partite!$E88="","",Partite!$E88&amp;"  -  "&amp;Partite!$F88)</f>
+        <v/>
+      </c>
+      <c r="D88" s="22">
+        <f>IF(Partite!$K88&lt;&gt;"Giocata","",IF(AND(Pronostici!$F88&lt;&gt;"",Pronostici!$G88&lt;&gt;"",Pronostici!$F88=Partite!$G88,Pronostici!$G88=Partite!$H88),Config!$D$6,IF(AND($J88&lt;&gt;"",$J88=Partite!$I88),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E88" s="22">
+        <f>IF(Partite!$K88&lt;&gt;"Giocata","",IF(AND(Pronostici!$I88&lt;&gt;"",Pronostici!$J88&lt;&gt;"",Pronostici!$I88=Partite!$G88,Pronostici!$J88=Partite!$H88),Config!$D$6,IF(AND($K88&lt;&gt;"",$K88=Partite!$I88),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F88" s="22">
+        <f>IF(Partite!$K88&lt;&gt;"Giocata","",IF(AND(Pronostici!$L88&lt;&gt;"",Pronostici!$M88&lt;&gt;"",Pronostici!$L88=Partite!$G88,Pronostici!$M88=Partite!$H88),Config!$D$6,IF(AND($L88&lt;&gt;"",$L88=Partite!$I88),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G88" s="22">
+        <f>IF(Partite!$K88&lt;&gt;"Giocata","",IF(AND(Pronostici!$O88&lt;&gt;"",Pronostici!$P88&lt;&gt;"",Pronostici!$O88=Partite!$G88,Pronostici!$P88=Partite!$H88),Config!$D$6,IF(AND($M88&lt;&gt;"",$M88=Partite!$I88),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H88" s="22">
+        <f>IF(Partite!$K88&lt;&gt;"Giocata","",IF(AND(Pronostici!$R88&lt;&gt;"",Pronostici!$S88&lt;&gt;"",Pronostici!$R88=Partite!$G88,Pronostici!$S88=Partite!$H88),Config!$D$6,IF(AND($N88&lt;&gt;"",$N88=Partite!$I88),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J88" s="63">
+        <f>IF(Pronostici!$E88&lt;&gt;"",UPPER(Pronostici!$E88),IF(OR(Pronostici!$F88="",Pronostici!$G88=""),"",IF(Pronostici!$F88&gt;Pronostici!$G88,"1",IF(Pronostici!$F88=Pronostici!$G88,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K88" s="63">
+        <f>IF(Pronostici!$H88&lt;&gt;"",UPPER(Pronostici!$H88),IF(OR(Pronostici!$I88="",Pronostici!$J88=""),"",IF(Pronostici!$I88&gt;Pronostici!$J88,"1",IF(Pronostici!$I88=Pronostici!$J88,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L88" s="63">
+        <f>IF(Pronostici!$K88&lt;&gt;"",UPPER(Pronostici!$K88),IF(OR(Pronostici!$L88="",Pronostici!$M88=""),"",IF(Pronostici!$L88&gt;Pronostici!$M88,"1",IF(Pronostici!$L88=Pronostici!$M88,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M88" s="63">
+        <f>IF(Pronostici!$N88&lt;&gt;"",UPPER(Pronostici!$N88),IF(OR(Pronostici!$O88="",Pronostici!$P88=""),"",IF(Pronostici!$O88&gt;Pronostici!$P88,"1",IF(Pronostici!$O88=Pronostici!$P88,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N88" s="63">
+        <f>IF(Pronostici!$Q88&lt;&gt;"",UPPER(Pronostici!$Q88),IF(OR(Pronostici!$R88="",Pronostici!$S88=""),"",IF(Pronostici!$R88&gt;Pronostici!$S88,"1",IF(Pronostici!$R88=Pronostici!$S88,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="69">
+        <f>Partite!$A89</f>
+        <v/>
+      </c>
+      <c r="B89" s="25">
+        <f>Partite!$B89</f>
+        <v/>
+      </c>
+      <c r="C89" s="43">
+        <f>IF(Partite!$E89="","",Partite!$E89&amp;"  -  "&amp;Partite!$F89)</f>
+        <v/>
+      </c>
+      <c r="D89" s="22">
+        <f>IF(Partite!$K89&lt;&gt;"Giocata","",IF(AND(Pronostici!$F89&lt;&gt;"",Pronostici!$G89&lt;&gt;"",Pronostici!$F89=Partite!$G89,Pronostici!$G89=Partite!$H89),Config!$D$6,IF(AND($J89&lt;&gt;"",$J89=Partite!$I89),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E89" s="22">
+        <f>IF(Partite!$K89&lt;&gt;"Giocata","",IF(AND(Pronostici!$I89&lt;&gt;"",Pronostici!$J89&lt;&gt;"",Pronostici!$I89=Partite!$G89,Pronostici!$J89=Partite!$H89),Config!$D$6,IF(AND($K89&lt;&gt;"",$K89=Partite!$I89),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F89" s="22">
+        <f>IF(Partite!$K89&lt;&gt;"Giocata","",IF(AND(Pronostici!$L89&lt;&gt;"",Pronostici!$M89&lt;&gt;"",Pronostici!$L89=Partite!$G89,Pronostici!$M89=Partite!$H89),Config!$D$6,IF(AND($L89&lt;&gt;"",$L89=Partite!$I89),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G89" s="22">
+        <f>IF(Partite!$K89&lt;&gt;"Giocata","",IF(AND(Pronostici!$O89&lt;&gt;"",Pronostici!$P89&lt;&gt;"",Pronostici!$O89=Partite!$G89,Pronostici!$P89=Partite!$H89),Config!$D$6,IF(AND($M89&lt;&gt;"",$M89=Partite!$I89),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H89" s="22">
+        <f>IF(Partite!$K89&lt;&gt;"Giocata","",IF(AND(Pronostici!$R89&lt;&gt;"",Pronostici!$S89&lt;&gt;"",Pronostici!$R89=Partite!$G89,Pronostici!$S89=Partite!$H89),Config!$D$6,IF(AND($N89&lt;&gt;"",$N89=Partite!$I89),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J89" s="63">
+        <f>IF(Pronostici!$E89&lt;&gt;"",UPPER(Pronostici!$E89),IF(OR(Pronostici!$F89="",Pronostici!$G89=""),"",IF(Pronostici!$F89&gt;Pronostici!$G89,"1",IF(Pronostici!$F89=Pronostici!$G89,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K89" s="63">
+        <f>IF(Pronostici!$H89&lt;&gt;"",UPPER(Pronostici!$H89),IF(OR(Pronostici!$I89="",Pronostici!$J89=""),"",IF(Pronostici!$I89&gt;Pronostici!$J89,"1",IF(Pronostici!$I89=Pronostici!$J89,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L89" s="63">
+        <f>IF(Pronostici!$K89&lt;&gt;"",UPPER(Pronostici!$K89),IF(OR(Pronostici!$L89="",Pronostici!$M89=""),"",IF(Pronostici!$L89&gt;Pronostici!$M89,"1",IF(Pronostici!$L89=Pronostici!$M89,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M89" s="63">
+        <f>IF(Pronostici!$N89&lt;&gt;"",UPPER(Pronostici!$N89),IF(OR(Pronostici!$O89="",Pronostici!$P89=""),"",IF(Pronostici!$O89&gt;Pronostici!$P89,"1",IF(Pronostici!$O89=Pronostici!$P89,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N89" s="63">
+        <f>IF(Pronostici!$Q89&lt;&gt;"",UPPER(Pronostici!$Q89),IF(OR(Pronostici!$R89="",Pronostici!$S89=""),"",IF(Pronostici!$R89&gt;Pronostici!$S89,"1",IF(Pronostici!$R89=Pronostici!$S89,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="69">
+        <f>Partite!$A90</f>
+        <v/>
+      </c>
+      <c r="B90" s="25">
+        <f>Partite!$B90</f>
+        <v/>
+      </c>
+      <c r="C90" s="43">
+        <f>IF(Partite!$E90="","",Partite!$E90&amp;"  -  "&amp;Partite!$F90)</f>
+        <v/>
+      </c>
+      <c r="D90" s="22">
+        <f>IF(Partite!$K90&lt;&gt;"Giocata","",IF(AND(Pronostici!$F90&lt;&gt;"",Pronostici!$G90&lt;&gt;"",Pronostici!$F90=Partite!$G90,Pronostici!$G90=Partite!$H90),Config!$D$6,IF(AND($J90&lt;&gt;"",$J90=Partite!$I90),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E90" s="22">
+        <f>IF(Partite!$K90&lt;&gt;"Giocata","",IF(AND(Pronostici!$I90&lt;&gt;"",Pronostici!$J90&lt;&gt;"",Pronostici!$I90=Partite!$G90,Pronostici!$J90=Partite!$H90),Config!$D$6,IF(AND($K90&lt;&gt;"",$K90=Partite!$I90),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F90" s="22">
+        <f>IF(Partite!$K90&lt;&gt;"Giocata","",IF(AND(Pronostici!$L90&lt;&gt;"",Pronostici!$M90&lt;&gt;"",Pronostici!$L90=Partite!$G90,Pronostici!$M90=Partite!$H90),Config!$D$6,IF(AND($L90&lt;&gt;"",$L90=Partite!$I90),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G90" s="22">
+        <f>IF(Partite!$K90&lt;&gt;"Giocata","",IF(AND(Pronostici!$O90&lt;&gt;"",Pronostici!$P90&lt;&gt;"",Pronostici!$O90=Partite!$G90,Pronostici!$P90=Partite!$H90),Config!$D$6,IF(AND($M90&lt;&gt;"",$M90=Partite!$I90),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H90" s="22">
+        <f>IF(Partite!$K90&lt;&gt;"Giocata","",IF(AND(Pronostici!$R90&lt;&gt;"",Pronostici!$S90&lt;&gt;"",Pronostici!$R90=Partite!$G90,Pronostici!$S90=Partite!$H90),Config!$D$6,IF(AND($N90&lt;&gt;"",$N90=Partite!$I90),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J90" s="63">
+        <f>IF(Pronostici!$E90&lt;&gt;"",UPPER(Pronostici!$E90),IF(OR(Pronostici!$F90="",Pronostici!$G90=""),"",IF(Pronostici!$F90&gt;Pronostici!$G90,"1",IF(Pronostici!$F90=Pronostici!$G90,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K90" s="63">
+        <f>IF(Pronostici!$H90&lt;&gt;"",UPPER(Pronostici!$H90),IF(OR(Pronostici!$I90="",Pronostici!$J90=""),"",IF(Pronostici!$I90&gt;Pronostici!$J90,"1",IF(Pronostici!$I90=Pronostici!$J90,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L90" s="63">
+        <f>IF(Pronostici!$K90&lt;&gt;"",UPPER(Pronostici!$K90),IF(OR(Pronostici!$L90="",Pronostici!$M90=""),"",IF(Pronostici!$L90&gt;Pronostici!$M90,"1",IF(Pronostici!$L90=Pronostici!$M90,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M90" s="63">
+        <f>IF(Pronostici!$N90&lt;&gt;"",UPPER(Pronostici!$N90),IF(OR(Pronostici!$O90="",Pronostici!$P90=""),"",IF(Pronostici!$O90&gt;Pronostici!$P90,"1",IF(Pronostici!$O90=Pronostici!$P90,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N90" s="63">
+        <f>IF(Pronostici!$Q90&lt;&gt;"",UPPER(Pronostici!$Q90),IF(OR(Pronostici!$R90="",Pronostici!$S90=""),"",IF(Pronostici!$R90&gt;Pronostici!$S90,"1",IF(Pronostici!$R90=Pronostici!$S90,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="69">
+        <f>Partite!$A91</f>
+        <v/>
+      </c>
+      <c r="B91" s="25">
+        <f>Partite!$B91</f>
+        <v/>
+      </c>
+      <c r="C91" s="43">
+        <f>IF(Partite!$E91="","",Partite!$E91&amp;"  -  "&amp;Partite!$F91)</f>
+        <v/>
+      </c>
+      <c r="D91" s="22">
+        <f>IF(Partite!$K91&lt;&gt;"Giocata","",IF(AND(Pronostici!$F91&lt;&gt;"",Pronostici!$G91&lt;&gt;"",Pronostici!$F91=Partite!$G91,Pronostici!$G91=Partite!$H91),Config!$D$6,IF(AND($J91&lt;&gt;"",$J91=Partite!$I91),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E91" s="22">
+        <f>IF(Partite!$K91&lt;&gt;"Giocata","",IF(AND(Pronostici!$I91&lt;&gt;"",Pronostici!$J91&lt;&gt;"",Pronostici!$I91=Partite!$G91,Pronostici!$J91=Partite!$H91),Config!$D$6,IF(AND($K91&lt;&gt;"",$K91=Partite!$I91),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F91" s="22">
+        <f>IF(Partite!$K91&lt;&gt;"Giocata","",IF(AND(Pronostici!$L91&lt;&gt;"",Pronostici!$M91&lt;&gt;"",Pronostici!$L91=Partite!$G91,Pronostici!$M91=Partite!$H91),Config!$D$6,IF(AND($L91&lt;&gt;"",$L91=Partite!$I91),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G91" s="22">
+        <f>IF(Partite!$K91&lt;&gt;"Giocata","",IF(AND(Pronostici!$O91&lt;&gt;"",Pronostici!$P91&lt;&gt;"",Pronostici!$O91=Partite!$G91,Pronostici!$P91=Partite!$H91),Config!$D$6,IF(AND($M91&lt;&gt;"",$M91=Partite!$I91),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H91" s="22">
+        <f>IF(Partite!$K91&lt;&gt;"Giocata","",IF(AND(Pronostici!$R91&lt;&gt;"",Pronostici!$S91&lt;&gt;"",Pronostici!$R91=Partite!$G91,Pronostici!$S91=Partite!$H91),Config!$D$6,IF(AND($N91&lt;&gt;"",$N91=Partite!$I91),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J91" s="63">
+        <f>IF(Pronostici!$E91&lt;&gt;"",UPPER(Pronostici!$E91),IF(OR(Pronostici!$F91="",Pronostici!$G91=""),"",IF(Pronostici!$F91&gt;Pronostici!$G91,"1",IF(Pronostici!$F91=Pronostici!$G91,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K91" s="63">
+        <f>IF(Pronostici!$H91&lt;&gt;"",UPPER(Pronostici!$H91),IF(OR(Pronostici!$I91="",Pronostici!$J91=""),"",IF(Pronostici!$I91&gt;Pronostici!$J91,"1",IF(Pronostici!$I91=Pronostici!$J91,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L91" s="63">
+        <f>IF(Pronostici!$K91&lt;&gt;"",UPPER(Pronostici!$K91),IF(OR(Pronostici!$L91="",Pronostici!$M91=""),"",IF(Pronostici!$L91&gt;Pronostici!$M91,"1",IF(Pronostici!$L91=Pronostici!$M91,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M91" s="63">
+        <f>IF(Pronostici!$N91&lt;&gt;"",UPPER(Pronostici!$N91),IF(OR(Pronostici!$O91="",Pronostici!$P91=""),"",IF(Pronostici!$O91&gt;Pronostici!$P91,"1",IF(Pronostici!$O91=Pronostici!$P91,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N91" s="63">
+        <f>IF(Pronostici!$Q91&lt;&gt;"",UPPER(Pronostici!$Q91),IF(OR(Pronostici!$R91="",Pronostici!$S91=""),"",IF(Pronostici!$R91&gt;Pronostici!$S91,"1",IF(Pronostici!$R91=Pronostici!$S91,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="69">
+        <f>Partite!$A92</f>
+        <v/>
+      </c>
+      <c r="B92" s="25">
+        <f>Partite!$B92</f>
+        <v/>
+      </c>
+      <c r="C92" s="43">
+        <f>IF(Partite!$E92="","",Partite!$E92&amp;"  -  "&amp;Partite!$F92)</f>
+        <v/>
+      </c>
+      <c r="D92" s="22">
+        <f>IF(Partite!$K92&lt;&gt;"Giocata","",IF(AND(Pronostici!$F92&lt;&gt;"",Pronostici!$G92&lt;&gt;"",Pronostici!$F92=Partite!$G92,Pronostici!$G92=Partite!$H92),Config!$D$6,IF(AND($J92&lt;&gt;"",$J92=Partite!$I92),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E92" s="22">
+        <f>IF(Partite!$K92&lt;&gt;"Giocata","",IF(AND(Pronostici!$I92&lt;&gt;"",Pronostici!$J92&lt;&gt;"",Pronostici!$I92=Partite!$G92,Pronostici!$J92=Partite!$H92),Config!$D$6,IF(AND($K92&lt;&gt;"",$K92=Partite!$I92),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F92" s="22">
+        <f>IF(Partite!$K92&lt;&gt;"Giocata","",IF(AND(Pronostici!$L92&lt;&gt;"",Pronostici!$M92&lt;&gt;"",Pronostici!$L92=Partite!$G92,Pronostici!$M92=Partite!$H92),Config!$D$6,IF(AND($L92&lt;&gt;"",$L92=Partite!$I92),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G92" s="22">
+        <f>IF(Partite!$K92&lt;&gt;"Giocata","",IF(AND(Pronostici!$O92&lt;&gt;"",Pronostici!$P92&lt;&gt;"",Pronostici!$O92=Partite!$G92,Pronostici!$P92=Partite!$H92),Config!$D$6,IF(AND($M92&lt;&gt;"",$M92=Partite!$I92),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H92" s="22">
+        <f>IF(Partite!$K92&lt;&gt;"Giocata","",IF(AND(Pronostici!$R92&lt;&gt;"",Pronostici!$S92&lt;&gt;"",Pronostici!$R92=Partite!$G92,Pronostici!$S92=Partite!$H92),Config!$D$6,IF(AND($N92&lt;&gt;"",$N92=Partite!$I92),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J92" s="63">
+        <f>IF(Pronostici!$E92&lt;&gt;"",UPPER(Pronostici!$E92),IF(OR(Pronostici!$F92="",Pronostici!$G92=""),"",IF(Pronostici!$F92&gt;Pronostici!$G92,"1",IF(Pronostici!$F92=Pronostici!$G92,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K92" s="63">
+        <f>IF(Pronostici!$H92&lt;&gt;"",UPPER(Pronostici!$H92),IF(OR(Pronostici!$I92="",Pronostici!$J92=""),"",IF(Pronostici!$I92&gt;Pronostici!$J92,"1",IF(Pronostici!$I92=Pronostici!$J92,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L92" s="63">
+        <f>IF(Pronostici!$K92&lt;&gt;"",UPPER(Pronostici!$K92),IF(OR(Pronostici!$L92="",Pronostici!$M92=""),"",IF(Pronostici!$L92&gt;Pronostici!$M92,"1",IF(Pronostici!$L92=Pronostici!$M92,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M92" s="63">
+        <f>IF(Pronostici!$N92&lt;&gt;"",UPPER(Pronostici!$N92),IF(OR(Pronostici!$O92="",Pronostici!$P92=""),"",IF(Pronostici!$O92&gt;Pronostici!$P92,"1",IF(Pronostici!$O92=Pronostici!$P92,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N92" s="63">
+        <f>IF(Pronostici!$Q92&lt;&gt;"",UPPER(Pronostici!$Q92),IF(OR(Pronostici!$R92="",Pronostici!$S92=""),"",IF(Pronostici!$R92&gt;Pronostici!$S92,"1",IF(Pronostici!$R92=Pronostici!$S92,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D82">
+  <conditionalFormatting sqref="D3:D92">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -16556,7 +17927,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E82">
+  <conditionalFormatting sqref="E3:E92">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -16564,7 +17935,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F82">
+  <conditionalFormatting sqref="F3:F92">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -16572,7 +17943,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G82">
+  <conditionalFormatting sqref="G3:G92">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -16580,7 +17951,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H82">
+  <conditionalFormatting sqref="H3:H92">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento automatico del 27/10/2026 alle 18:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -12292,21 +12292,61 @@
         <f>IF(Partite!$F73="","",Partite!$F73)</f>
         <v/>
       </c>
-      <c r="E73" s="71" t="n"/>
-      <c r="F73" s="71" t="n"/>
-      <c r="G73" s="71" t="n"/>
-      <c r="H73" s="71" t="n"/>
-      <c r="I73" s="71" t="n"/>
-      <c r="J73" s="71" t="n"/>
-      <c r="K73" s="71" t="n"/>
-      <c r="L73" s="71" t="n"/>
-      <c r="M73" s="71" t="n"/>
-      <c r="N73" s="71" t="n"/>
-      <c r="O73" s="71" t="n"/>
-      <c r="P73" s="71" t="n"/>
-      <c r="Q73" s="71" t="n"/>
-      <c r="R73" s="71" t="n"/>
-      <c r="S73" s="71" t="n"/>
+      <c r="E73" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F73" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I73" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J73" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K73" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L73" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M73" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N73" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O73" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q73" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R73" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S73" s="71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="74">
@@ -12325,21 +12365,61 @@
         <f>IF(Partite!$F74="","",Partite!$F74)</f>
         <v/>
       </c>
-      <c r="E74" s="71" t="n"/>
-      <c r="F74" s="71" t="n"/>
-      <c r="G74" s="71" t="n"/>
-      <c r="H74" s="71" t="n"/>
-      <c r="I74" s="71" t="n"/>
-      <c r="J74" s="71" t="n"/>
-      <c r="K74" s="71" t="n"/>
-      <c r="L74" s="71" t="n"/>
-      <c r="M74" s="71" t="n"/>
-      <c r="N74" s="71" t="n"/>
-      <c r="O74" s="71" t="n"/>
-      <c r="P74" s="71" t="n"/>
-      <c r="Q74" s="71" t="n"/>
-      <c r="R74" s="71" t="n"/>
-      <c r="S74" s="71" t="n"/>
+      <c r="E74" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F74" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G74" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I74" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J74" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K74" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L74" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M74" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N74" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O74" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P74" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q74" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R74" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S74" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="74">
@@ -12358,21 +12438,61 @@
         <f>IF(Partite!$F75="","",Partite!$F75)</f>
         <v/>
       </c>
-      <c r="E75" s="71" t="n"/>
-      <c r="F75" s="71" t="n"/>
-      <c r="G75" s="71" t="n"/>
-      <c r="H75" s="71" t="n"/>
-      <c r="I75" s="71" t="n"/>
-      <c r="J75" s="71" t="n"/>
-      <c r="K75" s="71" t="n"/>
-      <c r="L75" s="71" t="n"/>
-      <c r="M75" s="71" t="n"/>
-      <c r="N75" s="71" t="n"/>
-      <c r="O75" s="71" t="n"/>
-      <c r="P75" s="71" t="n"/>
-      <c r="Q75" s="71" t="n"/>
-      <c r="R75" s="71" t="n"/>
-      <c r="S75" s="71" t="n"/>
+      <c r="E75" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F75" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H75" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I75" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J75" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K75" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L75" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M75" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N75" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O75" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P75" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q75" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R75" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S75" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="74">
@@ -12391,21 +12511,61 @@
         <f>IF(Partite!$F76="","",Partite!$F76)</f>
         <v/>
       </c>
-      <c r="E76" s="71" t="n"/>
-      <c r="F76" s="71" t="n"/>
-      <c r="G76" s="71" t="n"/>
-      <c r="H76" s="71" t="n"/>
-      <c r="I76" s="71" t="n"/>
-      <c r="J76" s="71" t="n"/>
-      <c r="K76" s="71" t="n"/>
-      <c r="L76" s="71" t="n"/>
-      <c r="M76" s="71" t="n"/>
-      <c r="N76" s="71" t="n"/>
-      <c r="O76" s="71" t="n"/>
-      <c r="P76" s="71" t="n"/>
-      <c r="Q76" s="71" t="n"/>
-      <c r="R76" s="71" t="n"/>
-      <c r="S76" s="71" t="n"/>
+      <c r="E76" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G76" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L76" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P76" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q76" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S76" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="74">
@@ -12424,21 +12584,61 @@
         <f>IF(Partite!$F77="","",Partite!$F77)</f>
         <v/>
       </c>
-      <c r="E77" s="71" t="n"/>
-      <c r="F77" s="71" t="n"/>
-      <c r="G77" s="71" t="n"/>
-      <c r="H77" s="71" t="n"/>
-      <c r="I77" s="71" t="n"/>
-      <c r="J77" s="71" t="n"/>
-      <c r="K77" s="71" t="n"/>
-      <c r="L77" s="71" t="n"/>
-      <c r="M77" s="71" t="n"/>
-      <c r="N77" s="71" t="n"/>
-      <c r="O77" s="71" t="n"/>
-      <c r="P77" s="71" t="n"/>
-      <c r="Q77" s="71" t="n"/>
-      <c r="R77" s="71" t="n"/>
-      <c r="S77" s="71" t="n"/>
+      <c r="E77" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H77" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J77" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P77" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R77" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S77" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="74">
@@ -12457,21 +12657,61 @@
         <f>IF(Partite!$F78="","",Partite!$F78)</f>
         <v/>
       </c>
-      <c r="E78" s="71" t="n"/>
-      <c r="F78" s="71" t="n"/>
-      <c r="G78" s="71" t="n"/>
-      <c r="H78" s="71" t="n"/>
-      <c r="I78" s="71" t="n"/>
-      <c r="J78" s="71" t="n"/>
-      <c r="K78" s="71" t="n"/>
-      <c r="L78" s="71" t="n"/>
-      <c r="M78" s="71" t="n"/>
-      <c r="N78" s="71" t="n"/>
-      <c r="O78" s="71" t="n"/>
-      <c r="P78" s="71" t="n"/>
-      <c r="Q78" s="71" t="n"/>
-      <c r="R78" s="71" t="n"/>
-      <c r="S78" s="71" t="n"/>
+      <c r="E78" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F78" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H78" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I78" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K78" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L78" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="N78" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O78" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q78" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R78" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" s="71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="74">
@@ -12490,21 +12730,61 @@
         <f>IF(Partite!$F79="","",Partite!$F79)</f>
         <v/>
       </c>
-      <c r="E79" s="71" t="n"/>
-      <c r="F79" s="71" t="n"/>
-      <c r="G79" s="71" t="n"/>
-      <c r="H79" s="71" t="n"/>
-      <c r="I79" s="71" t="n"/>
-      <c r="J79" s="71" t="n"/>
-      <c r="K79" s="71" t="n"/>
-      <c r="L79" s="71" t="n"/>
-      <c r="M79" s="71" t="n"/>
-      <c r="N79" s="71" t="n"/>
-      <c r="O79" s="71" t="n"/>
-      <c r="P79" s="71" t="n"/>
-      <c r="Q79" s="71" t="n"/>
-      <c r="R79" s="71" t="n"/>
-      <c r="S79" s="71" t="n"/>
+      <c r="E79" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F79" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H79" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I79" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J79" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K79" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L79" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N79" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O79" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q79" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R79" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="74">
@@ -12523,21 +12803,61 @@
         <f>IF(Partite!$F80="","",Partite!$F80)</f>
         <v/>
       </c>
-      <c r="E80" s="71" t="n"/>
-      <c r="F80" s="71" t="n"/>
-      <c r="G80" s="71" t="n"/>
-      <c r="H80" s="71" t="n"/>
-      <c r="I80" s="71" t="n"/>
-      <c r="J80" s="71" t="n"/>
-      <c r="K80" s="71" t="n"/>
-      <c r="L80" s="71" t="n"/>
-      <c r="M80" s="71" t="n"/>
-      <c r="N80" s="71" t="n"/>
-      <c r="O80" s="71" t="n"/>
-      <c r="P80" s="71" t="n"/>
-      <c r="Q80" s="71" t="n"/>
-      <c r="R80" s="71" t="n"/>
-      <c r="S80" s="71" t="n"/>
+      <c r="E80" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F80" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H80" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I80" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J80" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K80" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L80" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N80" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O80" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P80" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q80" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R80" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S80" s="71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="74">
@@ -12556,21 +12876,61 @@
         <f>IF(Partite!$F81="","",Partite!$F81)</f>
         <v/>
       </c>
-      <c r="E81" s="71" t="n"/>
-      <c r="F81" s="71" t="n"/>
-      <c r="G81" s="71" t="n"/>
-      <c r="H81" s="71" t="n"/>
-      <c r="I81" s="71" t="n"/>
-      <c r="J81" s="71" t="n"/>
-      <c r="K81" s="71" t="n"/>
-      <c r="L81" s="71" t="n"/>
-      <c r="M81" s="71" t="n"/>
-      <c r="N81" s="71" t="n"/>
-      <c r="O81" s="71" t="n"/>
-      <c r="P81" s="71" t="n"/>
-      <c r="Q81" s="71" t="n"/>
-      <c r="R81" s="71" t="n"/>
-      <c r="S81" s="71" t="n"/>
+      <c r="E81" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F81" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I81" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J81" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K81" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L81" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M81" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O81" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P81" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q81" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R81" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S81" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="74">
@@ -12589,21 +12949,61 @@
         <f>IF(Partite!$F82="","",Partite!$F82)</f>
         <v/>
       </c>
-      <c r="E82" s="71" t="n"/>
-      <c r="F82" s="71" t="n"/>
-      <c r="G82" s="71" t="n"/>
-      <c r="H82" s="71" t="n"/>
-      <c r="I82" s="71" t="n"/>
-      <c r="J82" s="71" t="n"/>
-      <c r="K82" s="71" t="n"/>
-      <c r="L82" s="71" t="n"/>
-      <c r="M82" s="71" t="n"/>
-      <c r="N82" s="71" t="n"/>
-      <c r="O82" s="71" t="n"/>
-      <c r="P82" s="71" t="n"/>
-      <c r="Q82" s="71" t="n"/>
-      <c r="R82" s="71" t="n"/>
-      <c r="S82" s="71" t="n"/>
+      <c r="E82" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H82" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K82" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N82" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P82" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q82" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S82" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="69">

</xml_diff>

<commit_message>
Aggiornamento automatico del 27/10/2026 alle 20:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6130,8 +6130,12 @@
           <t>Lazio</t>
         </is>
       </c>
-      <c r="G73" s="71" t="n"/>
-      <c r="H73" s="71" t="n"/>
+      <c r="G73" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" s="71" t="n">
+        <v>6</v>
+      </c>
       <c r="I73" s="76">
         <f>IF(OR($G73="",$H73=""),"",IF($G73&gt;$H73,"1",IF($G73=$H73,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 27/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6178,8 +6178,12 @@
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="G74" s="71" t="n"/>
-      <c r="H74" s="71" t="n"/>
+      <c r="G74" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H74" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I74" s="76">
         <f>IF(OR($G74="",$H74=""),"",IF($G74&gt;$H74,"1",IF($G74=$H74,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 27/10/2026 alle 22:54
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6226,8 +6226,12 @@
           <t>Como</t>
         </is>
       </c>
-      <c r="G75" s="71" t="n"/>
-      <c r="H75" s="71" t="n"/>
+      <c r="G75" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="I75" s="76">
         <f>IF(OR($G75="",$H75=""),"",IF($G75&gt;$H75,"1",IF($G75=$H75,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 28/10/2026 alle 20:29
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6318,8 +6318,12 @@
           <t>Udinese</t>
         </is>
       </c>
-      <c r="G77" s="71" t="n"/>
-      <c r="H77" s="71" t="n"/>
+      <c r="G77" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I77" s="76">
         <f>IF(OR($G77="",$H77=""),"",IF($G77&gt;$H77,"1",IF($G77=$H77,"X","2")))</f>
         <v/>
@@ -6362,8 +6366,12 @@
           <t>Inter</t>
         </is>
       </c>
-      <c r="G78" s="71" t="n"/>
-      <c r="H78" s="71" t="n"/>
+      <c r="G78" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I78" s="76">
         <f>IF(OR($G78="",$H78=""),"",IF($G78&gt;$H78,"1",IF($G78=$H78,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 28/10/2026 alle 20:34
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6274,8 +6274,12 @@
           <t>Bologna</t>
         </is>
       </c>
-      <c r="G76" s="71" t="n"/>
-      <c r="H76" s="71" t="n"/>
+      <c r="G76" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H76" s="71" t="n">
+        <v>4</v>
+      </c>
       <c r="I76" s="76">
         <f>IF(OR($G76="",$H76=""),"",IF($G76&gt;$H76,"1",IF($G76=$H76,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 28/10/2026 alle 22:44
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6462,8 +6462,12 @@
           <t>Napoli</t>
         </is>
       </c>
-      <c r="G80" s="71" t="n"/>
-      <c r="H80" s="71" t="n"/>
+      <c r="G80" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="71" t="n">
+        <v>4</v>
+      </c>
       <c r="I80" s="76">
         <f>IF(OR($G80="",$H80=""),"",IF($G80&gt;$H80,"1",IF($G80=$H80,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 28/10/2026 alle 22:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6418,8 +6418,12 @@
           <t>Juventus</t>
         </is>
       </c>
-      <c r="G79" s="71" t="n"/>
-      <c r="H79" s="71" t="n"/>
+      <c r="G79" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H79" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I79" s="76">
         <f>IF(OR($G79="",$H79=""),"",IF($G79&gt;$H79,"1",IF($G79=$H79,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 29/10/2026 alle 20:39
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6514,8 +6514,12 @@
           <t>Lecce</t>
         </is>
       </c>
-      <c r="G81" s="71" t="n"/>
-      <c r="H81" s="71" t="n"/>
+      <c r="G81" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H81" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I81" s="76">
         <f>IF(OR($G81="",$H81=""),"",IF($G81&gt;$H81,"1",IF($G81=$H81,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 29/10/2026 alle 22:59
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Partite'!$A$2:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pronostici'!$A$2:$D$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$41</f>
+              <f>'Classifica'!$A$33:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$R$33:$R$41</f>
+              <f>'Classifica'!$R$33:$R$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -851,12 +851,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$41</f>
+              <f>'Classifica'!$A$33:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$S$33:$S$41</f>
+              <f>'Classifica'!$S$33:$S$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -888,12 +888,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$41</f>
+              <f>'Classifica'!$A$33:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$T$33:$T$41</f>
+              <f>'Classifica'!$T$33:$T$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -925,12 +925,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$41</f>
+              <f>'Classifica'!$A$33:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$U$33:$U$41</f>
+              <f>'Classifica'!$U$33:$U$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -962,12 +962,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Classifica'!$A$33:$A$41</f>
+              <f>'Classifica'!$A$33:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Classifica'!$V$33:$V$41</f>
+              <f>'Classifica'!$V$33:$V$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1043,7 +1043,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>43</row>
+      <row>44</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9720000" cy="3420000"/>
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>COUNTIF($B$33:$B$41,"Completata")</f>
+        <f>COUNTIF($B$33:$B$42,"Completata")</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>COUNTIF($B$33:$B$41,"Completata")+COUNTIF($B$33:$B$41,"In corso")</f>
+        <f>COUNTIF($B$33:$B$42,"Completata")+COUNTIF($B$33:$B$42,"In corso")</f>
         <v/>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L7" s="13">
-        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$41="Completata")*$A$33:$A$41)))</f>
+        <f>IF($L$5=0,"-",SUMPRODUCT(MAX(($B$33:$B$42="Completata")*$A$33:$A$42)))</f>
         <v/>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="L8" s="13">
-        <f>IF(SUMPRODUCT(MIN(($B$33:$B$41&lt;&gt;"Completata")*$A$33:$A$41+($B$33:$B$41="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$41&lt;&gt;"Completata")*$A$33:$A$41+($B$33:$B$41="Completata")*999)))</f>
+        <f>IF(SUMPRODUCT(MIN(($B$33:$B$42&lt;&gt;"Completata")*$A$33:$A$42+($B$33:$B$42="Completata")*999))&gt;=999,"-",SUMPRODUCT(MIN(($B$33:$B$42&lt;&gt;"Completata")*$A$33:$A$42+($B$33:$B$42="Completata")*999)))</f>
         <v/>
       </c>
     </row>
@@ -1591,19 +1591,19 @@
         <v/>
       </c>
       <c r="C12" s="24">
-        <f>SUM(Punti!$D$3:$D$92)</f>
+        <f>SUM(Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$92,Config!$D$7)+COUNTIF(Punti!$D$3:$D$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$102,Config!$D$7)+COUNTIF(Punti!$D$3:$D$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>SUMPRODUCT(((Pronostici!$E$3:$E$92&lt;&gt;"")+(Pronostici!$F$3:$F$92&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$E$3:$E$102&lt;&gt;"")+(Pronostici!$F$3:$F$102&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>SUMPRODUCT(($C$33:$C$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
+        <f>SUMPRODUCT(($C$33:$C$42=$H$33:$H$42)*($H$33:$H$42&gt;0)*($B$33:$B$42="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1625,19 +1625,19 @@
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>SUM(Punti!$E$3:$E$92)</f>
+        <f>SUM(Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$92,Config!$D$7)+COUNTIF(Punti!$E$3:$E$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$102,Config!$D$7)+COUNTIF(Punti!$E$3:$E$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F13" s="30">
-        <f>SUMPRODUCT(((Pronostici!$H$3:$H$92&lt;&gt;"")+(Pronostici!$I$3:$I$92&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$H$3:$H$102&lt;&gt;"")+(Pronostici!$I$3:$I$102&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G13" s="31">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="H13" s="30">
-        <f>SUMPRODUCT(($D$33:$D$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
+        <f>SUMPRODUCT(($D$33:$D$42=$H$33:$H$42)*($H$33:$H$42&gt;0)*($B$33:$B$42="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1659,19 @@
         <v/>
       </c>
       <c r="C14" s="24">
-        <f>SUM(Punti!$F$3:$F$92)</f>
+        <f>SUM(Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$92,Config!$D$7)+COUNTIF(Punti!$F$3:$F$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$102,Config!$D$7)+COUNTIF(Punti!$F$3:$F$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>SUMPRODUCT(((Pronostici!$K$3:$K$92&lt;&gt;"")+(Pronostici!$L$3:$L$92&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$K$3:$K$102&lt;&gt;"")+(Pronostici!$L$3:$L$102&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>SUMPRODUCT(($E$33:$E$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
+        <f>SUMPRODUCT(($E$33:$E$42=$H$33:$H$42)*($H$33:$H$42&gt;0)*($B$33:$B$42="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1693,19 +1693,19 @@
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>SUM(Punti!$G$3:$G$92)</f>
+        <f>SUM(Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$92,Config!$D$7)+COUNTIF(Punti!$G$3:$G$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$102,Config!$D$7)+COUNTIF(Punti!$G$3:$G$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F15" s="30">
-        <f>SUMPRODUCT(((Pronostici!$N$3:$N$92&lt;&gt;"")+(Pronostici!$O$3:$O$92&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$N$3:$N$102&lt;&gt;"")+(Pronostici!$O$3:$O$102&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G15" s="31">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="H15" s="30">
-        <f>SUMPRODUCT(($F$33:$F$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
+        <f>SUMPRODUCT(($F$33:$F$42=$H$33:$H$42)*($H$33:$H$42&gt;0)*($B$33:$B$42="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1727,19 +1727,19 @@
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>SUM(Punti!$H$3:$H$92)</f>
+        <f>SUM(Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$92,Config!$D$7)+COUNTIF(Punti!$H$3:$H$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$102,Config!$D$7)+COUNTIF(Punti!$H$3:$H$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$92,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$102,Config!$D$6)</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$92&lt;&gt;"")+(Pronostici!$R$3:$R$92&lt;&gt;""))*1&gt;0)</f>
+        <f>SUMPRODUCT(((Pronostici!$Q$3:$Q$102&lt;&gt;"")+(Pronostici!$R$3:$R$102&lt;&gt;""))*1&gt;0)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>SUMPRODUCT(($G$33:$G$41=$H$33:$H$41)*($H$33:$H$41&gt;0)*($B$33:$B$41="Completata"))</f>
+        <f>SUMPRODUCT(($G$33:$G$42=$H$33:$H$42)*($H$33:$H$42&gt;0)*($B$33:$B$42="Completata"))</f>
         <v/>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         <v/>
       </c>
       <c r="C20" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($C$33:$C$42,MATCH($L$7,$A$33:$A$42,0)),"-"))</f>
         <v/>
       </c>
       <c r="D20" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($C$33:$C$42,MATCH($L$7,$A$33:$A$42,0)),0)=IFERROR(INDEX($H$33:$H$42,MATCH($L$7,$A$33:$A$42,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E20" s="41" t="n"/>
       <c r="K20" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(1,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L20" s="43" t="n"/>
@@ -1826,7 +1826,7 @@
         <v/>
       </c>
       <c r="O20" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$E$3:$E$92&lt;&gt;"")+(Pronostici!$F$3:$F$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$102=$L$8)*(((Pronostici!$E$3:$E$102&lt;&gt;"")+(Pronostici!$F$3:$F$102&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1836,16 +1836,16 @@
         <v/>
       </c>
       <c r="C21" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($D$33:$D$42,MATCH($L$7,$A$33:$A$42,0)),"-"))</f>
         <v/>
       </c>
       <c r="D21" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($D$33:$D$42,MATCH($L$7,$A$33:$A$42,0)),0)=IFERROR(INDEX($H$33:$H$42,MATCH($L$7,$A$33:$A$42,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E21" s="41" t="n"/>
       <c r="K21" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(2,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L21" s="47" t="n"/>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="O21" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$H$3:$H$92&lt;&gt;"")+(Pronostici!$I$3:$I$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$102=$L$8)*(((Pronostici!$H$3:$H$102&lt;&gt;"")+(Pronostici!$I$3:$I$102&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v/>
       </c>
       <c r="C22" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($E$33:$E$42,MATCH($L$7,$A$33:$A$42,0)),"-"))</f>
         <v/>
       </c>
       <c r="D22" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($E$33:$E$42,MATCH($L$7,$A$33:$A$42,0)),0)=IFERROR(INDEX($H$33:$H$42,MATCH($L$7,$A$33:$A$42,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E22" s="41" t="n"/>
       <c r="K22" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(3,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L22" s="43" t="n"/>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="O22" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$K$3:$K$92&lt;&gt;"")+(Pronostici!$L$3:$L$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$102=$L$8)*(((Pronostici!$K$3:$K$102&lt;&gt;"")+(Pronostici!$L$3:$L$102&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1894,16 +1894,16 @@
         <v/>
       </c>
       <c r="C23" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($F$33:$F$42,MATCH($L$7,$A$33:$A$42,0)),"-"))</f>
         <v/>
       </c>
       <c r="D23" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($F$33:$F$42,MATCH($L$7,$A$33:$A$42,0)),0)=IFERROR(INDEX($H$33:$H$42,MATCH($L$7,$A$33:$A$42,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E23" s="41" t="n"/>
       <c r="K23" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(4,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L23" s="47" t="n"/>
@@ -1913,7 +1913,7 @@
         <v/>
       </c>
       <c r="O23" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$N$3:$N$92&lt;&gt;"")+(Pronostici!$O$3:$O$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$102=$L$8)*(((Pronostici!$N$3:$N$102&lt;&gt;"")+(Pronostici!$O$3:$O$102&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
@@ -1923,16 +1923,16 @@
         <v/>
       </c>
       <c r="C24" s="24">
-        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$41,MATCH($L$7,$A$33:$A$41,0)),"-"))</f>
+        <f>IF($L$7="-","-",IFERROR(INDEX($G$33:$G$42,MATCH($L$7,$A$33:$A$42,0)),"-"))</f>
         <v/>
       </c>
       <c r="D24" s="40">
-        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$41,MATCH($L$7,$A$33:$A$41,0)),0)=IFERROR(INDEX($H$33:$H$41,MATCH($L$7,$A$33:$A$41,0)),-1),"RE DELLA GIORNATA",""))</f>
+        <f>IF($L$7="-","",IF(IFERROR(INDEX($G$33:$G$42,MATCH($L$7,$A$33:$A$42,0)),0)=IFERROR(INDEX($H$33:$H$42,MATCH($L$7,$A$33:$A$42,0)),-1),"RE DELLA GIORNATA",""))</f>
         <v/>
       </c>
       <c r="E24" s="41" t="n"/>
       <c r="K24" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(5,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L24" s="43" t="n"/>
@@ -1942,13 +1942,13 @@
         <v/>
       </c>
       <c r="O24" s="45">
-        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$92=$L$8)*(((Pronostici!$Q$3:$Q$92&lt;&gt;"")+(Pronostici!$R$3:$R$92&lt;&gt;""))&gt;0))&amp;"/10")</f>
+        <f>IF($L$8="-","-",SUMPRODUCT((Pronostici!$B$3:$B$102=$L$8)*(((Pronostici!$Q$3:$Q$102&lt;&gt;"")+(Pronostici!$R$3:$R$102&lt;&gt;""))&gt;0))&amp;"/10")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(6,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L25" s="47" t="n"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="26">
       <c r="K26" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(7,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L26" s="43" t="n"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="27">
       <c r="K27" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(8,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L27" s="47" t="n"/>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="28">
       <c r="K28" s="42">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(9,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L28" s="43" t="n"/>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="29">
       <c r="K29" s="46">
-        <f>IFERROR(INDEX(Partite!$E$3:$E$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$92,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$92,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$92,0)),"-")</f>
+        <f>IFERROR(INDEX(Partite!$E$3:$E$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$102,0))&amp;"   -   "&amp;INDEX(Partite!$F$3:$F$102,MATCH("G"&amp;TEXT($L$8,"00")&amp;"-"&amp;TEXT(10,"00"),Partite!$A$3:$A$102,0)),"-")</f>
         <v/>
       </c>
       <c r="L29" s="47" t="n"/>
@@ -2070,27 +2070,27 @@
         <v>2</v>
       </c>
       <c r="B33" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A33,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A33,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A33,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A33,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A33,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A33,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A33,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A33,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A33,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A33,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A33,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H33" s="61">
@@ -2127,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="B34" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A34,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A34,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A34,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A34,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A34,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A34,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A34,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A34,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A34,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A34,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A34,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H34" s="61">
@@ -2184,27 +2184,27 @@
         <v>4</v>
       </c>
       <c r="B35" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A35,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A35,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A35,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A35,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A35,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A35,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A35,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A35,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A35,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G35" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A35,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A35,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H35" s="61">
@@ -2241,27 +2241,27 @@
         <v>5</v>
       </c>
       <c r="B36" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A36,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A36,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A36,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A36,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A36,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A36,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A36,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A36,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A36,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A36,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A36,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H36" s="61">
@@ -2298,27 +2298,27 @@
         <v>6</v>
       </c>
       <c r="B37" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A37,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A37,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A37,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A37,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A37,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A37,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A37,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A37,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A37,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A37,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A37,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H37" s="61">
@@ -2355,27 +2355,27 @@
         <v>7</v>
       </c>
       <c r="B38" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A38,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A38,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A38,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A38,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A38,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A38,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A38,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A38,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A38,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G38" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A38,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A38,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H38" s="61">
@@ -2412,27 +2412,27 @@
         <v>8</v>
       </c>
       <c r="B39" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A39,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A39,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A39,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A39,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A39,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A39,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A39,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A39,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A39,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G39" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A39,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A39,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H39" s="61">
@@ -2469,27 +2469,27 @@
         <v>9</v>
       </c>
       <c r="B40" s="47">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A40,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A40,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A40,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A40,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A40,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A40,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A40,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A40,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A40,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G40" s="30">
-        <f>SUMIF(Punti!$B$3:$B$92,$A40,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A40,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H40" s="61">
@@ -2526,27 +2526,27 @@
         <v>10</v>
       </c>
       <c r="B41" s="43">
-        <f>IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$E$3:$E$92,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$K$3:$K$92,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$K$3:$K$92,"Giocata")=COUNTIFS(Partite!$B$3:$B$92,$A41,Partite!$E$3:$E$92,"&lt;&gt;"),"Completata","In corso")))</f>
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A41,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A41,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A41,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A41,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
         <v/>
       </c>
       <c r="C41" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$D$3:$D$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A41,Punti!$D$3:$D$102)</f>
         <v/>
       </c>
       <c r="D41" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$E$3:$E$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A41,Punti!$E$3:$E$102)</f>
         <v/>
       </c>
       <c r="E41" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$F$3:$F$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A41,Punti!$F$3:$F$102)</f>
         <v/>
       </c>
       <c r="F41" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$G$3:$G$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A41,Punti!$G$3:$G$102)</f>
         <v/>
       </c>
       <c r="G41" s="25">
-        <f>SUMIF(Punti!$B$3:$B$92,$A41,Punti!$H$3:$H$92)</f>
+        <f>SUMIF(Punti!$B$3:$B$102,$A41,Punti!$H$3:$H$102)</f>
         <v/>
       </c>
       <c r="H41" s="61">
@@ -2575,6 +2575,63 @@
       </c>
       <c r="V41" s="63">
         <f>V40+G41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B42" s="47">
+        <f>IF(COUNTIFS(Partite!$B$3:$B$102,$A42,Partite!$E$3:$E$102,"&lt;&gt;")=0,"Calendario mancante",IF(COUNTIFS(Partite!$B$3:$B$102,$A42,Partite!$K$3:$K$102,"Giocata")=0,"Non giocata",IF(COUNTIFS(Partite!$B$3:$B$102,$A42,Partite!$K$3:$K$102,"Giocata")=COUNTIFS(Partite!$B$3:$B$102,$A42,Partite!$E$3:$E$102,"&lt;&gt;"),"Completata","In corso")))</f>
+        <v/>
+      </c>
+      <c r="C42" s="30">
+        <f>SUMIF(Punti!$B$3:$B$102,$A42,Punti!$D$3:$D$102)</f>
+        <v/>
+      </c>
+      <c r="D42" s="30">
+        <f>SUMIF(Punti!$B$3:$B$102,$A42,Punti!$E$3:$E$102)</f>
+        <v/>
+      </c>
+      <c r="E42" s="30">
+        <f>SUMIF(Punti!$B$3:$B$102,$A42,Punti!$F$3:$F$102)</f>
+        <v/>
+      </c>
+      <c r="F42" s="30">
+        <f>SUMIF(Punti!$B$3:$B$102,$A42,Punti!$G$3:$G$102)</f>
+        <v/>
+      </c>
+      <c r="G42" s="30">
+        <f>SUMIF(Punti!$B$3:$B$102,$A42,Punti!$H$3:$H$102)</f>
+        <v/>
+      </c>
+      <c r="H42" s="61">
+        <f>MAX($C42:$G42)</f>
+        <v/>
+      </c>
+      <c r="I42" s="64">
+        <f>IF($H42&lt;=0,"-",INDEX($C$32:$G$32,MATCH($H42,$C42:$G42,0))&amp;IF(COUNTIF($C42:$G42,$H42)&gt;1," (a pari)","")&amp;IF($B42="Completata",""," - in corso"))</f>
+        <v/>
+      </c>
+      <c r="R42" s="63">
+        <f>R41+C42</f>
+        <v/>
+      </c>
+      <c r="S42" s="63">
+        <f>S41+D42</f>
+        <v/>
+      </c>
+      <c r="T42" s="63">
+        <f>T41+E42</f>
+        <v/>
+      </c>
+      <c r="U42" s="63">
+        <f>U41+F42</f>
+        <v/>
+      </c>
+      <c r="V42" s="63">
+        <f>V41+G42</f>
         <v/>
       </c>
     </row>
@@ -2621,7 +2678,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:G41">
+  <conditionalFormatting sqref="C33:G42">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2643,7 +2700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6562,8 +6619,12 @@
           <t>Atalanta</t>
         </is>
       </c>
-      <c r="G82" s="71" t="n"/>
-      <c r="H82" s="71" t="n"/>
+      <c r="G82" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H82" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I82" s="76">
         <f>IF(OR($G82="",$H82=""),"",IF($G82&gt;$H82,"1",IF($G82=$H82,"X","2")))</f>
         <v/>
@@ -7017,14 +7078,454 @@
         <v/>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="74" t="inlineStr">
+        <is>
+          <t>G11-01</t>
+        </is>
+      </c>
+      <c r="B93" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C93" s="30" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="D93" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E93" s="75" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="F93" s="75" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="G93" s="71" t="n"/>
+      <c r="H93" s="71" t="n"/>
+      <c r="I93" s="76">
+        <f>IF(OR($G93="",$H93=""),"",IF($G93&gt;$H93,"1",IF($G93=$H93,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J93" s="30">
+        <f>IF(OR($G93="",$H93=""),"",$G93&amp;"-"&amp;$H93)</f>
+        <v/>
+      </c>
+      <c r="K93" s="77">
+        <f>IF($E93="","Calendario da inserire",IF(OR($G93="",$H93=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="74" t="inlineStr">
+        <is>
+          <t>G11-02</t>
+        </is>
+      </c>
+      <c r="B94" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C94" s="30" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="D94" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E94" s="75" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="F94" s="75" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="G94" s="71" t="n"/>
+      <c r="H94" s="71" t="n"/>
+      <c r="I94" s="76">
+        <f>IF(OR($G94="",$H94=""),"",IF($G94&gt;$H94,"1",IF($G94=$H94,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J94" s="30">
+        <f>IF(OR($G94="",$H94=""),"",$G94&amp;"-"&amp;$H94)</f>
+        <v/>
+      </c>
+      <c r="K94" s="77">
+        <f>IF($E94="","Calendario da inserire",IF(OR($G94="",$H94=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="74" t="inlineStr">
+        <is>
+          <t>G11-03</t>
+        </is>
+      </c>
+      <c r="B95" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C95" s="30" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="D95" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E95" s="75" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="F95" s="75" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="G95" s="71" t="n"/>
+      <c r="H95" s="71" t="n"/>
+      <c r="I95" s="76">
+        <f>IF(OR($G95="",$H95=""),"",IF($G95&gt;$H95,"1",IF($G95=$H95,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J95" s="30">
+        <f>IF(OR($G95="",$H95=""),"",$G95&amp;"-"&amp;$H95)</f>
+        <v/>
+      </c>
+      <c r="K95" s="77">
+        <f>IF($E95="","Calendario da inserire",IF(OR($G95="",$H95=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="74" t="inlineStr">
+        <is>
+          <t>G11-04</t>
+        </is>
+      </c>
+      <c r="B96" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C96" s="30" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="D96" s="30" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E96" s="75" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="F96" s="75" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="G96" s="71" t="n"/>
+      <c r="H96" s="71" t="n"/>
+      <c r="I96" s="76">
+        <f>IF(OR($G96="",$H96=""),"",IF($G96&gt;$H96,"1",IF($G96=$H96,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J96" s="30">
+        <f>IF(OR($G96="",$H96=""),"",$G96&amp;"-"&amp;$H96)</f>
+        <v/>
+      </c>
+      <c r="K96" s="77">
+        <f>IF($E96="","Calendario da inserire",IF(OR($G96="",$H96=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="74" t="inlineStr">
+        <is>
+          <t>G11-05</t>
+        </is>
+      </c>
+      <c r="B97" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C97" s="30" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="D97" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E97" s="75" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="F97" s="75" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="G97" s="71" t="n"/>
+      <c r="H97" s="71" t="n"/>
+      <c r="I97" s="76">
+        <f>IF(OR($G97="",$H97=""),"",IF($G97&gt;$H97,"1",IF($G97=$H97,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J97" s="30">
+        <f>IF(OR($G97="",$H97=""),"",$G97&amp;"-"&amp;$H97)</f>
+        <v/>
+      </c>
+      <c r="K97" s="77">
+        <f>IF($E97="","Calendario da inserire",IF(OR($G97="",$H97=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="74" t="inlineStr">
+        <is>
+          <t>G11-06</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E98" s="75" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="F98" s="75" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="G98" s="71" t="n"/>
+      <c r="H98" s="71" t="n"/>
+      <c r="I98" s="76">
+        <f>IF(OR($G98="",$H98=""),"",IF($G98&gt;$H98,"1",IF($G98=$H98,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J98" s="30">
+        <f>IF(OR($G98="",$H98=""),"",$G98&amp;"-"&amp;$H98)</f>
+        <v/>
+      </c>
+      <c r="K98" s="77">
+        <f>IF($E98="","Calendario da inserire",IF(OR($G98="",$H98=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="74" t="inlineStr">
+        <is>
+          <t>G11-07</t>
+        </is>
+      </c>
+      <c r="B99" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C99" s="30" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="D99" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E99" s="75" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="F99" s="75" t="inlineStr">
+        <is>
+          <t>Milan</t>
+        </is>
+      </c>
+      <c r="G99" s="71" t="n"/>
+      <c r="H99" s="71" t="n"/>
+      <c r="I99" s="76">
+        <f>IF(OR($G99="",$H99=""),"",IF($G99&gt;$H99,"1",IF($G99=$H99,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J99" s="30">
+        <f>IF(OR($G99="",$H99=""),"",$G99&amp;"-"&amp;$H99)</f>
+        <v/>
+      </c>
+      <c r="K99" s="77">
+        <f>IF($E99="","Calendario da inserire",IF(OR($G99="",$H99=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="74" t="inlineStr">
+        <is>
+          <t>G11-08</t>
+        </is>
+      </c>
+      <c r="B100" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C100" s="30" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="D100" s="30" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E100" s="75" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="F100" s="75" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="G100" s="71" t="n"/>
+      <c r="H100" s="71" t="n"/>
+      <c r="I100" s="76">
+        <f>IF(OR($G100="",$H100=""),"",IF($G100&gt;$H100,"1",IF($G100=$H100,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J100" s="30">
+        <f>IF(OR($G100="",$H100=""),"",$G100&amp;"-"&amp;$H100)</f>
+        <v/>
+      </c>
+      <c r="K100" s="77">
+        <f>IF($E100="","Calendario da inserire",IF(OR($G100="",$H100=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="74" t="inlineStr">
+        <is>
+          <t>G11-09</t>
+        </is>
+      </c>
+      <c r="B101" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C101" s="30" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="D101" s="30" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E101" s="75" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="F101" s="75" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="G101" s="71" t="n"/>
+      <c r="H101" s="71" t="n"/>
+      <c r="I101" s="76">
+        <f>IF(OR($G101="",$H101=""),"",IF($G101&gt;$H101,"1",IF($G101=$H101,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J101" s="30">
+        <f>IF(OR($G101="",$H101=""),"",$G101&amp;"-"&amp;$H101)</f>
+        <v/>
+      </c>
+      <c r="K101" s="77">
+        <f>IF($E101="","Calendario da inserire",IF(OR($G101="",$H101=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="74" t="inlineStr">
+        <is>
+          <t>G11-10</t>
+        </is>
+      </c>
+      <c r="B102" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="C102" s="30" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="D102" s="30" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="E102" s="75" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="F102" s="75" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="G102" s="71" t="n"/>
+      <c r="H102" s="71" t="n"/>
+      <c r="I102" s="76">
+        <f>IF(OR($G102="",$H102=""),"",IF($G102&gt;$H102,"1",IF($G102=$H102,"X","2")))</f>
+        <v/>
+      </c>
+      <c r="J102" s="30">
+        <f>IF(OR($G102="",$H102=""),"",$G102&amp;"-"&amp;$H102)</f>
+        <v/>
+      </c>
+      <c r="K102" s="77">
+        <f>IF($E102="","Calendario da inserire",IF(OR($G102="",$H102=""),"Da giocare","Giocata"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K92"/>
+  <autoFilter ref="A2:K102"/>
   <mergeCells count="3">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K3:K92">
+  <conditionalFormatting sqref="K3:K102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Giocata"</formula>
     </cfRule>
@@ -7040,7 +7541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S92"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13371,8 +13872,338 @@
       <c r="R92" s="71" t="n"/>
       <c r="S92" s="71" t="n"/>
     </row>
+    <row r="93">
+      <c r="A93" s="74">
+        <f>Partite!$A93</f>
+        <v/>
+      </c>
+      <c r="B93" s="30">
+        <f>Partite!$B93</f>
+        <v/>
+      </c>
+      <c r="C93" s="75">
+        <f>IF(Partite!$E93="","",Partite!$E93)</f>
+        <v/>
+      </c>
+      <c r="D93" s="75">
+        <f>IF(Partite!$F93="","",Partite!$F93)</f>
+        <v/>
+      </c>
+      <c r="E93" s="71" t="n"/>
+      <c r="F93" s="71" t="n"/>
+      <c r="G93" s="71" t="n"/>
+      <c r="H93" s="71" t="n"/>
+      <c r="I93" s="71" t="n"/>
+      <c r="J93" s="71" t="n"/>
+      <c r="K93" s="71" t="n"/>
+      <c r="L93" s="71" t="n"/>
+      <c r="M93" s="71" t="n"/>
+      <c r="N93" s="71" t="n"/>
+      <c r="O93" s="71" t="n"/>
+      <c r="P93" s="71" t="n"/>
+      <c r="Q93" s="71" t="n"/>
+      <c r="R93" s="71" t="n"/>
+      <c r="S93" s="71" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="74">
+        <f>Partite!$A94</f>
+        <v/>
+      </c>
+      <c r="B94" s="30">
+        <f>Partite!$B94</f>
+        <v/>
+      </c>
+      <c r="C94" s="75">
+        <f>IF(Partite!$E94="","",Partite!$E94)</f>
+        <v/>
+      </c>
+      <c r="D94" s="75">
+        <f>IF(Partite!$F94="","",Partite!$F94)</f>
+        <v/>
+      </c>
+      <c r="E94" s="71" t="n"/>
+      <c r="F94" s="71" t="n"/>
+      <c r="G94" s="71" t="n"/>
+      <c r="H94" s="71" t="n"/>
+      <c r="I94" s="71" t="n"/>
+      <c r="J94" s="71" t="n"/>
+      <c r="K94" s="71" t="n"/>
+      <c r="L94" s="71" t="n"/>
+      <c r="M94" s="71" t="n"/>
+      <c r="N94" s="71" t="n"/>
+      <c r="O94" s="71" t="n"/>
+      <c r="P94" s="71" t="n"/>
+      <c r="Q94" s="71" t="n"/>
+      <c r="R94" s="71" t="n"/>
+      <c r="S94" s="71" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="74">
+        <f>Partite!$A95</f>
+        <v/>
+      </c>
+      <c r="B95" s="30">
+        <f>Partite!$B95</f>
+        <v/>
+      </c>
+      <c r="C95" s="75">
+        <f>IF(Partite!$E95="","",Partite!$E95)</f>
+        <v/>
+      </c>
+      <c r="D95" s="75">
+        <f>IF(Partite!$F95="","",Partite!$F95)</f>
+        <v/>
+      </c>
+      <c r="E95" s="71" t="n"/>
+      <c r="F95" s="71" t="n"/>
+      <c r="G95" s="71" t="n"/>
+      <c r="H95" s="71" t="n"/>
+      <c r="I95" s="71" t="n"/>
+      <c r="J95" s="71" t="n"/>
+      <c r="K95" s="71" t="n"/>
+      <c r="L95" s="71" t="n"/>
+      <c r="M95" s="71" t="n"/>
+      <c r="N95" s="71" t="n"/>
+      <c r="O95" s="71" t="n"/>
+      <c r="P95" s="71" t="n"/>
+      <c r="Q95" s="71" t="n"/>
+      <c r="R95" s="71" t="n"/>
+      <c r="S95" s="71" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="74">
+        <f>Partite!$A96</f>
+        <v/>
+      </c>
+      <c r="B96" s="30">
+        <f>Partite!$B96</f>
+        <v/>
+      </c>
+      <c r="C96" s="75">
+        <f>IF(Partite!$E96="","",Partite!$E96)</f>
+        <v/>
+      </c>
+      <c r="D96" s="75">
+        <f>IF(Partite!$F96="","",Partite!$F96)</f>
+        <v/>
+      </c>
+      <c r="E96" s="71" t="n"/>
+      <c r="F96" s="71" t="n"/>
+      <c r="G96" s="71" t="n"/>
+      <c r="H96" s="71" t="n"/>
+      <c r="I96" s="71" t="n"/>
+      <c r="J96" s="71" t="n"/>
+      <c r="K96" s="71" t="n"/>
+      <c r="L96" s="71" t="n"/>
+      <c r="M96" s="71" t="n"/>
+      <c r="N96" s="71" t="n"/>
+      <c r="O96" s="71" t="n"/>
+      <c r="P96" s="71" t="n"/>
+      <c r="Q96" s="71" t="n"/>
+      <c r="R96" s="71" t="n"/>
+      <c r="S96" s="71" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="74">
+        <f>Partite!$A97</f>
+        <v/>
+      </c>
+      <c r="B97" s="30">
+        <f>Partite!$B97</f>
+        <v/>
+      </c>
+      <c r="C97" s="75">
+        <f>IF(Partite!$E97="","",Partite!$E97)</f>
+        <v/>
+      </c>
+      <c r="D97" s="75">
+        <f>IF(Partite!$F97="","",Partite!$F97)</f>
+        <v/>
+      </c>
+      <c r="E97" s="71" t="n"/>
+      <c r="F97" s="71" t="n"/>
+      <c r="G97" s="71" t="n"/>
+      <c r="H97" s="71" t="n"/>
+      <c r="I97" s="71" t="n"/>
+      <c r="J97" s="71" t="n"/>
+      <c r="K97" s="71" t="n"/>
+      <c r="L97" s="71" t="n"/>
+      <c r="M97" s="71" t="n"/>
+      <c r="N97" s="71" t="n"/>
+      <c r="O97" s="71" t="n"/>
+      <c r="P97" s="71" t="n"/>
+      <c r="Q97" s="71" t="n"/>
+      <c r="R97" s="71" t="n"/>
+      <c r="S97" s="71" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="74">
+        <f>Partite!$A98</f>
+        <v/>
+      </c>
+      <c r="B98" s="30">
+        <f>Partite!$B98</f>
+        <v/>
+      </c>
+      <c r="C98" s="75">
+        <f>IF(Partite!$E98="","",Partite!$E98)</f>
+        <v/>
+      </c>
+      <c r="D98" s="75">
+        <f>IF(Partite!$F98="","",Partite!$F98)</f>
+        <v/>
+      </c>
+      <c r="E98" s="71" t="n"/>
+      <c r="F98" s="71" t="n"/>
+      <c r="G98" s="71" t="n"/>
+      <c r="H98" s="71" t="n"/>
+      <c r="I98" s="71" t="n"/>
+      <c r="J98" s="71" t="n"/>
+      <c r="K98" s="71" t="n"/>
+      <c r="L98" s="71" t="n"/>
+      <c r="M98" s="71" t="n"/>
+      <c r="N98" s="71" t="n"/>
+      <c r="O98" s="71" t="n"/>
+      <c r="P98" s="71" t="n"/>
+      <c r="Q98" s="71" t="n"/>
+      <c r="R98" s="71" t="n"/>
+      <c r="S98" s="71" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="74">
+        <f>Partite!$A99</f>
+        <v/>
+      </c>
+      <c r="B99" s="30">
+        <f>Partite!$B99</f>
+        <v/>
+      </c>
+      <c r="C99" s="75">
+        <f>IF(Partite!$E99="","",Partite!$E99)</f>
+        <v/>
+      </c>
+      <c r="D99" s="75">
+        <f>IF(Partite!$F99="","",Partite!$F99)</f>
+        <v/>
+      </c>
+      <c r="E99" s="71" t="n"/>
+      <c r="F99" s="71" t="n"/>
+      <c r="G99" s="71" t="n"/>
+      <c r="H99" s="71" t="n"/>
+      <c r="I99" s="71" t="n"/>
+      <c r="J99" s="71" t="n"/>
+      <c r="K99" s="71" t="n"/>
+      <c r="L99" s="71" t="n"/>
+      <c r="M99" s="71" t="n"/>
+      <c r="N99" s="71" t="n"/>
+      <c r="O99" s="71" t="n"/>
+      <c r="P99" s="71" t="n"/>
+      <c r="Q99" s="71" t="n"/>
+      <c r="R99" s="71" t="n"/>
+      <c r="S99" s="71" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="74">
+        <f>Partite!$A100</f>
+        <v/>
+      </c>
+      <c r="B100" s="30">
+        <f>Partite!$B100</f>
+        <v/>
+      </c>
+      <c r="C100" s="75">
+        <f>IF(Partite!$E100="","",Partite!$E100)</f>
+        <v/>
+      </c>
+      <c r="D100" s="75">
+        <f>IF(Partite!$F100="","",Partite!$F100)</f>
+        <v/>
+      </c>
+      <c r="E100" s="71" t="n"/>
+      <c r="F100" s="71" t="n"/>
+      <c r="G100" s="71" t="n"/>
+      <c r="H100" s="71" t="n"/>
+      <c r="I100" s="71" t="n"/>
+      <c r="J100" s="71" t="n"/>
+      <c r="K100" s="71" t="n"/>
+      <c r="L100" s="71" t="n"/>
+      <c r="M100" s="71" t="n"/>
+      <c r="N100" s="71" t="n"/>
+      <c r="O100" s="71" t="n"/>
+      <c r="P100" s="71" t="n"/>
+      <c r="Q100" s="71" t="n"/>
+      <c r="R100" s="71" t="n"/>
+      <c r="S100" s="71" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="74">
+        <f>Partite!$A101</f>
+        <v/>
+      </c>
+      <c r="B101" s="30">
+        <f>Partite!$B101</f>
+        <v/>
+      </c>
+      <c r="C101" s="75">
+        <f>IF(Partite!$E101="","",Partite!$E101)</f>
+        <v/>
+      </c>
+      <c r="D101" s="75">
+        <f>IF(Partite!$F101="","",Partite!$F101)</f>
+        <v/>
+      </c>
+      <c r="E101" s="71" t="n"/>
+      <c r="F101" s="71" t="n"/>
+      <c r="G101" s="71" t="n"/>
+      <c r="H101" s="71" t="n"/>
+      <c r="I101" s="71" t="n"/>
+      <c r="J101" s="71" t="n"/>
+      <c r="K101" s="71" t="n"/>
+      <c r="L101" s="71" t="n"/>
+      <c r="M101" s="71" t="n"/>
+      <c r="N101" s="71" t="n"/>
+      <c r="O101" s="71" t="n"/>
+      <c r="P101" s="71" t="n"/>
+      <c r="Q101" s="71" t="n"/>
+      <c r="R101" s="71" t="n"/>
+      <c r="S101" s="71" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="74">
+        <f>Partite!$A102</f>
+        <v/>
+      </c>
+      <c r="B102" s="30">
+        <f>Partite!$B102</f>
+        <v/>
+      </c>
+      <c r="C102" s="75">
+        <f>IF(Partite!$E102="","",Partite!$E102)</f>
+        <v/>
+      </c>
+      <c r="D102" s="75">
+        <f>IF(Partite!$F102="","",Partite!$F102)</f>
+        <v/>
+      </c>
+      <c r="E102" s="71" t="n"/>
+      <c r="F102" s="71" t="n"/>
+      <c r="G102" s="71" t="n"/>
+      <c r="H102" s="71" t="n"/>
+      <c r="I102" s="71" t="n"/>
+      <c r="J102" s="71" t="n"/>
+      <c r="K102" s="71" t="n"/>
+      <c r="L102" s="71" t="n"/>
+      <c r="M102" s="71" t="n"/>
+      <c r="N102" s="71" t="n"/>
+      <c r="O102" s="71" t="n"/>
+      <c r="P102" s="71" t="n"/>
+      <c r="Q102" s="71" t="n"/>
+      <c r="R102" s="71" t="n"/>
+      <c r="S102" s="71" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:D92"/>
+  <autoFilter ref="A2:D102"/>
   <mergeCells count="6">
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A1:D1"/>
@@ -13382,7 +14213,7 @@
     <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 K92 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 N83 N84 N85 N86 N87 N88 N89 N90 N91 N92 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82 Q83 Q84 Q85 Q86 Q87 Q88 Q89 Q90 Q91 Q92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 K92 K93 K94 K95 K96 K97 K98 K99 K100 K101 K102 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 N83 N84 N85 N86 N87 N88 N89 N90 N91 N92 N93 N94 N95 N96 N97 N98 N99 N100 N101 N102 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82 Q83 Q84 Q85 Q86 Q87 Q88 Q89 Q90 Q91 Q92 Q93 Q94 Q95 Q96 Q97 Q98 Q99 Q100 Q101 Q102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Segno non valido" error="Scrivi 1 (vince la casa), X (pareggio) oppure 2 (vince l'ospite)." type="list">
       <formula1>"1,X,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13397,7 +14228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -18351,11 +19182,551 @@
         <v/>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="74">
+        <f>Partite!$A93</f>
+        <v/>
+      </c>
+      <c r="B93" s="30">
+        <f>Partite!$B93</f>
+        <v/>
+      </c>
+      <c r="C93" s="47">
+        <f>IF(Partite!$E93="","",Partite!$E93&amp;"  -  "&amp;Partite!$F93)</f>
+        <v/>
+      </c>
+      <c r="D93" s="27">
+        <f>IF(Partite!$K93&lt;&gt;"Giocata","",IF(AND(Pronostici!$F93&lt;&gt;"",Pronostici!$G93&lt;&gt;"",Pronostici!$F93=Partite!$G93,Pronostici!$G93=Partite!$H93),Config!$D$6,IF(AND($J93&lt;&gt;"",$J93=Partite!$I93),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E93" s="27">
+        <f>IF(Partite!$K93&lt;&gt;"Giocata","",IF(AND(Pronostici!$I93&lt;&gt;"",Pronostici!$J93&lt;&gt;"",Pronostici!$I93=Partite!$G93,Pronostici!$J93=Partite!$H93),Config!$D$6,IF(AND($K93&lt;&gt;"",$K93=Partite!$I93),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F93" s="27">
+        <f>IF(Partite!$K93&lt;&gt;"Giocata","",IF(AND(Pronostici!$L93&lt;&gt;"",Pronostici!$M93&lt;&gt;"",Pronostici!$L93=Partite!$G93,Pronostici!$M93=Partite!$H93),Config!$D$6,IF(AND($L93&lt;&gt;"",$L93=Partite!$I93),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G93" s="27">
+        <f>IF(Partite!$K93&lt;&gt;"Giocata","",IF(AND(Pronostici!$O93&lt;&gt;"",Pronostici!$P93&lt;&gt;"",Pronostici!$O93=Partite!$G93,Pronostici!$P93=Partite!$H93),Config!$D$6,IF(AND($M93&lt;&gt;"",$M93=Partite!$I93),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H93" s="27">
+        <f>IF(Partite!$K93&lt;&gt;"Giocata","",IF(AND(Pronostici!$R93&lt;&gt;"",Pronostici!$S93&lt;&gt;"",Pronostici!$R93=Partite!$G93,Pronostici!$S93=Partite!$H93),Config!$D$6,IF(AND($N93&lt;&gt;"",$N93=Partite!$I93),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J93" s="63">
+        <f>IF(Pronostici!$E93&lt;&gt;"",UPPER(Pronostici!$E93),IF(OR(Pronostici!$F93="",Pronostici!$G93=""),"",IF(Pronostici!$F93&gt;Pronostici!$G93,"1",IF(Pronostici!$F93=Pronostici!$G93,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K93" s="63">
+        <f>IF(Pronostici!$H93&lt;&gt;"",UPPER(Pronostici!$H93),IF(OR(Pronostici!$I93="",Pronostici!$J93=""),"",IF(Pronostici!$I93&gt;Pronostici!$J93,"1",IF(Pronostici!$I93=Pronostici!$J93,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L93" s="63">
+        <f>IF(Pronostici!$K93&lt;&gt;"",UPPER(Pronostici!$K93),IF(OR(Pronostici!$L93="",Pronostici!$M93=""),"",IF(Pronostici!$L93&gt;Pronostici!$M93,"1",IF(Pronostici!$L93=Pronostici!$M93,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M93" s="63">
+        <f>IF(Pronostici!$N93&lt;&gt;"",UPPER(Pronostici!$N93),IF(OR(Pronostici!$O93="",Pronostici!$P93=""),"",IF(Pronostici!$O93&gt;Pronostici!$P93,"1",IF(Pronostici!$O93=Pronostici!$P93,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N93" s="63">
+        <f>IF(Pronostici!$Q93&lt;&gt;"",UPPER(Pronostici!$Q93),IF(OR(Pronostici!$R93="",Pronostici!$S93=""),"",IF(Pronostici!$R93&gt;Pronostici!$S93,"1",IF(Pronostici!$R93=Pronostici!$S93,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="74">
+        <f>Partite!$A94</f>
+        <v/>
+      </c>
+      <c r="B94" s="30">
+        <f>Partite!$B94</f>
+        <v/>
+      </c>
+      <c r="C94" s="47">
+        <f>IF(Partite!$E94="","",Partite!$E94&amp;"  -  "&amp;Partite!$F94)</f>
+        <v/>
+      </c>
+      <c r="D94" s="27">
+        <f>IF(Partite!$K94&lt;&gt;"Giocata","",IF(AND(Pronostici!$F94&lt;&gt;"",Pronostici!$G94&lt;&gt;"",Pronostici!$F94=Partite!$G94,Pronostici!$G94=Partite!$H94),Config!$D$6,IF(AND($J94&lt;&gt;"",$J94=Partite!$I94),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E94" s="27">
+        <f>IF(Partite!$K94&lt;&gt;"Giocata","",IF(AND(Pronostici!$I94&lt;&gt;"",Pronostici!$J94&lt;&gt;"",Pronostici!$I94=Partite!$G94,Pronostici!$J94=Partite!$H94),Config!$D$6,IF(AND($K94&lt;&gt;"",$K94=Partite!$I94),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F94" s="27">
+        <f>IF(Partite!$K94&lt;&gt;"Giocata","",IF(AND(Pronostici!$L94&lt;&gt;"",Pronostici!$M94&lt;&gt;"",Pronostici!$L94=Partite!$G94,Pronostici!$M94=Partite!$H94),Config!$D$6,IF(AND($L94&lt;&gt;"",$L94=Partite!$I94),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G94" s="27">
+        <f>IF(Partite!$K94&lt;&gt;"Giocata","",IF(AND(Pronostici!$O94&lt;&gt;"",Pronostici!$P94&lt;&gt;"",Pronostici!$O94=Partite!$G94,Pronostici!$P94=Partite!$H94),Config!$D$6,IF(AND($M94&lt;&gt;"",$M94=Partite!$I94),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H94" s="27">
+        <f>IF(Partite!$K94&lt;&gt;"Giocata","",IF(AND(Pronostici!$R94&lt;&gt;"",Pronostici!$S94&lt;&gt;"",Pronostici!$R94=Partite!$G94,Pronostici!$S94=Partite!$H94),Config!$D$6,IF(AND($N94&lt;&gt;"",$N94=Partite!$I94),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J94" s="63">
+        <f>IF(Pronostici!$E94&lt;&gt;"",UPPER(Pronostici!$E94),IF(OR(Pronostici!$F94="",Pronostici!$G94=""),"",IF(Pronostici!$F94&gt;Pronostici!$G94,"1",IF(Pronostici!$F94=Pronostici!$G94,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K94" s="63">
+        <f>IF(Pronostici!$H94&lt;&gt;"",UPPER(Pronostici!$H94),IF(OR(Pronostici!$I94="",Pronostici!$J94=""),"",IF(Pronostici!$I94&gt;Pronostici!$J94,"1",IF(Pronostici!$I94=Pronostici!$J94,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L94" s="63">
+        <f>IF(Pronostici!$K94&lt;&gt;"",UPPER(Pronostici!$K94),IF(OR(Pronostici!$L94="",Pronostici!$M94=""),"",IF(Pronostici!$L94&gt;Pronostici!$M94,"1",IF(Pronostici!$L94=Pronostici!$M94,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M94" s="63">
+        <f>IF(Pronostici!$N94&lt;&gt;"",UPPER(Pronostici!$N94),IF(OR(Pronostici!$O94="",Pronostici!$P94=""),"",IF(Pronostici!$O94&gt;Pronostici!$P94,"1",IF(Pronostici!$O94=Pronostici!$P94,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N94" s="63">
+        <f>IF(Pronostici!$Q94&lt;&gt;"",UPPER(Pronostici!$Q94),IF(OR(Pronostici!$R94="",Pronostici!$S94=""),"",IF(Pronostici!$R94&gt;Pronostici!$S94,"1",IF(Pronostici!$R94=Pronostici!$S94,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="74">
+        <f>Partite!$A95</f>
+        <v/>
+      </c>
+      <c r="B95" s="30">
+        <f>Partite!$B95</f>
+        <v/>
+      </c>
+      <c r="C95" s="47">
+        <f>IF(Partite!$E95="","",Partite!$E95&amp;"  -  "&amp;Partite!$F95)</f>
+        <v/>
+      </c>
+      <c r="D95" s="27">
+        <f>IF(Partite!$K95&lt;&gt;"Giocata","",IF(AND(Pronostici!$F95&lt;&gt;"",Pronostici!$G95&lt;&gt;"",Pronostici!$F95=Partite!$G95,Pronostici!$G95=Partite!$H95),Config!$D$6,IF(AND($J95&lt;&gt;"",$J95=Partite!$I95),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E95" s="27">
+        <f>IF(Partite!$K95&lt;&gt;"Giocata","",IF(AND(Pronostici!$I95&lt;&gt;"",Pronostici!$J95&lt;&gt;"",Pronostici!$I95=Partite!$G95,Pronostici!$J95=Partite!$H95),Config!$D$6,IF(AND($K95&lt;&gt;"",$K95=Partite!$I95),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F95" s="27">
+        <f>IF(Partite!$K95&lt;&gt;"Giocata","",IF(AND(Pronostici!$L95&lt;&gt;"",Pronostici!$M95&lt;&gt;"",Pronostici!$L95=Partite!$G95,Pronostici!$M95=Partite!$H95),Config!$D$6,IF(AND($L95&lt;&gt;"",$L95=Partite!$I95),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G95" s="27">
+        <f>IF(Partite!$K95&lt;&gt;"Giocata","",IF(AND(Pronostici!$O95&lt;&gt;"",Pronostici!$P95&lt;&gt;"",Pronostici!$O95=Partite!$G95,Pronostici!$P95=Partite!$H95),Config!$D$6,IF(AND($M95&lt;&gt;"",$M95=Partite!$I95),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H95" s="27">
+        <f>IF(Partite!$K95&lt;&gt;"Giocata","",IF(AND(Pronostici!$R95&lt;&gt;"",Pronostici!$S95&lt;&gt;"",Pronostici!$R95=Partite!$G95,Pronostici!$S95=Partite!$H95),Config!$D$6,IF(AND($N95&lt;&gt;"",$N95=Partite!$I95),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J95" s="63">
+        <f>IF(Pronostici!$E95&lt;&gt;"",UPPER(Pronostici!$E95),IF(OR(Pronostici!$F95="",Pronostici!$G95=""),"",IF(Pronostici!$F95&gt;Pronostici!$G95,"1",IF(Pronostici!$F95=Pronostici!$G95,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K95" s="63">
+        <f>IF(Pronostici!$H95&lt;&gt;"",UPPER(Pronostici!$H95),IF(OR(Pronostici!$I95="",Pronostici!$J95=""),"",IF(Pronostici!$I95&gt;Pronostici!$J95,"1",IF(Pronostici!$I95=Pronostici!$J95,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L95" s="63">
+        <f>IF(Pronostici!$K95&lt;&gt;"",UPPER(Pronostici!$K95),IF(OR(Pronostici!$L95="",Pronostici!$M95=""),"",IF(Pronostici!$L95&gt;Pronostici!$M95,"1",IF(Pronostici!$L95=Pronostici!$M95,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M95" s="63">
+        <f>IF(Pronostici!$N95&lt;&gt;"",UPPER(Pronostici!$N95),IF(OR(Pronostici!$O95="",Pronostici!$P95=""),"",IF(Pronostici!$O95&gt;Pronostici!$P95,"1",IF(Pronostici!$O95=Pronostici!$P95,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N95" s="63">
+        <f>IF(Pronostici!$Q95&lt;&gt;"",UPPER(Pronostici!$Q95),IF(OR(Pronostici!$R95="",Pronostici!$S95=""),"",IF(Pronostici!$R95&gt;Pronostici!$S95,"1",IF(Pronostici!$R95=Pronostici!$S95,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="74">
+        <f>Partite!$A96</f>
+        <v/>
+      </c>
+      <c r="B96" s="30">
+        <f>Partite!$B96</f>
+        <v/>
+      </c>
+      <c r="C96" s="47">
+        <f>IF(Partite!$E96="","",Partite!$E96&amp;"  -  "&amp;Partite!$F96)</f>
+        <v/>
+      </c>
+      <c r="D96" s="27">
+        <f>IF(Partite!$K96&lt;&gt;"Giocata","",IF(AND(Pronostici!$F96&lt;&gt;"",Pronostici!$G96&lt;&gt;"",Pronostici!$F96=Partite!$G96,Pronostici!$G96=Partite!$H96),Config!$D$6,IF(AND($J96&lt;&gt;"",$J96=Partite!$I96),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E96" s="27">
+        <f>IF(Partite!$K96&lt;&gt;"Giocata","",IF(AND(Pronostici!$I96&lt;&gt;"",Pronostici!$J96&lt;&gt;"",Pronostici!$I96=Partite!$G96,Pronostici!$J96=Partite!$H96),Config!$D$6,IF(AND($K96&lt;&gt;"",$K96=Partite!$I96),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F96" s="27">
+        <f>IF(Partite!$K96&lt;&gt;"Giocata","",IF(AND(Pronostici!$L96&lt;&gt;"",Pronostici!$M96&lt;&gt;"",Pronostici!$L96=Partite!$G96,Pronostici!$M96=Partite!$H96),Config!$D$6,IF(AND($L96&lt;&gt;"",$L96=Partite!$I96),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G96" s="27">
+        <f>IF(Partite!$K96&lt;&gt;"Giocata","",IF(AND(Pronostici!$O96&lt;&gt;"",Pronostici!$P96&lt;&gt;"",Pronostici!$O96=Partite!$G96,Pronostici!$P96=Partite!$H96),Config!$D$6,IF(AND($M96&lt;&gt;"",$M96=Partite!$I96),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H96" s="27">
+        <f>IF(Partite!$K96&lt;&gt;"Giocata","",IF(AND(Pronostici!$R96&lt;&gt;"",Pronostici!$S96&lt;&gt;"",Pronostici!$R96=Partite!$G96,Pronostici!$S96=Partite!$H96),Config!$D$6,IF(AND($N96&lt;&gt;"",$N96=Partite!$I96),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J96" s="63">
+        <f>IF(Pronostici!$E96&lt;&gt;"",UPPER(Pronostici!$E96),IF(OR(Pronostici!$F96="",Pronostici!$G96=""),"",IF(Pronostici!$F96&gt;Pronostici!$G96,"1",IF(Pronostici!$F96=Pronostici!$G96,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K96" s="63">
+        <f>IF(Pronostici!$H96&lt;&gt;"",UPPER(Pronostici!$H96),IF(OR(Pronostici!$I96="",Pronostici!$J96=""),"",IF(Pronostici!$I96&gt;Pronostici!$J96,"1",IF(Pronostici!$I96=Pronostici!$J96,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L96" s="63">
+        <f>IF(Pronostici!$K96&lt;&gt;"",UPPER(Pronostici!$K96),IF(OR(Pronostici!$L96="",Pronostici!$M96=""),"",IF(Pronostici!$L96&gt;Pronostici!$M96,"1",IF(Pronostici!$L96=Pronostici!$M96,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M96" s="63">
+        <f>IF(Pronostici!$N96&lt;&gt;"",UPPER(Pronostici!$N96),IF(OR(Pronostici!$O96="",Pronostici!$P96=""),"",IF(Pronostici!$O96&gt;Pronostici!$P96,"1",IF(Pronostici!$O96=Pronostici!$P96,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N96" s="63">
+        <f>IF(Pronostici!$Q96&lt;&gt;"",UPPER(Pronostici!$Q96),IF(OR(Pronostici!$R96="",Pronostici!$S96=""),"",IF(Pronostici!$R96&gt;Pronostici!$S96,"1",IF(Pronostici!$R96=Pronostici!$S96,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="74">
+        <f>Partite!$A97</f>
+        <v/>
+      </c>
+      <c r="B97" s="30">
+        <f>Partite!$B97</f>
+        <v/>
+      </c>
+      <c r="C97" s="47">
+        <f>IF(Partite!$E97="","",Partite!$E97&amp;"  -  "&amp;Partite!$F97)</f>
+        <v/>
+      </c>
+      <c r="D97" s="27">
+        <f>IF(Partite!$K97&lt;&gt;"Giocata","",IF(AND(Pronostici!$F97&lt;&gt;"",Pronostici!$G97&lt;&gt;"",Pronostici!$F97=Partite!$G97,Pronostici!$G97=Partite!$H97),Config!$D$6,IF(AND($J97&lt;&gt;"",$J97=Partite!$I97),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E97" s="27">
+        <f>IF(Partite!$K97&lt;&gt;"Giocata","",IF(AND(Pronostici!$I97&lt;&gt;"",Pronostici!$J97&lt;&gt;"",Pronostici!$I97=Partite!$G97,Pronostici!$J97=Partite!$H97),Config!$D$6,IF(AND($K97&lt;&gt;"",$K97=Partite!$I97),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F97" s="27">
+        <f>IF(Partite!$K97&lt;&gt;"Giocata","",IF(AND(Pronostici!$L97&lt;&gt;"",Pronostici!$M97&lt;&gt;"",Pronostici!$L97=Partite!$G97,Pronostici!$M97=Partite!$H97),Config!$D$6,IF(AND($L97&lt;&gt;"",$L97=Partite!$I97),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G97" s="27">
+        <f>IF(Partite!$K97&lt;&gt;"Giocata","",IF(AND(Pronostici!$O97&lt;&gt;"",Pronostici!$P97&lt;&gt;"",Pronostici!$O97=Partite!$G97,Pronostici!$P97=Partite!$H97),Config!$D$6,IF(AND($M97&lt;&gt;"",$M97=Partite!$I97),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H97" s="27">
+        <f>IF(Partite!$K97&lt;&gt;"Giocata","",IF(AND(Pronostici!$R97&lt;&gt;"",Pronostici!$S97&lt;&gt;"",Pronostici!$R97=Partite!$G97,Pronostici!$S97=Partite!$H97),Config!$D$6,IF(AND($N97&lt;&gt;"",$N97=Partite!$I97),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J97" s="63">
+        <f>IF(Pronostici!$E97&lt;&gt;"",UPPER(Pronostici!$E97),IF(OR(Pronostici!$F97="",Pronostici!$G97=""),"",IF(Pronostici!$F97&gt;Pronostici!$G97,"1",IF(Pronostici!$F97=Pronostici!$G97,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K97" s="63">
+        <f>IF(Pronostici!$H97&lt;&gt;"",UPPER(Pronostici!$H97),IF(OR(Pronostici!$I97="",Pronostici!$J97=""),"",IF(Pronostici!$I97&gt;Pronostici!$J97,"1",IF(Pronostici!$I97=Pronostici!$J97,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L97" s="63">
+        <f>IF(Pronostici!$K97&lt;&gt;"",UPPER(Pronostici!$K97),IF(OR(Pronostici!$L97="",Pronostici!$M97=""),"",IF(Pronostici!$L97&gt;Pronostici!$M97,"1",IF(Pronostici!$L97=Pronostici!$M97,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M97" s="63">
+        <f>IF(Pronostici!$N97&lt;&gt;"",UPPER(Pronostici!$N97),IF(OR(Pronostici!$O97="",Pronostici!$P97=""),"",IF(Pronostici!$O97&gt;Pronostici!$P97,"1",IF(Pronostici!$O97=Pronostici!$P97,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N97" s="63">
+        <f>IF(Pronostici!$Q97&lt;&gt;"",UPPER(Pronostici!$Q97),IF(OR(Pronostici!$R97="",Pronostici!$S97=""),"",IF(Pronostici!$R97&gt;Pronostici!$S97,"1",IF(Pronostici!$R97=Pronostici!$S97,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="74">
+        <f>Partite!$A98</f>
+        <v/>
+      </c>
+      <c r="B98" s="30">
+        <f>Partite!$B98</f>
+        <v/>
+      </c>
+      <c r="C98" s="47">
+        <f>IF(Partite!$E98="","",Partite!$E98&amp;"  -  "&amp;Partite!$F98)</f>
+        <v/>
+      </c>
+      <c r="D98" s="27">
+        <f>IF(Partite!$K98&lt;&gt;"Giocata","",IF(AND(Pronostici!$F98&lt;&gt;"",Pronostici!$G98&lt;&gt;"",Pronostici!$F98=Partite!$G98,Pronostici!$G98=Partite!$H98),Config!$D$6,IF(AND($J98&lt;&gt;"",$J98=Partite!$I98),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E98" s="27">
+        <f>IF(Partite!$K98&lt;&gt;"Giocata","",IF(AND(Pronostici!$I98&lt;&gt;"",Pronostici!$J98&lt;&gt;"",Pronostici!$I98=Partite!$G98,Pronostici!$J98=Partite!$H98),Config!$D$6,IF(AND($K98&lt;&gt;"",$K98=Partite!$I98),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F98" s="27">
+        <f>IF(Partite!$K98&lt;&gt;"Giocata","",IF(AND(Pronostici!$L98&lt;&gt;"",Pronostici!$M98&lt;&gt;"",Pronostici!$L98=Partite!$G98,Pronostici!$M98=Partite!$H98),Config!$D$6,IF(AND($L98&lt;&gt;"",$L98=Partite!$I98),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G98" s="27">
+        <f>IF(Partite!$K98&lt;&gt;"Giocata","",IF(AND(Pronostici!$O98&lt;&gt;"",Pronostici!$P98&lt;&gt;"",Pronostici!$O98=Partite!$G98,Pronostici!$P98=Partite!$H98),Config!$D$6,IF(AND($M98&lt;&gt;"",$M98=Partite!$I98),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H98" s="27">
+        <f>IF(Partite!$K98&lt;&gt;"Giocata","",IF(AND(Pronostici!$R98&lt;&gt;"",Pronostici!$S98&lt;&gt;"",Pronostici!$R98=Partite!$G98,Pronostici!$S98=Partite!$H98),Config!$D$6,IF(AND($N98&lt;&gt;"",$N98=Partite!$I98),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J98" s="63">
+        <f>IF(Pronostici!$E98&lt;&gt;"",UPPER(Pronostici!$E98),IF(OR(Pronostici!$F98="",Pronostici!$G98=""),"",IF(Pronostici!$F98&gt;Pronostici!$G98,"1",IF(Pronostici!$F98=Pronostici!$G98,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K98" s="63">
+        <f>IF(Pronostici!$H98&lt;&gt;"",UPPER(Pronostici!$H98),IF(OR(Pronostici!$I98="",Pronostici!$J98=""),"",IF(Pronostici!$I98&gt;Pronostici!$J98,"1",IF(Pronostici!$I98=Pronostici!$J98,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L98" s="63">
+        <f>IF(Pronostici!$K98&lt;&gt;"",UPPER(Pronostici!$K98),IF(OR(Pronostici!$L98="",Pronostici!$M98=""),"",IF(Pronostici!$L98&gt;Pronostici!$M98,"1",IF(Pronostici!$L98=Pronostici!$M98,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M98" s="63">
+        <f>IF(Pronostici!$N98&lt;&gt;"",UPPER(Pronostici!$N98),IF(OR(Pronostici!$O98="",Pronostici!$P98=""),"",IF(Pronostici!$O98&gt;Pronostici!$P98,"1",IF(Pronostici!$O98=Pronostici!$P98,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N98" s="63">
+        <f>IF(Pronostici!$Q98&lt;&gt;"",UPPER(Pronostici!$Q98),IF(OR(Pronostici!$R98="",Pronostici!$S98=""),"",IF(Pronostici!$R98&gt;Pronostici!$S98,"1",IF(Pronostici!$R98=Pronostici!$S98,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="74">
+        <f>Partite!$A99</f>
+        <v/>
+      </c>
+      <c r="B99" s="30">
+        <f>Partite!$B99</f>
+        <v/>
+      </c>
+      <c r="C99" s="47">
+        <f>IF(Partite!$E99="","",Partite!$E99&amp;"  -  "&amp;Partite!$F99)</f>
+        <v/>
+      </c>
+      <c r="D99" s="27">
+        <f>IF(Partite!$K99&lt;&gt;"Giocata","",IF(AND(Pronostici!$F99&lt;&gt;"",Pronostici!$G99&lt;&gt;"",Pronostici!$F99=Partite!$G99,Pronostici!$G99=Partite!$H99),Config!$D$6,IF(AND($J99&lt;&gt;"",$J99=Partite!$I99),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E99" s="27">
+        <f>IF(Partite!$K99&lt;&gt;"Giocata","",IF(AND(Pronostici!$I99&lt;&gt;"",Pronostici!$J99&lt;&gt;"",Pronostici!$I99=Partite!$G99,Pronostici!$J99=Partite!$H99),Config!$D$6,IF(AND($K99&lt;&gt;"",$K99=Partite!$I99),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F99" s="27">
+        <f>IF(Partite!$K99&lt;&gt;"Giocata","",IF(AND(Pronostici!$L99&lt;&gt;"",Pronostici!$M99&lt;&gt;"",Pronostici!$L99=Partite!$G99,Pronostici!$M99=Partite!$H99),Config!$D$6,IF(AND($L99&lt;&gt;"",$L99=Partite!$I99),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G99" s="27">
+        <f>IF(Partite!$K99&lt;&gt;"Giocata","",IF(AND(Pronostici!$O99&lt;&gt;"",Pronostici!$P99&lt;&gt;"",Pronostici!$O99=Partite!$G99,Pronostici!$P99=Partite!$H99),Config!$D$6,IF(AND($M99&lt;&gt;"",$M99=Partite!$I99),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H99" s="27">
+        <f>IF(Partite!$K99&lt;&gt;"Giocata","",IF(AND(Pronostici!$R99&lt;&gt;"",Pronostici!$S99&lt;&gt;"",Pronostici!$R99=Partite!$G99,Pronostici!$S99=Partite!$H99),Config!$D$6,IF(AND($N99&lt;&gt;"",$N99=Partite!$I99),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J99" s="63">
+        <f>IF(Pronostici!$E99&lt;&gt;"",UPPER(Pronostici!$E99),IF(OR(Pronostici!$F99="",Pronostici!$G99=""),"",IF(Pronostici!$F99&gt;Pronostici!$G99,"1",IF(Pronostici!$F99=Pronostici!$G99,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K99" s="63">
+        <f>IF(Pronostici!$H99&lt;&gt;"",UPPER(Pronostici!$H99),IF(OR(Pronostici!$I99="",Pronostici!$J99=""),"",IF(Pronostici!$I99&gt;Pronostici!$J99,"1",IF(Pronostici!$I99=Pronostici!$J99,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L99" s="63">
+        <f>IF(Pronostici!$K99&lt;&gt;"",UPPER(Pronostici!$K99),IF(OR(Pronostici!$L99="",Pronostici!$M99=""),"",IF(Pronostici!$L99&gt;Pronostici!$M99,"1",IF(Pronostici!$L99=Pronostici!$M99,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M99" s="63">
+        <f>IF(Pronostici!$N99&lt;&gt;"",UPPER(Pronostici!$N99),IF(OR(Pronostici!$O99="",Pronostici!$P99=""),"",IF(Pronostici!$O99&gt;Pronostici!$P99,"1",IF(Pronostici!$O99=Pronostici!$P99,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N99" s="63">
+        <f>IF(Pronostici!$Q99&lt;&gt;"",UPPER(Pronostici!$Q99),IF(OR(Pronostici!$R99="",Pronostici!$S99=""),"",IF(Pronostici!$R99&gt;Pronostici!$S99,"1",IF(Pronostici!$R99=Pronostici!$S99,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="74">
+        <f>Partite!$A100</f>
+        <v/>
+      </c>
+      <c r="B100" s="30">
+        <f>Partite!$B100</f>
+        <v/>
+      </c>
+      <c r="C100" s="47">
+        <f>IF(Partite!$E100="","",Partite!$E100&amp;"  -  "&amp;Partite!$F100)</f>
+        <v/>
+      </c>
+      <c r="D100" s="27">
+        <f>IF(Partite!$K100&lt;&gt;"Giocata","",IF(AND(Pronostici!$F100&lt;&gt;"",Pronostici!$G100&lt;&gt;"",Pronostici!$F100=Partite!$G100,Pronostici!$G100=Partite!$H100),Config!$D$6,IF(AND($J100&lt;&gt;"",$J100=Partite!$I100),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E100" s="27">
+        <f>IF(Partite!$K100&lt;&gt;"Giocata","",IF(AND(Pronostici!$I100&lt;&gt;"",Pronostici!$J100&lt;&gt;"",Pronostici!$I100=Partite!$G100,Pronostici!$J100=Partite!$H100),Config!$D$6,IF(AND($K100&lt;&gt;"",$K100=Partite!$I100),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F100" s="27">
+        <f>IF(Partite!$K100&lt;&gt;"Giocata","",IF(AND(Pronostici!$L100&lt;&gt;"",Pronostici!$M100&lt;&gt;"",Pronostici!$L100=Partite!$G100,Pronostici!$M100=Partite!$H100),Config!$D$6,IF(AND($L100&lt;&gt;"",$L100=Partite!$I100),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G100" s="27">
+        <f>IF(Partite!$K100&lt;&gt;"Giocata","",IF(AND(Pronostici!$O100&lt;&gt;"",Pronostici!$P100&lt;&gt;"",Pronostici!$O100=Partite!$G100,Pronostici!$P100=Partite!$H100),Config!$D$6,IF(AND($M100&lt;&gt;"",$M100=Partite!$I100),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H100" s="27">
+        <f>IF(Partite!$K100&lt;&gt;"Giocata","",IF(AND(Pronostici!$R100&lt;&gt;"",Pronostici!$S100&lt;&gt;"",Pronostici!$R100=Partite!$G100,Pronostici!$S100=Partite!$H100),Config!$D$6,IF(AND($N100&lt;&gt;"",$N100=Partite!$I100),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J100" s="63">
+        <f>IF(Pronostici!$E100&lt;&gt;"",UPPER(Pronostici!$E100),IF(OR(Pronostici!$F100="",Pronostici!$G100=""),"",IF(Pronostici!$F100&gt;Pronostici!$G100,"1",IF(Pronostici!$F100=Pronostici!$G100,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K100" s="63">
+        <f>IF(Pronostici!$H100&lt;&gt;"",UPPER(Pronostici!$H100),IF(OR(Pronostici!$I100="",Pronostici!$J100=""),"",IF(Pronostici!$I100&gt;Pronostici!$J100,"1",IF(Pronostici!$I100=Pronostici!$J100,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L100" s="63">
+        <f>IF(Pronostici!$K100&lt;&gt;"",UPPER(Pronostici!$K100),IF(OR(Pronostici!$L100="",Pronostici!$M100=""),"",IF(Pronostici!$L100&gt;Pronostici!$M100,"1",IF(Pronostici!$L100=Pronostici!$M100,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M100" s="63">
+        <f>IF(Pronostici!$N100&lt;&gt;"",UPPER(Pronostici!$N100),IF(OR(Pronostici!$O100="",Pronostici!$P100=""),"",IF(Pronostici!$O100&gt;Pronostici!$P100,"1",IF(Pronostici!$O100=Pronostici!$P100,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N100" s="63">
+        <f>IF(Pronostici!$Q100&lt;&gt;"",UPPER(Pronostici!$Q100),IF(OR(Pronostici!$R100="",Pronostici!$S100=""),"",IF(Pronostici!$R100&gt;Pronostici!$S100,"1",IF(Pronostici!$R100=Pronostici!$S100,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="74">
+        <f>Partite!$A101</f>
+        <v/>
+      </c>
+      <c r="B101" s="30">
+        <f>Partite!$B101</f>
+        <v/>
+      </c>
+      <c r="C101" s="47">
+        <f>IF(Partite!$E101="","",Partite!$E101&amp;"  -  "&amp;Partite!$F101)</f>
+        <v/>
+      </c>
+      <c r="D101" s="27">
+        <f>IF(Partite!$K101&lt;&gt;"Giocata","",IF(AND(Pronostici!$F101&lt;&gt;"",Pronostici!$G101&lt;&gt;"",Pronostici!$F101=Partite!$G101,Pronostici!$G101=Partite!$H101),Config!$D$6,IF(AND($J101&lt;&gt;"",$J101=Partite!$I101),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E101" s="27">
+        <f>IF(Partite!$K101&lt;&gt;"Giocata","",IF(AND(Pronostici!$I101&lt;&gt;"",Pronostici!$J101&lt;&gt;"",Pronostici!$I101=Partite!$G101,Pronostici!$J101=Partite!$H101),Config!$D$6,IF(AND($K101&lt;&gt;"",$K101=Partite!$I101),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F101" s="27">
+        <f>IF(Partite!$K101&lt;&gt;"Giocata","",IF(AND(Pronostici!$L101&lt;&gt;"",Pronostici!$M101&lt;&gt;"",Pronostici!$L101=Partite!$G101,Pronostici!$M101=Partite!$H101),Config!$D$6,IF(AND($L101&lt;&gt;"",$L101=Partite!$I101),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G101" s="27">
+        <f>IF(Partite!$K101&lt;&gt;"Giocata","",IF(AND(Pronostici!$O101&lt;&gt;"",Pronostici!$P101&lt;&gt;"",Pronostici!$O101=Partite!$G101,Pronostici!$P101=Partite!$H101),Config!$D$6,IF(AND($M101&lt;&gt;"",$M101=Partite!$I101),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H101" s="27">
+        <f>IF(Partite!$K101&lt;&gt;"Giocata","",IF(AND(Pronostici!$R101&lt;&gt;"",Pronostici!$S101&lt;&gt;"",Pronostici!$R101=Partite!$G101,Pronostici!$S101=Partite!$H101),Config!$D$6,IF(AND($N101&lt;&gt;"",$N101=Partite!$I101),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J101" s="63">
+        <f>IF(Pronostici!$E101&lt;&gt;"",UPPER(Pronostici!$E101),IF(OR(Pronostici!$F101="",Pronostici!$G101=""),"",IF(Pronostici!$F101&gt;Pronostici!$G101,"1",IF(Pronostici!$F101=Pronostici!$G101,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K101" s="63">
+        <f>IF(Pronostici!$H101&lt;&gt;"",UPPER(Pronostici!$H101),IF(OR(Pronostici!$I101="",Pronostici!$J101=""),"",IF(Pronostici!$I101&gt;Pronostici!$J101,"1",IF(Pronostici!$I101=Pronostici!$J101,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L101" s="63">
+        <f>IF(Pronostici!$K101&lt;&gt;"",UPPER(Pronostici!$K101),IF(OR(Pronostici!$L101="",Pronostici!$M101=""),"",IF(Pronostici!$L101&gt;Pronostici!$M101,"1",IF(Pronostici!$L101=Pronostici!$M101,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M101" s="63">
+        <f>IF(Pronostici!$N101&lt;&gt;"",UPPER(Pronostici!$N101),IF(OR(Pronostici!$O101="",Pronostici!$P101=""),"",IF(Pronostici!$O101&gt;Pronostici!$P101,"1",IF(Pronostici!$O101=Pronostici!$P101,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N101" s="63">
+        <f>IF(Pronostici!$Q101&lt;&gt;"",UPPER(Pronostici!$Q101),IF(OR(Pronostici!$R101="",Pronostici!$S101=""),"",IF(Pronostici!$R101&gt;Pronostici!$S101,"1",IF(Pronostici!$R101=Pronostici!$S101,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="74">
+        <f>Partite!$A102</f>
+        <v/>
+      </c>
+      <c r="B102" s="30">
+        <f>Partite!$B102</f>
+        <v/>
+      </c>
+      <c r="C102" s="47">
+        <f>IF(Partite!$E102="","",Partite!$E102&amp;"  -  "&amp;Partite!$F102)</f>
+        <v/>
+      </c>
+      <c r="D102" s="27">
+        <f>IF(Partite!$K102&lt;&gt;"Giocata","",IF(AND(Pronostici!$F102&lt;&gt;"",Pronostici!$G102&lt;&gt;"",Pronostici!$F102=Partite!$G102,Pronostici!$G102=Partite!$H102),Config!$D$6,IF(AND($J102&lt;&gt;"",$J102=Partite!$I102),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="E102" s="27">
+        <f>IF(Partite!$K102&lt;&gt;"Giocata","",IF(AND(Pronostici!$I102&lt;&gt;"",Pronostici!$J102&lt;&gt;"",Pronostici!$I102=Partite!$G102,Pronostici!$J102=Partite!$H102),Config!$D$6,IF(AND($K102&lt;&gt;"",$K102=Partite!$I102),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="F102" s="27">
+        <f>IF(Partite!$K102&lt;&gt;"Giocata","",IF(AND(Pronostici!$L102&lt;&gt;"",Pronostici!$M102&lt;&gt;"",Pronostici!$L102=Partite!$G102,Pronostici!$M102=Partite!$H102),Config!$D$6,IF(AND($L102&lt;&gt;"",$L102=Partite!$I102),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="G102" s="27">
+        <f>IF(Partite!$K102&lt;&gt;"Giocata","",IF(AND(Pronostici!$O102&lt;&gt;"",Pronostici!$P102&lt;&gt;"",Pronostici!$O102=Partite!$G102,Pronostici!$P102=Partite!$H102),Config!$D$6,IF(AND($M102&lt;&gt;"",$M102=Partite!$I102),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="H102" s="27">
+        <f>IF(Partite!$K102&lt;&gt;"Giocata","",IF(AND(Pronostici!$R102&lt;&gt;"",Pronostici!$S102&lt;&gt;"",Pronostici!$R102=Partite!$G102,Pronostici!$S102=Partite!$H102),Config!$D$6,IF(AND($N102&lt;&gt;"",$N102=Partite!$I102),Config!$D$7,Config!$D$8)))</f>
+        <v/>
+      </c>
+      <c r="J102" s="63">
+        <f>IF(Pronostici!$E102&lt;&gt;"",UPPER(Pronostici!$E102),IF(OR(Pronostici!$F102="",Pronostici!$G102=""),"",IF(Pronostici!$F102&gt;Pronostici!$G102,"1",IF(Pronostici!$F102=Pronostici!$G102,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="K102" s="63">
+        <f>IF(Pronostici!$H102&lt;&gt;"",UPPER(Pronostici!$H102),IF(OR(Pronostici!$I102="",Pronostici!$J102=""),"",IF(Pronostici!$I102&gt;Pronostici!$J102,"1",IF(Pronostici!$I102=Pronostici!$J102,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="L102" s="63">
+        <f>IF(Pronostici!$K102&lt;&gt;"",UPPER(Pronostici!$K102),IF(OR(Pronostici!$L102="",Pronostici!$M102=""),"",IF(Pronostici!$L102&gt;Pronostici!$M102,"1",IF(Pronostici!$L102=Pronostici!$M102,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="M102" s="63">
+        <f>IF(Pronostici!$N102&lt;&gt;"",UPPER(Pronostici!$N102),IF(OR(Pronostici!$O102="",Pronostici!$P102=""),"",IF(Pronostici!$O102&gt;Pronostici!$P102,"1",IF(Pronostici!$O102=Pronostici!$P102,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="N102" s="63">
+        <f>IF(Pronostici!$Q102&lt;&gt;"",UPPER(Pronostici!$Q102),IF(OR(Pronostici!$R102="",Pronostici!$S102=""),"",IF(Pronostici!$R102&gt;Pronostici!$S102,"1",IF(Pronostici!$R102=Pronostici!$S102,"X","2"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D92">
+  <conditionalFormatting sqref="D3:D102">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -18363,7 +19734,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E92">
+  <conditionalFormatting sqref="E3:E102">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -18371,7 +19742,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F92">
+  <conditionalFormatting sqref="F3:F102">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -18379,7 +19750,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G92">
+  <conditionalFormatting sqref="G3:G102">
     <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
@@ -18387,7 +19758,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H92">
+  <conditionalFormatting sqref="H3:H102">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento automatico del 31/10/2026 alle 15:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -13559,21 +13559,61 @@
         <f>IF(Partite!$F83="","",Partite!$F83)</f>
         <v/>
       </c>
-      <c r="E83" s="71" t="n"/>
-      <c r="F83" s="71" t="n"/>
-      <c r="G83" s="71" t="n"/>
-      <c r="H83" s="71" t="n"/>
-      <c r="I83" s="71" t="n"/>
-      <c r="J83" s="71" t="n"/>
-      <c r="K83" s="71" t="n"/>
-      <c r="L83" s="71" t="n"/>
-      <c r="M83" s="71" t="n"/>
-      <c r="N83" s="71" t="n"/>
-      <c r="O83" s="71" t="n"/>
-      <c r="P83" s="71" t="n"/>
-      <c r="Q83" s="71" t="n"/>
-      <c r="R83" s="71" t="n"/>
-      <c r="S83" s="71" t="n"/>
+      <c r="E83" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F83" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G83" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I83" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J83" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K83" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L83" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M83" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O83" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P83" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q83" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R83" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S83" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="69">
@@ -13592,21 +13632,61 @@
         <f>IF(Partite!$F84="","",Partite!$F84)</f>
         <v/>
       </c>
-      <c r="E84" s="71" t="n"/>
-      <c r="F84" s="71" t="n"/>
-      <c r="G84" s="71" t="n"/>
-      <c r="H84" s="71" t="n"/>
-      <c r="I84" s="71" t="n"/>
-      <c r="J84" s="71" t="n"/>
-      <c r="K84" s="71" t="n"/>
-      <c r="L84" s="71" t="n"/>
-      <c r="M84" s="71" t="n"/>
-      <c r="N84" s="71" t="n"/>
-      <c r="O84" s="71" t="n"/>
-      <c r="P84" s="71" t="n"/>
-      <c r="Q84" s="71" t="n"/>
-      <c r="R84" s="71" t="n"/>
-      <c r="S84" s="71" t="n"/>
+      <c r="E84" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F84" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H84" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I84" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K84" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L84" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M84" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N84" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O84" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q84" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R84" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S84" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="69">
@@ -13625,21 +13705,61 @@
         <f>IF(Partite!$F85="","",Partite!$F85)</f>
         <v/>
       </c>
-      <c r="E85" s="71" t="n"/>
-      <c r="F85" s="71" t="n"/>
-      <c r="G85" s="71" t="n"/>
-      <c r="H85" s="71" t="n"/>
-      <c r="I85" s="71" t="n"/>
-      <c r="J85" s="71" t="n"/>
-      <c r="K85" s="71" t="n"/>
-      <c r="L85" s="71" t="n"/>
-      <c r="M85" s="71" t="n"/>
-      <c r="N85" s="71" t="n"/>
-      <c r="O85" s="71" t="n"/>
-      <c r="P85" s="71" t="n"/>
-      <c r="Q85" s="71" t="n"/>
-      <c r="R85" s="71" t="n"/>
-      <c r="S85" s="71" t="n"/>
+      <c r="E85" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F85" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I85" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J85" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L85" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M85" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N85" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O85" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P85" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q85" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R85" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S85" s="71" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="69">
@@ -13658,21 +13778,61 @@
         <f>IF(Partite!$F86="","",Partite!$F86)</f>
         <v/>
       </c>
-      <c r="E86" s="71" t="n"/>
-      <c r="F86" s="71" t="n"/>
-      <c r="G86" s="71" t="n"/>
-      <c r="H86" s="71" t="n"/>
-      <c r="I86" s="71" t="n"/>
-      <c r="J86" s="71" t="n"/>
-      <c r="K86" s="71" t="n"/>
-      <c r="L86" s="71" t="n"/>
-      <c r="M86" s="71" t="n"/>
-      <c r="N86" s="71" t="n"/>
-      <c r="O86" s="71" t="n"/>
-      <c r="P86" s="71" t="n"/>
-      <c r="Q86" s="71" t="n"/>
-      <c r="R86" s="71" t="n"/>
-      <c r="S86" s="71" t="n"/>
+      <c r="E86" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F86" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I86" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J86" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K86" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L86" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M86" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O86" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P86" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R86" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="S86" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="69">
@@ -13691,21 +13851,61 @@
         <f>IF(Partite!$F87="","",Partite!$F87)</f>
         <v/>
       </c>
-      <c r="E87" s="71" t="n"/>
-      <c r="F87" s="71" t="n"/>
-      <c r="G87" s="71" t="n"/>
-      <c r="H87" s="71" t="n"/>
-      <c r="I87" s="71" t="n"/>
-      <c r="J87" s="71" t="n"/>
-      <c r="K87" s="71" t="n"/>
-      <c r="L87" s="71" t="n"/>
-      <c r="M87" s="71" t="n"/>
-      <c r="N87" s="71" t="n"/>
-      <c r="O87" s="71" t="n"/>
-      <c r="P87" s="71" t="n"/>
-      <c r="Q87" s="71" t="n"/>
-      <c r="R87" s="71" t="n"/>
-      <c r="S87" s="71" t="n"/>
+      <c r="E87" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F87" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G87" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I87" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J87" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L87" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M87" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N87" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O87" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P87" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q87" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R87" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S87" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="69">
@@ -13724,21 +13924,61 @@
         <f>IF(Partite!$F88="","",Partite!$F88)</f>
         <v/>
       </c>
-      <c r="E88" s="71" t="n"/>
-      <c r="F88" s="71" t="n"/>
-      <c r="G88" s="71" t="n"/>
-      <c r="H88" s="71" t="n"/>
-      <c r="I88" s="71" t="n"/>
-      <c r="J88" s="71" t="n"/>
-      <c r="K88" s="71" t="n"/>
-      <c r="L88" s="71" t="n"/>
-      <c r="M88" s="71" t="n"/>
-      <c r="N88" s="71" t="n"/>
-      <c r="O88" s="71" t="n"/>
-      <c r="P88" s="71" t="n"/>
-      <c r="Q88" s="71" t="n"/>
-      <c r="R88" s="71" t="n"/>
-      <c r="S88" s="71" t="n"/>
+      <c r="E88" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F88" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G88" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H88" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I88" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J88" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K88" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L88" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M88" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O88" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P88" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R88" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S88" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="69">
@@ -13757,21 +13997,61 @@
         <f>IF(Partite!$F89="","",Partite!$F89)</f>
         <v/>
       </c>
-      <c r="E89" s="71" t="n"/>
-      <c r="F89" s="71" t="n"/>
-      <c r="G89" s="71" t="n"/>
-      <c r="H89" s="71" t="n"/>
-      <c r="I89" s="71" t="n"/>
-      <c r="J89" s="71" t="n"/>
-      <c r="K89" s="71" t="n"/>
-      <c r="L89" s="71" t="n"/>
-      <c r="M89" s="71" t="n"/>
-      <c r="N89" s="71" t="n"/>
-      <c r="O89" s="71" t="n"/>
-      <c r="P89" s="71" t="n"/>
-      <c r="Q89" s="71" t="n"/>
-      <c r="R89" s="71" t="n"/>
-      <c r="S89" s="71" t="n"/>
+      <c r="E89" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F89" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I89" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K89" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L89" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M89" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N89" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O89" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P89" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q89" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R89" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S89" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="69">
@@ -13790,21 +14070,61 @@
         <f>IF(Partite!$F90="","",Partite!$F90)</f>
         <v/>
       </c>
-      <c r="E90" s="71" t="n"/>
-      <c r="F90" s="71" t="n"/>
-      <c r="G90" s="71" t="n"/>
-      <c r="H90" s="71" t="n"/>
-      <c r="I90" s="71" t="n"/>
-      <c r="J90" s="71" t="n"/>
-      <c r="K90" s="71" t="n"/>
-      <c r="L90" s="71" t="n"/>
-      <c r="M90" s="71" t="n"/>
-      <c r="N90" s="71" t="n"/>
-      <c r="O90" s="71" t="n"/>
-      <c r="P90" s="71" t="n"/>
-      <c r="Q90" s="71" t="n"/>
-      <c r="R90" s="71" t="n"/>
-      <c r="S90" s="71" t="n"/>
+      <c r="E90" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F90" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H90" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I90" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J90" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L90" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="N90" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O90" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q90" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R90" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="S90" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="69">
@@ -13823,21 +14143,61 @@
         <f>IF(Partite!$F91="","",Partite!$F91)</f>
         <v/>
       </c>
-      <c r="E91" s="71" t="n"/>
-      <c r="F91" s="71" t="n"/>
-      <c r="G91" s="71" t="n"/>
-      <c r="H91" s="71" t="n"/>
-      <c r="I91" s="71" t="n"/>
-      <c r="J91" s="71" t="n"/>
-      <c r="K91" s="71" t="n"/>
-      <c r="L91" s="71" t="n"/>
-      <c r="M91" s="71" t="n"/>
-      <c r="N91" s="71" t="n"/>
-      <c r="O91" s="71" t="n"/>
-      <c r="P91" s="71" t="n"/>
-      <c r="Q91" s="71" t="n"/>
-      <c r="R91" s="71" t="n"/>
-      <c r="S91" s="71" t="n"/>
+      <c r="E91" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H91" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J91" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="K91" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N91" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O91" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P91" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q91" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R91" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="S91" s="71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="69">
@@ -13856,21 +14216,61 @@
         <f>IF(Partite!$F92="","",Partite!$F92)</f>
         <v/>
       </c>
-      <c r="E92" s="71" t="n"/>
-      <c r="F92" s="71" t="n"/>
-      <c r="G92" s="71" t="n"/>
-      <c r="H92" s="71" t="n"/>
-      <c r="I92" s="71" t="n"/>
-      <c r="J92" s="71" t="n"/>
-      <c r="K92" s="71" t="n"/>
-      <c r="L92" s="71" t="n"/>
-      <c r="M92" s="71" t="n"/>
-      <c r="N92" s="71" t="n"/>
-      <c r="O92" s="71" t="n"/>
-      <c r="P92" s="71" t="n"/>
-      <c r="Q92" s="71" t="n"/>
-      <c r="R92" s="71" t="n"/>
-      <c r="S92" s="71" t="n"/>
+      <c r="E92" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F92" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="G92" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I92" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K92" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L92" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M92" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O92" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P92" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R92" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="S92" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="74">

</xml_diff>

<commit_message>
Aggiornamento automatico del 31/10/2026 alle 17:04
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6667,8 +6667,12 @@
           <t>Monza</t>
         </is>
       </c>
-      <c r="G83" s="71" t="n"/>
-      <c r="H83" s="71" t="n"/>
+      <c r="G83" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H83" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I83" s="72">
         <f>IF(OR($G83="",$H83=""),"",IF($G83&gt;$H83,"1",IF($G83=$H83,"X","2")))</f>
         <v/>

</xml_diff>